<commit_message>
chore(SET-05): Redis 제거 및 Postgres 기반 캐싱으로 전환
개발설계서 v1.7 반영(구 v1.6은 /docs/archive/로 이동). SET-05(Upstash
Redis 생성) 취소 처리(코드 결번 유지), SET-09 선행TASK에서 SET-05 제거,
DATA-15를 캐시 정리 배치 구현(Postgres)으로 재정의. WBS.xlsx에 DATA-03
캐시 테이블 2종(chat_answer_cache, puuid_cache) 추가 및 API-11/CHAT-08
설명을 Postgres 기반으로 갱신. CLAUDE.md v1.5, 진행현황.md 동기화.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TFT_Hideout_WBS.xlsx
+++ b/TFT_Hideout_WBS.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'WBS'!$A$1:$K$94</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'WBS'!$A$1:$K$95</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K94"/>
+  <dimension ref="A1:K95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -823,17 +823,17 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Upstash Redis 생성</t>
+          <t>(취소) Upstash Redis 생성</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>무료 Redis 인스턴스 생성 및 연결 정보 발급</t>
+          <t>개발설계서 v1.7 반영 — 캐싱을 Postgres 테이블(chat_answer_cache, puuid_cache)로 대체하기로 결정해 별도 Redis 인프라 불필요. 코드는 결번으로 유지, 아래 완료기준/테스트요구사항 해당없음</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>필수</t>
+          <t>취소</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -843,17 +843,17 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>설계서 2장</t>
+          <t>개발설계서 v1.7 3장·4.6절(Redis 제거 결정, 2026-07-31 PM 결정)</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>연결 테스트 성공</t>
+          <t>해당 없음(취소)</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>스모크 테스트: Redis PING 응답 확인</t>
+          <t>해당 없음(취소)</t>
         </is>
       </c>
     </row>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>SET-04,SET-05,SET-06,SET-07,SET-08</t>
+          <t>SET-04,SET-06,SET-07,SET-08</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>match_analyses, chat_logs, link_click_events, account_link_events, patch_detection_runs, ragas_eval_results 마이그레이션 작성</t>
+          <t>match_analyses, chat_logs, link_click_events, account_link_events, patch_detection_runs, ragas_eval_results, chat_answer_cache, puuid_cache 마이그레이션 작성(캐시 테이블 2종은 v1.7 신설 — Redis 대체)</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -1589,12 +1589,12 @@
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>마이그레이션 적용 확인</t>
+          <t>마이그레이션 적용 확인(8개 테이블)</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>pytest: 6개 로그/분석 테이블 컬럼 존재 및 nullable 정책 assert</t>
+          <t>pytest: 8개 로그/분석/캐시 테이블 컬럼 존재 및 nullable 정책 assert</t>
         </is>
       </c>
     </row>
@@ -2248,12 +2248,12 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>캐시 무효화 로직 구현</t>
+          <t>캐시 정리 배치 구현</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>배치 완료 후 Redis 이전 패치 캐시 키 무효화</t>
+          <t>배치 완료 후 chat_answer_cache에서 이전 patch_version 캐시 행 삭제(Postgres DELETE, v1.7 — 이전 Redis 키 무효화 대체)</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -2263,22 +2263,22 @@
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>DATA-13,SET-05</t>
+          <t>DATA-13,DATA-03</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.3·4.6</t>
+          <t>설계서 v1.7 4.3·4.6</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>배치 완료 후 캐시 키 삭제 확인</t>
+          <t>배치 완료 후 이전 patch_version 캐시 행 삭제 확인</t>
         </is>
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>pytest: 배치 완료 이벤트 발생 시 이전 패치 관련 Redis 키가 삭제되는지 확인</t>
+          <t>pytest: 배치 완료 이벤트 발생 시 chat_answer_cache에서 이전 patch_version 행이 삭제되는지 확인</t>
         </is>
       </c>
     </row>
@@ -2880,7 +2880,7 @@
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>Riot ID→PUUID 변환, TTL 1시간 캐시</t>
+          <t>Riot ID→PUUID 변환, TTL 1시간 캐시(Postgres puuid_cache 테이블, v1.7)</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
@@ -2895,7 +2895,7 @@
       </c>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>PRD 9-1·설계서4.5</t>
+          <t>PRD 9-1·설계서v1.7 4.5</t>
         </is>
       </c>
       <c r="J42" s="3" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>첫턴 질문 Redis 캐시, 후속턴 캐시제외, 패치갱신시 무효화</t>
+          <t>첫턴 질문 Postgres(chat_answer_cache) 캐시, 후속턴 캐시제외, 패치갱신시 무효화</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
@@ -3522,7 +3522,7 @@
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>PRD 9-6·설계서4.4·4.6</t>
+          <t>PRD 9-6·설계서v1.7 4.4·4.6</t>
         </is>
       </c>
       <c r="J53" s="3" t="inlineStr">
@@ -5873,8 +5873,65 @@
         </is>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" s="6" t="inlineStr">
+        <is>
+          <t>REL-05</t>
+        </is>
+      </c>
+      <c r="B95" s="6" t="inlineStr">
+        <is>
+          <t>배포릴리즈</t>
+        </is>
+      </c>
+      <c r="C95" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>포트폴리오 공개 전환 준비 체크리스트</t>
+        </is>
+      </c>
+      <c r="F95" s="3" t="inlineStr">
+        <is>
+          <t>저장소를 private에서 public으로 전환하기 전 확인·조치한다: (1) gitleaks 등으로 커밋 히스토리 전체에서 시크릿·API 키 잔존 여부 스캔 (2) 테스트 fixture 전수 조사 — 실제 Riot ID/PUUID/닉네임/매치 데이터가 아닌 합성 데이터로만 구성됐는지 확인, 실데이터가 섞여 있으면 fixture 재작성 후 필요시 git 히스토리 정리 (3) README에 'Riot Games와 무관한 비공식 팬 프로젝트' 디스클레이머 추가 (4) 라이브 배포 URL을 README/공개 자료에 노출할지 결정 (5) 노출하기로 하면 챗봇/전적조회 진입점에 Cloudflare Turnstile 등 경량 봇 방지 적용 검토. 무료 호스팅 비용에는 영향 없음(저장소 공개 여부와 인프라 비용은 무관)</t>
+        </is>
+      </c>
+      <c r="G95" s="6" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H95" s="3" t="inlineStr">
+        <is>
+          <t>REL-04</t>
+        </is>
+      </c>
+      <c r="I95" s="3" t="inlineStr">
+        <is>
+          <t>PM 결정사항(2026-07-30 대화), policies.md 11번</t>
+        </is>
+      </c>
+      <c r="J95" s="3" t="inlineStr">
+        <is>
+          <t>체크리스트 5개 항목 모두 확인·조치 완료 및 PM 승인 후 저장소 visibility를 public으로 변경</t>
+        </is>
+      </c>
+      <c r="K95" s="3" t="inlineStr">
+        <is>
+          <t>정량 검증: gitleaks(또는 동급 도구) 스캔 결과 시크릿 탐지 0건, 전체 fixture 파일에서 실제 Riot ID 패턴(게임명#태그)·PUUID 패턴 검색 결과 0건</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K94"/>
+  <autoFilter ref="A1:K95"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5922,7 +5979,7 @@
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -6053,7 +6110,7 @@
       </c>
       <c r="B11" s="8" t="inlineStr"/>
       <c r="C11" s="8" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(API-01): FastAPI 프로젝트 스캐폴딩
catalog/chat/analysis/kpi 4개 APIRouter로 구조화(kpi는 SET-11 취소에
따른 자체 KPI 대시보드 백엔드용, CLAUDE.md v1.7 반영). 각 라우터는
현재 placeholder 루트 엔드포인트만 가지고 있고, 실제 엔드포인트는
API-02~06/09/11~14, KPI-01에서 채워질 예정.

pytest: 4개 라우터 마운트 확인(각 placeholder 응답 200). WBS API-01
TASK 설명/테스트 요구사항을 3개→4개 라우터 기준으로 갱신.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TFT_Hideout_WBS.xlsx
+++ b/TFT_Hideout_WBS.xlsx
@@ -2310,7 +2310,7 @@
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>단일 앱 + catalog/chat/analysis 라우터 구조, 헬스체크 엔드포인트</t>
+          <t>단일 앱 + catalog/chat/analysis/kpi 4개 라우터 구조(kpi는 SET-11 취소로 Metabase 대신 자체 KPI 대시보드 백엔드용으로 v1.7에서 추가), 헬스체크 엔드포인트</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
-          <t>pytest+FastAPI TestClient: /health 200 및 3개 라우터 마운트 확인</t>
+          <t>pytest+FastAPI TestClient: /health 200 및 4개 라우터(catalog/chat/analysis/kpi) 마운트 확인</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(SET-12): SET-12 취소 처리(PM 승인)
Figma MCP 커넥터가 세션에 연결되어 있지 않아 DoD(get_design_context
호출 성공)를 검증할 수 없었고, PM 결정으로 Figma를 사용하지 않기로
함. 이후 FE-* 작업은 design-tokens.md + 화면설계서만 참조.
FE-01 선행TASK에서 SET-12 제거.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TFT_Hideout_WBS.xlsx
+++ b/TFT_Hideout_WBS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="WBS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="요약" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'WBS'!$A$1:$K$95</definedName>
@@ -1222,17 +1222,17 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Figma 연동 및 프론트엔드 디자인 스킬 활성화</t>
+          <t>(취소) Figma 연동 및 프론트엔드 디자인 스킬 활성화</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Claude Code에 Figma MCP 커넥터 및 화면설계 관련 스킬 연동, 디자인가이드 v1.0·Figma "TFT_Hideout" 파일을 FE 작업 참조 소스로 등록</t>
+          <t>Claude Code 세션에 Figma MCP 커넥터가 연결되어 있지 않아 DoD(get_design_context 호출 성공)를 검증할 수 없었고, PM 결정으로 Figma MCP를 사용하지 않기로 함. 이후 FE-* 작업은 design-tokens.md + 화면설계서만을 참조 소스로 사용(CLAUDE.md 6장). 코드는 결번으로 유지</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>필수</t>
+          <t>취소</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
@@ -1242,17 +1242,17 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>디자인가이드 v1.0</t>
+          <t>PM 결정 2026-08-04</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>Figma MCP 호출 테스트 성공, FE 작업 시 디자인가이드 참조 확인</t>
+          <t>해당 없음(취소)</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>스모크 테스트: Figma MCP get_design_context 1회 호출 성공</t>
+          <t>해당 없음(취소)</t>
         </is>
       </c>
     </row>
@@ -4258,7 +4258,7 @@
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>SET-07,SET-12</t>
+          <t>SET-07</t>
         </is>
       </c>
       <c r="I66" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs(SET-10): SET-10 분리 — Groq/HF만 남기고 Riot은 SET-16 신설
PM 결정: 사후 패인 분석만 Riot API 키가 필요하고 카탈로그(op.gg)
쪽은 무관하다는 판단에 따라 SET-10을 Groq·HF 키 검증으로 재정의하고
(2026-08-03에 이미 200 확인, PM확인대기) Riot Personal Key는
SET-16으로 분리(진행중, 키 재발급 대기). DATA-05·DATA-06 선행TASK
제거로 즉시 착수 가능, API-11만 SET-16 의존으로 변경. WBS.xlsx에
SET-16 신규 삽입(전체 96개 TASK). 진행현황.md 반영은 이전 커밋에
포함됨.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TFT_Hideout_WBS.xlsx
+++ b/TFT_Hideout_WBS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="WBS" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="요약" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'WBS'!$A$1:$K$95</definedName>
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K96"/>
+  <dimension ref="A1:K97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1113,7 +1113,7 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Groq API 키, Hugging Face Inference API 키, Riot Personal Key 발급, op.gg MCP 연결 확인</t>
+          <t>Groq API 키, Hugging Face Inference API 키 발급 및 검증(Riot·op.gg는 SET-16/DATA-05로 분리, 2026-08-04 PM 결정)</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1133,12 +1133,12 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>4개 키 모두 1회 테스트 호출 성공</t>
+          <t>2개 키 모두 1회 테스트 호출 성공</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>스모크 테스트: Groq/HF/Riot/op.gg MCP 4개 API 각 1회 실호출 성공</t>
+          <t>스모크 테스트: Groq/HF 2개 API 각 1회 실호출 성공</t>
         </is>
       </c>
     </row>
@@ -1428,66 +1428,66 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>DATA-01</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>코딩</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>데이터파이프라인</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>공통(전 화면)</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>DB 스키마 설계-정적 테이블</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>patches/champions/traits/champion_traits/items/augments 마이그레이션 작성</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>필수</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>SET-04</t>
-        </is>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>설계서 5.1</t>
-        </is>
-      </c>
-      <c r="J17" s="3" t="inlineStr">
-        <is>
-          <t>마이그레이션 적용 후 테이블 생성 확인</t>
-        </is>
-      </c>
-      <c r="K17" s="3" t="inlineStr">
-        <is>
-          <t>pytest: 마이그레이션 적용 후 6개 테이블 컬럼/타입이 설계서 5.1과 일치하는지 assert</t>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SET-16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>시스템설정</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Riot Personal Key 발급 및 검증</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Riot Games Developer Portal에서 Personal API Key 발급, Match-V1/Account-V1 실호출 검증(SET-10에서 분리, 2026-08-04 PM 결정 — op.gg는 Riot 키 불필요)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>필수</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>PRD 9-1·11장</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Riot API 1회 테스트 호출 성공(200)</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>스모크 테스트: Riot Match-V1/Account-V1 API 1회 실호출 성공</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>DATA-02</t>
+          <t>DATA-01</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -1502,17 +1502,17 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>티어리스트·조합상세·아이템빌드</t>
+          <t>공통(전 화면)</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>DB 스키마 설계-메타조합 테이블</t>
+          <t>DB 스키마 설계-정적 테이블</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>comps/comp_champions/comp_augments/champion_item_builds 마이그레이션 작성</t>
+          <t>patches/champions/traits/champion_traits/items/augments 마이그레이션 작성</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1522,7 +1522,7 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>DATA-01</t>
+          <t>SET-04</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
@@ -1532,19 +1532,19 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>마이그레이션 적용 및 FK 제약 확인</t>
+          <t>마이그레이션 적용 후 테이블 생성 확인</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>pytest: comp_champions/comp_augments FK 제약 위반 시 IntegrityError 발생 확인</t>
+          <t>pytest: 마이그레이션 적용 후 6개 테이블 컬럼/타입이 설계서 5.1과 일치하는지 assert</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>DATA-03</t>
+          <t>DATA-02</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -1559,17 +1559,17 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석·분석리포트</t>
+          <t>티어리스트·조합상세·아이템빌드</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>DB 스키마 설계-분석/로그 테이블</t>
+          <t>DB 스키마 설계-메타조합 테이블</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>match_analyses, chat_logs, link_click_events, account_link_events, patch_detection_runs, ragas_eval_results, chat_answer_cache, puuid_cache 마이그레이션 작성(캐시 테이블 2종은 v1.7 신설 — Redis 대체)</t>
+          <t>comps/comp_champions/comp_augments/champion_item_builds 마이그레이션 작성</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -1584,24 +1584,24 @@
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>설계서 5.1·5.3</t>
+          <t>설계서 5.1</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>마이그레이션 적용 확인(8개 테이블)</t>
+          <t>마이그레이션 적용 및 FK 제약 확인</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>pytest: 8개 로그/분석/캐시 테이블 컬럼 존재 및 nullable 정책 assert</t>
+          <t>pytest: comp_champions/comp_augments FK 제약 위반 시 IntegrityError 발생 확인</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>DATA-04</t>
+          <t>DATA-03</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -1616,17 +1616,17 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>챗봇위젯</t>
+          <t>사후패인분석·분석리포트</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>벡터DB 스키마 및 인덱스 구성</t>
+          <t>DB 스키마 설계-분석/로그 테이블</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>meta_document_embeddings 테이블 생성, HNSW(vector_cosine_ops) 인덱스 및 (patch_version,doc_type) btree 인덱스 구성</t>
+          <t>match_analyses, chat_logs, link_click_events, account_link_events, patch_detection_runs, ragas_eval_results, chat_answer_cache, puuid_cache 마이그레이션 작성(캐시 테이블 2종은 v1.7 신설 — Redis 대체)</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -1636,29 +1636,29 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>DATA-01,SET-04</t>
+          <t>DATA-01</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>설계서 5.2</t>
+          <t>설계서 5.1·5.3</t>
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>인덱스 생성 확인, 샘플 벡터 검색 성공</t>
+          <t>마이그레이션 적용 확인(8개 테이블)</t>
         </is>
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>pytest: 더미 벡터 upsert 후 top-k 코사인 검색이 예상 순서로 반환되는지 확인, EXPLAIN으로 HNSW 인덱스 사용 확인</t>
+          <t>pytest: 8개 로그/분석/캐시 테이블 컬럼 존재 및 nullable 정책 assert</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>DATA-05</t>
+          <t>DATA-04</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -1673,17 +1673,17 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>챗봇위젯</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>op.gg MCP 응답 스키마 확인 스파이크</t>
+          <t>벡터DB 스키마 및 인덱스 구성</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>6개 TFT 도구 실호출로 응답 필드 전체 확인, patch_version 상당 필드 존재 여부 기록</t>
+          <t>meta_document_embeddings 테이블 생성, HNSW(vector_cosine_ops) 인덱스 및 (patch_version,doc_type) btree 인덱스 구성</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -1693,29 +1693,29 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>SET-10</t>
+          <t>DATA-01,SET-04</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>PRD 13-2·설계서 8장</t>
+          <t>설계서 5.2</t>
         </is>
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>확인 결과 스파이크 리포트 문서화</t>
+          <t>인덱스 생성 확인, 샘플 벡터 검색 성공</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>해당 없음(스파이크) — 실호출 결과를 /docs/spike/opgg-schema.md에 기록, DATA-08 테스트 fixture의 근거로 사용</t>
+          <t>pytest: 더미 벡터 upsert 후 top-k 코사인 검색이 예상 순서로 반환되는지 확인, EXPLAIN으로 HNSW 인덱스 사용 확인</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>DATA-06</t>
+          <t>DATA-05</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
@@ -1735,12 +1735,12 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>TFT DDragon 신규 구조 확인 스파이크</t>
+          <t>op.gg MCP 응답 스키마 확인 스파이크</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>Set 18 TFT DDragon 신규 엔드포인트·버전관리 방식 확인</t>
+          <t>6개 TFT 도구 실호출로 응답 필드 전체 확인, patch_version 상당 필드 존재 여부 기록</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1750,29 +1750,29 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>SET-10</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>PRD 12장·13-2</t>
+          <t>PRD 13-2·설계서 8장</t>
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>확인 결과 문서화</t>
+          <t>확인 결과 스파이크 리포트 문서화</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>해당 없음(스파이크) — 결과를 /docs/spike/tft-ddragon.md에 기록</t>
+          <t>해당 없음(스파이크) — 실호출 결과를 /docs/spike/opgg-schema.md에 기록, DATA-08 테스트 fixture의 근거로 사용</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>DATA-07</t>
+          <t>DATA-06</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -1787,17 +1787,17 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>증강체정보</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>is_legend_related 판별 방법 확인 스파이크</t>
+          <t>TFT DDragon 신규 구조 확인 스파이크</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>op.gg 응답 라벨 유무 확인, 없으면 수동 유지 목록 설계</t>
+          <t>Set 18 TFT DDragon 신규 엔드포인트·버전관리 방식 확인</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -1807,29 +1807,29 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>DATA-05</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>설계서 5.1·8장</t>
+          <t>PRD 12장·13-2</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>판별 로직 확정 및 문서화</t>
+          <t>확인 결과 문서화</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>해당 없음(스파이크) — 결과를 /docs/spike/legend-augment.md에 기록</t>
+          <t>해당 없음(스파이크) — 결과를 /docs/spike/tft-ddragon.md에 기록</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>DATA-08</t>
+          <t>DATA-07</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -1844,17 +1844,17 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>증강체정보</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>op.gg MCP 배치 수집 워커 구현</t>
+          <t>is_legend_related 판별 방법 확인 스파이크</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>6개 도구 순차 호출 클라이언트 구현</t>
+          <t>op.gg 응답 라벨 유무 확인, 없으면 수동 유지 목록 설계</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1869,24 +1869,24 @@
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.3</t>
+          <t>설계서 5.1·8장</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>스테이징에서 전체 도구 호출 성공</t>
+          <t>판별 로직 확정 및 문서화</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
-          <t>pytest: op.gg 응답을 스파이크 결과 기반 fixture로 고정해 6개 도구 호출·파싱 결과 검증(실 API 미호출)</t>
+          <t>해당 없음(스파이크) — 결과를 /docs/spike/legend-augment.md에 기록</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>DATA-09</t>
+          <t>DATA-08</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -1906,12 +1906,12 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>ID-이름 매핑 갱신 로직 구현</t>
+          <t>op.gg MCP 배치 수집 워커 구현</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>DDragon/TFT DDragon 조회 및 매핑 반영</t>
+          <t>6개 도구 순차 호출 클라이언트 구현</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -1921,7 +1921,7 @@
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>DATA-06,DATA-08</t>
+          <t>DATA-05</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
@@ -1931,19 +1931,19 @@
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t>매핑 결과 샘플 검증</t>
+          <t>스테이징에서 전체 도구 호출 성공</t>
         </is>
       </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
-          <t>pytest: DDragon mock 기준 ID→이름 매핑 정확도 케이스 + 매핑 누락 시 폴백 동작 검증</t>
+          <t>pytest: op.gg 응답을 스파이크 결과 기반 fixture로 고정해 6개 도구 호출·파싱 결과 검증(실 API 미호출)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>DATA-10</t>
+          <t>DATA-09</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
@@ -1963,12 +1963,12 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>데이터 정규화 및 patch_version 태깅 구현</t>
+          <t>ID-이름 매핑 갱신 로직 구현</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>raw 응답→구조화 테이블 upsert, 모든 레코드 patch_version 태깅</t>
+          <t>DDragon/TFT DDragon 조회 및 매핑 반영</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -1978,29 +1978,29 @@
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>DATA-02,DATA-08</t>
+          <t>DATA-06,DATA-08</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>PRD 9-2·12장</t>
+          <t>설계서 4.3</t>
         </is>
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>신규 패치 upsert 후 데이터 정합성 확인</t>
+          <t>매핑 결과 샘플 검증</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>pytest: 동일 엔티티 재수집 시 upsert(덮어쓰기 아님) 및 신규 행 patch_version 태깅 확인</t>
+          <t>pytest: DDragon mock 기준 ID→이름 매핑 정확도 케이스 + 매핑 누락 시 폴백 동작 검증</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>DATA-11</t>
+          <t>DATA-10</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
@@ -2020,12 +2020,12 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>임베딩 생성 파이프라인 구현</t>
+          <t>데이터 정규화 및 patch_version 태깅 구현</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>정규화 레코드→자연어 chunk 변환→BGE-M3 임베딩→upsert</t>
+          <t>raw 응답→구조화 테이블 upsert, 모든 레코드 patch_version 태깅</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -2035,29 +2035,29 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>DATA-04,DATA-10,SET-10</t>
+          <t>DATA-02,DATA-08</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.3·5.2</t>
+          <t>PRD 9-2·12장</t>
         </is>
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>임베딩 upsert 및 유사도 검색 성공</t>
+          <t>신규 패치 upsert 후 데이터 정합성 확인</t>
         </is>
       </c>
       <c r="K27" s="3" t="inlineStr">
         <is>
-          <t>pytest: mock 임베딩 클라이언트로 chunk→embedding upsert 동작, 임베딩 차원(1024) 검증</t>
+          <t>pytest: 동일 엔티티 재수집 시 upsert(덮어쓰기 아님) 및 신규 행 patch_version 태깅 확인</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>DATA-12</t>
+          <t>DATA-11</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
@@ -2077,12 +2077,12 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>자동 패치 감지 트리거 구현</t>
+          <t>임베딩 생성 파이프라인 구현</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>GitHub Actions 크론(매시간)으로 patch_version 비교 후 배치 트리거</t>
+          <t>정규화 레코드→자연어 chunk 변환→BGE-M3 임베딩→upsert</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -2092,29 +2092,29 @@
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>DATA-08,SET-08</t>
+          <t>DATA-04,DATA-10,SET-10</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>PRD 9-1·설계서4.3</t>
+          <t>설계서 4.3·5.2</t>
         </is>
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
-          <t>패치 변경 시뮬레이션 트리거 성공</t>
+          <t>임베딩 upsert 및 유사도 검색 성공</t>
         </is>
       </c>
       <c r="K28" s="3" t="inlineStr">
         <is>
-          <t>pytest: patch_version 변경을 mock으로 주입해 배치 트리거 호출 여부 확인</t>
+          <t>pytest: mock 임베딩 클라이언트로 chunk→embedding upsert 동작, 임베딩 차원(1024) 검증</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>DATA-13</t>
+          <t>DATA-12</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
@@ -2134,12 +2134,12 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>원자적 패치 전환 트랜잭션 구현</t>
+          <t>자동 패치 감지 트리거 구현</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>전체 성공시에만 patches.is_current 트랜잭션 전환, 실패시 롤백</t>
+          <t>GitHub Actions 크론(매시간)으로 patch_version 비교 후 배치 트리거</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -2149,29 +2149,29 @@
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>DATA-10,DATA-11</t>
+          <t>DATA-08,SET-08</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>PRD 12장</t>
+          <t>PRD 9-1·설계서4.3</t>
         </is>
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>중간 실패 시나리오에서 이전 패치 유지 확인</t>
+          <t>패치 변경 시뮬레이션 트리거 성공</t>
         </is>
       </c>
       <c r="K29" s="3" t="inlineStr">
         <is>
-          <t>pytest(필수·크리티컬, TEST-00 시나리오 선적용): 배치 중간 강제 실패 주입 시 is_current가 이전 값을 유지하는지, 전체 성공 시에만 전환되는지 두 시나리오 모두 검증</t>
+          <t>pytest: patch_version 변경을 mock으로 주입해 배치 트리거 호출 여부 확인</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>DATA-14</t>
+          <t>DATA-13</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -2191,12 +2191,12 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>배치 동시 실행 방지 구현</t>
+          <t>원자적 패치 전환 트랜잭션 구현</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>GitHub Actions concurrency 그룹 설정</t>
+          <t>전체 성공시에만 patches.is_current 트랜잭션 전환, 실패시 롤백</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -2206,29 +2206,29 @@
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>DATA-12</t>
+          <t>DATA-10,DATA-11</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.3</t>
+          <t>PRD 12장</t>
         </is>
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>중복 트리거 시 동작 확인</t>
+          <t>중간 실패 시나리오에서 이전 패치 유지 확인</t>
         </is>
       </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t>동시성 테스트: concurrency 그룹 설정 상태에서 동시 트리거 시 1개만 실행되는지 확인</t>
+          <t>pytest(필수·크리티컬, TEST-00 시나리오 선적용): 배치 중간 강제 실패 주입 시 is_current가 이전 값을 유지하는지, 전체 성공 시에만 전환되는지 두 시나리오 모두 검증</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>DATA-15</t>
+          <t>DATA-14</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -2248,12 +2248,12 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>캐시 정리 배치 구현</t>
+          <t>배치 동시 실행 방지 구현</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>배치 완료 후 chat_answer_cache에서 이전 patch_version 캐시 행 삭제(Postgres DELETE, v1.7 — 이전 Redis 키 무효화 대체)</t>
+          <t>GitHub Actions concurrency 그룹 설정</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -2263,29 +2263,29 @@
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>DATA-13,DATA-03</t>
+          <t>DATA-12</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>설계서 v1.7 4.3·4.6</t>
+          <t>설계서 4.3</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>배치 완료 후 이전 patch_version 캐시 행 삭제 확인</t>
+          <t>중복 트리거 시 동작 확인</t>
         </is>
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>pytest: 배치 완료 이벤트 발생 시 chat_answer_cache에서 이전 patch_version 행이 삭제되는지 확인</t>
+          <t>동시성 테스트: concurrency 그룹 설정 상태에서 동시 트리거 시 1개만 실행되는지 확인</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>API-01</t>
+          <t>DATA-15</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -2295,7 +2295,7 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>백엔드API</t>
+          <t>데이터파이프라인</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -2305,12 +2305,12 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>FastAPI 프로젝트 스캐폴딩</t>
+          <t>캐시 정리 배치 구현</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>단일 앱 + catalog/chat/analysis/kpi 4개 라우터 구조(kpi는 SET-11 취소로 Metabase 대신 자체 KPI 대시보드 백엔드용으로 v1.7에서 추가), 헬스체크 엔드포인트</t>
+          <t>배치 완료 후 chat_answer_cache에서 이전 patch_version 캐시 행 삭제(Postgres DELETE, v1.7 — 이전 Redis 키 무효화 대체)</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -2320,29 +2320,29 @@
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>SET-02,SET-03</t>
+          <t>DATA-13,DATA-03</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.2</t>
+          <t>설계서 v1.7 4.3·4.6</t>
         </is>
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>/health 200 응답 확인</t>
+          <t>배치 완료 후 이전 patch_version 캐시 행 삭제 확인</t>
         </is>
       </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
-          <t>pytest+FastAPI TestClient: /health 200 및 4개 라우터(catalog/chat/analysis/kpi) 마운트 확인</t>
+          <t>pytest: 배치 완료 이벤트 발생 시 chat_answer_cache에서 이전 patch_version 행이 삭제되는지 확인</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>API-02</t>
+          <t>API-01</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
@@ -2357,17 +2357,17 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>티어리스트</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>GET /catalog/tierlist 구현</t>
+          <t>FastAPI 프로젝트 스캐폴딩</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>패치·랭크 필터 지원, comps 테이블 SQL 조회</t>
+          <t>단일 앱 + catalog/chat/analysis/kpi 4개 라우터 구조(kpi는 SET-11 취소로 Metabase 대신 자체 KPI 대시보드 백엔드용으로 v1.7에서 추가), 헬스체크 엔드포인트</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -2377,29 +2377,29 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>DATA-02,API-01</t>
+          <t>SET-02,SET-03</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>PRD 7-1·설계서6장</t>
+          <t>설계서 4.2</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>응답 스키마·필터 동작 확인</t>
+          <t>/health 200 응답 확인</t>
         </is>
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>pytest: 패치/랭크 필터 조합별 응답, 빈 결과, 잘못된 파라미터 400 케이스</t>
+          <t>pytest+FastAPI TestClient: /health 200 및 4개 라우터(catalog/chat/analysis/kpi) 마운트 확인</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>API-03</t>
+          <t>API-02</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -2414,17 +2414,17 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>조합상세</t>
+          <t>티어리스트</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>GET /catalog/comps/{comp_id} 구현</t>
+          <t>GET /catalog/tierlist 구현</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>챔피언구성·증강체 우선순위 포함</t>
+          <t>패치·랭크 필터 지원, comps 테이블 SQL 조회</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -2439,24 +2439,24 @@
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>설계서 5.1·6장</t>
+          <t>PRD 7-1·설계서6장</t>
         </is>
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>응답 필드 검증</t>
+          <t>응답 스키마·필터 동작 확인</t>
         </is>
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t>pytest: 존재/미존재 comp_id 케이스, 캐리/서브 챔피언 구분 필드 정확성</t>
+          <t>pytest: 패치/랭크 필터 조합별 응답, 빈 결과, 잘못된 파라미터 400 케이스</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>API-04</t>
+          <t>API-03</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
@@ -2471,17 +2471,17 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>아이템빌드</t>
+          <t>조합상세</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>GET /catalog/items/builds 구현</t>
+          <t>GET /catalog/comps/{comp_id} 구현</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>챔피언 필터 지원</t>
+          <t>챔피언구성·증강체 우선순위 포함</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -2496,7 +2496,7 @@
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>설계서 6장</t>
+          <t>설계서 5.1·6장</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
@@ -2506,14 +2506,14 @@
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>pytest: champion_id 필터 유무 케이스, 정렬 순서 검증</t>
+          <t>pytest: 존재/미존재 comp_id 케이스, 캐리/서브 챔피언 구분 필드 정확성</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>API-05</t>
+          <t>API-04</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -2528,17 +2528,17 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>증강체정보</t>
+          <t>아이템빌드</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>GET /catalog/augments 구현</t>
+          <t>GET /catalog/items/builds 구현</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>is_legend_related=true 승률 마스킹 포함</t>
+          <t>챔피언 필터 지원</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -2548,29 +2548,29 @@
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>DATA-07,API-01</t>
+          <t>DATA-02,API-01</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>PRD 10-1·설계서4.4.3</t>
+          <t>설계서 6장</t>
         </is>
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>마스킹 동작 단위 테스트 통과</t>
+          <t>응답 필드 검증</t>
         </is>
       </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
-          <t>pytest(필수·정책, TEST-00 시나리오 선적용): is_legend_related=true 데이터로 응답에 win_rate 필드 자체가 없는지(=null 아님) 검증</t>
+          <t>pytest: champion_id 필터 유무 케이스, 정렬 순서 검증</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>API-06</t>
+          <t>API-05</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
@@ -2585,17 +2585,17 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>공통(GNB)</t>
+          <t>증강체정보</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>GET /catalog/patches/current 구현</t>
+          <t>GET /catalog/augments 구현</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>현재 패치 조회</t>
+          <t>is_legend_related=true 승률 마스킹 포함</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -2605,29 +2605,29 @@
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>DATA-01,API-01</t>
+          <t>DATA-07,API-01</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>설계서 6장</t>
+          <t>PRD 10-1·설계서4.4.3</t>
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
-          <t>응답 검증</t>
+          <t>마스킹 동작 단위 테스트 통과</t>
         </is>
       </c>
       <c r="K37" s="3" t="inlineStr">
         <is>
-          <t>pytest: is_current=true 패치 1건만 반환되는지 확인</t>
+          <t>pytest(필수·정책, TEST-00 시나리오 선적용): is_legend_related=true 데이터로 응답에 win_rate 필드 자체가 없는지(=null 아님) 검증</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>API-07</t>
+          <t>API-06</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
@@ -2642,17 +2642,17 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>공통(GNB)</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Rate Limiting 미들웨어 구현</t>
+          <t>GET /catalog/patches/current 구현</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>IP 기준 catalog 분당60/chat 분당10</t>
+          <t>현재 패치 조회</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -2662,29 +2662,29 @@
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>API-01</t>
+          <t>DATA-01,API-01</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.2·6장</t>
+          <t>설계서 6장</t>
         </is>
       </c>
       <c r="J38" s="3" t="inlineStr">
         <is>
-          <t>초과 요청 429 응답 확인</t>
+          <t>응답 검증</t>
         </is>
       </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
-          <t>pytest: 한도 초과 요청 시 429 응답 확인(catalog 60/분, chat 10/분 각각)</t>
+          <t>pytest: is_current=true 패치 1건만 반환되는지 확인</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>API-08</t>
+          <t>API-07</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
@@ -2699,17 +2699,17 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>챗봇위젯</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>session_id 발급/조회 로직 구현</t>
+          <t>Rate Limiting 미들웨어 구현</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>클라이언트 UUID 수신 및 대화 묶음 키로 사용</t>
+          <t>IP 기준 catalog 분당60/chat 분당10</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
@@ -2724,24 +2724,24 @@
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.2</t>
+          <t>설계서 4.2·6장</t>
         </is>
       </c>
       <c r="J39" s="3" t="inlineStr">
         <is>
-          <t>세션별 대화 구분 확인</t>
+          <t>초과 요청 429 응답 확인</t>
         </is>
       </c>
       <c r="K39" s="3" t="inlineStr">
         <is>
-          <t>pytest: 동일 session_id 재사용 시 동일 대화로 묶이는지, 신규 UUID는 분리되는지 확인</t>
+          <t>pytest: 한도 초과 요청 시 429 응답 확인(catalog 60/분, chat 10/분 각각)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>API-09</t>
+          <t>API-08</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
@@ -2761,12 +2761,12 @@
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>POST /chat/message 뼈대 구현(SSE)</t>
+          <t>session_id 발급/조회 로직 구현</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>스트리밍 응답 인프라 구현(RAG 로직은 CHAT 그룹에서 연동)</t>
+          <t>클라이언트 UUID 수신 및 대화 묶음 키로 사용</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
@@ -2776,29 +2776,29 @@
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>API-08</t>
+          <t>API-01</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.2·4.4</t>
+          <t>설계서 4.2</t>
         </is>
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>SSE 스트림 클라이언트 수신 확인</t>
+          <t>세션별 대화 구분 확인</t>
         </is>
       </c>
       <c r="K40" s="3" t="inlineStr">
         <is>
-          <t>pytest: SSE 스트림 청크 수신 순서 및 연결 종료 처리 확인(mock LLM 스트림)</t>
+          <t>pytest: 동일 session_id 재사용 시 동일 대화로 묶이는지, 신규 UUID는 분리되는지 확인</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>API-10</t>
+          <t>API-09</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
@@ -2818,12 +2818,12 @@
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>GET /chat/session/{id}/history 구현</t>
+          <t>POST /chat/message 뼈대 구현(SSE)</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>chat_logs 기반 대화이력 조회</t>
+          <t>스트리밍 응답 인프라 구현(RAG 로직은 CHAT 그룹에서 연동)</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
@@ -2833,29 +2833,29 @@
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>DATA-03,API-09</t>
+          <t>API-08</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.4</t>
+          <t>설계서 4.2·4.4</t>
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>최근 3턴 조회 확인</t>
+          <t>SSE 스트림 클라이언트 수신 확인</t>
         </is>
       </c>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>pytest: 최근 3턴만 반환, 4턴 이상 시 오래된 턴 제외 확인</t>
+          <t>pytest: SSE 스트림 청크 수신 순서 및 연결 종료 처리 확인(mock LLM 스트림)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>API-11</t>
+          <t>API-10</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
@@ -2870,17 +2870,17 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석</t>
+          <t>챗봇위젯</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>POST /analysis/link 구현</t>
+          <t>GET /chat/session/{id}/history 구현</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>Riot ID→PUUID 변환, TTL 1시간 캐시(Postgres puuid_cache 테이블, v1.7)</t>
+          <t>chat_logs 기반 대화이력 조회</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
@@ -2890,29 +2890,29 @@
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>SET-10,API-01</t>
+          <t>DATA-03,API-09</t>
         </is>
       </c>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>PRD 9-1·설계서v1.7 4.5</t>
+          <t>설계서 4.4</t>
         </is>
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t>변환 성공/실패 케이스 확인</t>
+          <t>최근 3턴 조회 확인</t>
         </is>
       </c>
       <c r="K42" s="3" t="inlineStr">
         <is>
-          <t>pytest: mock Riot API로 정상/미존재 계정/레이트리밋 초과 3케이스, TTL 1시간 캐시 hit 확인</t>
+          <t>pytest: 최근 3턴만 반환, 4턴 이상 시 오래된 턴 제외 확인</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>API-12</t>
+          <t>API-11</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
@@ -2932,12 +2932,12 @@
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>POST /analysis/recent 뼈대 구현</t>
+          <t>POST /analysis/link 구현</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>최신 매치ID 조회 및 캐시 재사용 분기(스코어링은 PGA 그룹에서 연동)</t>
+          <t>Riot ID→PUUID 변환, TTL 1시간 캐시(Postgres puuid_cache 테이블, v1.7)</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
@@ -2947,29 +2947,29 @@
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>API-11,DATA-03</t>
+          <t>SET-16,API-01</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>PRD 8-3·설계서4.5</t>
+          <t>PRD 9-1·설계서v1.7 4.5</t>
         </is>
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>캐시 hit/miss 분기 확인</t>
+          <t>변환 성공/실패 케이스 확인</t>
         </is>
       </c>
       <c r="K43" s="3" t="inlineStr">
         <is>
-          <t>pytest: match_analyses 캐시 hit 시 Riot API mock 호출 0회 확인</t>
+          <t>pytest: mock Riot API로 정상/미존재 계정/레이트리밋 초과 3케이스, TTL 1시간 캐시 hit 확인</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>API-13</t>
+          <t>API-12</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
@@ -2984,17 +2984,17 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>분석리포트</t>
+          <t>사후패인분석</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>GET /analysis/{match_id}/report 구현</t>
+          <t>POST /analysis/recent 뼈대 구현</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>match_analyses 기반 리포트 응답</t>
+          <t>최신 매치ID 조회 및 캐시 재사용 분기(스코어링은 PGA 그룹에서 연동)</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
@@ -3004,29 +3004,29 @@
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>DATA-03,API-12</t>
+          <t>API-11,DATA-03</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>PRD 8-3·설계서6장</t>
+          <t>PRD 8-3·설계서4.5</t>
         </is>
       </c>
       <c r="J44" s="3" t="inlineStr">
         <is>
-          <t>응답 스키마 검증</t>
+          <t>캐시 hit/miss 분기 확인</t>
         </is>
       </c>
       <c r="K44" s="3" t="inlineStr">
         <is>
-          <t>pytest: 존재/미존재 match_id 케이스, 응답 스키마 필드 전체 검증</t>
+          <t>pytest: match_analyses 캐시 hit 시 Riot API mock 호출 0회 확인</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>API-14</t>
+          <t>API-13</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
@@ -3041,17 +3041,17 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>분석리포트</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>KPI 계측 이벤트 API 구현</t>
+          <t>GET /analysis/{match_id}/report 구현</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>link_click_events, account_link_events 적재 엔드포인트/훅</t>
+          <t>match_analyses 기반 리포트 응답</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
@@ -3061,29 +3061,29 @@
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>DATA-03,API-01</t>
+          <t>DATA-03,API-12</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>PRD 3-3·설계서5.3</t>
+          <t>PRD 8-3·설계서6장</t>
         </is>
       </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t>이벤트 적재 확인</t>
+          <t>응답 스키마 검증</t>
         </is>
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>pytest: 이벤트 적재 후 DB row 생성 및 필드 값 정확성 확인</t>
+          <t>pytest: 존재/미존재 match_id 케이스, 응답 스키마 필드 전체 검증</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>CHAT-01</t>
+          <t>API-14</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
@@ -3093,22 +3093,22 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>챗봇RAG</t>
+          <t>백엔드API</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>챗봇위젯</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>의도 분류 로직 구현</t>
+          <t>KPI 계측 이벤트 API 구현</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>1차 키워드/정규식, 2차 Groq LLM 분류(4종)</t>
+          <t>link_click_events, account_link_events 적재 엔드포인트/훅</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
@@ -3118,29 +3118,29 @@
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>API-09</t>
+          <t>DATA-03,API-01</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
-          <t>PRD 7-2·설계서4.4</t>
+          <t>PRD 3-3·설계서5.3</t>
         </is>
       </c>
       <c r="J46" s="3" t="inlineStr">
         <is>
-          <t>4개 의도 분류 정확도 샘플 테스트</t>
+          <t>이벤트 적재 확인</t>
         </is>
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>pytest: 키워드 규칙 매칭 케이스(4종 각 2개 이상) + 애매한 질문의 mock LLM 분류 경로 확인</t>
+          <t>pytest: 이벤트 적재 후 DB row 생성 및 필드 값 정확성 확인</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>CHAT-02</t>
+          <t>CHAT-01</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
@@ -3160,12 +3160,12 @@
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>하이브리드 검색 구현</t>
+          <t>의도 분류 로직 구현</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>SQL 필터 + pgvector top-k 코사인 검색</t>
+          <t>1차 키워드/정규식, 2차 Groq LLM 분류(4종)</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
@@ -3175,29 +3175,29 @@
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>DATA-11,CHAT-01</t>
+          <t>API-09</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>PRD 9-4·설계서4.4</t>
+          <t>PRD 7-2·설계서4.4</t>
         </is>
       </c>
       <c r="J47" s="3" t="inlineStr">
         <is>
-          <t>의도별 검색 결과 검증</t>
+          <t>4개 의도 분류 정확도 샘플 테스트</t>
         </is>
       </c>
       <c r="K47" s="3" t="inlineStr">
         <is>
-          <t>pytest: 의도별 SQL 필터 조건 반영 여부, mock pgvector top-k 결과 병합 확인</t>
+          <t>pytest: 키워드 규칙 매칭 케이스(4종 각 2개 이상) + 애매한 질문의 mock LLM 분류 경로 확인</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>CHAT-03</t>
+          <t>CHAT-02</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
@@ -3217,12 +3217,12 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>프롬프트 조립 로직 구현</t>
+          <t>하이브리드 검색 구현</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>시스템프롬프트+검색문서+대화이력+질문 결합, few-shot 삽입</t>
+          <t>SQL 필터 + pgvector top-k 코사인 검색</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
@@ -3232,29 +3232,29 @@
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>CHAT-02,API-10</t>
+          <t>DATA-11,CHAT-01</t>
         </is>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.4.1</t>
+          <t>PRD 9-4·설계서4.4</t>
         </is>
       </c>
       <c r="J48" s="3" t="inlineStr">
         <is>
-          <t>프롬프트 스냅샷 테스트</t>
+          <t>의도별 검색 결과 검증</t>
         </is>
       </c>
       <c r="K48" s="3" t="inlineStr">
         <is>
-          <t>pytest: 프롬프트 스냅샷 테스트 — 시스템프롬프트/검색문서/대화이력/질문이 정해진 순서·구분자로 조립되는지 문자열 비교</t>
+          <t>pytest: 의도별 SQL 필터 조건 반영 여부, mock pgvector top-k 결과 병합 확인</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>CHAT-04</t>
+          <t>CHAT-03</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
@@ -3274,12 +3274,12 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>입력 전처리 구현</t>
+          <t>프롬프트 조립 로직 구현</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>질문정규화·은어치환·인젝션방어·길이제한·범위밖질문 안내</t>
+          <t>시스템프롬프트+검색문서+대화이력+질문 결합, few-shot 삽입</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
@@ -3289,29 +3289,29 @@
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>CHAT-01</t>
+          <t>CHAT-02,API-10</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.4.2</t>
+          <t>설계서 4.4.1</t>
         </is>
       </c>
       <c r="J49" s="3" t="inlineStr">
         <is>
-          <t>각 케이스 단위 테스트 통과</t>
+          <t>프롬프트 스냅샷 테스트</t>
         </is>
       </c>
       <c r="K49" s="3" t="inlineStr">
         <is>
-          <t>pytest(필수·보안, TEST-00 시나리오 선적용): 인젝션 문구가 [사용자 메시지] 델리미터 내부로만 들어가는지, 범위밖 질문 안내 문구 반환, 초과 길이 입력 truncate 확인</t>
+          <t>pytest: 프롬프트 스냅샷 테스트 — 시스템프롬프트/검색문서/대화이력/질문이 정해진 순서·구분자로 조립되는지 문자열 비교</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>CHAT-05</t>
+          <t>CHAT-04</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
@@ -3331,12 +3331,12 @@
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>sLLM 답변 생성 및 SSE 스트리밍 연동</t>
+          <t>입력 전처리 구현</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>Groq Llama 3.3 70B 호출, 스트리밍 응답</t>
+          <t>질문정규화·은어치환·인젝션방어·길이제한·범위밖질문 안내</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
@@ -3346,29 +3346,29 @@
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>CHAT-03,API-09,SET-10</t>
+          <t>CHAT-01</t>
         </is>
       </c>
       <c r="I50" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.4</t>
+          <t>설계서 4.4.2</t>
         </is>
       </c>
       <c r="J50" s="3" t="inlineStr">
         <is>
-          <t>스트리밍 응답 end-to-end 확인</t>
+          <t>각 케이스 단위 테스트 통과</t>
         </is>
       </c>
       <c r="K50" s="3" t="inlineStr">
         <is>
-          <t>pytest: mock Groq 클라이언트로 SSE 스트리밍 조립 확인, 타임아웃 예외 처리 확인</t>
+          <t>pytest(필수·보안, TEST-00 시나리오 선적용): 인젝션 문구가 [사용자 메시지] 델리미터 내부로만 들어가는지, 범위밖 질문 안내 문구 반환, 초과 길이 입력 truncate 확인</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>CHAT-06</t>
+          <t>CHAT-05</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
@@ -3388,12 +3388,12 @@
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>출력 후처리 구현</t>
+          <t>sLLM 답변 생성 및 SSE 스트리밍 연동</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>근거검증·Legend승률이중방어·닉네임마스킹·구조화출력·재시도폴백</t>
+          <t>Groq Llama 3.3 70B 호출, 스트리밍 응답</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
@@ -3403,29 +3403,29 @@
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>CHAT-05</t>
+          <t>CHAT-03,API-09,SET-10</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.4.3</t>
+          <t>설계서 4.4</t>
         </is>
       </c>
       <c r="J51" s="3" t="inlineStr">
         <is>
-          <t>각 방어 로직 단위 테스트 통과</t>
+          <t>스트리밍 응답 end-to-end 확인</t>
         </is>
       </c>
       <c r="K51" s="3" t="inlineStr">
         <is>
-          <t>pytest(필수·정책, TEST-00 시나리오 선적용): 근거 없는 고유명사 재생성/경고 처리, Legend 문서 승률 수치 후처리 제거, 상대 닉네임 정규식 마스킹 3케이스 모두 검증</t>
+          <t>pytest: mock Groq 클라이언트로 SSE 스트리밍 조립 확인, 타임아웃 예외 처리 확인</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>CHAT-07</t>
+          <t>CHAT-06</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
@@ -3445,12 +3445,12 @@
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>웹사이트 링크 자동 삽입 구현</t>
+          <t>출력 후처리 구현</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>답변 내 조합/아이템/증강체 id 파싱→상세페이지 링크 삽입</t>
+          <t>근거검증·Legend승률이중방어·닉네임마스킹·구조화출력·재시도폴백</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr">
@@ -3460,29 +3460,29 @@
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>CHAT-06</t>
+          <t>CHAT-05</t>
         </is>
       </c>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>PRD 7-2·설계서4.4</t>
+          <t>설계서 4.4.3</t>
         </is>
       </c>
       <c r="J52" s="3" t="inlineStr">
         <is>
-          <t>링크 삽입 정확도 샘플 테스트</t>
+          <t>각 방어 로직 단위 테스트 통과</t>
         </is>
       </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
-          <t>pytest: 답변 내 조합/아이템/증강체 언급 시 정확한 링크 삽입, 존재하지 않는 id 오탐 케이스 처리 확인</t>
+          <t>pytest(필수·정책, TEST-00 시나리오 선적용): 근거 없는 고유명사 재생성/경고 처리, Legend 문서 승률 수치 후처리 제거, 상대 닉네임 정규식 마스킹 3케이스 모두 검증</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>CHAT-08</t>
+          <t>CHAT-07</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
@@ -3502,12 +3502,12 @@
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>응답 캐싱 로직 구현</t>
+          <t>웹사이트 링크 자동 삽입 구현</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>첫턴 질문 Postgres(chat_answer_cache) 캐시, 후속턴 캐시제외, 패치갱신시 무효화</t>
+          <t>답변 내 조합/아이템/증강체 id 파싱→상세페이지 링크 삽입</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
@@ -3517,29 +3517,29 @@
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>CHAT-05,DATA-15</t>
+          <t>CHAT-06</t>
         </is>
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>PRD 9-6·설계서v1.7 4.4·4.6</t>
+          <t>PRD 7-2·설계서4.4</t>
         </is>
       </c>
       <c r="J53" s="3" t="inlineStr">
         <is>
-          <t>캐시 hit/무효화 시나리오 테스트</t>
+          <t>링크 삽입 정확도 샘플 테스트</t>
         </is>
       </c>
       <c r="K53" s="3" t="inlineStr">
         <is>
-          <t>pytest: 첫턴 캐시 hit, 후속턴 캐시 미적용, 패치갱신 후 캐시 무효화 확인</t>
+          <t>pytest: 답변 내 조합/아이템/증강체 언급 시 정확한 링크 삽입, 존재하지 않는 id 오탐 케이스 처리 확인</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>CHAT-09</t>
+          <t>CHAT-08</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
@@ -3559,12 +3559,12 @@
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>Q&amp;A 로깅 구현</t>
+          <t>응답 캐싱 로직 구현</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>chat_logs 적재(질의/의도/근거문서/patch/지연시간/콜드스타트)</t>
+          <t>첫턴 질문 Postgres(chat_answer_cache) 캐시, 후속턴 캐시제외, 패치갱신시 무효화</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
@@ -3574,29 +3574,29 @@
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>DATA-03,CHAT-05</t>
+          <t>CHAT-05,DATA-15</t>
         </is>
       </c>
       <c r="I54" s="3" t="inlineStr">
         <is>
-          <t>PRD 3-3·9-5</t>
+          <t>PRD 9-6·설계서v1.7 4.4·4.6</t>
         </is>
       </c>
       <c r="J54" s="3" t="inlineStr">
         <is>
-          <t>로그 적재 필드 확인</t>
+          <t>캐시 hit/무효화 시나리오 테스트</t>
         </is>
       </c>
       <c r="K54" s="3" t="inlineStr">
         <is>
-          <t>pytest: chat_logs row에 질의/의도/근거문서id/patch_version/답변/지연시간/콜드스타트 전체 필드 적재 확인</t>
+          <t>pytest: 첫턴 캐시 hit, 후속턴 캐시 미적용, 패치갱신 후 캐시 무효화 확인</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>CHAT-10</t>
+          <t>CHAT-09</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
@@ -3616,12 +3616,12 @@
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>사후분석 트리거 연동</t>
+          <t>Q&amp;A 로깅 구현</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>'방금 게임 분석해줘' 발화 시 분석 로직 호출 및 챗봇 답변 영역 요약 표시</t>
+          <t>chat_logs 적재(질의/의도/근거문서/patch/지연시간/콜드스타트)</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
@@ -3631,29 +3631,29 @@
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>CHAT-06,API-12</t>
+          <t>DATA-03,CHAT-05</t>
         </is>
       </c>
       <c r="I55" s="3" t="inlineStr">
         <is>
-          <t>PRD 8-3</t>
+          <t>PRD 3-3·9-5</t>
         </is>
       </c>
       <c r="J55" s="3" t="inlineStr">
         <is>
-          <t>트리거 발화 테스트 통과</t>
+          <t>로그 적재 필드 확인</t>
         </is>
       </c>
       <c r="K55" s="3" t="inlineStr">
         <is>
-          <t>pytest: '방금 게임 분석해줘' mock 발화 시 analysis 로직 호출(1회) 및 응답에 요약+링크 포함 확인</t>
+          <t>pytest: chat_logs row에 질의/의도/근거문서id/patch_version/답변/지연시간/콜드스타트 전체 필드 적재 확인</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>PGA-01</t>
+          <t>CHAT-10</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
@@ -3663,22 +3663,22 @@
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>사후패인분석</t>
+          <t>챗봇RAG</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석</t>
+          <t>챗봇위젯</t>
         </is>
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>Riot ID 계정 연동 로직 구현</t>
+          <t>사후분석 트리거 연동</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>게임명#태그+지역 입력→PUUID 변환, 임의계정 조회 허용</t>
+          <t>'방금 게임 분석해줘' 발화 시 분석 로직 호출 및 챗봇 답변 영역 요약 표시</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
@@ -3688,29 +3688,29 @@
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>API-11</t>
+          <t>CHAT-06,API-12</t>
         </is>
       </c>
       <c r="I56" s="3" t="inlineStr">
         <is>
-          <t>PRD 7-3·8-3·9-1</t>
+          <t>PRD 8-3</t>
         </is>
       </c>
       <c r="J56" s="3" t="inlineStr">
         <is>
-          <t>정상/비정상 계정 케이스 테스트</t>
+          <t>트리거 발화 테스트 통과</t>
         </is>
       </c>
       <c r="K56" s="3" t="inlineStr">
         <is>
-          <t>pytest: 정상 Riot ID/형식 오류/미존재 계정 3케이스</t>
+          <t>pytest: '방금 게임 분석해줘' mock 발화 시 analysis 로직 호출(1회) 및 응답에 요약+링크 포함 확인</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>PGA-02</t>
+          <t>PGA-01</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
@@ -3730,12 +3730,12 @@
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>최신 매치 조회 로직 구현</t>
+          <t>Riot ID 계정 연동 로직 구현</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>Match-V1으로 매치ID/매치상세 조회</t>
+          <t>게임명#태그+지역 입력→PUUID 변환, 임의계정 조회 허용</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
@@ -3745,29 +3745,29 @@
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>PGA-01</t>
+          <t>API-11</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
         <is>
-          <t>PRD 7-3·설계서4.5</t>
+          <t>PRD 7-3·8-3·9-1</t>
         </is>
       </c>
       <c r="J57" s="3" t="inlineStr">
         <is>
-          <t>매치 상세 파싱 검증</t>
+          <t>정상/비정상 계정 케이스 테스트</t>
         </is>
       </c>
       <c r="K57" s="3" t="inlineStr">
         <is>
-          <t>pytest: mock Match-V1 응답 기준 매치ID·매치상세 파싱 필드 전체 검증</t>
+          <t>pytest: 정상 Riot ID/형식 오류/미존재 계정 3케이스</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>PGA-03</t>
+          <t>PGA-02</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
@@ -3782,17 +3782,17 @@
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석·분석리포트</t>
+          <t>사후패인분석</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>분석 결과 캐시 재사용 로직 구현</t>
+          <t>최신 매치 조회 로직 구현</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>match_analyses 조회 우선, 없으면 신규계산</t>
+          <t>Match-V1으로 매치ID/매치상세 조회</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
@@ -3802,29 +3802,29 @@
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>DATA-03,PGA-02</t>
+          <t>PGA-01</t>
         </is>
       </c>
       <c r="I58" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.5·4.6·5.1</t>
+          <t>PRD 7-3·설계서4.5</t>
         </is>
       </c>
       <c r="J58" s="3" t="inlineStr">
         <is>
-          <t>재요청 시 캐시 히트 확인</t>
+          <t>매치 상세 파싱 검증</t>
         </is>
       </c>
       <c r="K58" s="3" t="inlineStr">
         <is>
-          <t>pytest: 동일 match_id+puuid 재요청 시 Riot API/Groq mock 호출 0회(캐시 hit), 신규 조합은 계산 경로 진입 확인</t>
+          <t>pytest: mock Match-V1 응답 기준 매치ID·매치상세 파싱 필드 전체 검증</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>PGA-04</t>
+          <t>PGA-03</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
@@ -3839,17 +3839,17 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>분석리포트</t>
+          <t>사후패인분석·분석리포트</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>조합 이탈도 계산 로직 구현</t>
+          <t>분석 결과 캐시 재사용 로직 구현</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>가중 자카드 유사도(캐리 가중치2), 구간분류</t>
+          <t>match_analyses 조회 우선, 없으면 신규계산</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">
@@ -3859,29 +3859,29 @@
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>PGA-02,DATA-02</t>
+          <t>DATA-03,PGA-02</t>
         </is>
       </c>
       <c r="I59" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.5.1</t>
+          <t>설계서 4.5·4.6·5.1</t>
         </is>
       </c>
       <c r="J59" s="3" t="inlineStr">
         <is>
-          <t>샘플 매치 계산값 수기검증 일치</t>
+          <t>재요청 시 캐시 히트 확인</t>
         </is>
       </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t>pytest(필수·크리티컬, TEST-00 시나리오 선적용): 수기 계산한 샘플 보드 3~5개에 대해 이탈도 값이 소수점 둘째자리까지 일치, 구간분류 경계값(0.3/0.6) 케이스 포함</t>
+          <t>pytest: 동일 match_id+puuid 재요청 시 Riot API/Groq mock 호출 0회(캐시 hit), 신규 조합은 계산 경로 진입 확인</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>PGA-05</t>
+          <t>PGA-04</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
@@ -3901,12 +3901,12 @@
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>아이템 집중도 계산 로직 구현</t>
+          <t>조합 이탈도 계산 로직 구현</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>캐리 완성아이템 비율, 추천빌드 멀티셋 교집합</t>
+          <t>가중 자카드 유사도(캐리 가중치2), 구간분류</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
@@ -3916,7 +3916,7 @@
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>PGA-04</t>
+          <t>PGA-02,DATA-02</t>
         </is>
       </c>
       <c r="I60" s="3" t="inlineStr">
@@ -3926,19 +3926,19 @@
       </c>
       <c r="J60" s="3" t="inlineStr">
         <is>
-          <t>샘플 계산값 검증</t>
+          <t>샘플 매치 계산값 수기검증 일치</t>
         </is>
       </c>
       <c r="K60" s="3" t="inlineStr">
         <is>
-          <t>pytest: 샘플 보드 기준 집중도 값 수기 계산과 일치, 중복 아이템 멀티셋 케이스 포함</t>
+          <t>pytest(필수·크리티컬, TEST-00 시나리오 선적용): 수기 계산한 샘플 보드 3~5개에 대해 이탈도 값이 소수점 둘째자리까지 일치, 구간분류 경계값(0.3/0.6) 케이스 포함</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>PGA-06</t>
+          <t>PGA-05</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
@@ -3958,12 +3958,12 @@
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>증강체 시너지 계산 로직 구현</t>
+          <t>아이템 집중도 계산 로직 구현</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>선택증강체 vs comp_augments 매칭 비율</t>
+          <t>캐리 완성아이템 비율, 추천빌드 멀티셋 교집합</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
@@ -3988,14 +3988,14 @@
       </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>pytest: 선택 증강체 0개/일부일치/전체일치 3케이스 시너지 점수 검증</t>
+          <t>pytest: 샘플 보드 기준 집중도 값 수기 계산과 일치, 중복 아이템 멀티셋 케이스 포함</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>PGA-07</t>
+          <t>PGA-06</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
@@ -4015,12 +4015,12 @@
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>코칭 문장 생성 로직 구현</t>
+          <t>증강체 시너지 계산 로직 구현</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>3개 지표+등수 근거로 잘한점/아쉬운점/제안 고정구조 생성, 수치 비노출</t>
+          <t>선택증강체 vs comp_augments 매칭 비율</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
@@ -4030,29 +4030,29 @@
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>PGA-04,PGA-05,PGA-06,SET-10</t>
+          <t>PGA-04</t>
         </is>
       </c>
       <c r="I62" s="3" t="inlineStr">
         <is>
-          <t>PRD 7-3·설계서4.5.2</t>
+          <t>설계서 4.5.1</t>
         </is>
       </c>
       <c r="J62" s="3" t="inlineStr">
         <is>
-          <t>출력 포맷 규칙 준수 확인</t>
+          <t>샘플 계산값 검증</t>
         </is>
       </c>
       <c r="K62" s="3" t="inlineStr">
         <is>
-          <t>pytest(필수·정책, TEST-00 시나리오 선적용): mock LLM 출력에 원 수치(예: '이탈도 0.42')가 노출되면 실패 처리되는 검증 로직 자체 테스트, 고정 3단 구조 파싱 확인</t>
+          <t>pytest: 선택 증강체 0개/일부일치/전체일치 3케이스 시너지 점수 검증</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>PGA-08</t>
+          <t>PGA-07</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
@@ -4072,12 +4072,12 @@
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>다음 게임 제안 근거 조회 로직 구현</t>
+          <t>코칭 문장 생성 로직 구현</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>matched_comp_id 기준 추천아이템·증강체 조회</t>
+          <t>3개 지표+등수 근거로 잘한점/아쉬운점/제안 고정구조 생성, 수치 비노출</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr">
@@ -4087,29 +4087,29 @@
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>PGA-04,DATA-02</t>
+          <t>PGA-04,PGA-05,PGA-06,SET-10</t>
         </is>
       </c>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.5.3</t>
+          <t>PRD 7-3·설계서4.5.2</t>
         </is>
       </c>
       <c r="J63" s="3" t="inlineStr">
         <is>
-          <t>추천 근거 정확성 검증</t>
+          <t>출력 포맷 규칙 준수 확인</t>
         </is>
       </c>
       <c r="K63" s="3" t="inlineStr">
         <is>
-          <t>pytest: matched_comp_id 기준 추천아이템/증강체 조회 결과가 champion_item_builds/comp_augments와 일치하는지 확인</t>
+          <t>pytest(필수·정책, TEST-00 시나리오 선적용): mock LLM 출력에 원 수치(예: '이탈도 0.42')가 노출되면 실패 처리되는 검증 로직 자체 테스트, 고정 3단 구조 파싱 확인</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>PGA-09</t>
+          <t>PGA-08</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
@@ -4129,12 +4129,12 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>프라이버시 마스킹 로직 구현</t>
+          <t>다음 게임 제안 근거 조회 로직 구현</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>상대 닉네임 마스킹 전처리+정규식 재마스킹 이중방어</t>
+          <t>matched_comp_id 기준 추천아이템·증강체 조회</t>
         </is>
       </c>
       <c r="G64" s="4" t="inlineStr">
@@ -4144,29 +4144,29 @@
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>PGA-07</t>
+          <t>PGA-04,DATA-02</t>
         </is>
       </c>
       <c r="I64" s="3" t="inlineStr">
         <is>
-          <t>PRD 7-3·설계서4.4.3·4.5.3</t>
+          <t>설계서 4.5.3</t>
         </is>
       </c>
       <c r="J64" s="3" t="inlineStr">
         <is>
-          <t>마스킹 누락 케이스 없음 확인</t>
+          <t>추천 근거 정확성 검증</t>
         </is>
       </c>
       <c r="K64" s="3" t="inlineStr">
         <is>
-          <t>pytest(필수·보안, TEST-00 시나리오 선적용): 상대 Riot ID 포함 mock LLM 출력에서 정규식 마스킹 후 원본 문자열이 전혀 남지 않는지(부분 마스킹 실패 케이스 포함) 확인</t>
+          <t>pytest: matched_comp_id 기준 추천아이템/증강체 조회 결과가 champion_item_builds/comp_augments와 일치하는지 확인</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>PGA-10</t>
+          <t>PGA-09</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
@@ -4181,17 +4181,17 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석·분석리포트</t>
+          <t>분석리포트</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>상세 리포트 데이터 조립 로직 구현</t>
+          <t>프라이버시 마스킹 로직 구현</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>코칭요약·매칭조합·등수변화·아이템타임라인 응답 조립</t>
+          <t>상대 닉네임 마스킹 전처리+정규식 재마스킹 이중방어</t>
         </is>
       </c>
       <c r="G65" s="4" t="inlineStr">
@@ -4201,29 +4201,29 @@
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
-          <t>PGA-07,PGA-08,PGA-09,API-13</t>
+          <t>PGA-07</t>
         </is>
       </c>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>PRD 8-3·IA4.6</t>
+          <t>PRD 7-3·설계서4.4.3·4.5.3</t>
         </is>
       </c>
       <c r="J65" s="3" t="inlineStr">
         <is>
-          <t>API-13 응답 필드 전체 채움 확인</t>
+          <t>마스킹 누락 케이스 없음 확인</t>
         </is>
       </c>
       <c r="K65" s="3" t="inlineStr">
         <is>
-          <t>pytest: API-13 응답 스키마 전체 필드가 null 없이 채워지는지 통합 테스트</t>
+          <t>pytest(필수·보안, TEST-00 시나리오 선적용): 상대 Riot ID 포함 mock LLM 출력에서 정규식 마스킹 후 원본 문자열이 전혀 남지 않는지(부분 마스킹 실패 케이스 포함) 확인</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>FE-01</t>
+          <t>PGA-10</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
@@ -4233,22 +4233,22 @@
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>프론트엔드</t>
+          <t>사후패인분석</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>사후패인분석·분석리포트</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>Next.js 프로젝트 스캐폴딩 및 Tailwind 설정</t>
+          <t>상세 리포트 데이터 조립 로직 구현</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>App Router, Tailwind 브레이크포인트(md768/lg1024) 매핑, 디자인가이드 토큰(컬러/타이포/spacing) 반영</t>
+          <t>코칭요약·매칭조합·등수변화·아이템타임라인 응답 조립</t>
         </is>
       </c>
       <c r="G66" s="4" t="inlineStr">
@@ -4258,29 +4258,29 @@
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>SET-07</t>
+          <t>PGA-07,PGA-08,PGA-09,API-13</t>
         </is>
       </c>
       <c r="I66" s="3" t="inlineStr">
         <is>
-          <t>설계서4.1.1·디자인가이드</t>
+          <t>PRD 8-3·IA4.6</t>
         </is>
       </c>
       <c r="J66" s="3" t="inlineStr">
         <is>
-          <t>기본 레이아웃 렌더링 확인</t>
+          <t>API-13 응답 필드 전체 채움 확인</t>
         </is>
       </c>
       <c r="K66" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: Tailwind 브레이크포인트 클래스 적용 여부, 디자인 토큰 색상값 매칭 확인</t>
+          <t>pytest: API-13 응답 스키마 전체 필드가 null 없이 채워지는지 통합 테스트</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>FE-02</t>
+          <t>FE-01</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
@@ -4295,17 +4295,17 @@
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>공통(GNB)</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>GNB 컴포넌트 구현</t>
+          <t>Next.js 프로젝트 스캐폴딩 및 Tailwind 설정</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>데스크톱/태블릿 가로바, 모바일 햄버거+드로어, 4개 진입점</t>
+          <t>App Router, Tailwind 브레이크포인트(md768/lg1024) 매핑, 디자인가이드 토큰(컬러/타이포/spacing) 반영</t>
         </is>
       </c>
       <c r="G67" s="4" t="inlineStr">
@@ -4315,29 +4315,29 @@
       </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
-          <t>FE-01</t>
+          <t>SET-07</t>
         </is>
       </c>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>PRD7-4·IA6.1·디자인가이드6.1</t>
+          <t>설계서4.1.1·디자인가이드</t>
         </is>
       </c>
       <c r="J67" s="3" t="inlineStr">
         <is>
-          <t>3개 브레이크포인트 시각 확인</t>
+          <t>기본 레이아웃 렌더링 확인</t>
         </is>
       </c>
       <c r="K67" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: 3개 브레이크포인트에서 GNB 렌더링 분기(가로바/드로어) 테스트 + Playwright 스모크(클릭 시 드로어 오픈)</t>
+          <t>Vitest+RTL: Tailwind 브레이크포인트 클래스 적용 여부, 디자인 토큰 색상값 매칭 확인</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>FE-03</t>
+          <t>FE-02</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
@@ -4352,17 +4352,17 @@
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>티어리스트</t>
+          <t>공통(GNB)</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>티어리스트(홈) 페이지 구현</t>
+          <t>GNB 컴포넌트 구현</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>필터바/카드그리드/챗봇슬롯, ISR 렌더링, 반응형(3~4열→2열→1열)</t>
+          <t>데스크톱/태블릿 가로바, 모바일 햄버거+드로어, 4개 진입점</t>
         </is>
       </c>
       <c r="G68" s="4" t="inlineStr">
@@ -4372,29 +4372,29 @@
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>FE-02,API-02,API-06</t>
+          <t>FE-01</t>
         </is>
       </c>
       <c r="I68" s="3" t="inlineStr">
         <is>
-          <t>PRD7-1·7-4·화면설계서2.1</t>
+          <t>PRD7-4·IA6.1·디자인가이드6.1</t>
         </is>
       </c>
       <c r="J68" s="3" t="inlineStr">
         <is>
-          <t>데스크톱/태블릿/모바일 와이어프레임 대비 시각 검증</t>
+          <t>3개 브레이크포인트 시각 확인</t>
         </is>
       </c>
       <c r="K68" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: 카드 그리드 컬럼 수 브레이크포인트별 렌더링, mock API 응답 데이터 바인딩 테스트(E2E는 TEST-08)</t>
+          <t>Vitest+RTL: 3개 브레이크포인트에서 GNB 렌더링 분기(가로바/드로어) 테스트 + Playwright 스모크(클릭 시 드로어 오픈)</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>FE-04</t>
+          <t>FE-03</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
@@ -4409,17 +4409,17 @@
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>조합상세</t>
+          <t>티어리스트</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>조합 상세 페이지 구현</t>
+          <t>티어리스트(홈) 페이지 구현</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>개요/챔피언구성(캐리강조)/증강체목록/CTA버튼, 모바일 full-width CTA</t>
+          <t>필터바/카드그리드/챗봇슬롯, ISR 렌더링, 반응형(3~4열→2열→1열)</t>
         </is>
       </c>
       <c r="G69" s="4" t="inlineStr">
@@ -4429,29 +4429,29 @@
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>FE-02,API-03</t>
+          <t>FE-02,API-02,API-06</t>
         </is>
       </c>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>화면설계서2.2</t>
+          <t>PRD7-1·7-4·화면설계서2.1</t>
         </is>
       </c>
       <c r="J69" s="3" t="inlineStr">
         <is>
-          <t>링크이동·반응형 검증</t>
+          <t>데스크톱/태블릿/모바일 와이어프레임 대비 시각 검증</t>
         </is>
       </c>
       <c r="K69" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: 캐리/서브 챔피언 보더 스타일 분기, CTA 버튼 모바일 full-width 렌더링 테스트</t>
+          <t>Vitest+RTL: 카드 그리드 컬럼 수 브레이크포인트별 렌더링, mock API 응답 데이터 바인딩 테스트(E2E는 TEST-08)</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>FE-05</t>
+          <t>FE-04</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
@@ -4466,17 +4466,17 @@
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>아이템빌드</t>
+          <t>조합상세</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>아이템 빌드 페이지 구현</t>
+          <t>조합 상세 페이지 구현</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>챔피언필터/조합리스트/상세패널(모바일 바텀시트)</t>
+          <t>개요/챔피언구성(캐리강조)/증강체목록/CTA버튼, 모바일 full-width CTA</t>
         </is>
       </c>
       <c r="G70" s="4" t="inlineStr">
@@ -4486,29 +4486,29 @@
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>FE-02,API-04</t>
+          <t>FE-02,API-03</t>
         </is>
       </c>
       <c r="I70" s="3" t="inlineStr">
         <is>
-          <t>화면설계서2.3</t>
+          <t>화면설계서2.2</t>
         </is>
       </c>
       <c r="J70" s="3" t="inlineStr">
         <is>
-          <t>필터-URL쿼리 동기화 검증</t>
+          <t>링크이동·반응형 검증</t>
         </is>
       </c>
       <c r="K70" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: 챔피언 필터 선택 시 URL 쿼리 동기화, 모바일 바텀시트 오픈/클로즈 테스트</t>
+          <t>Vitest+RTL: 캐리/서브 챔피언 보더 스타일 분기, CTA 버튼 모바일 full-width 렌더링 테스트</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>FE-06</t>
+          <t>FE-05</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
@@ -4523,17 +4523,17 @@
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>증강체정보</t>
+          <t>아이템빌드</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>증강체 정보 페이지 구현</t>
+          <t>아이템 빌드 페이지 구현</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>티어필터/카드리스트, Legend 승률 숨김 표시</t>
+          <t>챔피언필터/조합리스트/상세패널(모바일 바텀시트)</t>
         </is>
       </c>
       <c r="G71" s="4" t="inlineStr">
@@ -4543,29 +4543,29 @@
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
-          <t>FE-02,API-05</t>
+          <t>FE-02,API-04</t>
         </is>
       </c>
       <c r="I71" s="3" t="inlineStr">
         <is>
-          <t>PRD10-1·화면설계서2.4</t>
+          <t>화면설계서2.3</t>
         </is>
       </c>
       <c r="J71" s="3" t="inlineStr">
         <is>
-          <t>Legend 항목 승률 미노출 확인</t>
+          <t>필터-URL쿼리 동기화 검증</t>
         </is>
       </c>
       <c r="K71" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL(필수·정책): is_legend_related=true 카드에 '승률 표시 안함' 텍스트만 렌더링되고 숫자가 DOM에 없는지 확인</t>
+          <t>Vitest+RTL: 챔피언 필터 선택 시 URL 쿼리 동기화, 모바일 바텀시트 오픈/클로즈 테스트</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>FE-07</t>
+          <t>FE-06</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
@@ -4580,17 +4580,17 @@
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석</t>
+          <t>증강체정보</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>사후 패인 분석 페이지 구현</t>
+          <t>증강체 정보 페이지 구현</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>Riot ID 폼/최근계정목록(localStorage)/전적불러오기 버튼/진행상태</t>
+          <t>티어필터/카드리스트, Legend 승률 숨김 표시</t>
         </is>
       </c>
       <c r="G72" s="4" t="inlineStr">
@@ -4600,29 +4600,29 @@
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>FE-02,API-11,API-12</t>
+          <t>FE-02,API-05</t>
         </is>
       </c>
       <c r="I72" s="3" t="inlineStr">
         <is>
-          <t>PRD8-3·화면설계서2.5</t>
+          <t>PRD10-1·화면설계서2.4</t>
         </is>
       </c>
       <c r="J72" s="3" t="inlineStr">
         <is>
-          <t>로컬스토리지 저장/재사용 확인</t>
+          <t>Legend 항목 승률 미노출 확인</t>
         </is>
       </c>
       <c r="K72" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: localStorage mock 기준 최근 계정 목록 추가/조회/전환 테스트, 폼 검증 에러 메시지 테스트</t>
+          <t>Vitest+RTL(필수·정책): is_legend_related=true 카드에 '승률 표시 안함' 텍스트만 렌더링되고 숫자가 DOM에 없는지 확인</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>FE-08</t>
+          <t>FE-07</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
@@ -4637,17 +4637,17 @@
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>분석리포트</t>
+          <t>사후패인분석</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>분석 리포트 상세 페이지 구현</t>
+          <t>사후 패인 분석 페이지 구현</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>코칭요약/매칭조합카드/등수변화그래프/아이템타임라인</t>
+          <t>Riot ID 폼/최근계정목록(localStorage)/전적불러오기 버튼/진행상태</t>
         </is>
       </c>
       <c r="G73" s="4" t="inlineStr">
@@ -4657,29 +4657,29 @@
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>API-13,FE-02</t>
+          <t>FE-02,API-11,API-12</t>
         </is>
       </c>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>PRD8-3·화면설계서2.6</t>
+          <t>PRD8-3·화면설계서2.5</t>
         </is>
       </c>
       <c r="J73" s="3" t="inlineStr">
         <is>
-          <t>그래프/타임라인 렌더링 확인</t>
+          <t>로컬스토리지 저장/재사용 확인</t>
         </is>
       </c>
       <c r="K73" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: 그래프/타임라인 mock 데이터 렌더링, opponent-info 마스킹 텍스트 렌더링 확인</t>
+          <t>Vitest+RTL: localStorage mock 기준 최근 계정 목록 추가/조회/전환 테스트, 폼 검증 에러 메시지 테스트</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>FE-09</t>
+          <t>FE-08</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
@@ -4694,17 +4694,17 @@
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>챗봇위젯</t>
+          <t>분석리포트</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>챗봇 위젯 전역 컴포넌트 구현</t>
+          <t>분석 리포트 상세 페이지 구현</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>collapsed/expanded, SSE 연동, 모바일 바텀시트 전환, 후속질문칩</t>
+          <t>코칭요약/매칭조합카드/등수변화그래프/아이템타임라인</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr">
@@ -4714,29 +4714,29 @@
       </c>
       <c r="H74" s="3" t="inlineStr">
         <is>
-          <t>FE-01,API-09,CHAT-05</t>
+          <t>API-13,FE-02</t>
         </is>
       </c>
       <c r="I74" s="3" t="inlineStr">
         <is>
-          <t>PRD7-4·화면설계서2.7·디자인가이드6.6</t>
+          <t>PRD8-3·화면설계서2.6</t>
         </is>
       </c>
       <c r="J74" s="3" t="inlineStr">
         <is>
-          <t>전 페이지 삽입 및 반응형 동작 확인</t>
+          <t>그래프/타임라인 렌더링 확인</t>
         </is>
       </c>
       <c r="K74" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: collapsed/expanded 상태 전환, 모바일 바텀시트 전환, mock SSE 스트림 렌더링 테스트</t>
+          <t>Vitest+RTL: 그래프/타임라인 mock 데이터 렌더링, opponent-info 마스킹 텍스트 렌더링 확인</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>FE-10</t>
+          <t>FE-09</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
@@ -4751,49 +4751,49 @@
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>챗봇위젯</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>이미지 최적화 및 반응형 sizes 적용</t>
+          <t>챗봇 위젯 전역 컴포넌트 구현</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>Next Image 컴포넌트, 브레이크포인트별 해상도 서빙</t>
+          <t>collapsed/expanded, SSE 연동, 모바일 바텀시트 전환, 후속질문칩</t>
         </is>
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
-          <t>권장</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
-          <t>FE-03,FE-04,FE-05,FE-06,FE-07,FE-08</t>
+          <t>FE-01,API-09,CHAT-05</t>
         </is>
       </c>
       <c r="I75" s="3" t="inlineStr">
         <is>
-          <t>PRD7-4·설계서4.1.1</t>
+          <t>PRD7-4·화면설계서2.7·디자인가이드6.6</t>
         </is>
       </c>
       <c r="J75" s="3" t="inlineStr">
         <is>
-          <t>모바일 이미지 로딩 성능 확인</t>
+          <t>전 페이지 삽입 및 반응형 동작 확인</t>
         </is>
       </c>
       <c r="K75" s="3" t="inlineStr">
         <is>
-          <t>해당 없음 — Lighthouse 모바일 성능 점수로 갈음(수동 측정)</t>
+          <t>Vitest+RTL: collapsed/expanded 상태 전환, 모바일 바텀시트 전환, mock SSE 스트림 렌더링 테스트</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>FE-11</t>
+          <t>FE-10</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
@@ -4813,44 +4813,44 @@
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>필터 UI 반응형 공용 컴포넌트 구현</t>
+          <t>이미지 최적화 및 반응형 sizes 적용</t>
         </is>
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>데스크톱/태블릿 Dropdown, 모바일 BottomSheet 공용 컴포넌트</t>
+          <t>Next Image 컴포넌트, 브레이크포인트별 해상도 서빙</t>
         </is>
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t>필수</t>
+          <t>권장</t>
         </is>
       </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
-          <t>FE-01</t>
+          <t>FE-03,FE-04,FE-05,FE-06,FE-07,FE-08</t>
         </is>
       </c>
       <c r="I76" s="3" t="inlineStr">
         <is>
-          <t>디자인가이드6.2</t>
+          <t>PRD7-4·설계서4.1.1</t>
         </is>
       </c>
       <c r="J76" s="3" t="inlineStr">
         <is>
-          <t>3개 화면(티어리스트/아이템빌드/증강체)에서 재사용 확인</t>
+          <t>모바일 이미지 로딩 성능 확인</t>
         </is>
       </c>
       <c r="K76" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: 동일 필터 상태를 Dropdown/BottomSheet 두 컴포넌트가 공유하는지 상태 동기화 테스트</t>
+          <t>해당 없음 — Lighthouse 모바일 성능 점수로 갈음(수동 측정)</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>FE-12</t>
+          <t>FE-11</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
@@ -4865,17 +4865,17 @@
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>KPI 대시보드(비공개)</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>KPI 대시보드 페이지 구현(비공개)</t>
+          <t>필터 UI 반응형 공용 컴포넌트 구현</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>/kpi 페이지 — 비밀번호 입력 폼(미인증 시) + 5개 지표 카드/차트(최신성/근거율/전환율/이용률/응답지연). GNB·모바일 드로어에는 노출하지 않음(URL 직접 접근 전용)</t>
+          <t>데스크톱/태블릿 Dropdown, 모바일 BottomSheet 공용 컴포넌트</t>
         </is>
       </c>
       <c r="G77" s="4" t="inlineStr">
@@ -4885,86 +4885,86 @@
       </c>
       <c r="H77" s="3" t="inlineStr">
         <is>
-          <t>KPI-01</t>
+          <t>FE-01</t>
         </is>
       </c>
       <c r="I77" s="3" t="inlineStr">
         <is>
-          <t>IA v1.2 4.7절</t>
+          <t>디자인가이드6.2</t>
         </is>
       </c>
       <c r="J77" s="3" t="inlineStr">
         <is>
-          <t>비밀번호 게이트 통과 후 5개 지표 정상 렌더링 확인, 오답 시 게이트 재노출 확인</t>
+          <t>3개 화면(티어리스트/아이템빌드/증강체)에서 재사용 확인</t>
         </is>
       </c>
       <c r="K77" s="3" t="inlineStr">
         <is>
-          <t>Vitest: 비밀번호 게이트 컴포넌트 성공/실패 케이스, 지표 카드 렌더링 테스트</t>
+          <t>Vitest+RTL: 동일 필터 상태를 Dropdown/BottomSheet 두 컴포넌트가 공유하는지 상태 동기화 테스트</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
+          <t>FE-12</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>프론트엔드</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>KPI 대시보드(비공개)</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>KPI 대시보드 페이지 구현(비공개)</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>/kpi 페이지 — 비밀번호 입력 폼(미인증 시) + 5개 지표 카드/차트(최신성/근거율/전환율/이용률/응답지연). GNB·모바일 드로어에는 노출하지 않음(URL 직접 접근 전용)</t>
+        </is>
+      </c>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
+          <t>필수</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr">
+        <is>
           <t>KPI-01</t>
         </is>
       </c>
-      <c r="B78" s="4" t="inlineStr">
-        <is>
-          <t>코딩</t>
-        </is>
-      </c>
-      <c r="C78" s="4" t="inlineStr">
-        <is>
-          <t>KPI모니터링</t>
-        </is>
-      </c>
-      <c r="D78" s="3" t="inlineStr">
-        <is>
-          <t>공통</t>
-        </is>
-      </c>
-      <c r="E78" s="3" t="inlineStr">
-        <is>
-          <t>KPI 대시보드 백엔드 API 구현(자체, Metabase 대체)</t>
-        </is>
-      </c>
-      <c r="F78" s="3" t="inlineStr">
-        <is>
-          <t>5개 지표(최신성/근거율/전환율/이용률/응답지연) 집계 GET /kpi/summary 구현 + POST /kpi/auth 비밀번호 게이트(환경변수 KPI_DASHBOARD_PASSWORD 대조, 서명 토큰 발급) 구현. Metabase 대신 자체 페이지(FE-12)로 제공 (PM 결정 2026-08-03)</t>
-        </is>
-      </c>
-      <c r="G78" s="4" t="inlineStr">
-        <is>
-          <t>필수</t>
-        </is>
-      </c>
-      <c r="H78" s="3" t="inlineStr">
-        <is>
-          <t>DATA-03</t>
-        </is>
-      </c>
       <c r="I78" s="3" t="inlineStr">
         <is>
-          <t>PRD 3-3 / IA v1.2 4.7절 (자체구현 결정 2026-08-03)</t>
+          <t>IA v1.2 4.7절</t>
         </is>
       </c>
       <c r="J78" s="3" t="inlineStr">
         <is>
-          <t>5개 지표 API 정상 응답 확인, 비밀번호 게이트 통과/실패 동작 확인</t>
+          <t>비밀번호 게이트 통과 후 5개 지표 정상 렌더링 확인, 오답 시 게이트 재노출 확인</t>
         </is>
       </c>
       <c r="K78" s="3" t="inlineStr">
         <is>
-          <t>pytest: 비밀번호 게이트 성공/실패 케이스, mock 로그 데이터로 5개 지표 집계 쿼리 결과 검증</t>
+          <t>Vitest: 비밀번호 게이트 컴포넌트 성공/실패 케이스, 지표 카드 렌더링 테스트</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>KPI-02</t>
+          <t>KPI-01</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
@@ -4984,12 +4984,12 @@
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>RAGAS 주간 배치 평가 파이프라인 구현</t>
+          <t>KPI 대시보드 백엔드 API 구현(자체, Metabase 대체)</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>GitHub Actions 주간 배치로 Faithfulness/Answer Relevancy 산출, ragas_eval_results 적재</t>
+          <t>5개 지표(최신성/근거율/전환율/이용률/응답지연) 집계 GET /kpi/summary 구현 + POST /kpi/auth 비밀번호 게이트(환경변수 KPI_DASHBOARD_PASSWORD 대조, 서명 토큰 발급) 구현. Metabase 대신 자체 페이지(FE-12)로 제공 (PM 결정 2026-08-03)</t>
         </is>
       </c>
       <c r="G79" s="4" t="inlineStr">
@@ -4999,143 +4999,143 @@
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
-          <t>CHAT-09,SET-08</t>
+          <t>DATA-03</t>
         </is>
       </c>
       <c r="I79" s="3" t="inlineStr">
         <is>
-          <t>PRD3-3·설계서4.7</t>
+          <t>PRD 3-3 / IA v1.2 4.7절 (자체구현 결정 2026-08-03)</t>
         </is>
       </c>
       <c r="J79" s="3" t="inlineStr">
         <is>
-          <t>배치 실행 후 결과 적재 확인</t>
+          <t>5개 지표 API 정상 응답 확인, 비밀번호 게이트 통과/실패 동작 확인</t>
         </is>
       </c>
       <c r="K79" s="3" t="inlineStr">
         <is>
-          <t>pytest: mock 질의-답변 샘플로 RAGAS 스코어러 호출 및 ragas_eval_results 적재 필드 확인</t>
+          <t>pytest: 비밀번호 게이트 성공/실패 케이스, mock 로그 데이터로 5개 지표 집계 쿼리 결과 검증</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
+          <t>KPI-02</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>KPI모니터링</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>공통</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>RAGAS 주간 배치 평가 파이프라인 구현</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>GitHub Actions 주간 배치로 Faithfulness/Answer Relevancy 산출, ragas_eval_results 적재</t>
+        </is>
+      </c>
+      <c r="G80" s="4" t="inlineStr">
+        <is>
+          <t>필수</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="inlineStr">
+        <is>
+          <t>CHAT-09,SET-08</t>
+        </is>
+      </c>
+      <c r="I80" s="3" t="inlineStr">
+        <is>
+          <t>PRD3-3·설계서4.7</t>
+        </is>
+      </c>
+      <c r="J80" s="3" t="inlineStr">
+        <is>
+          <t>배치 실행 후 결과 적재 확인</t>
+        </is>
+      </c>
+      <c r="K80" s="3" t="inlineStr">
+        <is>
+          <t>pytest: mock 질의-답변 샘플로 RAGAS 스코어러 호출 및 ragas_eval_results 적재 필드 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
           <t>KPI-03</t>
         </is>
       </c>
-      <c r="B80" s="4" t="inlineStr">
-        <is>
-          <t>코딩</t>
-        </is>
-      </c>
-      <c r="C80" s="4" t="inlineStr">
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
         <is>
           <t>KPI모니터링</t>
         </is>
       </c>
-      <c r="D80" s="3" t="inlineStr">
+      <c r="D81" s="3" t="inlineStr">
         <is>
           <t>공통</t>
         </is>
       </c>
-      <c r="E80" s="3" t="inlineStr">
+      <c r="E81" s="3" t="inlineStr">
         <is>
           <t>목표 미달 알림 로직 구현</t>
         </is>
       </c>
-      <c r="F80" s="3" t="inlineStr">
+      <c r="F81" s="3" t="inlineStr">
         <is>
           <t>2주 연속 목표 미달 감지 시 알림 발송</t>
         </is>
       </c>
-      <c r="G80" s="4" t="inlineStr">
+      <c r="G81" s="4" t="inlineStr">
         <is>
           <t>권장</t>
         </is>
       </c>
-      <c r="H80" s="3" t="inlineStr">
+      <c r="H81" s="3" t="inlineStr">
         <is>
           <t>KPI-01</t>
         </is>
       </c>
-      <c r="I80" s="3" t="inlineStr">
+      <c r="I81" s="3" t="inlineStr">
         <is>
           <t>PRD3-3</t>
         </is>
       </c>
-      <c r="J80" s="3" t="inlineStr">
+      <c r="J81" s="3" t="inlineStr">
         <is>
           <t>알림 트리거 테스트 통과</t>
         </is>
       </c>
-      <c r="K80" s="3" t="inlineStr">
+      <c r="K81" s="3" t="inlineStr">
         <is>
           <t>pytest: 2주 연속 미달 mock 데이터 주입 시 알림 함수 호출 확인</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="5" t="inlineStr">
-        <is>
-          <t>TEST-00</t>
-        </is>
-      </c>
-      <c r="B81" s="5" t="inlineStr">
-        <is>
-          <t>테스트</t>
-        </is>
-      </c>
-      <c r="C81" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D81" s="3" t="inlineStr">
-        <is>
-          <t>공통(정책·로직 크리티컬 TASK)</t>
-        </is>
-      </c>
-      <c r="E81" s="3" t="inlineStr">
-        <is>
-          <t>핵심 정책/로직 테스트 시나리오 사전 정의</t>
-        </is>
-      </c>
-      <c r="F81" s="3" t="inlineStr">
-        <is>
-          <t>API-05, CHAT-04, CHAT-06, PGA-04~09, DATA-13 등 정책 준수·크리티컬 계산 로직이 걸린 TASK에 한해, 코딩 착수 전 입력값·기대출력·경계값을 포함한 테스트 시나리오를 문서화하고 PM과 합의한다. 해당 TASK의 구현자는 이 문서를 기준으로 단위 테스트를 먼저 작성한 뒤 구현한다</t>
-        </is>
-      </c>
-      <c r="G81" s="5" t="inlineStr">
-        <is>
-          <t>필수</t>
-        </is>
-      </c>
-      <c r="H81" s="3" t="inlineStr">
-        <is>
-          <t>SET-01</t>
-        </is>
-      </c>
-      <c r="I81" s="3" t="inlineStr">
-        <is>
-          <t>요구사항정의서 NFR-SEC·FR-PGA, 설계서 4.4.2·4.4.3·4.5.1·4.5.2</t>
-        </is>
-      </c>
-      <c r="J81" s="3" t="inlineStr">
-        <is>
-          <t>/docs/test-scenarios.md에 대상 TASK별 시나리오 표 작성 및 PM 승인 완료</t>
-        </is>
-      </c>
-      <c r="K81" s="3" t="inlineStr">
-        <is>
-          <t>해당 TASK 자체가 산출물 — /docs/test-scenarios.md 표 작성</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>TEST-01</t>
+          <t>TEST-00</t>
         </is>
       </c>
       <c r="B82" s="5" t="inlineStr">
@@ -5150,17 +5150,17 @@
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>공통(정책·로직 크리티컬 TASK)</t>
         </is>
       </c>
       <c r="E82" s="3" t="inlineStr">
         <is>
-          <t>DB 스키마/마이그레이션 검증</t>
+          <t>핵심 정책/로직 테스트 시나리오 사전 정의</t>
         </is>
       </c>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>전체 테이블·인덱스·제약조건 검증</t>
+          <t>API-05, CHAT-04, CHAT-06, PGA-04~09, DATA-13 등 정책 준수·크리티컬 계산 로직이 걸린 TASK에 한해, 코딩 착수 전 입력값·기대출력·경계값을 포함한 테스트 시나리오를 문서화하고 PM과 합의한다. 해당 TASK의 구현자는 이 문서를 기준으로 단위 테스트를 먼저 작성한 뒤 구현한다</t>
         </is>
       </c>
       <c r="G82" s="5" t="inlineStr">
@@ -5170,29 +5170,29 @@
       </c>
       <c r="H82" s="3" t="inlineStr">
         <is>
-          <t>DATA-01,DATA-02,DATA-03,DATA-04</t>
+          <t>SET-01</t>
         </is>
       </c>
       <c r="I82" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>요구사항정의서 NFR-SEC·FR-PGA, 설계서 4.4.2·4.4.3·4.5.1·4.5.2</t>
         </is>
       </c>
       <c r="J82" s="3" t="inlineStr">
         <is>
-          <t>마이그레이션 재실행 무결성 확인</t>
+          <t>/docs/test-scenarios.md에 대상 TASK별 시나리오 표 작성 및 PM 승인 완료</t>
         </is>
       </c>
       <c r="K82" s="3" t="inlineStr">
         <is>
-          <t>해당 TASK 자체가 테스트 작성/실행 TASK의 산출물</t>
+          <t>해당 TASK 자체가 산출물 — /docs/test-scenarios.md 표 작성</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>TEST-02</t>
+          <t>TEST-01</t>
         </is>
       </c>
       <c r="B83" s="5" t="inlineStr">
@@ -5207,17 +5207,17 @@
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>티어리스트~증강체정보</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>catalog API 단위/통합 테스트</t>
+          <t>DB 스키마/마이그레이션 검증</t>
         </is>
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>API-02~06 엔드포인트 테스트 코드 작성 및 실행</t>
+          <t>전체 테이블·인덱스·제약조건 검증</t>
         </is>
       </c>
       <c r="G83" s="5" t="inlineStr">
@@ -5227,7 +5227,7 @@
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>API-02,API-03,API-04,API-05,API-06</t>
+          <t>DATA-01,DATA-02,DATA-03,DATA-04</t>
         </is>
       </c>
       <c r="I83" s="3" t="inlineStr">
@@ -5237,7 +5237,7 @@
       </c>
       <c r="J83" s="3" t="inlineStr">
         <is>
-          <t>전체 테스트 통과</t>
+          <t>마이그레이션 재실행 무결성 확인</t>
         </is>
       </c>
       <c r="K83" s="3" t="inlineStr">
@@ -5249,7 +5249,7 @@
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>TEST-03</t>
+          <t>TEST-02</t>
         </is>
       </c>
       <c r="B84" s="5" t="inlineStr">
@@ -5264,17 +5264,17 @@
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>챗봇위젯</t>
+          <t>티어리스트~증강체정보</t>
         </is>
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>chat API 및 RAG 파이프라인 테스트</t>
+          <t>catalog API 단위/통합 테스트</t>
         </is>
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>의도분류/검색/생성/후처리/캐싱 테스트</t>
+          <t>API-02~06 엔드포인트 테스트 코드 작성 및 실행</t>
         </is>
       </c>
       <c r="G84" s="5" t="inlineStr">
@@ -5284,7 +5284,7 @@
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
-          <t>CHAT-01,CHAT-02,CHAT-03,CHAT-04,CHAT-05,CHAT-06,CHAT-07,CHAT-08,CHAT-09</t>
+          <t>API-02,API-03,API-04,API-05,API-06</t>
         </is>
       </c>
       <c r="I84" s="3" t="inlineStr">
@@ -5294,7 +5294,7 @@
       </c>
       <c r="J84" s="3" t="inlineStr">
         <is>
-          <t>전체 통과, 근거율 샘플 검증</t>
+          <t>전체 테스트 통과</t>
         </is>
       </c>
       <c r="K84" s="3" t="inlineStr">
@@ -5306,7 +5306,7 @@
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>TEST-04</t>
+          <t>TEST-03</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr">
@@ -5321,17 +5321,17 @@
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석·분석리포트</t>
+          <t>챗봇위젯</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>analysis API 및 스코어링 로직 테스트</t>
+          <t>chat API 및 RAG 파이프라인 테스트</t>
         </is>
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>PUUID변환/매치조회/3개지표계산/코칭생성 테스트</t>
+          <t>의도분류/검색/생성/후처리/캐싱 테스트</t>
         </is>
       </c>
       <c r="G85" s="5" t="inlineStr">
@@ -5341,7 +5341,7 @@
       </c>
       <c r="H85" s="3" t="inlineStr">
         <is>
-          <t>PGA-01,PGA-02,PGA-03,PGA-04,PGA-05,PGA-06,PGA-07,PGA-08,PGA-09,PGA-10</t>
+          <t>CHAT-01,CHAT-02,CHAT-03,CHAT-04,CHAT-05,CHAT-06,CHAT-07,CHAT-08,CHAT-09</t>
         </is>
       </c>
       <c r="I85" s="3" t="inlineStr">
@@ -5351,7 +5351,7 @@
       </c>
       <c r="J85" s="3" t="inlineStr">
         <is>
-          <t>전체 통과</t>
+          <t>전체 통과, 근거율 샘플 검증</t>
         </is>
       </c>
       <c r="K85" s="3" t="inlineStr">
@@ -5363,7 +5363,7 @@
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>TEST-05</t>
+          <t>TEST-04</t>
         </is>
       </c>
       <c r="B86" s="5" t="inlineStr">
@@ -5378,17 +5378,17 @@
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>사후패인분석·분석리포트</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>배치 파이프라인 통합 테스트</t>
+          <t>analysis API 및 스코어링 로직 테스트</t>
         </is>
       </c>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>패치감지→수집→정규화→임베딩→원자적전환 end-to-end 테스트</t>
+          <t>PUUID변환/매치조회/3개지표계산/코칭생성 테스트</t>
         </is>
       </c>
       <c r="G86" s="5" t="inlineStr">
@@ -5398,7 +5398,7 @@
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
-          <t>DATA-05,DATA-08,DATA-09,DATA-10,DATA-11,DATA-12,DATA-13,DATA-14,DATA-15</t>
+          <t>PGA-01,PGA-02,PGA-03,PGA-04,PGA-05,PGA-06,PGA-07,PGA-08,PGA-09,PGA-10</t>
         </is>
       </c>
       <c r="I86" s="3" t="inlineStr">
@@ -5408,7 +5408,7 @@
       </c>
       <c r="J86" s="3" t="inlineStr">
         <is>
-          <t>정상/중간실패 시나리오 모두 검증</t>
+          <t>전체 통과</t>
         </is>
       </c>
       <c r="K86" s="3" t="inlineStr">
@@ -5420,7 +5420,7 @@
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>TEST-06</t>
+          <t>TEST-05</t>
         </is>
       </c>
       <c r="B87" s="5" t="inlineStr">
@@ -5435,17 +5435,17 @@
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>챗봇위젯</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>챗봇 정책 준수 테스트</t>
+          <t>배치 파이프라인 통합 테스트</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>Legend 승률 비노출·프롬프트 인젝션 방어·범위밖 질문 안내 검증</t>
+          <t>패치감지→수집→정규화→임베딩→원자적전환 end-to-end 테스트</t>
         </is>
       </c>
       <c r="G87" s="5" t="inlineStr">
@@ -5455,17 +5455,17 @@
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
-          <t>CHAT-04,CHAT-06</t>
+          <t>DATA-05,DATA-08,DATA-09,DATA-10,DATA-11,DATA-12,DATA-13,DATA-14,DATA-15</t>
         </is>
       </c>
       <c r="I87" s="3" t="inlineStr">
         <is>
-          <t>PRD10-1·12장</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J87" s="3" t="inlineStr">
         <is>
-          <t>정책 위반 케이스 0건</t>
+          <t>정상/중간실패 시나리오 모두 검증</t>
         </is>
       </c>
       <c r="K87" s="3" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>TEST-07</t>
+          <t>TEST-06</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
@@ -5492,17 +5492,17 @@
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석·분석리포트</t>
+          <t>챗봇위젯</t>
         </is>
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>프라이버시 마스킹 테스트</t>
+          <t>챗봇 정책 준수 테스트</t>
         </is>
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>상대 닉네임 마스킹 누락 케이스 점검</t>
+          <t>Legend 승률 비노출·프롬프트 인젝션 방어·범위밖 질문 안내 검증</t>
         </is>
       </c>
       <c r="G88" s="5" t="inlineStr">
@@ -5512,17 +5512,17 @@
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>PGA-09</t>
+          <t>CHAT-04,CHAT-06</t>
         </is>
       </c>
       <c r="I88" s="3" t="inlineStr">
         <is>
-          <t>PRD7-3·12장</t>
+          <t>PRD10-1·12장</t>
         </is>
       </c>
       <c r="J88" s="3" t="inlineStr">
         <is>
-          <t>마스킹 누락 0건</t>
+          <t>정책 위반 케이스 0건</t>
         </is>
       </c>
       <c r="K88" s="3" t="inlineStr">
@@ -5534,7 +5534,7 @@
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>TEST-08</t>
+          <t>TEST-07</t>
         </is>
       </c>
       <c r="B89" s="5" t="inlineStr">
@@ -5549,17 +5549,17 @@
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>전체 7화면</t>
+          <t>사후패인분석·분석리포트</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>프론트엔드 E2E 테스트(Playwright)</t>
+          <t>프라이버시 마스킹 테스트</t>
         </is>
       </c>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>PRD 8-1/8-2/8-3 사용자 플로우 기준 시나리오 작성</t>
+          <t>상대 닉네임 마스킹 누락 케이스 점검</t>
         </is>
       </c>
       <c r="G89" s="5" t="inlineStr">
@@ -5569,17 +5569,17 @@
       </c>
       <c r="H89" s="3" t="inlineStr">
         <is>
-          <t>FE-03,FE-04,FE-05,FE-06,FE-07,FE-08,FE-09</t>
+          <t>PGA-09</t>
         </is>
       </c>
       <c r="I89" s="3" t="inlineStr">
         <is>
-          <t>PRD8장</t>
+          <t>PRD7-3·12장</t>
         </is>
       </c>
       <c r="J89" s="3" t="inlineStr">
         <is>
-          <t>전체 시나리오 통과</t>
+          <t>마스킹 누락 0건</t>
         </is>
       </c>
       <c r="K89" s="3" t="inlineStr">
@@ -5591,7 +5591,7 @@
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>TEST-09</t>
+          <t>TEST-08</t>
         </is>
       </c>
       <c r="B90" s="5" t="inlineStr">
@@ -5611,12 +5611,12 @@
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>반응형 크로스브라우저 테스트</t>
+          <t>프론트엔드 E2E 테스트(Playwright)</t>
         </is>
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>iOS Safari/Android Chrome/Desktop Chrome 3개 브레이크포인트 검증</t>
+          <t>PRD 8-1/8-2/8-3 사용자 플로우 기준 시나리오 작성</t>
         </is>
       </c>
       <c r="G90" s="5" t="inlineStr">
@@ -5631,12 +5631,12 @@
       </c>
       <c r="I90" s="3" t="inlineStr">
         <is>
-          <t>PRD12장(QA리소스제약)</t>
+          <t>PRD8장</t>
         </is>
       </c>
       <c r="J90" s="3" t="inlineStr">
         <is>
-          <t>주요 화면 시각 회귀 없음 확인</t>
+          <t>전체 시나리오 통과</t>
         </is>
       </c>
       <c r="K90" s="3" t="inlineStr">
@@ -5648,121 +5648,121 @@
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
+          <t>TEST-09</t>
+        </is>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>테스트</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>전체 7화면</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="inlineStr">
+        <is>
+          <t>반응형 크로스브라우저 테스트</t>
+        </is>
+      </c>
+      <c r="F91" s="3" t="inlineStr">
+        <is>
+          <t>iOS Safari/Android Chrome/Desktop Chrome 3개 브레이크포인트 검증</t>
+        </is>
+      </c>
+      <c r="G91" s="5" t="inlineStr">
+        <is>
+          <t>필수</t>
+        </is>
+      </c>
+      <c r="H91" s="3" t="inlineStr">
+        <is>
+          <t>FE-03,FE-04,FE-05,FE-06,FE-07,FE-08,FE-09</t>
+        </is>
+      </c>
+      <c r="I91" s="3" t="inlineStr">
+        <is>
+          <t>PRD12장(QA리소스제약)</t>
+        </is>
+      </c>
+      <c r="J91" s="3" t="inlineStr">
+        <is>
+          <t>주요 화면 시각 회귀 없음 확인</t>
+        </is>
+      </c>
+      <c r="K91" s="3" t="inlineStr">
+        <is>
+          <t>해당 TASK 자체가 테스트 작성/실행 TASK의 산출물</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="5" t="inlineStr">
+        <is>
           <t>TEST-10</t>
         </is>
       </c>
-      <c r="B91" s="5" t="inlineStr">
+      <c r="B92" s="5" t="inlineStr">
         <is>
           <t>테스트</t>
         </is>
       </c>
-      <c r="C91" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D91" s="3" t="inlineStr">
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
         <is>
           <t>공통</t>
         </is>
       </c>
-      <c r="E91" s="3" t="inlineStr">
+      <c r="E92" s="3" t="inlineStr">
         <is>
           <t>Rate Limiting/보안 테스트</t>
         </is>
       </c>
-      <c r="F91" s="3" t="inlineStr">
+      <c r="F92" s="3" t="inlineStr">
         <is>
           <t>요청 한도 초과·비정상 입력 처리 검증</t>
         </is>
       </c>
-      <c r="G91" s="5" t="inlineStr">
+      <c r="G92" s="5" t="inlineStr">
         <is>
           <t>권장</t>
         </is>
       </c>
-      <c r="H91" s="3" t="inlineStr">
+      <c r="H92" s="3" t="inlineStr">
         <is>
           <t>API-07</t>
         </is>
       </c>
-      <c r="I91" s="3" t="inlineStr">
+      <c r="I92" s="3" t="inlineStr">
         <is>
           <t>설계서4.2·6장</t>
         </is>
       </c>
-      <c r="J91" s="3" t="inlineStr">
+      <c r="J92" s="3" t="inlineStr">
         <is>
           <t>429 응답 및 로그 확인</t>
         </is>
       </c>
-      <c r="K91" s="3" t="inlineStr">
+      <c r="K92" s="3" t="inlineStr">
         <is>
           <t>해당 TASK 자체가 테스트 작성/실행 TASK의 산출물</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="6" t="inlineStr">
-        <is>
-          <t>REL-01</t>
-        </is>
-      </c>
-      <c r="B92" s="6" t="inlineStr">
-        <is>
-          <t>배포릴리즈</t>
-        </is>
-      </c>
-      <c r="C92" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D92" s="3" t="inlineStr">
-        <is>
-          <t>전체</t>
-        </is>
-      </c>
-      <c r="E92" s="3" t="inlineStr">
-        <is>
-          <t>스테이징 통합 배포 및 QA</t>
-        </is>
-      </c>
-      <c r="F92" s="3" t="inlineStr">
-        <is>
-          <t>전체 기능 스테이징 환경 배포 후 PM 검수</t>
-        </is>
-      </c>
-      <c r="G92" s="6" t="inlineStr">
-        <is>
-          <t>필수</t>
-        </is>
-      </c>
-      <c r="H92" s="3" t="inlineStr">
-        <is>
-          <t>TEST-01,TEST-02,TEST-03,TEST-04,TEST-05,TEST-06,TEST-07,TEST-08,TEST-09</t>
-        </is>
-      </c>
-      <c r="I92" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J92" s="3" t="inlineStr">
-        <is>
-          <t>PM 승인 획득</t>
-        </is>
-      </c>
-      <c r="K92" s="3" t="inlineStr">
-        <is>
-          <t>TEST-00~10 전체 그린 상태를 배포 전제조건으로 확인</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>REL-02</t>
+          <t>REL-01</t>
         </is>
       </c>
       <c r="B93" s="6" t="inlineStr">
@@ -5782,12 +5782,12 @@
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>프로덕션 배포</t>
+          <t>스테이징 통합 배포 및 QA</t>
         </is>
       </c>
       <c r="F93" s="3" t="inlineStr">
         <is>
-          <t>Cloudflare Pages+Render 프로덕션 반영, PM 최종 승인 후 커밋/푸시</t>
+          <t>전체 기능 스테이징 환경 배포 후 PM 검수</t>
         </is>
       </c>
       <c r="G93" s="6" t="inlineStr">
@@ -5797,7 +5797,7 @@
       </c>
       <c r="H93" s="3" t="inlineStr">
         <is>
-          <t>REL-01</t>
+          <t>TEST-01,TEST-02,TEST-03,TEST-04,TEST-05,TEST-06,TEST-07,TEST-08,TEST-09</t>
         </is>
       </c>
       <c r="I93" s="3" t="inlineStr">
@@ -5807,19 +5807,19 @@
       </c>
       <c r="J93" s="3" t="inlineStr">
         <is>
-          <t>프로덕션 URL 정상 서비스 확인</t>
+          <t>PM 승인 획득</t>
         </is>
       </c>
       <c r="K93" s="3" t="inlineStr">
         <is>
-          <t>프로덕션 스모크 테스트: 핵심 URL 200 확인, 챗봇 질의 1회 왕복 확인</t>
+          <t>TEST-00~10 전체 그린 상태를 배포 전제조건으로 확인</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>REL-03</t>
+          <t>REL-02</t>
         </is>
       </c>
       <c r="B94" s="6" t="inlineStr">
@@ -5834,17 +5834,17 @@
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>전체</t>
         </is>
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>배포 후 모니터링 점검</t>
+          <t>프로덕션 배포</t>
         </is>
       </c>
       <c r="F94" s="3" t="inlineStr">
         <is>
-          <t>콜드스타트 비중·응답지연 p50/p95 확인</t>
+          <t>Cloudflare Pages+Render 프로덕션 반영, PM 최종 승인 후 커밋/푸시</t>
         </is>
       </c>
       <c r="G94" s="6" t="inlineStr">
@@ -5854,29 +5854,29 @@
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>REL-02,KPI-01</t>
+          <t>REL-01</t>
         </is>
       </c>
       <c r="I94" s="3" t="inlineStr">
         <is>
-          <t>PRD3-3</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J94" s="3" t="inlineStr">
         <is>
-          <t>초기 1주 지표 리뷰 완료</t>
+          <t>프로덕션 URL 정상 서비스 확인</t>
         </is>
       </c>
       <c r="K94" s="3" t="inlineStr">
         <is>
-          <t>해당 없음 — 모니터링 지표 수동 리뷰</t>
+          <t>프로덕션 스모크 테스트: 핵심 URL 200 확인, 챗봇 질의 1회 왕복 확인</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>REL-04</t>
+          <t>REL-03</t>
         </is>
       </c>
       <c r="B95" s="6" t="inlineStr">
@@ -5896,92 +5896,149 @@
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>1.0 출시 회고 및 KPI 재보정 계획 수립</t>
+          <t>배포 후 모니터링 점검</t>
         </is>
       </c>
       <c r="F95" s="3" t="inlineStr">
         <is>
-          <t>2~4주 실측 데이터 수집 계획 및 재보정 일정 수립</t>
+          <t>콜드스타트 비중·응답지연 p50/p95 확인</t>
         </is>
       </c>
       <c r="G95" s="6" t="inlineStr">
         <is>
-          <t>권장</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="H95" s="3" t="inlineStr">
         <is>
-          <t>REL-03</t>
+          <t>REL-02,KPI-01</t>
         </is>
       </c>
       <c r="I95" s="3" t="inlineStr">
         <is>
-          <t>PRD3-2·3-3</t>
+          <t>PRD3-3</t>
         </is>
       </c>
       <c r="J95" s="3" t="inlineStr">
         <is>
-          <t>재보정 일정 문서화</t>
+          <t>초기 1주 지표 리뷰 완료</t>
         </is>
       </c>
       <c r="K95" s="3" t="inlineStr">
         <is>
-          <t>해당 없음 — 문서화 작업</t>
+          <t>해당 없음 — 모니터링 지표 수동 리뷰</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="6" t="inlineStr">
         <is>
+          <t>REL-04</t>
+        </is>
+      </c>
+      <c r="B96" s="6" t="inlineStr">
+        <is>
+          <t>배포릴리즈</t>
+        </is>
+      </c>
+      <c r="C96" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>공통</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>1.0 출시 회고 및 KPI 재보정 계획 수립</t>
+        </is>
+      </c>
+      <c r="F96" s="3" t="inlineStr">
+        <is>
+          <t>2~4주 실측 데이터 수집 계획 및 재보정 일정 수립</t>
+        </is>
+      </c>
+      <c r="G96" s="6" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H96" s="3" t="inlineStr">
+        <is>
+          <t>REL-03</t>
+        </is>
+      </c>
+      <c r="I96" s="3" t="inlineStr">
+        <is>
+          <t>PRD3-2·3-3</t>
+        </is>
+      </c>
+      <c r="J96" s="3" t="inlineStr">
+        <is>
+          <t>재보정 일정 문서화</t>
+        </is>
+      </c>
+      <c r="K96" s="3" t="inlineStr">
+        <is>
+          <t>해당 없음 — 문서화 작업</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="6" t="inlineStr">
+        <is>
           <t>REL-05</t>
         </is>
       </c>
-      <c r="B96" s="6" t="inlineStr">
+      <c r="B97" s="6" t="inlineStr">
         <is>
           <t>배포릴리즈</t>
         </is>
       </c>
-      <c r="C96" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D96" s="3" t="inlineStr">
+      <c r="C97" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
         <is>
           <t>전체</t>
         </is>
       </c>
-      <c r="E96" s="3" t="inlineStr">
+      <c r="E97" s="3" t="inlineStr">
         <is>
           <t>포트폴리오 공개 전환 준비 체크리스트</t>
         </is>
       </c>
-      <c r="F96" s="3" t="inlineStr">
+      <c r="F97" s="3" t="inlineStr">
         <is>
           <t>저장소를 private에서 public으로 전환하기 전 확인·조치한다: (1) gitleaks 등으로 커밋 히스토리 전체에서 시크릿·API 키 잔존 여부 스캔 (2) 테스트 fixture 전수 조사 — 실제 Riot ID/PUUID/닉네임/매치 데이터가 아닌 합성 데이터로만 구성됐는지 확인, 실데이터가 섞여 있으면 fixture 재작성 후 필요시 git 히스토리 정리 (3) README에 'Riot Games와 무관한 비공식 팬 프로젝트' 디스클레이머 추가 (4) 라이브 배포 URL을 README/공개 자료에 노출할지 결정 (5) 노출하기로 하면 챗봇/전적조회 진입점에 Cloudflare Turnstile 등 경량 봇 방지 적용 검토. 무료 호스팅 비용에는 영향 없음(저장소 공개 여부와 인프라 비용은 무관)</t>
         </is>
       </c>
-      <c r="G96" s="6" t="inlineStr">
+      <c r="G97" s="6" t="inlineStr">
         <is>
           <t>권장</t>
         </is>
       </c>
-      <c r="H96" s="3" t="inlineStr">
+      <c r="H97" s="3" t="inlineStr">
         <is>
           <t>REL-04</t>
         </is>
       </c>
-      <c r="I96" s="3" t="inlineStr">
+      <c r="I97" s="3" t="inlineStr">
         <is>
           <t>PM 결정사항(2026-07-30 대화), policies.md 11번</t>
         </is>
       </c>
-      <c r="J96" s="3" t="inlineStr">
+      <c r="J97" s="3" t="inlineStr">
         <is>
           <t>체크리스트 5개 항목 모두 확인·조치 완료 및 PM 승인 후 저장소 visibility를 public으로 변경</t>
         </is>
       </c>
-      <c r="K96" s="3" t="inlineStr">
+      <c r="K97" s="3" t="inlineStr">
         <is>
           <t>정량 검증: gitleaks(또는 동급 도구) 스캔 결과 시크릿 탐지 0건, 전체 fixture 파일에서 실제 Riot ID 패턴(게임명#태그)·PUUID 패턴 검색 결과 0건</t>
         </is>

</xml_diff>

<commit_message>
docs(DATA-05): DATA-05 완료 처리(PM 승인), tft_get_play_style을 PGA-07로 재배치
PM 결정 3가지 반영: (1) DATA-12 패치 감지는
tft_list_item_combinations.version 기준으로 확정, (2) DATA-07은
op.gg 라벨 없음 확정으로 수동 목록 방식 확정, (3) tft_get_play_style
(PUUID 필수)은 DATA-08에서 제외하고 PGA-07로 이동. WBS.xlsx
DATA-08/PGA-07 TASK 설명, glossary.md/api-spec.md의 "개인 전적 조회
기능 없음" 문구 갱신.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TFT_Hideout_WBS.xlsx
+++ b/TFT_Hideout_WBS.xlsx
@@ -1911,7 +1911,7 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>6개 도구 순차 호출 클라이언트 구현</t>
+          <t>5개 도구 순차 호출 클라이언트 구현(tft_get_play_style은 PUUID 필수라 PGA-07로 이동, 2026-08-04 PM 결정)</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -4077,7 +4077,7 @@
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>3개 지표+등수 근거로 잘한점/아쉬운점/제안 고정구조 생성, 수치 비노출</t>
+          <t>3개 지표+등수 근거로 잘한점/아쉬운점/제안 고정구조 생성, 수치 비노출. op.gg tft_get_play_style(PUUID 필요, DATA-08에서 이동)을 호출해 코칭 근거로 활용</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr">

</xml_diff>

<commit_message>
docs(CHAT-08): CHAT-08 완료 처리(PM 승인), FE-03 ISR->CSR 결정 반영
CHAT 그룹(01~09) 전체 완료.

WBS FE-03 TASK 설명의 "ISR 렌더링"이 FE-01의 정적 export 결정과
모순되던 걸 해소 — ISR은 서버 런타임이 필요해 정적 export와 양립
불가하고 Cloudflare 정적 Worker(SET-07)와도 안 맞음. 티어리스트
데이터는 배치가 하루 1회 갱신하므로 ISR/빌드시점고정 둘 다 완전한
최신성을 보장 못 해, 정적 export + 클라이언트 사이드 fetch(CSR)로
확정(TFT_Hideout_WBS.xlsx F69 갱신, diff 1셀만).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TFT_Hideout_WBS.xlsx
+++ b/TFT_Hideout_WBS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="WBS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="요약" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'WBS'!$A$1:$K$95</definedName>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>필터바/카드그리드/챗봇슬롯, ISR 렌더링, 반응형(3~4열→2열→1열)</t>
+          <t>필터바/카드그리드/챗봇슬롯, 정적 export(FE-01 결정) + 클라이언트 사이드 fetch(CSR), 반응형(3~4열→2열→1열)</t>
         </is>
       </c>
       <c r="G69" s="4" t="inlineStr">

</xml_diff>

<commit_message>
docs(FE-06): FE-06 완료 처리(PM 승인) 및 DATA-16 신규 TASK 추가
FE-06 실데이터 검증 중 발견한 증강체 설명 템플릿 플레이스홀더
(<br> 리터럴·미해석 @TFTUnitProperty...@) 정리를 PM 결정으로 별도
TASK 분리 — DATA-16(권장, 선행TASK DATA-08) 신설. WBS.xlsx·
진행현황.md 동시 반영, 전체 97개 TASK(활성 94개).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TFT_Hideout_WBS.xlsx
+++ b/TFT_Hideout_WBS.xlsx
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K97"/>
+  <dimension ref="A1:K98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2342,7 +2342,7 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>API-01</t>
+          <t>DATA-16</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
@@ -2352,54 +2352,54 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>백엔드API</t>
+          <t>데이터파이프라인</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>증강체정보</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>FastAPI 프로젝트 스캐폴딩</t>
+          <t>증강체 설명 템플릿 플레이스홀더 정리</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>단일 앱 + catalog/chat/analysis/kpi 4개 라우터 구조(kpi는 SET-11 취소로 Metabase 대신 자체 KPI 대시보드 백엔드용으로 v1.7에서 추가), 헬스체크 엔드포인트</t>
+          <t>op.gg 증강체(augments) 설명 원문에 남아있는 &lt;br&gt; 리터럴 태그와 @TFTUnitProperty...@ 형태의 미해석 수치 템플릿을 실제 표시 가능한 형태로 정리(치환 또는 안전한 스트립). FE-06 실데이터 검증 중 발견 — 해당 텍스트가 줄바꿈 없이 길게 남아 모바일 레이아웃 뷰포트 팽창 버그의 원인이기도 했음(FE-06에서 wrap-break-word로 레이아웃 증상은 우선 보정, 텍스트 자체는 원문 그대로).</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>필수</t>
+          <t>권장</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>SET-02,SET-03</t>
+          <t>DATA-08</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.2</t>
+          <t>docs/verification/FE-06-작업결과.md(2026-08-05 발견)</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>/health 200 응답 확인</t>
+          <t>증강체 설명에 &lt;br&gt; 리터럴 문자열·미해석 @...@ 템플릿이 노출되지 않음</t>
         </is>
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>pytest+FastAPI TestClient: /health 200 및 4개 라우터(catalog/chat/analysis/kpi) 마운트 확인</t>
+          <t>pytest: 정규화된 augment description에 &lt;br&gt;·@...@ 템플릿 패턴이 남지 않는지 확인</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>API-02</t>
+          <t>API-01</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -2414,17 +2414,17 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>티어리스트</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>GET /catalog/tierlist 구현</t>
+          <t>FastAPI 프로젝트 스캐폴딩</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>패치·랭크 필터 지원, comps 테이블 SQL 조회</t>
+          <t>단일 앱 + catalog/chat/analysis/kpi 4개 라우터 구조(kpi는 SET-11 취소로 Metabase 대신 자체 KPI 대시보드 백엔드용으로 v1.7에서 추가), 헬스체크 엔드포인트</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -2434,29 +2434,29 @@
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>DATA-02,API-01</t>
+          <t>SET-02,SET-03</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>PRD 7-1·설계서6장</t>
+          <t>설계서 4.2</t>
         </is>
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>응답 스키마·필터 동작 확인</t>
+          <t>/health 200 응답 확인</t>
         </is>
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t>pytest: 패치/랭크 필터 조합별 응답, 빈 결과, 잘못된 파라미터 400 케이스</t>
+          <t>pytest+FastAPI TestClient: /health 200 및 4개 라우터(catalog/chat/analysis/kpi) 마운트 확인</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>API-03</t>
+          <t>API-02</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
@@ -2471,17 +2471,17 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>조합상세</t>
+          <t>티어리스트</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>GET /catalog/comps/{comp_id} 구현</t>
+          <t>GET /catalog/tierlist 구현</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>챔피언구성·증강체 우선순위 포함</t>
+          <t>패치·랭크 필터 지원, comps 테이블 SQL 조회</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -2496,24 +2496,24 @@
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>설계서 5.1·6장</t>
+          <t>PRD 7-1·설계서6장</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>응답 필드 검증</t>
+          <t>응답 스키마·필터 동작 확인</t>
         </is>
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>pytest: 존재/미존재 comp_id 케이스, 캐리/서브 챔피언 구분 필드 정확성</t>
+          <t>pytest: 패치/랭크 필터 조합별 응답, 빈 결과, 잘못된 파라미터 400 케이스</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>API-04</t>
+          <t>API-03</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -2528,17 +2528,17 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>아이템빌드</t>
+          <t>조합상세</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>GET /catalog/items/builds 구현</t>
+          <t>GET /catalog/comps/{comp_id} 구현</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>챔피언 필터 지원</t>
+          <t>챔피언구성·증강체 우선순위 포함</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -2553,7 +2553,7 @@
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>설계서 6장</t>
+          <t>설계서 5.1·6장</t>
         </is>
       </c>
       <c r="J36" s="3" t="inlineStr">
@@ -2563,14 +2563,14 @@
       </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
-          <t>pytest: champion_id 필터 유무 케이스, 정렬 순서 검증</t>
+          <t>pytest: 존재/미존재 comp_id 케이스, 캐리/서브 챔피언 구분 필드 정확성</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>API-05</t>
+          <t>API-04</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
@@ -2585,17 +2585,17 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>증강체정보</t>
+          <t>아이템빌드</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>GET /catalog/augments 구현</t>
+          <t>GET /catalog/items/builds 구현</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>is_legend_related=true 승률 마스킹 포함</t>
+          <t>챔피언 필터 지원</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -2605,29 +2605,29 @@
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>DATA-07,API-01</t>
+          <t>DATA-02,API-01</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>PRD 10-1·설계서4.4.3</t>
+          <t>설계서 6장</t>
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
-          <t>마스킹 동작 단위 테스트 통과</t>
+          <t>응답 필드 검증</t>
         </is>
       </c>
       <c r="K37" s="3" t="inlineStr">
         <is>
-          <t>pytest(필수·정책, TEST-00 시나리오 선적용): is_legend_related=true 데이터로 응답에 win_rate 필드 자체가 없는지(=null 아님) 검증</t>
+          <t>pytest: champion_id 필터 유무 케이스, 정렬 순서 검증</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>API-06</t>
+          <t>API-05</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
@@ -2642,17 +2642,17 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>공통(GNB)</t>
+          <t>증강체정보</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>GET /catalog/patches/current 구현</t>
+          <t>GET /catalog/augments 구현</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>현재 패치 조회</t>
+          <t>is_legend_related=true 승률 마스킹 포함</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -2662,29 +2662,29 @@
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>DATA-01,API-01</t>
+          <t>DATA-07,API-01</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>설계서 6장</t>
+          <t>PRD 10-1·설계서4.4.3</t>
         </is>
       </c>
       <c r="J38" s="3" t="inlineStr">
         <is>
-          <t>응답 검증</t>
+          <t>마스킹 동작 단위 테스트 통과</t>
         </is>
       </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
-          <t>pytest: is_current=true 패치 1건만 반환되는지 확인</t>
+          <t>pytest(필수·정책, TEST-00 시나리오 선적용): is_legend_related=true 데이터로 응답에 win_rate 필드 자체가 없는지(=null 아님) 검증</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>API-07</t>
+          <t>API-06</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
@@ -2699,17 +2699,17 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>공통(GNB)</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Rate Limiting 미들웨어 구현</t>
+          <t>GET /catalog/patches/current 구현</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>IP 기준 catalog 분당60/chat 분당10</t>
+          <t>현재 패치 조회</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
@@ -2719,29 +2719,29 @@
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>API-01</t>
+          <t>DATA-01,API-01</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.2·6장</t>
+          <t>설계서 6장</t>
         </is>
       </c>
       <c r="J39" s="3" t="inlineStr">
         <is>
-          <t>초과 요청 429 응답 확인</t>
+          <t>응답 검증</t>
         </is>
       </c>
       <c r="K39" s="3" t="inlineStr">
         <is>
-          <t>pytest: 한도 초과 요청 시 429 응답 확인(catalog 60/분, chat 10/분 각각)</t>
+          <t>pytest: is_current=true 패치 1건만 반환되는지 확인</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>API-08</t>
+          <t>API-07</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
@@ -2756,17 +2756,17 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>챗봇위젯</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>session_id 발급/조회 로직 구현</t>
+          <t>Rate Limiting 미들웨어 구현</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>클라이언트 UUID 수신 및 대화 묶음 키로 사용</t>
+          <t>IP 기준 catalog 분당60/chat 분당10</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
@@ -2781,24 +2781,24 @@
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.2</t>
+          <t>설계서 4.2·6장</t>
         </is>
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>세션별 대화 구분 확인</t>
+          <t>초과 요청 429 응답 확인</t>
         </is>
       </c>
       <c r="K40" s="3" t="inlineStr">
         <is>
-          <t>pytest: 동일 session_id 재사용 시 동일 대화로 묶이는지, 신규 UUID는 분리되는지 확인</t>
+          <t>pytest: 한도 초과 요청 시 429 응답 확인(catalog 60/분, chat 10/분 각각)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>API-09</t>
+          <t>API-08</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
@@ -2818,12 +2818,12 @@
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>POST /chat/message 뼈대 구현(SSE)</t>
+          <t>session_id 발급/조회 로직 구현</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>스트리밍 응답 인프라 구현(RAG 로직은 CHAT 그룹에서 연동)</t>
+          <t>클라이언트 UUID 수신 및 대화 묶음 키로 사용</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
@@ -2833,29 +2833,29 @@
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>API-08</t>
+          <t>API-01</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.2·4.4</t>
+          <t>설계서 4.2</t>
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>SSE 스트림 클라이언트 수신 확인</t>
+          <t>세션별 대화 구분 확인</t>
         </is>
       </c>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>pytest: SSE 스트림 청크 수신 순서 및 연결 종료 처리 확인(mock LLM 스트림)</t>
+          <t>pytest: 동일 session_id 재사용 시 동일 대화로 묶이는지, 신규 UUID는 분리되는지 확인</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>API-10</t>
+          <t>API-09</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
@@ -2875,12 +2875,12 @@
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>GET /chat/session/{id}/history 구현</t>
+          <t>POST /chat/message 뼈대 구현(SSE)</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>chat_logs 기반 대화이력 조회</t>
+          <t>스트리밍 응답 인프라 구현(RAG 로직은 CHAT 그룹에서 연동)</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
@@ -2890,29 +2890,29 @@
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>DATA-03,API-09</t>
+          <t>API-08</t>
         </is>
       </c>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.4</t>
+          <t>설계서 4.2·4.4</t>
         </is>
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t>최근 3턴 조회 확인</t>
+          <t>SSE 스트림 클라이언트 수신 확인</t>
         </is>
       </c>
       <c r="K42" s="3" t="inlineStr">
         <is>
-          <t>pytest: 최근 3턴만 반환, 4턴 이상 시 오래된 턴 제외 확인</t>
+          <t>pytest: SSE 스트림 청크 수신 순서 및 연결 종료 처리 확인(mock LLM 스트림)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>API-11</t>
+          <t>API-10</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
@@ -2927,17 +2927,17 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석</t>
+          <t>챗봇위젯</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>POST /analysis/link 구현</t>
+          <t>GET /chat/session/{id}/history 구현</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>Riot ID→PUUID 변환, TTL 1시간 캐시(Postgres puuid_cache 테이블, v1.7)</t>
+          <t>chat_logs 기반 대화이력 조회</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
@@ -2947,29 +2947,29 @@
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>SET-16,API-01</t>
+          <t>DATA-03,API-09</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>PRD 9-1·설계서v1.7 4.5</t>
+          <t>설계서 4.4</t>
         </is>
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>변환 성공/실패 케이스 확인</t>
+          <t>최근 3턴 조회 확인</t>
         </is>
       </c>
       <c r="K43" s="3" t="inlineStr">
         <is>
-          <t>pytest: mock Riot API로 정상/미존재 계정/레이트리밋 초과 3케이스, TTL 1시간 캐시 hit 확인</t>
+          <t>pytest: 최근 3턴만 반환, 4턴 이상 시 오래된 턴 제외 확인</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>API-12</t>
+          <t>API-11</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
@@ -2989,12 +2989,12 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>POST /analysis/recent 뼈대 구현</t>
+          <t>POST /analysis/link 구현</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>최신 매치ID 조회 및 캐시 재사용 분기(스코어링은 PGA 그룹에서 연동)</t>
+          <t>Riot ID→PUUID 변환, TTL 1시간 캐시(Postgres puuid_cache 테이블, v1.7)</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
@@ -3004,29 +3004,29 @@
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>API-11,DATA-03</t>
+          <t>SET-16,API-01</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>PRD 8-3·설계서4.5</t>
+          <t>PRD 9-1·설계서v1.7 4.5</t>
         </is>
       </c>
       <c r="J44" s="3" t="inlineStr">
         <is>
-          <t>캐시 hit/miss 분기 확인</t>
+          <t>변환 성공/실패 케이스 확인</t>
         </is>
       </c>
       <c r="K44" s="3" t="inlineStr">
         <is>
-          <t>pytest: match_analyses 캐시 hit 시 Riot API mock 호출 0회 확인</t>
+          <t>pytest: mock Riot API로 정상/미존재 계정/레이트리밋 초과 3케이스, TTL 1시간 캐시 hit 확인</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>API-13</t>
+          <t>API-12</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
@@ -3041,17 +3041,17 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>분석리포트</t>
+          <t>사후패인분석</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>GET /analysis/{match_id}/report 구현</t>
+          <t>POST /analysis/recent 뼈대 구현</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>match_analyses 기반 리포트 응답</t>
+          <t>최신 매치ID 조회 및 캐시 재사용 분기(스코어링은 PGA 그룹에서 연동)</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
@@ -3061,29 +3061,29 @@
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>DATA-03,API-12</t>
+          <t>API-11,DATA-03</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>PRD 8-3·설계서6장</t>
+          <t>PRD 8-3·설계서4.5</t>
         </is>
       </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t>응답 스키마 검증</t>
+          <t>캐시 hit/miss 분기 확인</t>
         </is>
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>pytest: 존재/미존재 match_id 케이스, 응답 스키마 필드 전체 검증</t>
+          <t>pytest: match_analyses 캐시 hit 시 Riot API mock 호출 0회 확인</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>API-14</t>
+          <t>API-13</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
@@ -3098,17 +3098,17 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>분석리포트</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>KPI 계측 이벤트 API 구현</t>
+          <t>GET /analysis/{match_id}/report 구현</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>link_click_events, account_link_events 적재 엔드포인트/훅</t>
+          <t>match_analyses 기반 리포트 응답</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
@@ -3118,29 +3118,29 @@
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>DATA-03,API-01</t>
+          <t>DATA-03,API-12</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
-          <t>PRD 3-3·설계서5.3</t>
+          <t>PRD 8-3·설계서6장</t>
         </is>
       </c>
       <c r="J46" s="3" t="inlineStr">
         <is>
-          <t>이벤트 적재 확인</t>
+          <t>응답 스키마 검증</t>
         </is>
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>pytest: 이벤트 적재 후 DB row 생성 및 필드 값 정확성 확인</t>
+          <t>pytest: 존재/미존재 match_id 케이스, 응답 스키마 필드 전체 검증</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>CHAT-01</t>
+          <t>API-14</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
@@ -3150,22 +3150,22 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>챗봇RAG</t>
+          <t>백엔드API</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>챗봇위젯</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>의도 분류 로직 구현</t>
+          <t>KPI 계측 이벤트 API 구현</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>1차 키워드/정규식, 2차 Groq LLM 분류(4종)</t>
+          <t>link_click_events, account_link_events 적재 엔드포인트/훅</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
@@ -3175,29 +3175,29 @@
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>API-09</t>
+          <t>DATA-03,API-01</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>PRD 7-2·설계서4.4</t>
+          <t>PRD 3-3·설계서5.3</t>
         </is>
       </c>
       <c r="J47" s="3" t="inlineStr">
         <is>
-          <t>4개 의도 분류 정확도 샘플 테스트</t>
+          <t>이벤트 적재 확인</t>
         </is>
       </c>
       <c r="K47" s="3" t="inlineStr">
         <is>
-          <t>pytest: 키워드 규칙 매칭 케이스(4종 각 2개 이상) + 애매한 질문의 mock LLM 분류 경로 확인</t>
+          <t>pytest: 이벤트 적재 후 DB row 생성 및 필드 값 정확성 확인</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>CHAT-02</t>
+          <t>CHAT-01</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
@@ -3217,12 +3217,12 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>하이브리드 검색 구현</t>
+          <t>의도 분류 로직 구현</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>SQL 필터 + pgvector top-k 코사인 검색</t>
+          <t>1차 키워드/정규식, 2차 Groq LLM 분류(4종)</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
@@ -3232,29 +3232,29 @@
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>DATA-11,CHAT-01</t>
+          <t>API-09</t>
         </is>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
-          <t>PRD 9-4·설계서4.4</t>
+          <t>PRD 7-2·설계서4.4</t>
         </is>
       </c>
       <c r="J48" s="3" t="inlineStr">
         <is>
-          <t>의도별 검색 결과 검증</t>
+          <t>4개 의도 분류 정확도 샘플 테스트</t>
         </is>
       </c>
       <c r="K48" s="3" t="inlineStr">
         <is>
-          <t>pytest: 의도별 SQL 필터 조건 반영 여부, mock pgvector top-k 결과 병합 확인</t>
+          <t>pytest: 키워드 규칙 매칭 케이스(4종 각 2개 이상) + 애매한 질문의 mock LLM 분류 경로 확인</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>CHAT-03</t>
+          <t>CHAT-02</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
@@ -3274,12 +3274,12 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>프롬프트 조립 로직 구현</t>
+          <t>하이브리드 검색 구현</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>시스템프롬프트+검색문서+대화이력+질문 결합, few-shot 삽입</t>
+          <t>SQL 필터 + pgvector top-k 코사인 검색</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
@@ -3289,29 +3289,29 @@
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>CHAT-02,API-10</t>
+          <t>DATA-11,CHAT-01</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.4.1</t>
+          <t>PRD 9-4·설계서4.4</t>
         </is>
       </c>
       <c r="J49" s="3" t="inlineStr">
         <is>
-          <t>프롬프트 스냅샷 테스트</t>
+          <t>의도별 검색 결과 검증</t>
         </is>
       </c>
       <c r="K49" s="3" t="inlineStr">
         <is>
-          <t>pytest: 프롬프트 스냅샷 테스트 — 시스템프롬프트/검색문서/대화이력/질문이 정해진 순서·구분자로 조립되는지 문자열 비교</t>
+          <t>pytest: 의도별 SQL 필터 조건 반영 여부, mock pgvector top-k 결과 병합 확인</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>CHAT-04</t>
+          <t>CHAT-03</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
@@ -3331,12 +3331,12 @@
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>입력 전처리 구현</t>
+          <t>프롬프트 조립 로직 구현</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>질문정규화·은어치환·인젝션방어·길이제한·범위밖질문 안내</t>
+          <t>시스템프롬프트+검색문서+대화이력+질문 결합, few-shot 삽입</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
@@ -3346,29 +3346,29 @@
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>CHAT-01</t>
+          <t>CHAT-02,API-10</t>
         </is>
       </c>
       <c r="I50" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.4.2</t>
+          <t>설계서 4.4.1</t>
         </is>
       </c>
       <c r="J50" s="3" t="inlineStr">
         <is>
-          <t>각 케이스 단위 테스트 통과</t>
+          <t>프롬프트 스냅샷 테스트</t>
         </is>
       </c>
       <c r="K50" s="3" t="inlineStr">
         <is>
-          <t>pytest(필수·보안, TEST-00 시나리오 선적용): 인젝션 문구가 [사용자 메시지] 델리미터 내부로만 들어가는지, 범위밖 질문 안내 문구 반환, 초과 길이 입력 truncate 확인</t>
+          <t>pytest: 프롬프트 스냅샷 테스트 — 시스템프롬프트/검색문서/대화이력/질문이 정해진 순서·구분자로 조립되는지 문자열 비교</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>CHAT-05</t>
+          <t>CHAT-04</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
@@ -3388,12 +3388,12 @@
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>sLLM 답변 생성 및 SSE 스트리밍 연동</t>
+          <t>입력 전처리 구현</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>Groq Llama 3.3 70B 호출, 스트리밍 응답</t>
+          <t>질문정규화·은어치환·인젝션방어·길이제한·범위밖질문 안내</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
@@ -3403,29 +3403,29 @@
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>CHAT-03,API-09,SET-10</t>
+          <t>CHAT-01</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.4</t>
+          <t>설계서 4.4.2</t>
         </is>
       </c>
       <c r="J51" s="3" t="inlineStr">
         <is>
-          <t>스트리밍 응답 end-to-end 확인</t>
+          <t>각 케이스 단위 테스트 통과</t>
         </is>
       </c>
       <c r="K51" s="3" t="inlineStr">
         <is>
-          <t>pytest: mock Groq 클라이언트로 SSE 스트리밍 조립 확인, 타임아웃 예외 처리 확인</t>
+          <t>pytest(필수·보안, TEST-00 시나리오 선적용): 인젝션 문구가 [사용자 메시지] 델리미터 내부로만 들어가는지, 범위밖 질문 안내 문구 반환, 초과 길이 입력 truncate 확인</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>CHAT-06</t>
+          <t>CHAT-05</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
@@ -3445,12 +3445,12 @@
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>출력 후처리 구현</t>
+          <t>sLLM 답변 생성 및 SSE 스트리밍 연동</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>근거검증·Legend승률이중방어·닉네임마스킹·구조화출력·재시도폴백</t>
+          <t>Groq Llama 3.3 70B 호출, 스트리밍 응답</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr">
@@ -3460,29 +3460,29 @@
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>CHAT-05</t>
+          <t>CHAT-03,API-09,SET-10</t>
         </is>
       </c>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.4.3</t>
+          <t>설계서 4.4</t>
         </is>
       </c>
       <c r="J52" s="3" t="inlineStr">
         <is>
-          <t>각 방어 로직 단위 테스트 통과</t>
+          <t>스트리밍 응답 end-to-end 확인</t>
         </is>
       </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
-          <t>pytest(필수·정책, TEST-00 시나리오 선적용): 근거 없는 고유명사 재생성/경고 처리, Legend 문서 승률 수치 후처리 제거, 상대 닉네임 정규식 마스킹 3케이스 모두 검증</t>
+          <t>pytest: mock Groq 클라이언트로 SSE 스트리밍 조립 확인, 타임아웃 예외 처리 확인</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>CHAT-07</t>
+          <t>CHAT-06</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
@@ -3502,12 +3502,12 @@
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>웹사이트 링크 자동 삽입 구현</t>
+          <t>출력 후처리 구현</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>답변 내 조합/아이템/증강체 id 파싱→상세페이지 링크 삽입</t>
+          <t>근거검증·Legend승률이중방어·닉네임마스킹·구조화출력·재시도폴백</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
@@ -3517,29 +3517,29 @@
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>CHAT-06</t>
+          <t>CHAT-05</t>
         </is>
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>PRD 7-2·설계서4.4</t>
+          <t>설계서 4.4.3</t>
         </is>
       </c>
       <c r="J53" s="3" t="inlineStr">
         <is>
-          <t>링크 삽입 정확도 샘플 테스트</t>
+          <t>각 방어 로직 단위 테스트 통과</t>
         </is>
       </c>
       <c r="K53" s="3" t="inlineStr">
         <is>
-          <t>pytest: 답변 내 조합/아이템/증강체 언급 시 정확한 링크 삽입, 존재하지 않는 id 오탐 케이스 처리 확인</t>
+          <t>pytest(필수·정책, TEST-00 시나리오 선적용): 근거 없는 고유명사 재생성/경고 처리, Legend 문서 승률 수치 후처리 제거, 상대 닉네임 정규식 마스킹 3케이스 모두 검증</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>CHAT-08</t>
+          <t>CHAT-07</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
@@ -3559,12 +3559,12 @@
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>응답 캐싱 로직 구현</t>
+          <t>웹사이트 링크 자동 삽입 구현</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>첫턴 질문 Postgres(chat_answer_cache) 캐시, 후속턴 캐시제외, 패치갱신시 무효화</t>
+          <t>답변 내 조합/아이템/증강체 id 파싱→상세페이지 링크 삽입</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
@@ -3574,29 +3574,29 @@
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>CHAT-05,DATA-15</t>
+          <t>CHAT-06</t>
         </is>
       </c>
       <c r="I54" s="3" t="inlineStr">
         <is>
-          <t>PRD 9-6·설계서v1.7 4.4·4.6</t>
+          <t>PRD 7-2·설계서4.4</t>
         </is>
       </c>
       <c r="J54" s="3" t="inlineStr">
         <is>
-          <t>캐시 hit/무효화 시나리오 테스트</t>
+          <t>링크 삽입 정확도 샘플 테스트</t>
         </is>
       </c>
       <c r="K54" s="3" t="inlineStr">
         <is>
-          <t>pytest: 첫턴 캐시 hit, 후속턴 캐시 미적용, 패치갱신 후 캐시 무효화 확인</t>
+          <t>pytest: 답변 내 조합/아이템/증강체 언급 시 정확한 링크 삽입, 존재하지 않는 id 오탐 케이스 처리 확인</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>CHAT-09</t>
+          <t>CHAT-08</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
@@ -3616,12 +3616,12 @@
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>Q&amp;A 로깅 구현</t>
+          <t>응답 캐싱 로직 구현</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>chat_logs 적재(질의/의도/근거문서/patch/지연시간/콜드스타트)</t>
+          <t>첫턴 질문 Postgres(chat_answer_cache) 캐시, 후속턴 캐시제외, 패치갱신시 무효화</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
@@ -3631,29 +3631,29 @@
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>DATA-03,CHAT-05</t>
+          <t>CHAT-05,DATA-15</t>
         </is>
       </c>
       <c r="I55" s="3" t="inlineStr">
         <is>
-          <t>PRD 3-3·9-5</t>
+          <t>PRD 9-6·설계서v1.7 4.4·4.6</t>
         </is>
       </c>
       <c r="J55" s="3" t="inlineStr">
         <is>
-          <t>로그 적재 필드 확인</t>
+          <t>캐시 hit/무효화 시나리오 테스트</t>
         </is>
       </c>
       <c r="K55" s="3" t="inlineStr">
         <is>
-          <t>pytest: chat_logs row에 질의/의도/근거문서id/patch_version/답변/지연시간/콜드스타트 전체 필드 적재 확인</t>
+          <t>pytest: 첫턴 캐시 hit, 후속턴 캐시 미적용, 패치갱신 후 캐시 무효화 확인</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>CHAT-10</t>
+          <t>CHAT-09</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
@@ -3673,12 +3673,12 @@
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>사후분석 트리거 연동</t>
+          <t>Q&amp;A 로깅 구현</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>'방금 게임 분석해줘' 발화 시 분석 로직 호출 및 챗봇 답변 영역 요약 표시</t>
+          <t>chat_logs 적재(질의/의도/근거문서/patch/지연시간/콜드스타트)</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
@@ -3688,29 +3688,29 @@
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>CHAT-06,API-12</t>
+          <t>DATA-03,CHAT-05</t>
         </is>
       </c>
       <c r="I56" s="3" t="inlineStr">
         <is>
-          <t>PRD 8-3</t>
+          <t>PRD 3-3·9-5</t>
         </is>
       </c>
       <c r="J56" s="3" t="inlineStr">
         <is>
-          <t>트리거 발화 테스트 통과</t>
+          <t>로그 적재 필드 확인</t>
         </is>
       </c>
       <c r="K56" s="3" t="inlineStr">
         <is>
-          <t>pytest: '방금 게임 분석해줘' mock 발화 시 analysis 로직 호출(1회) 및 응답에 요약+링크 포함 확인</t>
+          <t>pytest: chat_logs row에 질의/의도/근거문서id/patch_version/답변/지연시간/콜드스타트 전체 필드 적재 확인</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>PGA-01</t>
+          <t>CHAT-10</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
@@ -3720,22 +3720,22 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>사후패인분석</t>
+          <t>챗봇RAG</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석</t>
+          <t>챗봇위젯</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>Riot ID 계정 연동 로직 구현</t>
+          <t>사후분석 트리거 연동</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>게임명#태그+지역 입력→PUUID 변환, 임의계정 조회 허용</t>
+          <t>'방금 게임 분석해줘' 발화 시 분석 로직 호출 및 챗봇 답변 영역 요약 표시</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
@@ -3745,29 +3745,29 @@
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>API-11</t>
+          <t>CHAT-06,API-12</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
         <is>
-          <t>PRD 7-3·8-3·9-1</t>
+          <t>PRD 8-3</t>
         </is>
       </c>
       <c r="J57" s="3" t="inlineStr">
         <is>
-          <t>정상/비정상 계정 케이스 테스트</t>
+          <t>트리거 발화 테스트 통과</t>
         </is>
       </c>
       <c r="K57" s="3" t="inlineStr">
         <is>
-          <t>pytest: 정상 Riot ID/형식 오류/미존재 계정 3케이스</t>
+          <t>pytest: '방금 게임 분석해줘' mock 발화 시 analysis 로직 호출(1회) 및 응답에 요약+링크 포함 확인</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>PGA-02</t>
+          <t>PGA-01</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
@@ -3787,12 +3787,12 @@
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>최신 매치 조회 로직 구현</t>
+          <t>Riot ID 계정 연동 로직 구현</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>Match-V1으로 매치ID/매치상세 조회</t>
+          <t>게임명#태그+지역 입력→PUUID 변환, 임의계정 조회 허용</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
@@ -3802,29 +3802,29 @@
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>PGA-01</t>
+          <t>API-11</t>
         </is>
       </c>
       <c r="I58" s="3" t="inlineStr">
         <is>
-          <t>PRD 7-3·설계서4.5</t>
+          <t>PRD 7-3·8-3·9-1</t>
         </is>
       </c>
       <c r="J58" s="3" t="inlineStr">
         <is>
-          <t>매치 상세 파싱 검증</t>
+          <t>정상/비정상 계정 케이스 테스트</t>
         </is>
       </c>
       <c r="K58" s="3" t="inlineStr">
         <is>
-          <t>pytest: mock Match-V1 응답 기준 매치ID·매치상세 파싱 필드 전체 검증</t>
+          <t>pytest: 정상 Riot ID/형식 오류/미존재 계정 3케이스</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>PGA-03</t>
+          <t>PGA-02</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
@@ -3839,17 +3839,17 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석·분석리포트</t>
+          <t>사후패인분석</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>분석 결과 캐시 재사용 로직 구현</t>
+          <t>최신 매치 조회 로직 구현</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>match_analyses 조회 우선, 없으면 신규계산</t>
+          <t>Match-V1으로 매치ID/매치상세 조회</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">
@@ -3859,29 +3859,29 @@
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>DATA-03,PGA-02</t>
+          <t>PGA-01</t>
         </is>
       </c>
       <c r="I59" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.5·4.6·5.1</t>
+          <t>PRD 7-3·설계서4.5</t>
         </is>
       </c>
       <c r="J59" s="3" t="inlineStr">
         <is>
-          <t>재요청 시 캐시 히트 확인</t>
+          <t>매치 상세 파싱 검증</t>
         </is>
       </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t>pytest: 동일 match_id+puuid 재요청 시 Riot API/Groq mock 호출 0회(캐시 hit), 신규 조합은 계산 경로 진입 확인</t>
+          <t>pytest: mock Match-V1 응답 기준 매치ID·매치상세 파싱 필드 전체 검증</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>PGA-04</t>
+          <t>PGA-03</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
@@ -3896,17 +3896,17 @@
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>분석리포트</t>
+          <t>사후패인분석·분석리포트</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>조합 이탈도 계산 로직 구현</t>
+          <t>분석 결과 캐시 재사용 로직 구현</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>가중 자카드 유사도(캐리 가중치2), 구간분류</t>
+          <t>match_analyses 조회 우선, 없으면 신규계산</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
@@ -3916,29 +3916,29 @@
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>PGA-02,DATA-02</t>
+          <t>DATA-03,PGA-02</t>
         </is>
       </c>
       <c r="I60" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.5.1</t>
+          <t>설계서 4.5·4.6·5.1</t>
         </is>
       </c>
       <c r="J60" s="3" t="inlineStr">
         <is>
-          <t>샘플 매치 계산값 수기검증 일치</t>
+          <t>재요청 시 캐시 히트 확인</t>
         </is>
       </c>
       <c r="K60" s="3" t="inlineStr">
         <is>
-          <t>pytest(필수·크리티컬, TEST-00 시나리오 선적용): 수기 계산한 샘플 보드 3~5개에 대해 이탈도 값이 소수점 둘째자리까지 일치, 구간분류 경계값(0.3/0.6) 케이스 포함</t>
+          <t>pytest: 동일 match_id+puuid 재요청 시 Riot API/Groq mock 호출 0회(캐시 hit), 신규 조합은 계산 경로 진입 확인</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>PGA-05</t>
+          <t>PGA-04</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
@@ -3958,12 +3958,12 @@
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>아이템 집중도 계산 로직 구현</t>
+          <t>조합 이탈도 계산 로직 구현</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>캐리 완성아이템 비율, 추천빌드 멀티셋 교집합</t>
+          <t>가중 자카드 유사도(캐리 가중치2), 구간분류</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
@@ -3973,7 +3973,7 @@
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>PGA-04</t>
+          <t>PGA-02,DATA-02</t>
         </is>
       </c>
       <c r="I61" s="3" t="inlineStr">
@@ -3983,19 +3983,19 @@
       </c>
       <c r="J61" s="3" t="inlineStr">
         <is>
-          <t>샘플 계산값 검증</t>
+          <t>샘플 매치 계산값 수기검증 일치</t>
         </is>
       </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>pytest: 샘플 보드 기준 집중도 값 수기 계산과 일치, 중복 아이템 멀티셋 케이스 포함</t>
+          <t>pytest(필수·크리티컬, TEST-00 시나리오 선적용): 수기 계산한 샘플 보드 3~5개에 대해 이탈도 값이 소수점 둘째자리까지 일치, 구간분류 경계값(0.3/0.6) 케이스 포함</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>PGA-06</t>
+          <t>PGA-05</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
@@ -4015,12 +4015,12 @@
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>증강체 시너지 계산 로직 구현</t>
+          <t>아이템 집중도 계산 로직 구현</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>선택증강체 vs comp_augments 매칭 비율</t>
+          <t>캐리 완성아이템 비율, 추천빌드 멀티셋 교집합</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
@@ -4045,14 +4045,14 @@
       </c>
       <c r="K62" s="3" t="inlineStr">
         <is>
-          <t>pytest: 선택 증강체 0개/일부일치/전체일치 3케이스 시너지 점수 검증</t>
+          <t>pytest: 샘플 보드 기준 집중도 값 수기 계산과 일치, 중복 아이템 멀티셋 케이스 포함</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>PGA-07</t>
+          <t>PGA-06</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
@@ -4072,12 +4072,12 @@
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>코칭 문장 생성 로직 구현</t>
+          <t>증강체 시너지 계산 로직 구현</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>3개 지표+등수 근거로 잘한점/아쉬운점/제안 고정구조 생성, 수치 비노출. op.gg tft_get_play_style(PUUID 필요, DATA-08에서 이동)을 호출해 코칭 근거로 활용</t>
+          <t>선택증강체 vs comp_augments 매칭 비율</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr">
@@ -4087,29 +4087,29 @@
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>PGA-04,PGA-05,PGA-06,SET-10</t>
+          <t>PGA-04</t>
         </is>
       </c>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>PRD 7-3·설계서4.5.2</t>
+          <t>설계서 4.5.1</t>
         </is>
       </c>
       <c r="J63" s="3" t="inlineStr">
         <is>
-          <t>출력 포맷 규칙 준수 확인</t>
+          <t>샘플 계산값 검증</t>
         </is>
       </c>
       <c r="K63" s="3" t="inlineStr">
         <is>
-          <t>pytest(필수·정책, TEST-00 시나리오 선적용): mock LLM 출력에 원 수치(예: '이탈도 0.42')가 노출되면 실패 처리되는 검증 로직 자체 테스트, 고정 3단 구조 파싱 확인</t>
+          <t>pytest: 선택 증강체 0개/일부일치/전체일치 3케이스 시너지 점수 검증</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>PGA-08</t>
+          <t>PGA-07</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
@@ -4129,12 +4129,12 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>다음 게임 제안 근거 조회 로직 구현</t>
+          <t>코칭 문장 생성 로직 구현</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>matched_comp_id 기준 추천아이템·증강체 조회</t>
+          <t>3개 지표+등수 근거로 잘한점/아쉬운점/제안 고정구조 생성, 수치 비노출. op.gg tft_get_play_style(PUUID 필요, DATA-08에서 이동)을 호출해 코칭 근거로 활용</t>
         </is>
       </c>
       <c r="G64" s="4" t="inlineStr">
@@ -4144,29 +4144,29 @@
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>PGA-04,DATA-02</t>
+          <t>PGA-04,PGA-05,PGA-06,SET-10</t>
         </is>
       </c>
       <c r="I64" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.5.3</t>
+          <t>PRD 7-3·설계서4.5.2</t>
         </is>
       </c>
       <c r="J64" s="3" t="inlineStr">
         <is>
-          <t>추천 근거 정확성 검증</t>
+          <t>출력 포맷 규칙 준수 확인</t>
         </is>
       </c>
       <c r="K64" s="3" t="inlineStr">
         <is>
-          <t>pytest: matched_comp_id 기준 추천아이템/증강체 조회 결과가 champion_item_builds/comp_augments와 일치하는지 확인</t>
+          <t>pytest(필수·정책, TEST-00 시나리오 선적용): mock LLM 출력에 원 수치(예: '이탈도 0.42')가 노출되면 실패 처리되는 검증 로직 자체 테스트, 고정 3단 구조 파싱 확인</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>PGA-09</t>
+          <t>PGA-08</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
@@ -4186,12 +4186,12 @@
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>프라이버시 마스킹 로직 구현</t>
+          <t>다음 게임 제안 근거 조회 로직 구현</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>상대 닉네임 마스킹 전처리+정규식 재마스킹 이중방어</t>
+          <t>matched_comp_id 기준 추천아이템·증강체 조회</t>
         </is>
       </c>
       <c r="G65" s="4" t="inlineStr">
@@ -4201,29 +4201,29 @@
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
-          <t>PGA-07</t>
+          <t>PGA-04,DATA-02</t>
         </is>
       </c>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>PRD 7-3·설계서4.4.3·4.5.3</t>
+          <t>설계서 4.5.3</t>
         </is>
       </c>
       <c r="J65" s="3" t="inlineStr">
         <is>
-          <t>마스킹 누락 케이스 없음 확인</t>
+          <t>추천 근거 정확성 검증</t>
         </is>
       </c>
       <c r="K65" s="3" t="inlineStr">
         <is>
-          <t>pytest(필수·보안, TEST-00 시나리오 선적용): 상대 Riot ID 포함 mock LLM 출력에서 정규식 마스킹 후 원본 문자열이 전혀 남지 않는지(부분 마스킹 실패 케이스 포함) 확인</t>
+          <t>pytest: matched_comp_id 기준 추천아이템/증강체 조회 결과가 champion_item_builds/comp_augments와 일치하는지 확인</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>PGA-10</t>
+          <t>PGA-09</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
@@ -4238,17 +4238,17 @@
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석·분석리포트</t>
+          <t>분석리포트</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>상세 리포트 데이터 조립 로직 구현</t>
+          <t>프라이버시 마스킹 로직 구현</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>코칭요약·매칭조합·등수변화·아이템타임라인 응답 조립</t>
+          <t>상대 닉네임 마스킹 전처리+정규식 재마스킹 이중방어</t>
         </is>
       </c>
       <c r="G66" s="4" t="inlineStr">
@@ -4258,29 +4258,29 @@
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>PGA-07,PGA-08,PGA-09,API-13</t>
+          <t>PGA-07</t>
         </is>
       </c>
       <c r="I66" s="3" t="inlineStr">
         <is>
-          <t>PRD 8-3·IA4.6</t>
+          <t>PRD 7-3·설계서4.4.3·4.5.3</t>
         </is>
       </c>
       <c r="J66" s="3" t="inlineStr">
         <is>
-          <t>API-13 응답 필드 전체 채움 확인</t>
+          <t>마스킹 누락 케이스 없음 확인</t>
         </is>
       </c>
       <c r="K66" s="3" t="inlineStr">
         <is>
-          <t>pytest: API-13 응답 스키마 전체 필드가 null 없이 채워지는지 통합 테스트</t>
+          <t>pytest(필수·보안, TEST-00 시나리오 선적용): 상대 Riot ID 포함 mock LLM 출력에서 정규식 마스킹 후 원본 문자열이 전혀 남지 않는지(부분 마스킹 실패 케이스 포함) 확인</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>FE-01</t>
+          <t>PGA-10</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
@@ -4290,22 +4290,22 @@
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>프론트엔드</t>
+          <t>사후패인분석</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>사후패인분석·분석리포트</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Next.js 프로젝트 스캐폴딩 및 Tailwind 설정</t>
+          <t>상세 리포트 데이터 조립 로직 구현</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>App Router, Tailwind 브레이크포인트(md768/lg1024) 매핑, 디자인가이드 토큰(컬러/타이포/spacing) 반영</t>
+          <t>코칭요약·매칭조합·등수변화·아이템타임라인 응답 조립</t>
         </is>
       </c>
       <c r="G67" s="4" t="inlineStr">
@@ -4315,29 +4315,29 @@
       </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
-          <t>SET-07</t>
+          <t>PGA-07,PGA-08,PGA-09,API-13</t>
         </is>
       </c>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>설계서4.1.1·디자인가이드</t>
+          <t>PRD 8-3·IA4.6</t>
         </is>
       </c>
       <c r="J67" s="3" t="inlineStr">
         <is>
-          <t>기본 레이아웃 렌더링 확인</t>
+          <t>API-13 응답 필드 전체 채움 확인</t>
         </is>
       </c>
       <c r="K67" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: Tailwind 브레이크포인트 클래스 적용 여부, 디자인 토큰 색상값 매칭 확인</t>
+          <t>pytest: API-13 응답 스키마 전체 필드가 null 없이 채워지는지 통합 테스트</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>FE-02</t>
+          <t>FE-01</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
@@ -4352,17 +4352,17 @@
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>공통(GNB)</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>GNB 컴포넌트 구현</t>
+          <t>Next.js 프로젝트 스캐폴딩 및 Tailwind 설정</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>데스크톱/태블릿 가로바, 모바일 햄버거+드로어, 4개 진입점</t>
+          <t>App Router, Tailwind 브레이크포인트(md768/lg1024) 매핑, 디자인가이드 토큰(컬러/타이포/spacing) 반영</t>
         </is>
       </c>
       <c r="G68" s="4" t="inlineStr">
@@ -4372,29 +4372,29 @@
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>FE-01</t>
+          <t>SET-07</t>
         </is>
       </c>
       <c r="I68" s="3" t="inlineStr">
         <is>
-          <t>PRD7-4·IA6.1·디자인가이드6.1</t>
+          <t>설계서4.1.1·디자인가이드</t>
         </is>
       </c>
       <c r="J68" s="3" t="inlineStr">
         <is>
-          <t>3개 브레이크포인트 시각 확인</t>
+          <t>기본 레이아웃 렌더링 확인</t>
         </is>
       </c>
       <c r="K68" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: 3개 브레이크포인트에서 GNB 렌더링 분기(가로바/드로어) 테스트 + Playwright 스모크(클릭 시 드로어 오픈)</t>
+          <t>Vitest+RTL: Tailwind 브레이크포인트 클래스 적용 여부, 디자인 토큰 색상값 매칭 확인</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>FE-03</t>
+          <t>FE-02</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
@@ -4409,17 +4409,17 @@
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>티어리스트</t>
+          <t>공통(GNB)</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>티어리스트(홈) 페이지 구현</t>
+          <t>GNB 컴포넌트 구현</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>필터바/카드그리드/챗봇슬롯, 정적 export(FE-01 결정) + 클라이언트 사이드 fetch(CSR), 반응형(3~4열→2열→1열)</t>
+          <t>데스크톱/태블릿 가로바, 모바일 햄버거+드로어, 4개 진입점</t>
         </is>
       </c>
       <c r="G69" s="4" t="inlineStr">
@@ -4429,29 +4429,29 @@
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>FE-02,API-02,API-06</t>
+          <t>FE-01</t>
         </is>
       </c>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>PRD7-1·7-4·화면설계서2.1</t>
+          <t>PRD7-4·IA6.1·디자인가이드6.1</t>
         </is>
       </c>
       <c r="J69" s="3" t="inlineStr">
         <is>
-          <t>데스크톱/태블릿/모바일 와이어프레임 대비 시각 검증</t>
+          <t>3개 브레이크포인트 시각 확인</t>
         </is>
       </c>
       <c r="K69" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: 카드 그리드 컬럼 수 브레이크포인트별 렌더링, mock API 응답 데이터 바인딩 테스트(E2E는 TEST-08)</t>
+          <t>Vitest+RTL: 3개 브레이크포인트에서 GNB 렌더링 분기(가로바/드로어) 테스트 + Playwright 스모크(클릭 시 드로어 오픈)</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>FE-04</t>
+          <t>FE-03</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
@@ -4466,17 +4466,17 @@
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>조합상세</t>
+          <t>티어리스트</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>조합 상세 페이지 구현</t>
+          <t>티어리스트(홈) 페이지 구현</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>개요/챔피언구성(캐리강조)/증강체목록/CTA버튼, 모바일 full-width CTA</t>
+          <t>필터바/카드그리드/챗봇슬롯, 정적 export(FE-01 결정) + 클라이언트 사이드 fetch(CSR), 반응형(3~4열→2열→1열)</t>
         </is>
       </c>
       <c r="G70" s="4" t="inlineStr">
@@ -4486,29 +4486,29 @@
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>FE-02,API-03</t>
+          <t>FE-02,API-02,API-06</t>
         </is>
       </c>
       <c r="I70" s="3" t="inlineStr">
         <is>
-          <t>화면설계서2.2</t>
+          <t>PRD7-1·7-4·화면설계서2.1</t>
         </is>
       </c>
       <c r="J70" s="3" t="inlineStr">
         <is>
-          <t>링크이동·반응형 검증</t>
+          <t>데스크톱/태블릿/모바일 와이어프레임 대비 시각 검증</t>
         </is>
       </c>
       <c r="K70" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: 캐리/서브 챔피언 보더 스타일 분기, CTA 버튼 모바일 full-width 렌더링 테스트</t>
+          <t>Vitest+RTL: 카드 그리드 컬럼 수 브레이크포인트별 렌더링, mock API 응답 데이터 바인딩 테스트(E2E는 TEST-08)</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>FE-05</t>
+          <t>FE-04</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
@@ -4523,17 +4523,17 @@
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>아이템빌드</t>
+          <t>조합상세</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>아이템 빌드 페이지 구현</t>
+          <t>조합 상세 페이지 구현</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>챔피언필터/조합리스트/상세패널(모바일 바텀시트)</t>
+          <t>개요/챔피언구성(캐리강조)/증강체목록/CTA버튼, 모바일 full-width CTA</t>
         </is>
       </c>
       <c r="G71" s="4" t="inlineStr">
@@ -4543,29 +4543,29 @@
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
-          <t>FE-02,API-04</t>
+          <t>FE-02,API-03</t>
         </is>
       </c>
       <c r="I71" s="3" t="inlineStr">
         <is>
-          <t>화면설계서2.3</t>
+          <t>화면설계서2.2</t>
         </is>
       </c>
       <c r="J71" s="3" t="inlineStr">
         <is>
-          <t>필터-URL쿼리 동기화 검증</t>
+          <t>링크이동·반응형 검증</t>
         </is>
       </c>
       <c r="K71" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: 챔피언 필터 선택 시 URL 쿼리 동기화, 모바일 바텀시트 오픈/클로즈 테스트</t>
+          <t>Vitest+RTL: 캐리/서브 챔피언 보더 스타일 분기, CTA 버튼 모바일 full-width 렌더링 테스트</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>FE-06</t>
+          <t>FE-05</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
@@ -4580,17 +4580,17 @@
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>증강체정보</t>
+          <t>아이템빌드</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>증강체 정보 페이지 구현</t>
+          <t>아이템 빌드 페이지 구현</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>티어필터/카드리스트, Legend 승률 숨김 표시</t>
+          <t>챔피언필터/조합리스트/상세패널(모바일 바텀시트)</t>
         </is>
       </c>
       <c r="G72" s="4" t="inlineStr">
@@ -4600,29 +4600,29 @@
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>FE-02,API-05</t>
+          <t>FE-02,API-04</t>
         </is>
       </c>
       <c r="I72" s="3" t="inlineStr">
         <is>
-          <t>PRD10-1·화면설계서2.4</t>
+          <t>화면설계서2.3</t>
         </is>
       </c>
       <c r="J72" s="3" t="inlineStr">
         <is>
-          <t>Legend 항목 승률 미노출 확인</t>
+          <t>필터-URL쿼리 동기화 검증</t>
         </is>
       </c>
       <c r="K72" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL(필수·정책): is_legend_related=true 카드에 '승률 표시 안함' 텍스트만 렌더링되고 숫자가 DOM에 없는지 확인</t>
+          <t>Vitest+RTL: 챔피언 필터 선택 시 URL 쿼리 동기화, 모바일 바텀시트 오픈/클로즈 테스트</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>FE-07</t>
+          <t>FE-06</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
@@ -4637,17 +4637,17 @@
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석</t>
+          <t>증강체정보</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>사후 패인 분석 페이지 구현</t>
+          <t>증강체 정보 페이지 구현</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>Riot ID 폼/최근계정목록(localStorage)/전적불러오기 버튼/진행상태</t>
+          <t>티어필터/카드리스트, Legend 승률 숨김 표시</t>
         </is>
       </c>
       <c r="G73" s="4" t="inlineStr">
@@ -4657,29 +4657,29 @@
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>FE-02,API-11,API-12</t>
+          <t>FE-02,API-05</t>
         </is>
       </c>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>PRD8-3·화면설계서2.5</t>
+          <t>PRD10-1·화면설계서2.4</t>
         </is>
       </c>
       <c r="J73" s="3" t="inlineStr">
         <is>
-          <t>로컬스토리지 저장/재사용 확인</t>
+          <t>Legend 항목 승률 미노출 확인</t>
         </is>
       </c>
       <c r="K73" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: localStorage mock 기준 최근 계정 목록 추가/조회/전환 테스트, 폼 검증 에러 메시지 테스트</t>
+          <t>Vitest+RTL(필수·정책): is_legend_related=true 카드에 '승률 표시 안함' 텍스트만 렌더링되고 숫자가 DOM에 없는지 확인</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>FE-08</t>
+          <t>FE-07</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
@@ -4694,17 +4694,17 @@
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>분석리포트</t>
+          <t>사후패인분석</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>분석 리포트 상세 페이지 구현</t>
+          <t>사후 패인 분석 페이지 구현</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>코칭요약/매칭조합카드/등수변화그래프/아이템타임라인</t>
+          <t>Riot ID 폼/최근계정목록(localStorage)/전적불러오기 버튼/진행상태</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr">
@@ -4714,29 +4714,29 @@
       </c>
       <c r="H74" s="3" t="inlineStr">
         <is>
-          <t>API-13,FE-02</t>
+          <t>FE-02,API-11,API-12</t>
         </is>
       </c>
       <c r="I74" s="3" t="inlineStr">
         <is>
-          <t>PRD8-3·화면설계서2.6</t>
+          <t>PRD8-3·화면설계서2.5</t>
         </is>
       </c>
       <c r="J74" s="3" t="inlineStr">
         <is>
-          <t>그래프/타임라인 렌더링 확인</t>
+          <t>로컬스토리지 저장/재사용 확인</t>
         </is>
       </c>
       <c r="K74" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: 그래프/타임라인 mock 데이터 렌더링, opponent-info 마스킹 텍스트 렌더링 확인</t>
+          <t>Vitest+RTL: localStorage mock 기준 최근 계정 목록 추가/조회/전환 테스트, 폼 검증 에러 메시지 테스트</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>FE-09</t>
+          <t>FE-08</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
@@ -4751,17 +4751,17 @@
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>챗봇위젯</t>
+          <t>분석리포트</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>챗봇 위젯 전역 컴포넌트 구현</t>
+          <t>분석 리포트 상세 페이지 구현</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>collapsed/expanded, SSE 연동, 모바일 바텀시트 전환, 후속질문칩</t>
+          <t>코칭요약/매칭조합카드/등수변화그래프/아이템타임라인</t>
         </is>
       </c>
       <c r="G75" s="4" t="inlineStr">
@@ -4771,29 +4771,29 @@
       </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
-          <t>FE-01,API-09,CHAT-05</t>
+          <t>API-13,FE-02</t>
         </is>
       </c>
       <c r="I75" s="3" t="inlineStr">
         <is>
-          <t>PRD7-4·화면설계서2.7·디자인가이드6.6</t>
+          <t>PRD8-3·화면설계서2.6</t>
         </is>
       </c>
       <c r="J75" s="3" t="inlineStr">
         <is>
-          <t>전 페이지 삽입 및 반응형 동작 확인</t>
+          <t>그래프/타임라인 렌더링 확인</t>
         </is>
       </c>
       <c r="K75" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: collapsed/expanded 상태 전환, 모바일 바텀시트 전환, mock SSE 스트림 렌더링 테스트</t>
+          <t>Vitest+RTL: 그래프/타임라인 mock 데이터 렌더링, opponent-info 마스킹 텍스트 렌더링 확인</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>FE-10</t>
+          <t>FE-09</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
@@ -4808,49 +4808,49 @@
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>챗봇위젯</t>
         </is>
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>이미지 최적화 및 반응형 sizes 적용</t>
+          <t>챗봇 위젯 전역 컴포넌트 구현</t>
         </is>
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>Next Image 컴포넌트, 브레이크포인트별 해상도 서빙</t>
+          <t>collapsed/expanded, SSE 연동, 모바일 바텀시트 전환, 후속질문칩</t>
         </is>
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t>권장</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
-          <t>FE-03,FE-04,FE-05,FE-06,FE-07,FE-08</t>
+          <t>FE-01,API-09,CHAT-05</t>
         </is>
       </c>
       <c r="I76" s="3" t="inlineStr">
         <is>
-          <t>PRD7-4·설계서4.1.1</t>
+          <t>PRD7-4·화면설계서2.7·디자인가이드6.6</t>
         </is>
       </c>
       <c r="J76" s="3" t="inlineStr">
         <is>
-          <t>모바일 이미지 로딩 성능 확인</t>
+          <t>전 페이지 삽입 및 반응형 동작 확인</t>
         </is>
       </c>
       <c r="K76" s="3" t="inlineStr">
         <is>
-          <t>해당 없음 — Lighthouse 모바일 성능 점수로 갈음(수동 측정)</t>
+          <t>Vitest+RTL: collapsed/expanded 상태 전환, 모바일 바텀시트 전환, mock SSE 스트림 렌더링 테스트</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>FE-11</t>
+          <t>FE-10</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
@@ -4870,44 +4870,44 @@
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>필터 UI 반응형 공용 컴포넌트 구현</t>
+          <t>이미지 최적화 및 반응형 sizes 적용</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>데스크톱/태블릿 Dropdown, 모바일 BottomSheet 공용 컴포넌트</t>
+          <t>Next Image 컴포넌트, 브레이크포인트별 해상도 서빙</t>
         </is>
       </c>
       <c r="G77" s="4" t="inlineStr">
         <is>
-          <t>필수</t>
+          <t>권장</t>
         </is>
       </c>
       <c r="H77" s="3" t="inlineStr">
         <is>
-          <t>FE-01</t>
+          <t>FE-03,FE-04,FE-05,FE-06,FE-07,FE-08</t>
         </is>
       </c>
       <c r="I77" s="3" t="inlineStr">
         <is>
-          <t>디자인가이드6.2</t>
+          <t>PRD7-4·설계서4.1.1</t>
         </is>
       </c>
       <c r="J77" s="3" t="inlineStr">
         <is>
-          <t>3개 화면(티어리스트/아이템빌드/증강체)에서 재사용 확인</t>
+          <t>모바일 이미지 로딩 성능 확인</t>
         </is>
       </c>
       <c r="K77" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: 동일 필터 상태를 Dropdown/BottomSheet 두 컴포넌트가 공유하는지 상태 동기화 테스트</t>
+          <t>해당 없음 — Lighthouse 모바일 성능 점수로 갈음(수동 측정)</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>FE-12</t>
+          <t>FE-11</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
@@ -4922,17 +4922,17 @@
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>KPI 대시보드(비공개)</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>KPI 대시보드 페이지 구현(비공개)</t>
+          <t>필터 UI 반응형 공용 컴포넌트 구현</t>
         </is>
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>/kpi 페이지 — 비밀번호 입력 폼(미인증 시) + 5개 지표 카드/차트(최신성/근거율/전환율/이용률/응답지연). GNB·모바일 드로어에는 노출하지 않음(URL 직접 접근 전용)</t>
+          <t>데스크톱/태블릿 Dropdown, 모바일 BottomSheet 공용 컴포넌트</t>
         </is>
       </c>
       <c r="G78" s="4" t="inlineStr">
@@ -4942,86 +4942,86 @@
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
-          <t>KPI-01</t>
+          <t>FE-01</t>
         </is>
       </c>
       <c r="I78" s="3" t="inlineStr">
         <is>
-          <t>IA v1.2 4.7절</t>
+          <t>디자인가이드6.2</t>
         </is>
       </c>
       <c r="J78" s="3" t="inlineStr">
         <is>
-          <t>비밀번호 게이트 통과 후 5개 지표 정상 렌더링 확인, 오답 시 게이트 재노출 확인</t>
+          <t>3개 화면(티어리스트/아이템빌드/증강체)에서 재사용 확인</t>
         </is>
       </c>
       <c r="K78" s="3" t="inlineStr">
         <is>
-          <t>Vitest: 비밀번호 게이트 컴포넌트 성공/실패 케이스, 지표 카드 렌더링 테스트</t>
+          <t>Vitest+RTL: 동일 필터 상태를 Dropdown/BottomSheet 두 컴포넌트가 공유하는지 상태 동기화 테스트</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
+          <t>FE-12</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>프론트엔드</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>KPI 대시보드(비공개)</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>KPI 대시보드 페이지 구현(비공개)</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="inlineStr">
+        <is>
+          <t>/kpi 페이지 — 비밀번호 입력 폼(미인증 시) + 5개 지표 카드/차트(최신성/근거율/전환율/이용률/응답지연). GNB·모바일 드로어에는 노출하지 않음(URL 직접 접근 전용)</t>
+        </is>
+      </c>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>필수</t>
+        </is>
+      </c>
+      <c r="H79" s="3" t="inlineStr">
+        <is>
           <t>KPI-01</t>
         </is>
       </c>
-      <c r="B79" s="4" t="inlineStr">
-        <is>
-          <t>코딩</t>
-        </is>
-      </c>
-      <c r="C79" s="4" t="inlineStr">
-        <is>
-          <t>KPI모니터링</t>
-        </is>
-      </c>
-      <c r="D79" s="3" t="inlineStr">
-        <is>
-          <t>공통</t>
-        </is>
-      </c>
-      <c r="E79" s="3" t="inlineStr">
-        <is>
-          <t>KPI 대시보드 백엔드 API 구현(자체, Metabase 대체)</t>
-        </is>
-      </c>
-      <c r="F79" s="3" t="inlineStr">
-        <is>
-          <t>5개 지표(최신성/근거율/전환율/이용률/응답지연) 집계 GET /kpi/summary 구현 + POST /kpi/auth 비밀번호 게이트(환경변수 KPI_DASHBOARD_PASSWORD 대조, 서명 토큰 발급) 구현. Metabase 대신 자체 페이지(FE-12)로 제공 (PM 결정 2026-08-03)</t>
-        </is>
-      </c>
-      <c r="G79" s="4" t="inlineStr">
-        <is>
-          <t>필수</t>
-        </is>
-      </c>
-      <c r="H79" s="3" t="inlineStr">
-        <is>
-          <t>DATA-03</t>
-        </is>
-      </c>
       <c r="I79" s="3" t="inlineStr">
         <is>
-          <t>PRD 3-3 / IA v1.2 4.7절 (자체구현 결정 2026-08-03)</t>
+          <t>IA v1.2 4.7절</t>
         </is>
       </c>
       <c r="J79" s="3" t="inlineStr">
         <is>
-          <t>5개 지표 API 정상 응답 확인, 비밀번호 게이트 통과/실패 동작 확인</t>
+          <t>비밀번호 게이트 통과 후 5개 지표 정상 렌더링 확인, 오답 시 게이트 재노출 확인</t>
         </is>
       </c>
       <c r="K79" s="3" t="inlineStr">
         <is>
-          <t>pytest: 비밀번호 게이트 성공/실패 케이스, mock 로그 데이터로 5개 지표 집계 쿼리 결과 검증</t>
+          <t>Vitest: 비밀번호 게이트 컴포넌트 성공/실패 케이스, 지표 카드 렌더링 테스트</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>KPI-02</t>
+          <t>KPI-01</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
@@ -5041,12 +5041,12 @@
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>RAGAS 주간 배치 평가 파이프라인 구현</t>
+          <t>KPI 대시보드 백엔드 API 구현(자체, Metabase 대체)</t>
         </is>
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>GitHub Actions 주간 배치로 Faithfulness/Answer Relevancy 산출, ragas_eval_results 적재</t>
+          <t>5개 지표(최신성/근거율/전환율/이용률/응답지연) 집계 GET /kpi/summary 구현 + POST /kpi/auth 비밀번호 게이트(환경변수 KPI_DASHBOARD_PASSWORD 대조, 서명 토큰 발급) 구현. Metabase 대신 자체 페이지(FE-12)로 제공 (PM 결정 2026-08-03)</t>
         </is>
       </c>
       <c r="G80" s="4" t="inlineStr">
@@ -5056,143 +5056,143 @@
       </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
-          <t>CHAT-09,SET-08</t>
+          <t>DATA-03</t>
         </is>
       </c>
       <c r="I80" s="3" t="inlineStr">
         <is>
-          <t>PRD3-3·설계서4.7</t>
+          <t>PRD 3-3 / IA v1.2 4.7절 (자체구현 결정 2026-08-03)</t>
         </is>
       </c>
       <c r="J80" s="3" t="inlineStr">
         <is>
-          <t>배치 실행 후 결과 적재 확인</t>
+          <t>5개 지표 API 정상 응답 확인, 비밀번호 게이트 통과/실패 동작 확인</t>
         </is>
       </c>
       <c r="K80" s="3" t="inlineStr">
         <is>
-          <t>pytest: mock 질의-답변 샘플로 RAGAS 스코어러 호출 및 ragas_eval_results 적재 필드 확인</t>
+          <t>pytest: 비밀번호 게이트 성공/실패 케이스, mock 로그 데이터로 5개 지표 집계 쿼리 결과 검증</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
+          <t>KPI-02</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>KPI모니터링</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>공통</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="inlineStr">
+        <is>
+          <t>RAGAS 주간 배치 평가 파이프라인 구현</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="inlineStr">
+        <is>
+          <t>GitHub Actions 주간 배치로 Faithfulness/Answer Relevancy 산출, ragas_eval_results 적재</t>
+        </is>
+      </c>
+      <c r="G81" s="4" t="inlineStr">
+        <is>
+          <t>필수</t>
+        </is>
+      </c>
+      <c r="H81" s="3" t="inlineStr">
+        <is>
+          <t>CHAT-09,SET-08</t>
+        </is>
+      </c>
+      <c r="I81" s="3" t="inlineStr">
+        <is>
+          <t>PRD3-3·설계서4.7</t>
+        </is>
+      </c>
+      <c r="J81" s="3" t="inlineStr">
+        <is>
+          <t>배치 실행 후 결과 적재 확인</t>
+        </is>
+      </c>
+      <c r="K81" s="3" t="inlineStr">
+        <is>
+          <t>pytest: mock 질의-답변 샘플로 RAGAS 스코어러 호출 및 ragas_eval_results 적재 필드 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
           <t>KPI-03</t>
         </is>
       </c>
-      <c r="B81" s="4" t="inlineStr">
-        <is>
-          <t>코딩</t>
-        </is>
-      </c>
-      <c r="C81" s="4" t="inlineStr">
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
         <is>
           <t>KPI모니터링</t>
         </is>
       </c>
-      <c r="D81" s="3" t="inlineStr">
+      <c r="D82" s="3" t="inlineStr">
         <is>
           <t>공통</t>
         </is>
       </c>
-      <c r="E81" s="3" t="inlineStr">
+      <c r="E82" s="3" t="inlineStr">
         <is>
           <t>목표 미달 알림 로직 구현</t>
         </is>
       </c>
-      <c r="F81" s="3" t="inlineStr">
+      <c r="F82" s="3" t="inlineStr">
         <is>
           <t>2주 연속 목표 미달 감지 시 알림 발송</t>
         </is>
       </c>
-      <c r="G81" s="4" t="inlineStr">
+      <c r="G82" s="4" t="inlineStr">
         <is>
           <t>권장</t>
         </is>
       </c>
-      <c r="H81" s="3" t="inlineStr">
+      <c r="H82" s="3" t="inlineStr">
         <is>
           <t>KPI-01</t>
         </is>
       </c>
-      <c r="I81" s="3" t="inlineStr">
+      <c r="I82" s="3" t="inlineStr">
         <is>
           <t>PRD3-3</t>
         </is>
       </c>
-      <c r="J81" s="3" t="inlineStr">
+      <c r="J82" s="3" t="inlineStr">
         <is>
           <t>알림 트리거 테스트 통과</t>
         </is>
       </c>
-      <c r="K81" s="3" t="inlineStr">
+      <c r="K82" s="3" t="inlineStr">
         <is>
           <t>pytest: 2주 연속 미달 mock 데이터 주입 시 알림 함수 호출 확인</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="5" t="inlineStr">
-        <is>
-          <t>TEST-00</t>
-        </is>
-      </c>
-      <c r="B82" s="5" t="inlineStr">
-        <is>
-          <t>테스트</t>
-        </is>
-      </c>
-      <c r="C82" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D82" s="3" t="inlineStr">
-        <is>
-          <t>공통(정책·로직 크리티컬 TASK)</t>
-        </is>
-      </c>
-      <c r="E82" s="3" t="inlineStr">
-        <is>
-          <t>핵심 정책/로직 테스트 시나리오 사전 정의</t>
-        </is>
-      </c>
-      <c r="F82" s="3" t="inlineStr">
-        <is>
-          <t>API-05, CHAT-04, CHAT-06, PGA-04~09, DATA-13 등 정책 준수·크리티컬 계산 로직이 걸린 TASK에 한해, 코딩 착수 전 입력값·기대출력·경계값을 포함한 테스트 시나리오를 문서화하고 PM과 합의한다. 해당 TASK의 구현자는 이 문서를 기준으로 단위 테스트를 먼저 작성한 뒤 구현한다</t>
-        </is>
-      </c>
-      <c r="G82" s="5" t="inlineStr">
-        <is>
-          <t>필수</t>
-        </is>
-      </c>
-      <c r="H82" s="3" t="inlineStr">
-        <is>
-          <t>SET-01</t>
-        </is>
-      </c>
-      <c r="I82" s="3" t="inlineStr">
-        <is>
-          <t>요구사항정의서 NFR-SEC·FR-PGA, 설계서 4.4.2·4.4.3·4.5.1·4.5.2</t>
-        </is>
-      </c>
-      <c r="J82" s="3" t="inlineStr">
-        <is>
-          <t>/docs/test-scenarios.md에 대상 TASK별 시나리오 표 작성 및 PM 승인 완료</t>
-        </is>
-      </c>
-      <c r="K82" s="3" t="inlineStr">
-        <is>
-          <t>해당 TASK 자체가 산출물 — /docs/test-scenarios.md 표 작성</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>TEST-01</t>
+          <t>TEST-00</t>
         </is>
       </c>
       <c r="B83" s="5" t="inlineStr">
@@ -5207,17 +5207,17 @@
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>공통(정책·로직 크리티컬 TASK)</t>
         </is>
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>DB 스키마/마이그레이션 검증</t>
+          <t>핵심 정책/로직 테스트 시나리오 사전 정의</t>
         </is>
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>전체 테이블·인덱스·제약조건 검증</t>
+          <t>API-05, CHAT-04, CHAT-06, PGA-04~09, DATA-13 등 정책 준수·크리티컬 계산 로직이 걸린 TASK에 한해, 코딩 착수 전 입력값·기대출력·경계값을 포함한 테스트 시나리오를 문서화하고 PM과 합의한다. 해당 TASK의 구현자는 이 문서를 기준으로 단위 테스트를 먼저 작성한 뒤 구현한다</t>
         </is>
       </c>
       <c r="G83" s="5" t="inlineStr">
@@ -5227,29 +5227,29 @@
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>DATA-01,DATA-02,DATA-03,DATA-04</t>
+          <t>SET-01</t>
         </is>
       </c>
       <c r="I83" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>요구사항정의서 NFR-SEC·FR-PGA, 설계서 4.4.2·4.4.3·4.5.1·4.5.2</t>
         </is>
       </c>
       <c r="J83" s="3" t="inlineStr">
         <is>
-          <t>마이그레이션 재실행 무결성 확인</t>
+          <t>/docs/test-scenarios.md에 대상 TASK별 시나리오 표 작성 및 PM 승인 완료</t>
         </is>
       </c>
       <c r="K83" s="3" t="inlineStr">
         <is>
-          <t>해당 TASK 자체가 테스트 작성/실행 TASK의 산출물</t>
+          <t>해당 TASK 자체가 산출물 — /docs/test-scenarios.md 표 작성</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>TEST-02</t>
+          <t>TEST-01</t>
         </is>
       </c>
       <c r="B84" s="5" t="inlineStr">
@@ -5264,17 +5264,17 @@
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>티어리스트~증강체정보</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>catalog API 단위/통합 테스트</t>
+          <t>DB 스키마/마이그레이션 검증</t>
         </is>
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>API-02~06 엔드포인트 테스트 코드 작성 및 실행</t>
+          <t>전체 테이블·인덱스·제약조건 검증</t>
         </is>
       </c>
       <c r="G84" s="5" t="inlineStr">
@@ -5284,7 +5284,7 @@
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
-          <t>API-02,API-03,API-04,API-05,API-06</t>
+          <t>DATA-01,DATA-02,DATA-03,DATA-04</t>
         </is>
       </c>
       <c r="I84" s="3" t="inlineStr">
@@ -5294,7 +5294,7 @@
       </c>
       <c r="J84" s="3" t="inlineStr">
         <is>
-          <t>전체 테스트 통과</t>
+          <t>마이그레이션 재실행 무결성 확인</t>
         </is>
       </c>
       <c r="K84" s="3" t="inlineStr">
@@ -5306,7 +5306,7 @@
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>TEST-03</t>
+          <t>TEST-02</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr">
@@ -5321,17 +5321,17 @@
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>챗봇위젯</t>
+          <t>티어리스트~증강체정보</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>chat API 및 RAG 파이프라인 테스트</t>
+          <t>catalog API 단위/통합 테스트</t>
         </is>
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>의도분류/검색/생성/후처리/캐싱 테스트</t>
+          <t>API-02~06 엔드포인트 테스트 코드 작성 및 실행</t>
         </is>
       </c>
       <c r="G85" s="5" t="inlineStr">
@@ -5341,7 +5341,7 @@
       </c>
       <c r="H85" s="3" t="inlineStr">
         <is>
-          <t>CHAT-01,CHAT-02,CHAT-03,CHAT-04,CHAT-05,CHAT-06,CHAT-07,CHAT-08,CHAT-09</t>
+          <t>API-02,API-03,API-04,API-05,API-06</t>
         </is>
       </c>
       <c r="I85" s="3" t="inlineStr">
@@ -5351,7 +5351,7 @@
       </c>
       <c r="J85" s="3" t="inlineStr">
         <is>
-          <t>전체 통과, 근거율 샘플 검증</t>
+          <t>전체 테스트 통과</t>
         </is>
       </c>
       <c r="K85" s="3" t="inlineStr">
@@ -5363,7 +5363,7 @@
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>TEST-04</t>
+          <t>TEST-03</t>
         </is>
       </c>
       <c r="B86" s="5" t="inlineStr">
@@ -5378,17 +5378,17 @@
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석·분석리포트</t>
+          <t>챗봇위젯</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>analysis API 및 스코어링 로직 테스트</t>
+          <t>chat API 및 RAG 파이프라인 테스트</t>
         </is>
       </c>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>PUUID변환/매치조회/3개지표계산/코칭생성 테스트</t>
+          <t>의도분류/검색/생성/후처리/캐싱 테스트</t>
         </is>
       </c>
       <c r="G86" s="5" t="inlineStr">
@@ -5398,7 +5398,7 @@
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
-          <t>PGA-01,PGA-02,PGA-03,PGA-04,PGA-05,PGA-06,PGA-07,PGA-08,PGA-09,PGA-10</t>
+          <t>CHAT-01,CHAT-02,CHAT-03,CHAT-04,CHAT-05,CHAT-06,CHAT-07,CHAT-08,CHAT-09</t>
         </is>
       </c>
       <c r="I86" s="3" t="inlineStr">
@@ -5408,7 +5408,7 @@
       </c>
       <c r="J86" s="3" t="inlineStr">
         <is>
-          <t>전체 통과</t>
+          <t>전체 통과, 근거율 샘플 검증</t>
         </is>
       </c>
       <c r="K86" s="3" t="inlineStr">
@@ -5420,7 +5420,7 @@
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>TEST-05</t>
+          <t>TEST-04</t>
         </is>
       </c>
       <c r="B87" s="5" t="inlineStr">
@@ -5435,17 +5435,17 @@
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>사후패인분석·분석리포트</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>배치 파이프라인 통합 테스트</t>
+          <t>analysis API 및 스코어링 로직 테스트</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>패치감지→수집→정규화→임베딩→원자적전환 end-to-end 테스트</t>
+          <t>PUUID변환/매치조회/3개지표계산/코칭생성 테스트</t>
         </is>
       </c>
       <c r="G87" s="5" t="inlineStr">
@@ -5455,7 +5455,7 @@
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
-          <t>DATA-05,DATA-08,DATA-09,DATA-10,DATA-11,DATA-12,DATA-13,DATA-14,DATA-15</t>
+          <t>PGA-01,PGA-02,PGA-03,PGA-04,PGA-05,PGA-06,PGA-07,PGA-08,PGA-09,PGA-10</t>
         </is>
       </c>
       <c r="I87" s="3" t="inlineStr">
@@ -5465,7 +5465,7 @@
       </c>
       <c r="J87" s="3" t="inlineStr">
         <is>
-          <t>정상/중간실패 시나리오 모두 검증</t>
+          <t>전체 통과</t>
         </is>
       </c>
       <c r="K87" s="3" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>TEST-06</t>
+          <t>TEST-05</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
@@ -5492,17 +5492,17 @@
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>챗봇위젯</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>챗봇 정책 준수 테스트</t>
+          <t>배치 파이프라인 통합 테스트</t>
         </is>
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>Legend 승률 비노출·프롬프트 인젝션 방어·범위밖 질문 안내 검증</t>
+          <t>패치감지→수집→정규화→임베딩→원자적전환 end-to-end 테스트</t>
         </is>
       </c>
       <c r="G88" s="5" t="inlineStr">
@@ -5512,17 +5512,17 @@
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>CHAT-04,CHAT-06</t>
+          <t>DATA-05,DATA-08,DATA-09,DATA-10,DATA-11,DATA-12,DATA-13,DATA-14,DATA-15</t>
         </is>
       </c>
       <c r="I88" s="3" t="inlineStr">
         <is>
-          <t>PRD10-1·12장</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J88" s="3" t="inlineStr">
         <is>
-          <t>정책 위반 케이스 0건</t>
+          <t>정상/중간실패 시나리오 모두 검증</t>
         </is>
       </c>
       <c r="K88" s="3" t="inlineStr">
@@ -5534,7 +5534,7 @@
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>TEST-07</t>
+          <t>TEST-06</t>
         </is>
       </c>
       <c r="B89" s="5" t="inlineStr">
@@ -5549,17 +5549,17 @@
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석·분석리포트</t>
+          <t>챗봇위젯</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>프라이버시 마스킹 테스트</t>
+          <t>챗봇 정책 준수 테스트</t>
         </is>
       </c>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>상대 닉네임 마스킹 누락 케이스 점검</t>
+          <t>Legend 승률 비노출·프롬프트 인젝션 방어·범위밖 질문 안내 검증</t>
         </is>
       </c>
       <c r="G89" s="5" t="inlineStr">
@@ -5569,17 +5569,17 @@
       </c>
       <c r="H89" s="3" t="inlineStr">
         <is>
-          <t>PGA-09</t>
+          <t>CHAT-04,CHAT-06</t>
         </is>
       </c>
       <c r="I89" s="3" t="inlineStr">
         <is>
-          <t>PRD7-3·12장</t>
+          <t>PRD10-1·12장</t>
         </is>
       </c>
       <c r="J89" s="3" t="inlineStr">
         <is>
-          <t>마스킹 누락 0건</t>
+          <t>정책 위반 케이스 0건</t>
         </is>
       </c>
       <c r="K89" s="3" t="inlineStr">
@@ -5591,7 +5591,7 @@
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>TEST-08</t>
+          <t>TEST-07</t>
         </is>
       </c>
       <c r="B90" s="5" t="inlineStr">
@@ -5606,17 +5606,17 @@
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>전체 7화면</t>
+          <t>사후패인분석·분석리포트</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>프론트엔드 E2E 테스트(Playwright)</t>
+          <t>프라이버시 마스킹 테스트</t>
         </is>
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>PRD 8-1/8-2/8-3 사용자 플로우 기준 시나리오 작성</t>
+          <t>상대 닉네임 마스킹 누락 케이스 점검</t>
         </is>
       </c>
       <c r="G90" s="5" t="inlineStr">
@@ -5626,17 +5626,17 @@
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>FE-03,FE-04,FE-05,FE-06,FE-07,FE-08,FE-09</t>
+          <t>PGA-09</t>
         </is>
       </c>
       <c r="I90" s="3" t="inlineStr">
         <is>
-          <t>PRD8장</t>
+          <t>PRD7-3·12장</t>
         </is>
       </c>
       <c r="J90" s="3" t="inlineStr">
         <is>
-          <t>전체 시나리오 통과</t>
+          <t>마스킹 누락 0건</t>
         </is>
       </c>
       <c r="K90" s="3" t="inlineStr">
@@ -5648,7 +5648,7 @@
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>TEST-09</t>
+          <t>TEST-08</t>
         </is>
       </c>
       <c r="B91" s="5" t="inlineStr">
@@ -5668,12 +5668,12 @@
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>반응형 크로스브라우저 테스트</t>
+          <t>프론트엔드 E2E 테스트(Playwright)</t>
         </is>
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>iOS Safari/Android Chrome/Desktop Chrome 3개 브레이크포인트 검증</t>
+          <t>PRD 8-1/8-2/8-3 사용자 플로우 기준 시나리오 작성</t>
         </is>
       </c>
       <c r="G91" s="5" t="inlineStr">
@@ -5688,12 +5688,12 @@
       </c>
       <c r="I91" s="3" t="inlineStr">
         <is>
-          <t>PRD12장(QA리소스제약)</t>
+          <t>PRD8장</t>
         </is>
       </c>
       <c r="J91" s="3" t="inlineStr">
         <is>
-          <t>주요 화면 시각 회귀 없음 확인</t>
+          <t>전체 시나리오 통과</t>
         </is>
       </c>
       <c r="K91" s="3" t="inlineStr">
@@ -5705,121 +5705,121 @@
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
         <is>
+          <t>TEST-09</t>
+        </is>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>테스트</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>전체 7화면</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>반응형 크로스브라우저 테스트</t>
+        </is>
+      </c>
+      <c r="F92" s="3" t="inlineStr">
+        <is>
+          <t>iOS Safari/Android Chrome/Desktop Chrome 3개 브레이크포인트 검증</t>
+        </is>
+      </c>
+      <c r="G92" s="5" t="inlineStr">
+        <is>
+          <t>필수</t>
+        </is>
+      </c>
+      <c r="H92" s="3" t="inlineStr">
+        <is>
+          <t>FE-03,FE-04,FE-05,FE-06,FE-07,FE-08,FE-09</t>
+        </is>
+      </c>
+      <c r="I92" s="3" t="inlineStr">
+        <is>
+          <t>PRD12장(QA리소스제약)</t>
+        </is>
+      </c>
+      <c r="J92" s="3" t="inlineStr">
+        <is>
+          <t>주요 화면 시각 회귀 없음 확인</t>
+        </is>
+      </c>
+      <c r="K92" s="3" t="inlineStr">
+        <is>
+          <t>해당 TASK 자체가 테스트 작성/실행 TASK의 산출물</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="5" t="inlineStr">
+        <is>
           <t>TEST-10</t>
         </is>
       </c>
-      <c r="B92" s="5" t="inlineStr">
+      <c r="B93" s="5" t="inlineStr">
         <is>
           <t>테스트</t>
         </is>
       </c>
-      <c r="C92" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D92" s="3" t="inlineStr">
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
         <is>
           <t>공통</t>
         </is>
       </c>
-      <c r="E92" s="3" t="inlineStr">
+      <c r="E93" s="3" t="inlineStr">
         <is>
           <t>Rate Limiting/보안 테스트</t>
         </is>
       </c>
-      <c r="F92" s="3" t="inlineStr">
+      <c r="F93" s="3" t="inlineStr">
         <is>
           <t>요청 한도 초과·비정상 입력 처리 검증</t>
         </is>
       </c>
-      <c r="G92" s="5" t="inlineStr">
+      <c r="G93" s="5" t="inlineStr">
         <is>
           <t>권장</t>
         </is>
       </c>
-      <c r="H92" s="3" t="inlineStr">
+      <c r="H93" s="3" t="inlineStr">
         <is>
           <t>API-07</t>
         </is>
       </c>
-      <c r="I92" s="3" t="inlineStr">
+      <c r="I93" s="3" t="inlineStr">
         <is>
           <t>설계서4.2·6장</t>
         </is>
       </c>
-      <c r="J92" s="3" t="inlineStr">
+      <c r="J93" s="3" t="inlineStr">
         <is>
           <t>429 응답 및 로그 확인</t>
         </is>
       </c>
-      <c r="K92" s="3" t="inlineStr">
+      <c r="K93" s="3" t="inlineStr">
         <is>
           <t>해당 TASK 자체가 테스트 작성/실행 TASK의 산출물</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="6" t="inlineStr">
-        <is>
-          <t>REL-01</t>
-        </is>
-      </c>
-      <c r="B93" s="6" t="inlineStr">
-        <is>
-          <t>배포릴리즈</t>
-        </is>
-      </c>
-      <c r="C93" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D93" s="3" t="inlineStr">
-        <is>
-          <t>전체</t>
-        </is>
-      </c>
-      <c r="E93" s="3" t="inlineStr">
-        <is>
-          <t>스테이징 통합 배포 및 QA</t>
-        </is>
-      </c>
-      <c r="F93" s="3" t="inlineStr">
-        <is>
-          <t>전체 기능 스테이징 환경 배포 후 PM 검수</t>
-        </is>
-      </c>
-      <c r="G93" s="6" t="inlineStr">
-        <is>
-          <t>필수</t>
-        </is>
-      </c>
-      <c r="H93" s="3" t="inlineStr">
-        <is>
-          <t>TEST-01,TEST-02,TEST-03,TEST-04,TEST-05,TEST-06,TEST-07,TEST-08,TEST-09</t>
-        </is>
-      </c>
-      <c r="I93" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J93" s="3" t="inlineStr">
-        <is>
-          <t>PM 승인 획득</t>
-        </is>
-      </c>
-      <c r="K93" s="3" t="inlineStr">
-        <is>
-          <t>TEST-00~10 전체 그린 상태를 배포 전제조건으로 확인</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>REL-02</t>
+          <t>REL-01</t>
         </is>
       </c>
       <c r="B94" s="6" t="inlineStr">
@@ -5839,12 +5839,12 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>프로덕션 배포</t>
+          <t>스테이징 통합 배포 및 QA</t>
         </is>
       </c>
       <c r="F94" s="3" t="inlineStr">
         <is>
-          <t>Cloudflare Pages+Render 프로덕션 반영, PM 최종 승인 후 커밋/푸시</t>
+          <t>전체 기능 스테이징 환경 배포 후 PM 검수</t>
         </is>
       </c>
       <c r="G94" s="6" t="inlineStr">
@@ -5854,7 +5854,7 @@
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>REL-01</t>
+          <t>TEST-01,TEST-02,TEST-03,TEST-04,TEST-05,TEST-06,TEST-07,TEST-08,TEST-09</t>
         </is>
       </c>
       <c r="I94" s="3" t="inlineStr">
@@ -5864,19 +5864,19 @@
       </c>
       <c r="J94" s="3" t="inlineStr">
         <is>
-          <t>프로덕션 URL 정상 서비스 확인</t>
+          <t>PM 승인 획득</t>
         </is>
       </c>
       <c r="K94" s="3" t="inlineStr">
         <is>
-          <t>프로덕션 스모크 테스트: 핵심 URL 200 확인, 챗봇 질의 1회 왕복 확인</t>
+          <t>TEST-00~10 전체 그린 상태를 배포 전제조건으로 확인</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>REL-03</t>
+          <t>REL-02</t>
         </is>
       </c>
       <c r="B95" s="6" t="inlineStr">
@@ -5891,17 +5891,17 @@
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>전체</t>
         </is>
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>배포 후 모니터링 점검</t>
+          <t>프로덕션 배포</t>
         </is>
       </c>
       <c r="F95" s="3" t="inlineStr">
         <is>
-          <t>콜드스타트 비중·응답지연 p50/p95 확인</t>
+          <t>Cloudflare Pages+Render 프로덕션 반영, PM 최종 승인 후 커밋/푸시</t>
         </is>
       </c>
       <c r="G95" s="6" t="inlineStr">
@@ -5911,29 +5911,29 @@
       </c>
       <c r="H95" s="3" t="inlineStr">
         <is>
-          <t>REL-02,KPI-01</t>
+          <t>REL-01</t>
         </is>
       </c>
       <c r="I95" s="3" t="inlineStr">
         <is>
-          <t>PRD3-3</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J95" s="3" t="inlineStr">
         <is>
-          <t>초기 1주 지표 리뷰 완료</t>
+          <t>프로덕션 URL 정상 서비스 확인</t>
         </is>
       </c>
       <c r="K95" s="3" t="inlineStr">
         <is>
-          <t>해당 없음 — 모니터링 지표 수동 리뷰</t>
+          <t>프로덕션 스모크 테스트: 핵심 URL 200 확인, 챗봇 질의 1회 왕복 확인</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="6" t="inlineStr">
         <is>
-          <t>REL-04</t>
+          <t>REL-03</t>
         </is>
       </c>
       <c r="B96" s="6" t="inlineStr">
@@ -5953,92 +5953,149 @@
       </c>
       <c r="E96" s="3" t="inlineStr">
         <is>
-          <t>1.0 출시 회고 및 KPI 재보정 계획 수립</t>
+          <t>배포 후 모니터링 점검</t>
         </is>
       </c>
       <c r="F96" s="3" t="inlineStr">
         <is>
-          <t>2~4주 실측 데이터 수집 계획 및 재보정 일정 수립</t>
+          <t>콜드스타트 비중·응답지연 p50/p95 확인</t>
         </is>
       </c>
       <c r="G96" s="6" t="inlineStr">
         <is>
-          <t>권장</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="H96" s="3" t="inlineStr">
         <is>
-          <t>REL-03</t>
+          <t>REL-02,KPI-01</t>
         </is>
       </c>
       <c r="I96" s="3" t="inlineStr">
         <is>
-          <t>PRD3-2·3-3</t>
+          <t>PRD3-3</t>
         </is>
       </c>
       <c r="J96" s="3" t="inlineStr">
         <is>
-          <t>재보정 일정 문서화</t>
+          <t>초기 1주 지표 리뷰 완료</t>
         </is>
       </c>
       <c r="K96" s="3" t="inlineStr">
         <is>
-          <t>해당 없음 — 문서화 작업</t>
+          <t>해당 없음 — 모니터링 지표 수동 리뷰</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="6" t="inlineStr">
         <is>
+          <t>REL-04</t>
+        </is>
+      </c>
+      <c r="B97" s="6" t="inlineStr">
+        <is>
+          <t>배포릴리즈</t>
+        </is>
+      </c>
+      <c r="C97" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>공통</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>1.0 출시 회고 및 KPI 재보정 계획 수립</t>
+        </is>
+      </c>
+      <c r="F97" s="3" t="inlineStr">
+        <is>
+          <t>2~4주 실측 데이터 수집 계획 및 재보정 일정 수립</t>
+        </is>
+      </c>
+      <c r="G97" s="6" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H97" s="3" t="inlineStr">
+        <is>
+          <t>REL-03</t>
+        </is>
+      </c>
+      <c r="I97" s="3" t="inlineStr">
+        <is>
+          <t>PRD3-2·3-3</t>
+        </is>
+      </c>
+      <c r="J97" s="3" t="inlineStr">
+        <is>
+          <t>재보정 일정 문서화</t>
+        </is>
+      </c>
+      <c r="K97" s="3" t="inlineStr">
+        <is>
+          <t>해당 없음 — 문서화 작업</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="6" t="inlineStr">
+        <is>
           <t>REL-05</t>
         </is>
       </c>
-      <c r="B97" s="6" t="inlineStr">
+      <c r="B98" s="6" t="inlineStr">
         <is>
           <t>배포릴리즈</t>
         </is>
       </c>
-      <c r="C97" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D97" s="3" t="inlineStr">
+      <c r="C98" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
         <is>
           <t>전체</t>
         </is>
       </c>
-      <c r="E97" s="3" t="inlineStr">
+      <c r="E98" s="3" t="inlineStr">
         <is>
           <t>포트폴리오 공개 전환 준비 체크리스트</t>
         </is>
       </c>
-      <c r="F97" s="3" t="inlineStr">
+      <c r="F98" s="3" t="inlineStr">
         <is>
           <t>저장소를 private에서 public으로 전환하기 전 확인·조치한다: (1) gitleaks 등으로 커밋 히스토리 전체에서 시크릿·API 키 잔존 여부 스캔 (2) 테스트 fixture 전수 조사 — 실제 Riot ID/PUUID/닉네임/매치 데이터가 아닌 합성 데이터로만 구성됐는지 확인, 실데이터가 섞여 있으면 fixture 재작성 후 필요시 git 히스토리 정리 (3) README에 'Riot Games와 무관한 비공식 팬 프로젝트' 디스클레이머 추가 (4) 라이브 배포 URL을 README/공개 자료에 노출할지 결정 (5) 노출하기로 하면 챗봇/전적조회 진입점에 Cloudflare Turnstile 등 경량 봇 방지 적용 검토. 무료 호스팅 비용에는 영향 없음(저장소 공개 여부와 인프라 비용은 무관)</t>
         </is>
       </c>
-      <c r="G97" s="6" t="inlineStr">
+      <c r="G98" s="6" t="inlineStr">
         <is>
           <t>권장</t>
         </is>
       </c>
-      <c r="H97" s="3" t="inlineStr">
+      <c r="H98" s="3" t="inlineStr">
         <is>
           <t>REL-04</t>
         </is>
       </c>
-      <c r="I97" s="3" t="inlineStr">
+      <c r="I98" s="3" t="inlineStr">
         <is>
           <t>PM 결정사항(2026-07-30 대화), policies.md 11번</t>
         </is>
       </c>
-      <c r="J97" s="3" t="inlineStr">
+      <c r="J98" s="3" t="inlineStr">
         <is>
           <t>체크리스트 5개 항목 모두 확인·조치 완료 및 PM 승인 후 저장소 visibility를 public으로 변경</t>
         </is>
       </c>
-      <c r="K97" s="3" t="inlineStr">
+      <c r="K98" s="3" t="inlineStr">
         <is>
           <t>정량 검증: gitleaks(또는 동급 도구) 스캔 결과 시크릿 탐지 0건, 전체 fixture 파일에서 실제 Riot ID 패턴(게임명#태그)·PUUID 패턴 검색 결과 0건</t>
         </is>

</xml_diff>

<commit_message>
docs(FE-13): FE-13 완료 처리(PM 승인) 및 WBS 신규 TASK 반영
FE-13(티어리스트 카드 챔피언 이미지 표시) WBS.xlsx 신규 반영, 진행현황.md
완료 처리. 운영 DB 백필은 배포 확인 후 별도 진행.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TFT_Hideout_WBS.xlsx
+++ b/TFT_Hideout_WBS.xlsx
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K98"/>
+  <dimension ref="A1:K99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5021,7 +5021,7 @@
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>KPI-01</t>
+          <t>FE-13</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
@@ -5031,54 +5031,54 @@
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>KPI모니터링</t>
+          <t>프론트엔드</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>티어리스트</t>
         </is>
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>KPI 대시보드 백엔드 API 구현(자체, Metabase 대체)</t>
+          <t>티어리스트 카드 챔피언 이미지 표시</t>
         </is>
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>5개 지표(최신성/근거율/전환율/이용률/응답지연) 집계 GET /kpi/summary 구현 + POST /kpi/auth 비밀번호 게이트(환경변수 KPI_DASHBOARD_PASSWORD 대조, 서명 토큰 발급) 구현. Metabase 대신 자체 페이지(FE-12)로 제공 (PM 결정 2026-08-03)</t>
+          <t>CompCard의 캐리 챔피언 점(●) placeholder를 Community Dragon 실제 챔피언 아이콘 이미지로 교체. champions 테이블에 square_icon_url 컬럼 추가(배치, Community Dragon squareIcon .tex 경로를 raw.communitydragon.org PNG URL로 변환), GET /catalog/tierlist 응답(CompSummary)에 캐리 챔피언 이름·이미지 URL 포함하도록 확장(API-02), CompCard에 next/image로 렌더링(이미지 없으면 기존 placeholder 폴백).</t>
         </is>
       </c>
       <c r="G80" s="4" t="inlineStr">
         <is>
-          <t>필수</t>
+          <t>권장</t>
         </is>
       </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
-          <t>DATA-03</t>
+          <t>FE-03</t>
         </is>
       </c>
       <c r="I80" s="3" t="inlineStr">
         <is>
-          <t>PRD 3-3 / IA v1.2 4.7절 (자체구현 결정 2026-08-03)</t>
+          <t>PM 요청 2026-08-05, Community Dragon squareIcon 필드 실호출로 URL 변환 가능 확인</t>
         </is>
       </c>
       <c r="J80" s="3" t="inlineStr">
         <is>
-          <t>5개 지표 API 정상 응답 확인, 비밀번호 게이트 통과/실패 동작 확인</t>
+          <t>티어리스트 카드에 캐리 챔피언 실제 이미지가 표시됨(이미지 URL 없으면 기존 placeholder로 폴백)</t>
         </is>
       </c>
       <c r="K80" s="3" t="inlineStr">
         <is>
-          <t>pytest: 비밀번호 게이트 성공/실패 케이스, mock 로그 데이터로 5개 지표 집계 쿼리 결과 검증</t>
+          <t>pytest(batch): squareIcon .tex 경로 -&gt; PNG URL 변환 함수 단위 테스트 / pytest(backend): GET /catalog/tierlist 응답에 캐리 챔피언 이름·이미지 URL 포함 확인 / Vitest+RTL: CompCard가 이미지 URL 있으면 이미지, 없으면 placeholder 렌더링 확인</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>KPI-02</t>
+          <t>KPI-01</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
@@ -5098,12 +5098,12 @@
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>RAGAS 주간 배치 평가 파이프라인 구현</t>
+          <t>KPI 대시보드 백엔드 API 구현(자체, Metabase 대체)</t>
         </is>
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>GitHub Actions 주간 배치로 Faithfulness/Answer Relevancy 산출, ragas_eval_results 적재</t>
+          <t>5개 지표(최신성/근거율/전환율/이용률/응답지연) 집계 GET /kpi/summary 구현 + POST /kpi/auth 비밀번호 게이트(환경변수 KPI_DASHBOARD_PASSWORD 대조, 서명 토큰 발급) 구현. Metabase 대신 자체 페이지(FE-12)로 제공 (PM 결정 2026-08-03)</t>
         </is>
       </c>
       <c r="G81" s="4" t="inlineStr">
@@ -5113,143 +5113,143 @@
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
-          <t>CHAT-09,SET-08</t>
+          <t>DATA-03</t>
         </is>
       </c>
       <c r="I81" s="3" t="inlineStr">
         <is>
-          <t>PRD3-3·설계서4.7</t>
+          <t>PRD 3-3 / IA v1.2 4.7절 (자체구현 결정 2026-08-03)</t>
         </is>
       </c>
       <c r="J81" s="3" t="inlineStr">
         <is>
-          <t>배치 실행 후 결과 적재 확인</t>
+          <t>5개 지표 API 정상 응답 확인, 비밀번호 게이트 통과/실패 동작 확인</t>
         </is>
       </c>
       <c r="K81" s="3" t="inlineStr">
         <is>
-          <t>pytest: mock 질의-답변 샘플로 RAGAS 스코어러 호출 및 ragas_eval_results 적재 필드 확인</t>
+          <t>pytest: 비밀번호 게이트 성공/실패 케이스, mock 로그 데이터로 5개 지표 집계 쿼리 결과 검증</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
+          <t>KPI-02</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>KPI모니터링</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>공통</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>RAGAS 주간 배치 평가 파이프라인 구현</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>GitHub Actions 주간 배치로 Faithfulness/Answer Relevancy 산출, ragas_eval_results 적재</t>
+        </is>
+      </c>
+      <c r="G82" s="4" t="inlineStr">
+        <is>
+          <t>필수</t>
+        </is>
+      </c>
+      <c r="H82" s="3" t="inlineStr">
+        <is>
+          <t>CHAT-09,SET-08</t>
+        </is>
+      </c>
+      <c r="I82" s="3" t="inlineStr">
+        <is>
+          <t>PRD3-3·설계서4.7</t>
+        </is>
+      </c>
+      <c r="J82" s="3" t="inlineStr">
+        <is>
+          <t>배치 실행 후 결과 적재 확인</t>
+        </is>
+      </c>
+      <c r="K82" s="3" t="inlineStr">
+        <is>
+          <t>pytest: mock 질의-답변 샘플로 RAGAS 스코어러 호출 및 ragas_eval_results 적재 필드 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
           <t>KPI-03</t>
         </is>
       </c>
-      <c r="B82" s="4" t="inlineStr">
-        <is>
-          <t>코딩</t>
-        </is>
-      </c>
-      <c r="C82" s="4" t="inlineStr">
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
         <is>
           <t>KPI모니터링</t>
         </is>
       </c>
-      <c r="D82" s="3" t="inlineStr">
+      <c r="D83" s="3" t="inlineStr">
         <is>
           <t>공통</t>
         </is>
       </c>
-      <c r="E82" s="3" t="inlineStr">
+      <c r="E83" s="3" t="inlineStr">
         <is>
           <t>목표 미달 알림 로직 구현</t>
         </is>
       </c>
-      <c r="F82" s="3" t="inlineStr">
+      <c r="F83" s="3" t="inlineStr">
         <is>
           <t>2주 연속 목표 미달 감지 시 알림 발송</t>
         </is>
       </c>
-      <c r="G82" s="4" t="inlineStr">
+      <c r="G83" s="4" t="inlineStr">
         <is>
           <t>권장</t>
         </is>
       </c>
-      <c r="H82" s="3" t="inlineStr">
+      <c r="H83" s="3" t="inlineStr">
         <is>
           <t>KPI-01</t>
         </is>
       </c>
-      <c r="I82" s="3" t="inlineStr">
+      <c r="I83" s="3" t="inlineStr">
         <is>
           <t>PRD3-3</t>
         </is>
       </c>
-      <c r="J82" s="3" t="inlineStr">
+      <c r="J83" s="3" t="inlineStr">
         <is>
           <t>알림 트리거 테스트 통과</t>
         </is>
       </c>
-      <c r="K82" s="3" t="inlineStr">
+      <c r="K83" s="3" t="inlineStr">
         <is>
           <t>pytest: 2주 연속 미달 mock 데이터 주입 시 알림 함수 호출 확인</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="5" t="inlineStr">
-        <is>
-          <t>TEST-00</t>
-        </is>
-      </c>
-      <c r="B83" s="5" t="inlineStr">
-        <is>
-          <t>테스트</t>
-        </is>
-      </c>
-      <c r="C83" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D83" s="3" t="inlineStr">
-        <is>
-          <t>공통(정책·로직 크리티컬 TASK)</t>
-        </is>
-      </c>
-      <c r="E83" s="3" t="inlineStr">
-        <is>
-          <t>핵심 정책/로직 테스트 시나리오 사전 정의</t>
-        </is>
-      </c>
-      <c r="F83" s="3" t="inlineStr">
-        <is>
-          <t>API-05, CHAT-04, CHAT-06, PGA-04~09, DATA-13 등 정책 준수·크리티컬 계산 로직이 걸린 TASK에 한해, 코딩 착수 전 입력값·기대출력·경계값을 포함한 테스트 시나리오를 문서화하고 PM과 합의한다. 해당 TASK의 구현자는 이 문서를 기준으로 단위 테스트를 먼저 작성한 뒤 구현한다</t>
-        </is>
-      </c>
-      <c r="G83" s="5" t="inlineStr">
-        <is>
-          <t>필수</t>
-        </is>
-      </c>
-      <c r="H83" s="3" t="inlineStr">
-        <is>
-          <t>SET-01</t>
-        </is>
-      </c>
-      <c r="I83" s="3" t="inlineStr">
-        <is>
-          <t>요구사항정의서 NFR-SEC·FR-PGA, 설계서 4.4.2·4.4.3·4.5.1·4.5.2</t>
-        </is>
-      </c>
-      <c r="J83" s="3" t="inlineStr">
-        <is>
-          <t>/docs/test-scenarios.md에 대상 TASK별 시나리오 표 작성 및 PM 승인 완료</t>
-        </is>
-      </c>
-      <c r="K83" s="3" t="inlineStr">
-        <is>
-          <t>해당 TASK 자체가 산출물 — /docs/test-scenarios.md 표 작성</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>TEST-01</t>
+          <t>TEST-00</t>
         </is>
       </c>
       <c r="B84" s="5" t="inlineStr">
@@ -5264,17 +5264,17 @@
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>공통(정책·로직 크리티컬 TASK)</t>
         </is>
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>DB 스키마/마이그레이션 검증</t>
+          <t>핵심 정책/로직 테스트 시나리오 사전 정의</t>
         </is>
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>전체 테이블·인덱스·제약조건 검증</t>
+          <t>API-05, CHAT-04, CHAT-06, PGA-04~09, DATA-13 등 정책 준수·크리티컬 계산 로직이 걸린 TASK에 한해, 코딩 착수 전 입력값·기대출력·경계값을 포함한 테스트 시나리오를 문서화하고 PM과 합의한다. 해당 TASK의 구현자는 이 문서를 기준으로 단위 테스트를 먼저 작성한 뒤 구현한다</t>
         </is>
       </c>
       <c r="G84" s="5" t="inlineStr">
@@ -5284,29 +5284,29 @@
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
-          <t>DATA-01,DATA-02,DATA-03,DATA-04</t>
+          <t>SET-01</t>
         </is>
       </c>
       <c r="I84" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>요구사항정의서 NFR-SEC·FR-PGA, 설계서 4.4.2·4.4.3·4.5.1·4.5.2</t>
         </is>
       </c>
       <c r="J84" s="3" t="inlineStr">
         <is>
-          <t>마이그레이션 재실행 무결성 확인</t>
+          <t>/docs/test-scenarios.md에 대상 TASK별 시나리오 표 작성 및 PM 승인 완료</t>
         </is>
       </c>
       <c r="K84" s="3" t="inlineStr">
         <is>
-          <t>해당 TASK 자체가 테스트 작성/실행 TASK의 산출물</t>
+          <t>해당 TASK 자체가 산출물 — /docs/test-scenarios.md 표 작성</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>TEST-02</t>
+          <t>TEST-01</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr">
@@ -5321,17 +5321,17 @@
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>티어리스트~증강체정보</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>catalog API 단위/통합 테스트</t>
+          <t>DB 스키마/마이그레이션 검증</t>
         </is>
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>API-02~06 엔드포인트 테스트 코드 작성 및 실행</t>
+          <t>전체 테이블·인덱스·제약조건 검증</t>
         </is>
       </c>
       <c r="G85" s="5" t="inlineStr">
@@ -5341,7 +5341,7 @@
       </c>
       <c r="H85" s="3" t="inlineStr">
         <is>
-          <t>API-02,API-03,API-04,API-05,API-06</t>
+          <t>DATA-01,DATA-02,DATA-03,DATA-04</t>
         </is>
       </c>
       <c r="I85" s="3" t="inlineStr">
@@ -5351,7 +5351,7 @@
       </c>
       <c r="J85" s="3" t="inlineStr">
         <is>
-          <t>전체 테스트 통과</t>
+          <t>마이그레이션 재실행 무결성 확인</t>
         </is>
       </c>
       <c r="K85" s="3" t="inlineStr">
@@ -5363,7 +5363,7 @@
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>TEST-03</t>
+          <t>TEST-02</t>
         </is>
       </c>
       <c r="B86" s="5" t="inlineStr">
@@ -5378,17 +5378,17 @@
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>챗봇위젯</t>
+          <t>티어리스트~증강체정보</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>chat API 및 RAG 파이프라인 테스트</t>
+          <t>catalog API 단위/통합 테스트</t>
         </is>
       </c>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>의도분류/검색/생성/후처리/캐싱 테스트</t>
+          <t>API-02~06 엔드포인트 테스트 코드 작성 및 실행</t>
         </is>
       </c>
       <c r="G86" s="5" t="inlineStr">
@@ -5398,7 +5398,7 @@
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
-          <t>CHAT-01,CHAT-02,CHAT-03,CHAT-04,CHAT-05,CHAT-06,CHAT-07,CHAT-08,CHAT-09</t>
+          <t>API-02,API-03,API-04,API-05,API-06</t>
         </is>
       </c>
       <c r="I86" s="3" t="inlineStr">
@@ -5408,7 +5408,7 @@
       </c>
       <c r="J86" s="3" t="inlineStr">
         <is>
-          <t>전체 통과, 근거율 샘플 검증</t>
+          <t>전체 테스트 통과</t>
         </is>
       </c>
       <c r="K86" s="3" t="inlineStr">
@@ -5420,7 +5420,7 @@
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>TEST-04</t>
+          <t>TEST-03</t>
         </is>
       </c>
       <c r="B87" s="5" t="inlineStr">
@@ -5435,17 +5435,17 @@
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석·분석리포트</t>
+          <t>챗봇위젯</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>analysis API 및 스코어링 로직 테스트</t>
+          <t>chat API 및 RAG 파이프라인 테스트</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>PUUID변환/매치조회/3개지표계산/코칭생성 테스트</t>
+          <t>의도분류/검색/생성/후처리/캐싱 테스트</t>
         </is>
       </c>
       <c r="G87" s="5" t="inlineStr">
@@ -5455,7 +5455,7 @@
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
-          <t>PGA-01,PGA-02,PGA-03,PGA-04,PGA-05,PGA-06,PGA-07,PGA-08,PGA-09,PGA-10</t>
+          <t>CHAT-01,CHAT-02,CHAT-03,CHAT-04,CHAT-05,CHAT-06,CHAT-07,CHAT-08,CHAT-09</t>
         </is>
       </c>
       <c r="I87" s="3" t="inlineStr">
@@ -5465,7 +5465,7 @@
       </c>
       <c r="J87" s="3" t="inlineStr">
         <is>
-          <t>전체 통과</t>
+          <t>전체 통과, 근거율 샘플 검증</t>
         </is>
       </c>
       <c r="K87" s="3" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>TEST-05</t>
+          <t>TEST-04</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
@@ -5492,17 +5492,17 @@
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>사후패인분석·분석리포트</t>
         </is>
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>배치 파이프라인 통합 테스트</t>
+          <t>analysis API 및 스코어링 로직 테스트</t>
         </is>
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>패치감지→수집→정규화→임베딩→원자적전환 end-to-end 테스트</t>
+          <t>PUUID변환/매치조회/3개지표계산/코칭생성 테스트</t>
         </is>
       </c>
       <c r="G88" s="5" t="inlineStr">
@@ -5512,7 +5512,7 @@
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>DATA-05,DATA-08,DATA-09,DATA-10,DATA-11,DATA-12,DATA-13,DATA-14,DATA-15</t>
+          <t>PGA-01,PGA-02,PGA-03,PGA-04,PGA-05,PGA-06,PGA-07,PGA-08,PGA-09,PGA-10</t>
         </is>
       </c>
       <c r="I88" s="3" t="inlineStr">
@@ -5522,7 +5522,7 @@
       </c>
       <c r="J88" s="3" t="inlineStr">
         <is>
-          <t>정상/중간실패 시나리오 모두 검증</t>
+          <t>전체 통과</t>
         </is>
       </c>
       <c r="K88" s="3" t="inlineStr">
@@ -5534,7 +5534,7 @@
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>TEST-06</t>
+          <t>TEST-05</t>
         </is>
       </c>
       <c r="B89" s="5" t="inlineStr">
@@ -5549,17 +5549,17 @@
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>챗봇위젯</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>챗봇 정책 준수 테스트</t>
+          <t>배치 파이프라인 통합 테스트</t>
         </is>
       </c>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>Legend 승률 비노출·프롬프트 인젝션 방어·범위밖 질문 안내 검증</t>
+          <t>패치감지→수집→정규화→임베딩→원자적전환 end-to-end 테스트</t>
         </is>
       </c>
       <c r="G89" s="5" t="inlineStr">
@@ -5569,17 +5569,17 @@
       </c>
       <c r="H89" s="3" t="inlineStr">
         <is>
-          <t>CHAT-04,CHAT-06</t>
+          <t>DATA-05,DATA-08,DATA-09,DATA-10,DATA-11,DATA-12,DATA-13,DATA-14,DATA-15</t>
         </is>
       </c>
       <c r="I89" s="3" t="inlineStr">
         <is>
-          <t>PRD10-1·12장</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J89" s="3" t="inlineStr">
         <is>
-          <t>정책 위반 케이스 0건</t>
+          <t>정상/중간실패 시나리오 모두 검증</t>
         </is>
       </c>
       <c r="K89" s="3" t="inlineStr">
@@ -5591,7 +5591,7 @@
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>TEST-07</t>
+          <t>TEST-06</t>
         </is>
       </c>
       <c r="B90" s="5" t="inlineStr">
@@ -5606,17 +5606,17 @@
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석·분석리포트</t>
+          <t>챗봇위젯</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>프라이버시 마스킹 테스트</t>
+          <t>챗봇 정책 준수 테스트</t>
         </is>
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>상대 닉네임 마스킹 누락 케이스 점검</t>
+          <t>Legend 승률 비노출·프롬프트 인젝션 방어·범위밖 질문 안내 검증</t>
         </is>
       </c>
       <c r="G90" s="5" t="inlineStr">
@@ -5626,17 +5626,17 @@
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>PGA-09</t>
+          <t>CHAT-04,CHAT-06</t>
         </is>
       </c>
       <c r="I90" s="3" t="inlineStr">
         <is>
-          <t>PRD7-3·12장</t>
+          <t>PRD10-1·12장</t>
         </is>
       </c>
       <c r="J90" s="3" t="inlineStr">
         <is>
-          <t>마스킹 누락 0건</t>
+          <t>정책 위반 케이스 0건</t>
         </is>
       </c>
       <c r="K90" s="3" t="inlineStr">
@@ -5648,7 +5648,7 @@
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>TEST-08</t>
+          <t>TEST-07</t>
         </is>
       </c>
       <c r="B91" s="5" t="inlineStr">
@@ -5663,17 +5663,17 @@
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>전체 7화면</t>
+          <t>사후패인분석·분석리포트</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>프론트엔드 E2E 테스트(Playwright)</t>
+          <t>프라이버시 마스킹 테스트</t>
         </is>
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>PRD 8-1/8-2/8-3 사용자 플로우 기준 시나리오 작성</t>
+          <t>상대 닉네임 마스킹 누락 케이스 점검</t>
         </is>
       </c>
       <c r="G91" s="5" t="inlineStr">
@@ -5683,17 +5683,17 @@
       </c>
       <c r="H91" s="3" t="inlineStr">
         <is>
-          <t>FE-03,FE-04,FE-05,FE-06,FE-07,FE-08,FE-09</t>
+          <t>PGA-09</t>
         </is>
       </c>
       <c r="I91" s="3" t="inlineStr">
         <is>
-          <t>PRD8장</t>
+          <t>PRD7-3·12장</t>
         </is>
       </c>
       <c r="J91" s="3" t="inlineStr">
         <is>
-          <t>전체 시나리오 통과</t>
+          <t>마스킹 누락 0건</t>
         </is>
       </c>
       <c r="K91" s="3" t="inlineStr">
@@ -5705,7 +5705,7 @@
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
         <is>
-          <t>TEST-09</t>
+          <t>TEST-08</t>
         </is>
       </c>
       <c r="B92" s="5" t="inlineStr">
@@ -5725,12 +5725,12 @@
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>반응형 크로스브라우저 테스트</t>
+          <t>프론트엔드 E2E 테스트(Playwright)</t>
         </is>
       </c>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>iOS Safari/Android Chrome/Desktop Chrome 3개 브레이크포인트 검증</t>
+          <t>PRD 8-1/8-2/8-3 사용자 플로우 기준 시나리오 작성</t>
         </is>
       </c>
       <c r="G92" s="5" t="inlineStr">
@@ -5745,12 +5745,12 @@
       </c>
       <c r="I92" s="3" t="inlineStr">
         <is>
-          <t>PRD12장(QA리소스제약)</t>
+          <t>PRD8장</t>
         </is>
       </c>
       <c r="J92" s="3" t="inlineStr">
         <is>
-          <t>주요 화면 시각 회귀 없음 확인</t>
+          <t>전체 시나리오 통과</t>
         </is>
       </c>
       <c r="K92" s="3" t="inlineStr">
@@ -5762,121 +5762,121 @@
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
+          <t>TEST-09</t>
+        </is>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>테스트</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>전체 7화면</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="inlineStr">
+        <is>
+          <t>반응형 크로스브라우저 테스트</t>
+        </is>
+      </c>
+      <c r="F93" s="3" t="inlineStr">
+        <is>
+          <t>iOS Safari/Android Chrome/Desktop Chrome 3개 브레이크포인트 검증</t>
+        </is>
+      </c>
+      <c r="G93" s="5" t="inlineStr">
+        <is>
+          <t>필수</t>
+        </is>
+      </c>
+      <c r="H93" s="3" t="inlineStr">
+        <is>
+          <t>FE-03,FE-04,FE-05,FE-06,FE-07,FE-08,FE-09</t>
+        </is>
+      </c>
+      <c r="I93" s="3" t="inlineStr">
+        <is>
+          <t>PRD12장(QA리소스제약)</t>
+        </is>
+      </c>
+      <c r="J93" s="3" t="inlineStr">
+        <is>
+          <t>주요 화면 시각 회귀 없음 확인</t>
+        </is>
+      </c>
+      <c r="K93" s="3" t="inlineStr">
+        <is>
+          <t>해당 TASK 자체가 테스트 작성/실행 TASK의 산출물</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="5" t="inlineStr">
+        <is>
           <t>TEST-10</t>
         </is>
       </c>
-      <c r="B93" s="5" t="inlineStr">
+      <c r="B94" s="5" t="inlineStr">
         <is>
           <t>테스트</t>
         </is>
       </c>
-      <c r="C93" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D93" s="3" t="inlineStr">
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
         <is>
           <t>공통</t>
         </is>
       </c>
-      <c r="E93" s="3" t="inlineStr">
+      <c r="E94" s="3" t="inlineStr">
         <is>
           <t>Rate Limiting/보안 테스트</t>
         </is>
       </c>
-      <c r="F93" s="3" t="inlineStr">
+      <c r="F94" s="3" t="inlineStr">
         <is>
           <t>요청 한도 초과·비정상 입력 처리 검증</t>
         </is>
       </c>
-      <c r="G93" s="5" t="inlineStr">
+      <c r="G94" s="5" t="inlineStr">
         <is>
           <t>권장</t>
         </is>
       </c>
-      <c r="H93" s="3" t="inlineStr">
+      <c r="H94" s="3" t="inlineStr">
         <is>
           <t>API-07</t>
         </is>
       </c>
-      <c r="I93" s="3" t="inlineStr">
+      <c r="I94" s="3" t="inlineStr">
         <is>
           <t>설계서4.2·6장</t>
         </is>
       </c>
-      <c r="J93" s="3" t="inlineStr">
+      <c r="J94" s="3" t="inlineStr">
         <is>
           <t>429 응답 및 로그 확인</t>
         </is>
       </c>
-      <c r="K93" s="3" t="inlineStr">
+      <c r="K94" s="3" t="inlineStr">
         <is>
           <t>해당 TASK 자체가 테스트 작성/실행 TASK의 산출물</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="6" t="inlineStr">
-        <is>
-          <t>REL-01</t>
-        </is>
-      </c>
-      <c r="B94" s="6" t="inlineStr">
-        <is>
-          <t>배포릴리즈</t>
-        </is>
-      </c>
-      <c r="C94" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D94" s="3" t="inlineStr">
-        <is>
-          <t>전체</t>
-        </is>
-      </c>
-      <c r="E94" s="3" t="inlineStr">
-        <is>
-          <t>스테이징 통합 배포 및 QA</t>
-        </is>
-      </c>
-      <c r="F94" s="3" t="inlineStr">
-        <is>
-          <t>전체 기능 스테이징 환경 배포 후 PM 검수</t>
-        </is>
-      </c>
-      <c r="G94" s="6" t="inlineStr">
-        <is>
-          <t>필수</t>
-        </is>
-      </c>
-      <c r="H94" s="3" t="inlineStr">
-        <is>
-          <t>TEST-01,TEST-02,TEST-03,TEST-04,TEST-05,TEST-06,TEST-07,TEST-08,TEST-09</t>
-        </is>
-      </c>
-      <c r="I94" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J94" s="3" t="inlineStr">
-        <is>
-          <t>PM 승인 획득</t>
-        </is>
-      </c>
-      <c r="K94" s="3" t="inlineStr">
-        <is>
-          <t>TEST-00~10 전체 그린 상태를 배포 전제조건으로 확인</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>REL-02</t>
+          <t>REL-01</t>
         </is>
       </c>
       <c r="B95" s="6" t="inlineStr">
@@ -5896,12 +5896,12 @@
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>프로덕션 배포</t>
+          <t>스테이징 통합 배포 및 QA</t>
         </is>
       </c>
       <c r="F95" s="3" t="inlineStr">
         <is>
-          <t>Cloudflare Pages+Render 프로덕션 반영, PM 최종 승인 후 커밋/푸시</t>
+          <t>전체 기능 스테이징 환경 배포 후 PM 검수</t>
         </is>
       </c>
       <c r="G95" s="6" t="inlineStr">
@@ -5911,7 +5911,7 @@
       </c>
       <c r="H95" s="3" t="inlineStr">
         <is>
-          <t>REL-01</t>
+          <t>TEST-01,TEST-02,TEST-03,TEST-04,TEST-05,TEST-06,TEST-07,TEST-08,TEST-09</t>
         </is>
       </c>
       <c r="I95" s="3" t="inlineStr">
@@ -5921,19 +5921,19 @@
       </c>
       <c r="J95" s="3" t="inlineStr">
         <is>
-          <t>프로덕션 URL 정상 서비스 확인</t>
+          <t>PM 승인 획득</t>
         </is>
       </c>
       <c r="K95" s="3" t="inlineStr">
         <is>
-          <t>프로덕션 스모크 테스트: 핵심 URL 200 확인, 챗봇 질의 1회 왕복 확인</t>
+          <t>TEST-00~10 전체 그린 상태를 배포 전제조건으로 확인</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="6" t="inlineStr">
         <is>
-          <t>REL-03</t>
+          <t>REL-02</t>
         </is>
       </c>
       <c r="B96" s="6" t="inlineStr">
@@ -5948,17 +5948,17 @@
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>전체</t>
         </is>
       </c>
       <c r="E96" s="3" t="inlineStr">
         <is>
-          <t>배포 후 모니터링 점검</t>
+          <t>프로덕션 배포</t>
         </is>
       </c>
       <c r="F96" s="3" t="inlineStr">
         <is>
-          <t>콜드스타트 비중·응답지연 p50/p95 확인</t>
+          <t>Cloudflare Pages+Render 프로덕션 반영, PM 최종 승인 후 커밋/푸시</t>
         </is>
       </c>
       <c r="G96" s="6" t="inlineStr">
@@ -5968,29 +5968,29 @@
       </c>
       <c r="H96" s="3" t="inlineStr">
         <is>
-          <t>REL-02,KPI-01</t>
+          <t>REL-01</t>
         </is>
       </c>
       <c r="I96" s="3" t="inlineStr">
         <is>
-          <t>PRD3-3</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J96" s="3" t="inlineStr">
         <is>
-          <t>초기 1주 지표 리뷰 완료</t>
+          <t>프로덕션 URL 정상 서비스 확인</t>
         </is>
       </c>
       <c r="K96" s="3" t="inlineStr">
         <is>
-          <t>해당 없음 — 모니터링 지표 수동 리뷰</t>
+          <t>프로덕션 스모크 테스트: 핵심 URL 200 확인, 챗봇 질의 1회 왕복 확인</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="6" t="inlineStr">
         <is>
-          <t>REL-04</t>
+          <t>REL-03</t>
         </is>
       </c>
       <c r="B97" s="6" t="inlineStr">
@@ -6010,92 +6010,149 @@
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>1.0 출시 회고 및 KPI 재보정 계획 수립</t>
+          <t>배포 후 모니터링 점검</t>
         </is>
       </c>
       <c r="F97" s="3" t="inlineStr">
         <is>
-          <t>2~4주 실측 데이터 수집 계획 및 재보정 일정 수립</t>
+          <t>콜드스타트 비중·응답지연 p50/p95 확인</t>
         </is>
       </c>
       <c r="G97" s="6" t="inlineStr">
         <is>
-          <t>권장</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="H97" s="3" t="inlineStr">
         <is>
-          <t>REL-03</t>
+          <t>REL-02,KPI-01</t>
         </is>
       </c>
       <c r="I97" s="3" t="inlineStr">
         <is>
-          <t>PRD3-2·3-3</t>
+          <t>PRD3-3</t>
         </is>
       </c>
       <c r="J97" s="3" t="inlineStr">
         <is>
-          <t>재보정 일정 문서화</t>
+          <t>초기 1주 지표 리뷰 완료</t>
         </is>
       </c>
       <c r="K97" s="3" t="inlineStr">
         <is>
-          <t>해당 없음 — 문서화 작업</t>
+          <t>해당 없음 — 모니터링 지표 수동 리뷰</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="6" t="inlineStr">
         <is>
+          <t>REL-04</t>
+        </is>
+      </c>
+      <c r="B98" s="6" t="inlineStr">
+        <is>
+          <t>배포릴리즈</t>
+        </is>
+      </c>
+      <c r="C98" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>공통</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr">
+        <is>
+          <t>1.0 출시 회고 및 KPI 재보정 계획 수립</t>
+        </is>
+      </c>
+      <c r="F98" s="3" t="inlineStr">
+        <is>
+          <t>2~4주 실측 데이터 수집 계획 및 재보정 일정 수립</t>
+        </is>
+      </c>
+      <c r="G98" s="6" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H98" s="3" t="inlineStr">
+        <is>
+          <t>REL-03</t>
+        </is>
+      </c>
+      <c r="I98" s="3" t="inlineStr">
+        <is>
+          <t>PRD3-2·3-3</t>
+        </is>
+      </c>
+      <c r="J98" s="3" t="inlineStr">
+        <is>
+          <t>재보정 일정 문서화</t>
+        </is>
+      </c>
+      <c r="K98" s="3" t="inlineStr">
+        <is>
+          <t>해당 없음 — 문서화 작업</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="6" t="inlineStr">
+        <is>
           <t>REL-05</t>
         </is>
       </c>
-      <c r="B98" s="6" t="inlineStr">
+      <c r="B99" s="6" t="inlineStr">
         <is>
           <t>배포릴리즈</t>
         </is>
       </c>
-      <c r="C98" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D98" s="3" t="inlineStr">
+      <c r="C99" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr">
         <is>
           <t>전체</t>
         </is>
       </c>
-      <c r="E98" s="3" t="inlineStr">
+      <c r="E99" s="3" t="inlineStr">
         <is>
           <t>포트폴리오 공개 전환 준비 체크리스트</t>
         </is>
       </c>
-      <c r="F98" s="3" t="inlineStr">
+      <c r="F99" s="3" t="inlineStr">
         <is>
           <t>저장소를 private에서 public으로 전환하기 전 확인·조치한다: (1) gitleaks 등으로 커밋 히스토리 전체에서 시크릿·API 키 잔존 여부 스캔 (2) 테스트 fixture 전수 조사 — 실제 Riot ID/PUUID/닉네임/매치 데이터가 아닌 합성 데이터로만 구성됐는지 확인, 실데이터가 섞여 있으면 fixture 재작성 후 필요시 git 히스토리 정리 (3) README에 'Riot Games와 무관한 비공식 팬 프로젝트' 디스클레이머 추가 (4) 라이브 배포 URL을 README/공개 자료에 노출할지 결정 (5) 노출하기로 하면 챗봇/전적조회 진입점에 Cloudflare Turnstile 등 경량 봇 방지 적용 검토. 무료 호스팅 비용에는 영향 없음(저장소 공개 여부와 인프라 비용은 무관)</t>
         </is>
       </c>
-      <c r="G98" s="6" t="inlineStr">
+      <c r="G99" s="6" t="inlineStr">
         <is>
           <t>권장</t>
         </is>
       </c>
-      <c r="H98" s="3" t="inlineStr">
+      <c r="H99" s="3" t="inlineStr">
         <is>
           <t>REL-04</t>
         </is>
       </c>
-      <c r="I98" s="3" t="inlineStr">
+      <c r="I99" s="3" t="inlineStr">
         <is>
           <t>PM 결정사항(2026-07-30 대화), policies.md 11번</t>
         </is>
       </c>
-      <c r="J98" s="3" t="inlineStr">
+      <c r="J99" s="3" t="inlineStr">
         <is>
           <t>체크리스트 5개 항목 모두 확인·조치 완료 및 PM 승인 후 저장소 visibility를 public으로 변경</t>
         </is>
       </c>
-      <c r="K98" s="3" t="inlineStr">
+      <c r="K99" s="3" t="inlineStr">
         <is>
           <t>정량 검증: gitleaks(또는 동급 도구) 스캔 결과 시크릿 탐지 0건, 전체 fixture 파일에서 실제 Riot ID 패턴(게임명#태그)·PUUID 패턴 검색 결과 0건</t>
         </is>

</xml_diff>

<commit_message>
docs(FE-09): FE-09 완료 처리(PM 승인) 및 CHAT-11 신규 등록 반영
FE-09(챗봇 위젯 전역 컴포넌트) PM 승인에 따라 진행현황.md 상태를
완료로 갱신하고 작업결과 문서를 확정.

PM 확인 과정에서 후속질문칩의 맥락 기반 동적 생성 여부를 논의,
LLM 기반으로 채택하기로 결정해 CHAT-11(권장, 선행TASK CHAT-05·FE-09)을
WBS.xlsx·진행현황.md에 신규 등록(프롬프트 설계·SSE 신규 이벤트·
무료 티어 레이트리밋 검토를 DoD에 포함).

진행현황.md 대그룹별 TASK 수 표의 기존 오기(프론트엔드 13→14)도
함께 정정.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TFT_Hideout_WBS.xlsx
+++ b/TFT_Hideout_WBS.xlsx
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K100"/>
+  <dimension ref="A1:K101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3767,7 +3767,7 @@
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>PGA-01</t>
+          <t>CHAT-11</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
@@ -3777,54 +3777,54 @@
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>사후패인분석</t>
+          <t>챗봇RAG</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석</t>
+          <t>챗봇위젯</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>Riot ID 계정 연동 로직 구현</t>
+          <t>후속질문 동적 생성(LLM 기반) 구현</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>게임명#태그+지역 입력→PUUID 변환, 임의계정 조회 허용</t>
+          <t>CHAT-05 답변 생성 이후 Groq에 맥락 기반 후속 질문 2~3개 생성을 추가 요청(프롬프트 설계), SSE에 신규 이벤트(event: followups) 추가해 FE-09가 만든 고정 4개 칩을 동적 목록으로 교체. 무료 티어 레이트리밋/응답 지연 영향 검토 포함(PM 결정 2026-08-06, LLM 기반 채택).</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
-          <t>필수</t>
+          <t>권장</t>
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>API-11</t>
+          <t>CHAT-05,FE-09</t>
         </is>
       </c>
       <c r="I58" s="3" t="inlineStr">
         <is>
-          <t>PRD 7-3·8-3·9-1</t>
+          <t>PRD7-4·화면설계서2.7(SuggestedFollowupChips)·개발설계서4.4(프롬프트 조립)</t>
         </is>
       </c>
       <c r="J58" s="3" t="inlineStr">
         <is>
-          <t>정상/비정상 계정 케이스 테스트</t>
+          <t>Groq 추가 호출로 후속 질문 2~3개 생성, SSE event: followups로 프론트에 전달, FE-09 정적 칩이 동적 목록으로 교체됨, 무료 티어 레이트리밋 영향(호출 증가율·콜드스타트 비중 변화) 검토 결과 기록</t>
         </is>
       </c>
       <c r="K58" s="3" t="inlineStr">
         <is>
-          <t>pytest: 정상 Riot ID/형식 오류/미존재 계정 3케이스</t>
+          <t>pytest: 후속질문 생성 함수 고정 fixture 입력 → 질문 형식/개수 검증, Groq 실패 시 후속질문 없이도 기존 답변 스트리밍은 정상 동작하는지(폴백) 확인 | Vitest+RTL: followups 이벤트 포함 mock SSE로 동적 칩 렌더링, 칩 클릭 시 해당 질문이 전송되는지 테스트</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>PGA-02</t>
+          <t>PGA-01</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
@@ -3844,12 +3844,12 @@
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>최신 매치 조회 로직 구현</t>
+          <t>Riot ID 계정 연동 로직 구현</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>Match-V1으로 매치ID/매치상세 조회</t>
+          <t>게임명#태그+지역 입력→PUUID 변환, 임의계정 조회 허용</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">
@@ -3859,29 +3859,29 @@
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>PGA-01</t>
+          <t>API-11</t>
         </is>
       </c>
       <c r="I59" s="3" t="inlineStr">
         <is>
-          <t>PRD 7-3·설계서4.5</t>
+          <t>PRD 7-3·8-3·9-1</t>
         </is>
       </c>
       <c r="J59" s="3" t="inlineStr">
         <is>
-          <t>매치 상세 파싱 검증</t>
+          <t>정상/비정상 계정 케이스 테스트</t>
         </is>
       </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t>pytest: mock Match-V1 응답 기준 매치ID·매치상세 파싱 필드 전체 검증</t>
+          <t>pytest: 정상 Riot ID/형식 오류/미존재 계정 3케이스</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>PGA-03</t>
+          <t>PGA-02</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
@@ -3896,17 +3896,17 @@
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석·분석리포트</t>
+          <t>사후패인분석</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>분석 결과 캐시 재사용 로직 구현</t>
+          <t>최신 매치 조회 로직 구현</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>match_analyses 조회 우선, 없으면 신규계산</t>
+          <t>Match-V1으로 매치ID/매치상세 조회</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
@@ -3916,29 +3916,29 @@
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>DATA-03,PGA-02</t>
+          <t>PGA-01</t>
         </is>
       </c>
       <c r="I60" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.5·4.6·5.1</t>
+          <t>PRD 7-3·설계서4.5</t>
         </is>
       </c>
       <c r="J60" s="3" t="inlineStr">
         <is>
-          <t>재요청 시 캐시 히트 확인</t>
+          <t>매치 상세 파싱 검증</t>
         </is>
       </c>
       <c r="K60" s="3" t="inlineStr">
         <is>
-          <t>pytest: 동일 match_id+puuid 재요청 시 Riot API/Groq mock 호출 0회(캐시 hit), 신규 조합은 계산 경로 진입 확인</t>
+          <t>pytest: mock Match-V1 응답 기준 매치ID·매치상세 파싱 필드 전체 검증</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>PGA-04</t>
+          <t>PGA-03</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
@@ -3953,17 +3953,17 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>분석리포트</t>
+          <t>사후패인분석·분석리포트</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>조합 이탈도 계산 로직 구현</t>
+          <t>분석 결과 캐시 재사용 로직 구현</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>가중 자카드 유사도(캐리 가중치2), 구간분류</t>
+          <t>match_analyses 조회 우선, 없으면 신규계산</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
@@ -3973,29 +3973,29 @@
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>PGA-02,DATA-02</t>
+          <t>DATA-03,PGA-02</t>
         </is>
       </c>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.5.1</t>
+          <t>설계서 4.5·4.6·5.1</t>
         </is>
       </c>
       <c r="J61" s="3" t="inlineStr">
         <is>
-          <t>샘플 매치 계산값 수기검증 일치</t>
+          <t>재요청 시 캐시 히트 확인</t>
         </is>
       </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>pytest(필수·크리티컬, TEST-00 시나리오 선적용): 수기 계산한 샘플 보드 3~5개에 대해 이탈도 값이 소수점 둘째자리까지 일치, 구간분류 경계값(0.3/0.6) 케이스 포함</t>
+          <t>pytest: 동일 match_id+puuid 재요청 시 Riot API/Groq mock 호출 0회(캐시 hit), 신규 조합은 계산 경로 진입 확인</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>PGA-05</t>
+          <t>PGA-04</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
@@ -4015,12 +4015,12 @@
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>아이템 집중도 계산 로직 구현</t>
+          <t>조합 이탈도 계산 로직 구현</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>캐리 완성아이템 비율, 추천빌드 멀티셋 교집합</t>
+          <t>가중 자카드 유사도(캐리 가중치2), 구간분류</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
@@ -4030,7 +4030,7 @@
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>PGA-04</t>
+          <t>PGA-02,DATA-02</t>
         </is>
       </c>
       <c r="I62" s="3" t="inlineStr">
@@ -4040,19 +4040,19 @@
       </c>
       <c r="J62" s="3" t="inlineStr">
         <is>
-          <t>샘플 계산값 검증</t>
+          <t>샘플 매치 계산값 수기검증 일치</t>
         </is>
       </c>
       <c r="K62" s="3" t="inlineStr">
         <is>
-          <t>pytest: 샘플 보드 기준 집중도 값 수기 계산과 일치, 중복 아이템 멀티셋 케이스 포함</t>
+          <t>pytest(필수·크리티컬, TEST-00 시나리오 선적용): 수기 계산한 샘플 보드 3~5개에 대해 이탈도 값이 소수점 둘째자리까지 일치, 구간분류 경계값(0.3/0.6) 케이스 포함</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>PGA-06</t>
+          <t>PGA-05</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
@@ -4072,12 +4072,12 @@
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>증강체 시너지 계산 로직 구현</t>
+          <t>아이템 집중도 계산 로직 구현</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>선택증강체 vs comp_augments 매칭 비율</t>
+          <t>캐리 완성아이템 비율, 추천빌드 멀티셋 교집합</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr">
@@ -4102,14 +4102,14 @@
       </c>
       <c r="K63" s="3" t="inlineStr">
         <is>
-          <t>pytest: 선택 증강체 0개/일부일치/전체일치 3케이스 시너지 점수 검증</t>
+          <t>pytest: 샘플 보드 기준 집중도 값 수기 계산과 일치, 중복 아이템 멀티셋 케이스 포함</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>PGA-07</t>
+          <t>PGA-06</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
@@ -4129,12 +4129,12 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>코칭 문장 생성 로직 구현</t>
+          <t>증강체 시너지 계산 로직 구현</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>3개 지표+등수 근거로 잘한점/아쉬운점/제안 고정구조 생성, 수치 비노출. op.gg tft_get_play_style(PUUID 필요, DATA-08에서 이동)을 호출해 코칭 근거로 활용</t>
+          <t>선택증강체 vs comp_augments 매칭 비율</t>
         </is>
       </c>
       <c r="G64" s="4" t="inlineStr">
@@ -4144,29 +4144,29 @@
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>PGA-04,PGA-05,PGA-06,SET-10</t>
+          <t>PGA-04</t>
         </is>
       </c>
       <c r="I64" s="3" t="inlineStr">
         <is>
-          <t>PRD 7-3·설계서4.5.2</t>
+          <t>설계서 4.5.1</t>
         </is>
       </c>
       <c r="J64" s="3" t="inlineStr">
         <is>
-          <t>출력 포맷 규칙 준수 확인</t>
+          <t>샘플 계산값 검증</t>
         </is>
       </c>
       <c r="K64" s="3" t="inlineStr">
         <is>
-          <t>pytest(필수·정책, TEST-00 시나리오 선적용): mock LLM 출력에 원 수치(예: '이탈도 0.42')가 노출되면 실패 처리되는 검증 로직 자체 테스트, 고정 3단 구조 파싱 확인</t>
+          <t>pytest: 선택 증강체 0개/일부일치/전체일치 3케이스 시너지 점수 검증</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>PGA-08</t>
+          <t>PGA-07</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
@@ -4186,12 +4186,12 @@
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>다음 게임 제안 근거 조회 로직 구현</t>
+          <t>코칭 문장 생성 로직 구현</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>matched_comp_id 기준 추천아이템·증강체 조회</t>
+          <t>3개 지표+등수 근거로 잘한점/아쉬운점/제안 고정구조 생성, 수치 비노출. op.gg tft_get_play_style(PUUID 필요, DATA-08에서 이동)을 호출해 코칭 근거로 활용</t>
         </is>
       </c>
       <c r="G65" s="4" t="inlineStr">
@@ -4201,29 +4201,29 @@
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
-          <t>PGA-04,DATA-02</t>
+          <t>PGA-04,PGA-05,PGA-06,SET-10</t>
         </is>
       </c>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.5.3</t>
+          <t>PRD 7-3·설계서4.5.2</t>
         </is>
       </c>
       <c r="J65" s="3" t="inlineStr">
         <is>
-          <t>추천 근거 정확성 검증</t>
+          <t>출력 포맷 규칙 준수 확인</t>
         </is>
       </c>
       <c r="K65" s="3" t="inlineStr">
         <is>
-          <t>pytest: matched_comp_id 기준 추천아이템/증강체 조회 결과가 champion_item_builds/comp_augments와 일치하는지 확인</t>
+          <t>pytest(필수·정책, TEST-00 시나리오 선적용): mock LLM 출력에 원 수치(예: '이탈도 0.42')가 노출되면 실패 처리되는 검증 로직 자체 테스트, 고정 3단 구조 파싱 확인</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>PGA-09</t>
+          <t>PGA-08</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
@@ -4243,12 +4243,12 @@
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>프라이버시 마스킹 로직 구현</t>
+          <t>다음 게임 제안 근거 조회 로직 구현</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>상대 닉네임 마스킹 전처리+정규식 재마스킹 이중방어</t>
+          <t>matched_comp_id 기준 추천아이템·증강체 조회</t>
         </is>
       </c>
       <c r="G66" s="4" t="inlineStr">
@@ -4258,29 +4258,29 @@
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>PGA-07</t>
+          <t>PGA-04,DATA-02</t>
         </is>
       </c>
       <c r="I66" s="3" t="inlineStr">
         <is>
-          <t>PRD 7-3·설계서4.4.3·4.5.3</t>
+          <t>설계서 4.5.3</t>
         </is>
       </c>
       <c r="J66" s="3" t="inlineStr">
         <is>
-          <t>마스킹 누락 케이스 없음 확인</t>
+          <t>추천 근거 정확성 검증</t>
         </is>
       </c>
       <c r="K66" s="3" t="inlineStr">
         <is>
-          <t>pytest(필수·보안, TEST-00 시나리오 선적용): 상대 Riot ID 포함 mock LLM 출력에서 정규식 마스킹 후 원본 문자열이 전혀 남지 않는지(부분 마스킹 실패 케이스 포함) 확인</t>
+          <t>pytest: matched_comp_id 기준 추천아이템/증강체 조회 결과가 champion_item_builds/comp_augments와 일치하는지 확인</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>PGA-10</t>
+          <t>PGA-09</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
@@ -4295,17 +4295,17 @@
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석·분석리포트</t>
+          <t>분석리포트</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>상세 리포트 데이터 조립 로직 구현</t>
+          <t>프라이버시 마스킹 로직 구현</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>코칭요약·매칭조합·등수변화·아이템타임라인 응답 조립</t>
+          <t>상대 닉네임 마스킹 전처리+정규식 재마스킹 이중방어</t>
         </is>
       </c>
       <c r="G67" s="4" t="inlineStr">
@@ -4315,29 +4315,29 @@
       </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
-          <t>PGA-07,PGA-08,PGA-09,API-13</t>
+          <t>PGA-07</t>
         </is>
       </c>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>PRD 8-3·IA4.6</t>
+          <t>PRD 7-3·설계서4.4.3·4.5.3</t>
         </is>
       </c>
       <c r="J67" s="3" t="inlineStr">
         <is>
-          <t>API-13 응답 필드 전체 채움 확인</t>
+          <t>마스킹 누락 케이스 없음 확인</t>
         </is>
       </c>
       <c r="K67" s="3" t="inlineStr">
         <is>
-          <t>pytest: API-13 응답 스키마 전체 필드가 null 없이 채워지는지 통합 테스트</t>
+          <t>pytest(필수·보안, TEST-00 시나리오 선적용): 상대 Riot ID 포함 mock LLM 출력에서 정규식 마스킹 후 원본 문자열이 전혀 남지 않는지(부분 마스킹 실패 케이스 포함) 확인</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>FE-01</t>
+          <t>PGA-10</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
@@ -4347,22 +4347,22 @@
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>프론트엔드</t>
+          <t>사후패인분석</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>사후패인분석·분석리포트</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>Next.js 프로젝트 스캐폴딩 및 Tailwind 설정</t>
+          <t>상세 리포트 데이터 조립 로직 구현</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>App Router, Tailwind 브레이크포인트(md768/lg1024) 매핑, 디자인가이드 토큰(컬러/타이포/spacing) 반영</t>
+          <t>코칭요약·매칭조합·등수변화·아이템타임라인 응답 조립</t>
         </is>
       </c>
       <c r="G68" s="4" t="inlineStr">
@@ -4372,29 +4372,29 @@
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>SET-07</t>
+          <t>PGA-07,PGA-08,PGA-09,API-13</t>
         </is>
       </c>
       <c r="I68" s="3" t="inlineStr">
         <is>
-          <t>설계서4.1.1·디자인가이드</t>
+          <t>PRD 8-3·IA4.6</t>
         </is>
       </c>
       <c r="J68" s="3" t="inlineStr">
         <is>
-          <t>기본 레이아웃 렌더링 확인</t>
+          <t>API-13 응답 필드 전체 채움 확인</t>
         </is>
       </c>
       <c r="K68" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: Tailwind 브레이크포인트 클래스 적용 여부, 디자인 토큰 색상값 매칭 확인</t>
+          <t>pytest: API-13 응답 스키마 전체 필드가 null 없이 채워지는지 통합 테스트</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>FE-02</t>
+          <t>FE-01</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
@@ -4409,17 +4409,17 @@
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>공통(GNB)</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>GNB 컴포넌트 구현</t>
+          <t>Next.js 프로젝트 스캐폴딩 및 Tailwind 설정</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>데스크톱/태블릿 가로바, 모바일 햄버거+드로어, 4개 진입점</t>
+          <t>App Router, Tailwind 브레이크포인트(md768/lg1024) 매핑, 디자인가이드 토큰(컬러/타이포/spacing) 반영</t>
         </is>
       </c>
       <c r="G69" s="4" t="inlineStr">
@@ -4429,29 +4429,29 @@
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>FE-01</t>
+          <t>SET-07</t>
         </is>
       </c>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>PRD7-4·IA6.1·디자인가이드6.1</t>
+          <t>설계서4.1.1·디자인가이드</t>
         </is>
       </c>
       <c r="J69" s="3" t="inlineStr">
         <is>
-          <t>3개 브레이크포인트 시각 확인</t>
+          <t>기본 레이아웃 렌더링 확인</t>
         </is>
       </c>
       <c r="K69" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: 3개 브레이크포인트에서 GNB 렌더링 분기(가로바/드로어) 테스트 + Playwright 스모크(클릭 시 드로어 오픈)</t>
+          <t>Vitest+RTL: Tailwind 브레이크포인트 클래스 적용 여부, 디자인 토큰 색상값 매칭 확인</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>FE-03</t>
+          <t>FE-02</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
@@ -4466,17 +4466,17 @@
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>티어리스트</t>
+          <t>공통(GNB)</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>티어리스트(홈) 페이지 구현</t>
+          <t>GNB 컴포넌트 구현</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>필터바/카드그리드/챗봇슬롯, 정적 export(FE-01 결정) + 클라이언트 사이드 fetch(CSR), 반응형(3~4열→2열→1열)</t>
+          <t>데스크톱/태블릿 가로바, 모바일 햄버거+드로어, 4개 진입점</t>
         </is>
       </c>
       <c r="G70" s="4" t="inlineStr">
@@ -4486,29 +4486,29 @@
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>FE-02,API-02,API-06</t>
+          <t>FE-01</t>
         </is>
       </c>
       <c r="I70" s="3" t="inlineStr">
         <is>
-          <t>PRD7-1·7-4·화면설계서2.1</t>
+          <t>PRD7-4·IA6.1·디자인가이드6.1</t>
         </is>
       </c>
       <c r="J70" s="3" t="inlineStr">
         <is>
-          <t>데스크톱/태블릿/모바일 와이어프레임 대비 시각 검증</t>
+          <t>3개 브레이크포인트 시각 확인</t>
         </is>
       </c>
       <c r="K70" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: 카드 그리드 컬럼 수 브레이크포인트별 렌더링, mock API 응답 데이터 바인딩 테스트(E2E는 TEST-08)</t>
+          <t>Vitest+RTL: 3개 브레이크포인트에서 GNB 렌더링 분기(가로바/드로어) 테스트 + Playwright 스모크(클릭 시 드로어 오픈)</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>FE-04</t>
+          <t>FE-03</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
@@ -4523,17 +4523,17 @@
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>조합상세</t>
+          <t>티어리스트</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>조합 상세 페이지 구현</t>
+          <t>티어리스트(홈) 페이지 구현</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>개요/챔피언구성(캐리강조)/증강체목록/CTA버튼, 모바일 full-width CTA</t>
+          <t>필터바/카드그리드/챗봇슬롯, 정적 export(FE-01 결정) + 클라이언트 사이드 fetch(CSR), 반응형(3~4열→2열→1열)</t>
         </is>
       </c>
       <c r="G71" s="4" t="inlineStr">
@@ -4543,29 +4543,29 @@
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
-          <t>FE-02,API-03</t>
+          <t>FE-02,API-02,API-06</t>
         </is>
       </c>
       <c r="I71" s="3" t="inlineStr">
         <is>
-          <t>화면설계서2.2</t>
+          <t>PRD7-1·7-4·화면설계서2.1</t>
         </is>
       </c>
       <c r="J71" s="3" t="inlineStr">
         <is>
-          <t>링크이동·반응형 검증</t>
+          <t>데스크톱/태블릿/모바일 와이어프레임 대비 시각 검증</t>
         </is>
       </c>
       <c r="K71" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: 캐리/서브 챔피언 보더 스타일 분기, CTA 버튼 모바일 full-width 렌더링 테스트</t>
+          <t>Vitest+RTL: 카드 그리드 컬럼 수 브레이크포인트별 렌더링, mock API 응답 데이터 바인딩 테스트(E2E는 TEST-08)</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>FE-05</t>
+          <t>FE-04</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
@@ -4580,17 +4580,17 @@
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>아이템빌드</t>
+          <t>조합상세</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>아이템 빌드 페이지 구현</t>
+          <t>조합 상세 페이지 구현</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>챔피언필터/조합리스트/상세패널(모바일 바텀시트)</t>
+          <t>개요/챔피언구성(캐리강조)/증강체목록/CTA버튼, 모바일 full-width CTA</t>
         </is>
       </c>
       <c r="G72" s="4" t="inlineStr">
@@ -4600,29 +4600,29 @@
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>FE-02,API-04</t>
+          <t>FE-02,API-03</t>
         </is>
       </c>
       <c r="I72" s="3" t="inlineStr">
         <is>
-          <t>화면설계서2.3</t>
+          <t>화면설계서2.2</t>
         </is>
       </c>
       <c r="J72" s="3" t="inlineStr">
         <is>
-          <t>필터-URL쿼리 동기화 검증</t>
+          <t>링크이동·반응형 검증</t>
         </is>
       </c>
       <c r="K72" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: 챔피언 필터 선택 시 URL 쿼리 동기화, 모바일 바텀시트 오픈/클로즈 테스트</t>
+          <t>Vitest+RTL: 캐리/서브 챔피언 보더 스타일 분기, CTA 버튼 모바일 full-width 렌더링 테스트</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>FE-06</t>
+          <t>FE-05</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
@@ -4637,17 +4637,17 @@
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>증강체정보</t>
+          <t>아이템빌드</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>증강체 정보 페이지 구현</t>
+          <t>아이템 빌드 페이지 구현</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>티어필터/카드리스트, Legend 승률 숨김 표시</t>
+          <t>챔피언필터/조합리스트/상세패널(모바일 바텀시트)</t>
         </is>
       </c>
       <c r="G73" s="4" t="inlineStr">
@@ -4657,29 +4657,29 @@
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>FE-02,API-05</t>
+          <t>FE-02,API-04</t>
         </is>
       </c>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>PRD10-1·화면설계서2.4</t>
+          <t>화면설계서2.3</t>
         </is>
       </c>
       <c r="J73" s="3" t="inlineStr">
         <is>
-          <t>Legend 항목 승률 미노출 확인</t>
+          <t>필터-URL쿼리 동기화 검증</t>
         </is>
       </c>
       <c r="K73" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL(필수·정책): is_legend_related=true 카드에 '승률 표시 안함' 텍스트만 렌더링되고 숫자가 DOM에 없는지 확인</t>
+          <t>Vitest+RTL: 챔피언 필터 선택 시 URL 쿼리 동기화, 모바일 바텀시트 오픈/클로즈 테스트</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>FE-07</t>
+          <t>FE-06</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
@@ -4694,17 +4694,17 @@
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석</t>
+          <t>증강체정보</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>사후 패인 분석 페이지 구현</t>
+          <t>증강체 정보 페이지 구현</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>Riot ID 폼/최근계정목록(localStorage)/전적불러오기 버튼/진행상태</t>
+          <t>티어필터/카드리스트, Legend 승률 숨김 표시</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr">
@@ -4714,29 +4714,29 @@
       </c>
       <c r="H74" s="3" t="inlineStr">
         <is>
-          <t>FE-02,API-11,API-12</t>
+          <t>FE-02,API-05</t>
         </is>
       </c>
       <c r="I74" s="3" t="inlineStr">
         <is>
-          <t>PRD8-3·화면설계서2.5</t>
+          <t>PRD10-1·화면설계서2.4</t>
         </is>
       </c>
       <c r="J74" s="3" t="inlineStr">
         <is>
-          <t>로컬스토리지 저장/재사용 확인</t>
+          <t>Legend 항목 승률 미노출 확인</t>
         </is>
       </c>
       <c r="K74" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: localStorage mock 기준 최근 계정 목록 추가/조회/전환 테스트, 폼 검증 에러 메시지 테스트</t>
+          <t>Vitest+RTL(필수·정책): is_legend_related=true 카드에 '승률 표시 안함' 텍스트만 렌더링되고 숫자가 DOM에 없는지 확인</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>FE-08</t>
+          <t>FE-07</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
@@ -4751,17 +4751,17 @@
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>분석리포트</t>
+          <t>사후패인분석</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>분석 리포트 상세 페이지 구현</t>
+          <t>사후 패인 분석 페이지 구현</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>코칭요약/매칭조합카드/등수변화그래프/아이템타임라인</t>
+          <t>Riot ID 폼/최근계정목록(localStorage)/전적불러오기 버튼/진행상태</t>
         </is>
       </c>
       <c r="G75" s="4" t="inlineStr">
@@ -4771,29 +4771,29 @@
       </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
-          <t>API-13,FE-02</t>
+          <t>FE-02,API-11,API-12</t>
         </is>
       </c>
       <c r="I75" s="3" t="inlineStr">
         <is>
-          <t>PRD8-3·화면설계서2.6</t>
+          <t>PRD8-3·화면설계서2.5</t>
         </is>
       </c>
       <c r="J75" s="3" t="inlineStr">
         <is>
-          <t>그래프/타임라인 렌더링 확인</t>
+          <t>로컬스토리지 저장/재사용 확인</t>
         </is>
       </c>
       <c r="K75" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: 그래프/타임라인 mock 데이터 렌더링, opponent-info 마스킹 텍스트 렌더링 확인</t>
+          <t>Vitest+RTL: localStorage mock 기준 최근 계정 목록 추가/조회/전환 테스트, 폼 검증 에러 메시지 테스트</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>FE-09</t>
+          <t>FE-08</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
@@ -4808,17 +4808,17 @@
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>챗봇위젯</t>
+          <t>분석리포트</t>
         </is>
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>챗봇 위젯 전역 컴포넌트 구현</t>
+          <t>분석 리포트 상세 페이지 구현</t>
         </is>
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>collapsed/expanded, SSE 연동, 모바일 바텀시트 전환, 후속질문칩</t>
+          <t>코칭요약/매칭조합카드/등수변화그래프/아이템타임라인</t>
         </is>
       </c>
       <c r="G76" s="4" t="inlineStr">
@@ -4828,29 +4828,29 @@
       </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
-          <t>FE-01,API-09,CHAT-05</t>
+          <t>API-13,FE-02</t>
         </is>
       </c>
       <c r="I76" s="3" t="inlineStr">
         <is>
-          <t>PRD7-4·화면설계서2.7·디자인가이드6.6</t>
+          <t>PRD8-3·화면설계서2.6</t>
         </is>
       </c>
       <c r="J76" s="3" t="inlineStr">
         <is>
-          <t>전 페이지 삽입 및 반응형 동작 확인</t>
+          <t>그래프/타임라인 렌더링 확인</t>
         </is>
       </c>
       <c r="K76" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: collapsed/expanded 상태 전환, 모바일 바텀시트 전환, mock SSE 스트림 렌더링 테스트</t>
+          <t>Vitest+RTL: 그래프/타임라인 mock 데이터 렌더링, opponent-info 마스킹 텍스트 렌더링 확인</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>FE-10</t>
+          <t>FE-09</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
@@ -4865,49 +4865,49 @@
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>챗봇위젯</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>이미지 최적화 및 반응형 sizes 적용</t>
+          <t>챗봇 위젯 전역 컴포넌트 구현</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>Next Image 컴포넌트, 브레이크포인트별 해상도 서빙</t>
+          <t>collapsed/expanded, SSE 연동, 모바일 바텀시트 전환, 후속질문칩</t>
         </is>
       </c>
       <c r="G77" s="4" t="inlineStr">
         <is>
-          <t>권장</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="H77" s="3" t="inlineStr">
         <is>
-          <t>FE-03,FE-04,FE-05,FE-06,FE-07,FE-08</t>
+          <t>FE-01,API-09,CHAT-05</t>
         </is>
       </c>
       <c r="I77" s="3" t="inlineStr">
         <is>
-          <t>PRD7-4·설계서4.1.1</t>
+          <t>PRD7-4·화면설계서2.7·디자인가이드6.6</t>
         </is>
       </c>
       <c r="J77" s="3" t="inlineStr">
         <is>
-          <t>모바일 이미지 로딩 성능 확인</t>
+          <t>전 페이지 삽입 및 반응형 동작 확인</t>
         </is>
       </c>
       <c r="K77" s="3" t="inlineStr">
         <is>
-          <t>해당 없음 — Lighthouse 모바일 성능 점수로 갈음(수동 측정)</t>
+          <t>Vitest+RTL: collapsed/expanded 상태 전환, 모바일 바텀시트 전환, mock SSE 스트림 렌더링 테스트</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>FE-11</t>
+          <t>FE-10</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
@@ -4927,44 +4927,44 @@
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>필터 UI 반응형 공용 컴포넌트 구현</t>
+          <t>이미지 최적화 및 반응형 sizes 적용</t>
         </is>
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>데스크톱/태블릿 Dropdown, 모바일 BottomSheet 공용 컴포넌트</t>
+          <t>Next Image 컴포넌트, 브레이크포인트별 해상도 서빙</t>
         </is>
       </c>
       <c r="G78" s="4" t="inlineStr">
         <is>
-          <t>필수</t>
+          <t>권장</t>
         </is>
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
-          <t>FE-01</t>
+          <t>FE-03,FE-04,FE-05,FE-06,FE-07,FE-08</t>
         </is>
       </c>
       <c r="I78" s="3" t="inlineStr">
         <is>
-          <t>디자인가이드6.2</t>
+          <t>PRD7-4·설계서4.1.1</t>
         </is>
       </c>
       <c r="J78" s="3" t="inlineStr">
         <is>
-          <t>3개 화면(티어리스트/아이템빌드/증강체)에서 재사용 확인</t>
+          <t>모바일 이미지 로딩 성능 확인</t>
         </is>
       </c>
       <c r="K78" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: 동일 필터 상태를 Dropdown/BottomSheet 두 컴포넌트가 공유하는지 상태 동기화 테스트</t>
+          <t>해당 없음 — Lighthouse 모바일 성능 점수로 갈음(수동 측정)</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>FE-12</t>
+          <t>FE-11</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
@@ -4979,17 +4979,17 @@
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>KPI 대시보드(비공개)</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>KPI 대시보드 페이지 구현(비공개)</t>
+          <t>필터 UI 반응형 공용 컴포넌트 구현</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>/kpi 페이지 — 비밀번호 입력 폼(미인증 시) + 5개 지표 카드/차트(최신성/근거율/전환율/이용률/응답지연). GNB·모바일 드로어에는 노출하지 않음(URL 직접 접근 전용)</t>
+          <t>데스크톱/태블릿 Dropdown, 모바일 BottomSheet 공용 컴포넌트</t>
         </is>
       </c>
       <c r="G79" s="4" t="inlineStr">
@@ -4999,29 +4999,29 @@
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
-          <t>KPI-01</t>
+          <t>FE-01</t>
         </is>
       </c>
       <c r="I79" s="3" t="inlineStr">
         <is>
-          <t>IA v1.2 4.7절</t>
+          <t>디자인가이드6.2</t>
         </is>
       </c>
       <c r="J79" s="3" t="inlineStr">
         <is>
-          <t>비밀번호 게이트 통과 후 5개 지표 정상 렌더링 확인, 오답 시 게이트 재노출 확인</t>
+          <t>3개 화면(티어리스트/아이템빌드/증강체)에서 재사용 확인</t>
         </is>
       </c>
       <c r="K79" s="3" t="inlineStr">
         <is>
-          <t>Vitest: 비밀번호 게이트 컴포넌트 성공/실패 케이스, 지표 카드 렌더링 테스트</t>
+          <t>Vitest+RTL: 동일 필터 상태를 Dropdown/BottomSheet 두 컴포넌트가 공유하는지 상태 동기화 테스트</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>FE-13</t>
+          <t>FE-12</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
@@ -5036,49 +5036,49 @@
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>티어리스트</t>
+          <t>KPI 대시보드(비공개)</t>
         </is>
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>티어리스트 카드 챔피언 이미지 표시</t>
+          <t>KPI 대시보드 페이지 구현(비공개)</t>
         </is>
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>CompCard의 캐리 챔피언 점(●) placeholder를 Community Dragon 실제 챔피언 아이콘 이미지로 교체. champions 테이블에 square_icon_url 컬럼 추가(배치, Community Dragon squareIcon .tex 경로를 raw.communitydragon.org PNG URL로 변환), GET /catalog/tierlist 응답(CompSummary)에 캐리 챔피언 이름·이미지 URL 포함하도록 확장(API-02), CompCard에 next/image로 렌더링(이미지 없으면 기존 placeholder 폴백).</t>
+          <t>/kpi 페이지 — 비밀번호 입력 폼(미인증 시) + 5개 지표 카드/차트(최신성/근거율/전환율/이용률/응답지연). GNB·모바일 드로어에는 노출하지 않음(URL 직접 접근 전용)</t>
         </is>
       </c>
       <c r="G80" s="4" t="inlineStr">
         <is>
-          <t>권장</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
-          <t>FE-03</t>
+          <t>KPI-01</t>
         </is>
       </c>
       <c r="I80" s="3" t="inlineStr">
         <is>
-          <t>PM 요청 2026-08-05, Community Dragon squareIcon 필드 실호출로 URL 변환 가능 확인</t>
+          <t>IA v1.2 4.7절</t>
         </is>
       </c>
       <c r="J80" s="3" t="inlineStr">
         <is>
-          <t>티어리스트 카드에 캐리 챔피언 실제 이미지가 표시됨(이미지 URL 없으면 기존 placeholder로 폴백)</t>
+          <t>비밀번호 게이트 통과 후 5개 지표 정상 렌더링 확인, 오답 시 게이트 재노출 확인</t>
         </is>
       </c>
       <c r="K80" s="3" t="inlineStr">
         <is>
-          <t>pytest(batch): squareIcon .tex 경로 -&gt; PNG URL 변환 함수 단위 테스트 / pytest(backend): GET /catalog/tierlist 응답에 캐리 챔피언 이름·이미지 URL 포함 확인 / Vitest+RTL: CompCard가 이미지 URL 있으면 이미지, 없으면 placeholder 렌더링 확인</t>
+          <t>Vitest: 비밀번호 게이트 컴포넌트 성공/실패 케이스, 지표 카드 렌더링 테스트</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>FE-14</t>
+          <t>FE-13</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
@@ -5093,17 +5093,17 @@
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>조합상세</t>
+          <t>티어리스트</t>
         </is>
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>조합 상세 헥스 배치도 실좌표 반영</t>
+          <t>티어리스트 카드 챔피언 이미지 표시</t>
         </is>
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>HexBoard의 is_carry 기반 전열/후열 휴리스틱 배치를 op.gg tft_list_meta_decks 응답의 units[].cell.{x,y}(실제 랭커 배치 좌표, 4행x7열, 2026-08-06 실호출로 확인)로 교체. comp_champions 테이블에 cell_x/cell_y 컬럼 추가(배치, comp_champion_rows()에서 unit.cell 추출), GET /comps/{comp_id} 응답(ChampionInComp)에 cell_x/cell_y 포함(API-03), HexBoard가 좌표 있으면 실제 4x7 헥스 그리드(오프셋 스태거)로 렌더링하고 좌표 없는 기존 데이터는 기존 휴리스틱 배치로 폴백.</t>
+          <t>CompCard의 캐리 챔피언 점(●) placeholder를 Community Dragon 실제 챔피언 아이콘 이미지로 교체. champions 테이블에 square_icon_url 컬럼 추가(배치, Community Dragon squareIcon .tex 경로를 raw.communitydragon.org PNG URL로 변환), GET /catalog/tierlist 응답(CompSummary)에 캐리 챔피언 이름·이미지 URL 포함하도록 확장(API-02), CompCard에 next/image로 렌더링(이미지 없으면 기존 placeholder 폴백).</t>
         </is>
       </c>
       <c r="G81" s="4" t="inlineStr">
@@ -5113,29 +5113,29 @@
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
-          <t>FE-04</t>
+          <t>FE-03</t>
         </is>
       </c>
       <c r="I81" s="3" t="inlineStr">
         <is>
-          <t>PM 요청 2026-08-06, op.gg tft_list_meta_decks 실호출로 units[].cell 필드(x:1-7, y:1-4) 확인</t>
+          <t>PM 요청 2026-08-05, Community Dragon squareIcon 필드 실호출로 URL 변환 가능 확인</t>
         </is>
       </c>
       <c r="J81" s="3" t="inlineStr">
         <is>
-          <t>조합 상세 페이지 태블릿/데스크톱에서 실제 좌표 기반 헥스 배치도가 표시됨(좌표 없는 구 데이터는 기존 휴리스틱 폴백 유지, 콘솔 에러 0건)</t>
+          <t>티어리스트 카드에 캐리 챔피언 실제 이미지가 표시됨(이미지 URL 없으면 기존 placeholder로 폴백)</t>
         </is>
       </c>
       <c r="K81" s="3" t="inlineStr">
         <is>
-          <t>pytest(batch): comp_champion_rows()가 unit.cell에서 cell_x/cell_y를 추출하는 단위 테스트 / pytest(backend): GET /comps/{comp_id} 응답에 cell_x/cell_y 포함 및 null 폴백 확인 / Vitest+RTL: HexBoard가 좌표 있으면 실좌표 그리드, 없으면(cell_x/y null) 기존 휴리스틱 렌더링 확인</t>
+          <t>pytest(batch): squareIcon .tex 경로 -&gt; PNG URL 변환 함수 단위 테스트 / pytest(backend): GET /catalog/tierlist 응답에 캐리 챔피언 이름·이미지 URL 포함 확인 / Vitest+RTL: CompCard가 이미지 URL 있으면 이미지, 없으면 placeholder 렌더링 확인</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>KPI-01</t>
+          <t>FE-14</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
@@ -5145,54 +5145,54 @@
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>KPI모니터링</t>
+          <t>프론트엔드</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>조합상세</t>
         </is>
       </c>
       <c r="E82" s="3" t="inlineStr">
         <is>
-          <t>KPI 대시보드 백엔드 API 구현(자체, Metabase 대체)</t>
+          <t>조합 상세 헥스 배치도 실좌표 반영</t>
         </is>
       </c>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>5개 지표(최신성/근거율/전환율/이용률/응답지연) 집계 GET /kpi/summary 구현 + POST /kpi/auth 비밀번호 게이트(환경변수 KPI_DASHBOARD_PASSWORD 대조, 서명 토큰 발급) 구현. Metabase 대신 자체 페이지(FE-12)로 제공 (PM 결정 2026-08-03)</t>
+          <t>HexBoard의 is_carry 기반 전열/후열 휴리스틱 배치를 op.gg tft_list_meta_decks 응답의 units[].cell.{x,y}(실제 랭커 배치 좌표, 4행x7열, 2026-08-06 실호출로 확인)로 교체. comp_champions 테이블에 cell_x/cell_y 컬럼 추가(배치, comp_champion_rows()에서 unit.cell 추출), GET /comps/{comp_id} 응답(ChampionInComp)에 cell_x/cell_y 포함(API-03), HexBoard가 좌표 있으면 실제 4x7 헥스 그리드(오프셋 스태거)로 렌더링하고 좌표 없는 기존 데이터는 기존 휴리스틱 배치로 폴백.</t>
         </is>
       </c>
       <c r="G82" s="4" t="inlineStr">
         <is>
-          <t>필수</t>
+          <t>권장</t>
         </is>
       </c>
       <c r="H82" s="3" t="inlineStr">
         <is>
-          <t>DATA-03</t>
+          <t>FE-04</t>
         </is>
       </c>
       <c r="I82" s="3" t="inlineStr">
         <is>
-          <t>PRD 3-3 / IA v1.2 4.7절 (자체구현 결정 2026-08-03)</t>
+          <t>PM 요청 2026-08-06, op.gg tft_list_meta_decks 실호출로 units[].cell 필드(x:1-7, y:1-4) 확인</t>
         </is>
       </c>
       <c r="J82" s="3" t="inlineStr">
         <is>
-          <t>5개 지표 API 정상 응답 확인, 비밀번호 게이트 통과/실패 동작 확인</t>
+          <t>조합 상세 페이지 태블릿/데스크톱에서 실제 좌표 기반 헥스 배치도가 표시됨(좌표 없는 구 데이터는 기존 휴리스틱 폴백 유지, 콘솔 에러 0건)</t>
         </is>
       </c>
       <c r="K82" s="3" t="inlineStr">
         <is>
-          <t>pytest: 비밀번호 게이트 성공/실패 케이스, mock 로그 데이터로 5개 지표 집계 쿼리 결과 검증</t>
+          <t>pytest(batch): comp_champion_rows()가 unit.cell에서 cell_x/cell_y를 추출하는 단위 테스트 / pytest(backend): GET /comps/{comp_id} 응답에 cell_x/cell_y 포함 및 null 폴백 확인 / Vitest+RTL: HexBoard가 좌표 있으면 실좌표 그리드, 없으면(cell_x/y null) 기존 휴리스틱 렌더링 확인</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>KPI-02</t>
+          <t>KPI-01</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
@@ -5212,12 +5212,12 @@
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>RAGAS 주간 배치 평가 파이프라인 구현</t>
+          <t>KPI 대시보드 백엔드 API 구현(자체, Metabase 대체)</t>
         </is>
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>GitHub Actions 주간 배치로 Faithfulness/Answer Relevancy 산출, ragas_eval_results 적재</t>
+          <t>5개 지표(최신성/근거율/전환율/이용률/응답지연) 집계 GET /kpi/summary 구현 + POST /kpi/auth 비밀번호 게이트(환경변수 KPI_DASHBOARD_PASSWORD 대조, 서명 토큰 발급) 구현. Metabase 대신 자체 페이지(FE-12)로 제공 (PM 결정 2026-08-03)</t>
         </is>
       </c>
       <c r="G83" s="4" t="inlineStr">
@@ -5227,143 +5227,143 @@
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>CHAT-09,SET-08</t>
+          <t>DATA-03</t>
         </is>
       </c>
       <c r="I83" s="3" t="inlineStr">
         <is>
-          <t>PRD3-3·설계서4.7</t>
+          <t>PRD 3-3 / IA v1.2 4.7절 (자체구현 결정 2026-08-03)</t>
         </is>
       </c>
       <c r="J83" s="3" t="inlineStr">
         <is>
-          <t>배치 실행 후 결과 적재 확인</t>
+          <t>5개 지표 API 정상 응답 확인, 비밀번호 게이트 통과/실패 동작 확인</t>
         </is>
       </c>
       <c r="K83" s="3" t="inlineStr">
         <is>
-          <t>pytest: mock 질의-답변 샘플로 RAGAS 스코어러 호출 및 ragas_eval_results 적재 필드 확인</t>
+          <t>pytest: 비밀번호 게이트 성공/실패 케이스, mock 로그 데이터로 5개 지표 집계 쿼리 결과 검증</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
+          <t>KPI-02</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>KPI모니터링</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>공통</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>RAGAS 주간 배치 평가 파이프라인 구현</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>GitHub Actions 주간 배치로 Faithfulness/Answer Relevancy 산출, ragas_eval_results 적재</t>
+        </is>
+      </c>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
+          <t>필수</t>
+        </is>
+      </c>
+      <c r="H84" s="3" t="inlineStr">
+        <is>
+          <t>CHAT-09,SET-08</t>
+        </is>
+      </c>
+      <c r="I84" s="3" t="inlineStr">
+        <is>
+          <t>PRD3-3·설계서4.7</t>
+        </is>
+      </c>
+      <c r="J84" s="3" t="inlineStr">
+        <is>
+          <t>배치 실행 후 결과 적재 확인</t>
+        </is>
+      </c>
+      <c r="K84" s="3" t="inlineStr">
+        <is>
+          <t>pytest: mock 질의-답변 샘플로 RAGAS 스코어러 호출 및 ragas_eval_results 적재 필드 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
           <t>KPI-03</t>
         </is>
       </c>
-      <c r="B84" s="4" t="inlineStr">
-        <is>
-          <t>코딩</t>
-        </is>
-      </c>
-      <c r="C84" s="4" t="inlineStr">
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
         <is>
           <t>KPI모니터링</t>
         </is>
       </c>
-      <c r="D84" s="3" t="inlineStr">
+      <c r="D85" s="3" t="inlineStr">
         <is>
           <t>공통</t>
         </is>
       </c>
-      <c r="E84" s="3" t="inlineStr">
+      <c r="E85" s="3" t="inlineStr">
         <is>
           <t>목표 미달 알림 로직 구현</t>
         </is>
       </c>
-      <c r="F84" s="3" t="inlineStr">
+      <c r="F85" s="3" t="inlineStr">
         <is>
           <t>2주 연속 목표 미달 감지 시 알림 발송</t>
         </is>
       </c>
-      <c r="G84" s="4" t="inlineStr">
+      <c r="G85" s="4" t="inlineStr">
         <is>
           <t>권장</t>
         </is>
       </c>
-      <c r="H84" s="3" t="inlineStr">
+      <c r="H85" s="3" t="inlineStr">
         <is>
           <t>KPI-01</t>
         </is>
       </c>
-      <c r="I84" s="3" t="inlineStr">
+      <c r="I85" s="3" t="inlineStr">
         <is>
           <t>PRD3-3</t>
         </is>
       </c>
-      <c r="J84" s="3" t="inlineStr">
+      <c r="J85" s="3" t="inlineStr">
         <is>
           <t>알림 트리거 테스트 통과</t>
         </is>
       </c>
-      <c r="K84" s="3" t="inlineStr">
+      <c r="K85" s="3" t="inlineStr">
         <is>
           <t>pytest: 2주 연속 미달 mock 데이터 주입 시 알림 함수 호출 확인</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="5" t="inlineStr">
-        <is>
-          <t>TEST-00</t>
-        </is>
-      </c>
-      <c r="B85" s="5" t="inlineStr">
-        <is>
-          <t>테스트</t>
-        </is>
-      </c>
-      <c r="C85" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D85" s="3" t="inlineStr">
-        <is>
-          <t>공통(정책·로직 크리티컬 TASK)</t>
-        </is>
-      </c>
-      <c r="E85" s="3" t="inlineStr">
-        <is>
-          <t>핵심 정책/로직 테스트 시나리오 사전 정의</t>
-        </is>
-      </c>
-      <c r="F85" s="3" t="inlineStr">
-        <is>
-          <t>API-05, CHAT-04, CHAT-06, PGA-04~09, DATA-13 등 정책 준수·크리티컬 계산 로직이 걸린 TASK에 한해, 코딩 착수 전 입력값·기대출력·경계값을 포함한 테스트 시나리오를 문서화하고 PM과 합의한다. 해당 TASK의 구현자는 이 문서를 기준으로 단위 테스트를 먼저 작성한 뒤 구현한다</t>
-        </is>
-      </c>
-      <c r="G85" s="5" t="inlineStr">
-        <is>
-          <t>필수</t>
-        </is>
-      </c>
-      <c r="H85" s="3" t="inlineStr">
-        <is>
-          <t>SET-01</t>
-        </is>
-      </c>
-      <c r="I85" s="3" t="inlineStr">
-        <is>
-          <t>요구사항정의서 NFR-SEC·FR-PGA, 설계서 4.4.2·4.4.3·4.5.1·4.5.2</t>
-        </is>
-      </c>
-      <c r="J85" s="3" t="inlineStr">
-        <is>
-          <t>/docs/test-scenarios.md에 대상 TASK별 시나리오 표 작성 및 PM 승인 완료</t>
-        </is>
-      </c>
-      <c r="K85" s="3" t="inlineStr">
-        <is>
-          <t>해당 TASK 자체가 산출물 — /docs/test-scenarios.md 표 작성</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>TEST-01</t>
+          <t>TEST-00</t>
         </is>
       </c>
       <c r="B86" s="5" t="inlineStr">
@@ -5378,17 +5378,17 @@
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>공통(정책·로직 크리티컬 TASK)</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>DB 스키마/마이그레이션 검증</t>
+          <t>핵심 정책/로직 테스트 시나리오 사전 정의</t>
         </is>
       </c>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>전체 테이블·인덱스·제약조건 검증</t>
+          <t>API-05, CHAT-04, CHAT-06, PGA-04~09, DATA-13 등 정책 준수·크리티컬 계산 로직이 걸린 TASK에 한해, 코딩 착수 전 입력값·기대출력·경계값을 포함한 테스트 시나리오를 문서화하고 PM과 합의한다. 해당 TASK의 구현자는 이 문서를 기준으로 단위 테스트를 먼저 작성한 뒤 구현한다</t>
         </is>
       </c>
       <c r="G86" s="5" t="inlineStr">
@@ -5398,29 +5398,29 @@
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
-          <t>DATA-01,DATA-02,DATA-03,DATA-04</t>
+          <t>SET-01</t>
         </is>
       </c>
       <c r="I86" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>요구사항정의서 NFR-SEC·FR-PGA, 설계서 4.4.2·4.4.3·4.5.1·4.5.2</t>
         </is>
       </c>
       <c r="J86" s="3" t="inlineStr">
         <is>
-          <t>마이그레이션 재실행 무결성 확인</t>
+          <t>/docs/test-scenarios.md에 대상 TASK별 시나리오 표 작성 및 PM 승인 완료</t>
         </is>
       </c>
       <c r="K86" s="3" t="inlineStr">
         <is>
-          <t>해당 TASK 자체가 테스트 작성/실행 TASK의 산출물</t>
+          <t>해당 TASK 자체가 산출물 — /docs/test-scenarios.md 표 작성</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>TEST-02</t>
+          <t>TEST-01</t>
         </is>
       </c>
       <c r="B87" s="5" t="inlineStr">
@@ -5435,17 +5435,17 @@
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>티어리스트~증강체정보</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>catalog API 단위/통합 테스트</t>
+          <t>DB 스키마/마이그레이션 검증</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>API-02~06 엔드포인트 테스트 코드 작성 및 실행</t>
+          <t>전체 테이블·인덱스·제약조건 검증</t>
         </is>
       </c>
       <c r="G87" s="5" t="inlineStr">
@@ -5455,7 +5455,7 @@
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
-          <t>API-02,API-03,API-04,API-05,API-06</t>
+          <t>DATA-01,DATA-02,DATA-03,DATA-04</t>
         </is>
       </c>
       <c r="I87" s="3" t="inlineStr">
@@ -5465,7 +5465,7 @@
       </c>
       <c r="J87" s="3" t="inlineStr">
         <is>
-          <t>전체 테스트 통과</t>
+          <t>마이그레이션 재실행 무결성 확인</t>
         </is>
       </c>
       <c r="K87" s="3" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>TEST-03</t>
+          <t>TEST-02</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
@@ -5492,17 +5492,17 @@
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>챗봇위젯</t>
+          <t>티어리스트~증강체정보</t>
         </is>
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>chat API 및 RAG 파이프라인 테스트</t>
+          <t>catalog API 단위/통합 테스트</t>
         </is>
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>의도분류/검색/생성/후처리/캐싱 테스트</t>
+          <t>API-02~06 엔드포인트 테스트 코드 작성 및 실행</t>
         </is>
       </c>
       <c r="G88" s="5" t="inlineStr">
@@ -5512,7 +5512,7 @@
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>CHAT-01,CHAT-02,CHAT-03,CHAT-04,CHAT-05,CHAT-06,CHAT-07,CHAT-08,CHAT-09</t>
+          <t>API-02,API-03,API-04,API-05,API-06</t>
         </is>
       </c>
       <c r="I88" s="3" t="inlineStr">
@@ -5522,7 +5522,7 @@
       </c>
       <c r="J88" s="3" t="inlineStr">
         <is>
-          <t>전체 통과, 근거율 샘플 검증</t>
+          <t>전체 테스트 통과</t>
         </is>
       </c>
       <c r="K88" s="3" t="inlineStr">
@@ -5534,7 +5534,7 @@
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>TEST-04</t>
+          <t>TEST-03</t>
         </is>
       </c>
       <c r="B89" s="5" t="inlineStr">
@@ -5549,17 +5549,17 @@
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석·분석리포트</t>
+          <t>챗봇위젯</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>analysis API 및 스코어링 로직 테스트</t>
+          <t>chat API 및 RAG 파이프라인 테스트</t>
         </is>
       </c>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>PUUID변환/매치조회/3개지표계산/코칭생성 테스트</t>
+          <t>의도분류/검색/생성/후처리/캐싱 테스트</t>
         </is>
       </c>
       <c r="G89" s="5" t="inlineStr">
@@ -5569,7 +5569,7 @@
       </c>
       <c r="H89" s="3" t="inlineStr">
         <is>
-          <t>PGA-01,PGA-02,PGA-03,PGA-04,PGA-05,PGA-06,PGA-07,PGA-08,PGA-09,PGA-10</t>
+          <t>CHAT-01,CHAT-02,CHAT-03,CHAT-04,CHAT-05,CHAT-06,CHAT-07,CHAT-08,CHAT-09</t>
         </is>
       </c>
       <c r="I89" s="3" t="inlineStr">
@@ -5579,7 +5579,7 @@
       </c>
       <c r="J89" s="3" t="inlineStr">
         <is>
-          <t>전체 통과</t>
+          <t>전체 통과, 근거율 샘플 검증</t>
         </is>
       </c>
       <c r="K89" s="3" t="inlineStr">
@@ -5591,7 +5591,7 @@
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>TEST-05</t>
+          <t>TEST-04</t>
         </is>
       </c>
       <c r="B90" s="5" t="inlineStr">
@@ -5606,17 +5606,17 @@
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>사후패인분석·분석리포트</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>배치 파이프라인 통합 테스트</t>
+          <t>analysis API 및 스코어링 로직 테스트</t>
         </is>
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>패치감지→수집→정규화→임베딩→원자적전환 end-to-end 테스트</t>
+          <t>PUUID변환/매치조회/3개지표계산/코칭생성 테스트</t>
         </is>
       </c>
       <c r="G90" s="5" t="inlineStr">
@@ -5626,7 +5626,7 @@
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>DATA-05,DATA-08,DATA-09,DATA-10,DATA-11,DATA-12,DATA-13,DATA-14,DATA-15</t>
+          <t>PGA-01,PGA-02,PGA-03,PGA-04,PGA-05,PGA-06,PGA-07,PGA-08,PGA-09,PGA-10</t>
         </is>
       </c>
       <c r="I90" s="3" t="inlineStr">
@@ -5636,7 +5636,7 @@
       </c>
       <c r="J90" s="3" t="inlineStr">
         <is>
-          <t>정상/중간실패 시나리오 모두 검증</t>
+          <t>전체 통과</t>
         </is>
       </c>
       <c r="K90" s="3" t="inlineStr">
@@ -5648,7 +5648,7 @@
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>TEST-06</t>
+          <t>TEST-05</t>
         </is>
       </c>
       <c r="B91" s="5" t="inlineStr">
@@ -5663,17 +5663,17 @@
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>챗봇위젯</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>챗봇 정책 준수 테스트</t>
+          <t>배치 파이프라인 통합 테스트</t>
         </is>
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>Legend 승률 비노출·프롬프트 인젝션 방어·범위밖 질문 안내 검증</t>
+          <t>패치감지→수집→정규화→임베딩→원자적전환 end-to-end 테스트</t>
         </is>
       </c>
       <c r="G91" s="5" t="inlineStr">
@@ -5683,17 +5683,17 @@
       </c>
       <c r="H91" s="3" t="inlineStr">
         <is>
-          <t>CHAT-04,CHAT-06</t>
+          <t>DATA-05,DATA-08,DATA-09,DATA-10,DATA-11,DATA-12,DATA-13,DATA-14,DATA-15</t>
         </is>
       </c>
       <c r="I91" s="3" t="inlineStr">
         <is>
-          <t>PRD10-1·12장</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J91" s="3" t="inlineStr">
         <is>
-          <t>정책 위반 케이스 0건</t>
+          <t>정상/중간실패 시나리오 모두 검증</t>
         </is>
       </c>
       <c r="K91" s="3" t="inlineStr">
@@ -5705,7 +5705,7 @@
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
         <is>
-          <t>TEST-07</t>
+          <t>TEST-06</t>
         </is>
       </c>
       <c r="B92" s="5" t="inlineStr">
@@ -5720,17 +5720,17 @@
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석·분석리포트</t>
+          <t>챗봇위젯</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>프라이버시 마스킹 테스트</t>
+          <t>챗봇 정책 준수 테스트</t>
         </is>
       </c>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>상대 닉네임 마스킹 누락 케이스 점검</t>
+          <t>Legend 승률 비노출·프롬프트 인젝션 방어·범위밖 질문 안내 검증</t>
         </is>
       </c>
       <c r="G92" s="5" t="inlineStr">
@@ -5740,17 +5740,17 @@
       </c>
       <c r="H92" s="3" t="inlineStr">
         <is>
-          <t>PGA-09</t>
+          <t>CHAT-04,CHAT-06</t>
         </is>
       </c>
       <c r="I92" s="3" t="inlineStr">
         <is>
-          <t>PRD7-3·12장</t>
+          <t>PRD10-1·12장</t>
         </is>
       </c>
       <c r="J92" s="3" t="inlineStr">
         <is>
-          <t>마스킹 누락 0건</t>
+          <t>정책 위반 케이스 0건</t>
         </is>
       </c>
       <c r="K92" s="3" t="inlineStr">
@@ -5762,7 +5762,7 @@
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>TEST-08</t>
+          <t>TEST-07</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
@@ -5777,17 +5777,17 @@
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>전체 7화면</t>
+          <t>사후패인분석·분석리포트</t>
         </is>
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>프론트엔드 E2E 테스트(Playwright)</t>
+          <t>프라이버시 마스킹 테스트</t>
         </is>
       </c>
       <c r="F93" s="3" t="inlineStr">
         <is>
-          <t>PRD 8-1/8-2/8-3 사용자 플로우 기준 시나리오 작성</t>
+          <t>상대 닉네임 마스킹 누락 케이스 점검</t>
         </is>
       </c>
       <c r="G93" s="5" t="inlineStr">
@@ -5797,17 +5797,17 @@
       </c>
       <c r="H93" s="3" t="inlineStr">
         <is>
-          <t>FE-03,FE-04,FE-05,FE-06,FE-07,FE-08,FE-09</t>
+          <t>PGA-09</t>
         </is>
       </c>
       <c r="I93" s="3" t="inlineStr">
         <is>
-          <t>PRD8장</t>
+          <t>PRD7-3·12장</t>
         </is>
       </c>
       <c r="J93" s="3" t="inlineStr">
         <is>
-          <t>전체 시나리오 통과</t>
+          <t>마스킹 누락 0건</t>
         </is>
       </c>
       <c r="K93" s="3" t="inlineStr">
@@ -5819,7 +5819,7 @@
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>TEST-09</t>
+          <t>TEST-08</t>
         </is>
       </c>
       <c r="B94" s="5" t="inlineStr">
@@ -5839,12 +5839,12 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>반응형 크로스브라우저 테스트</t>
+          <t>프론트엔드 E2E 테스트(Playwright)</t>
         </is>
       </c>
       <c r="F94" s="3" t="inlineStr">
         <is>
-          <t>iOS Safari/Android Chrome/Desktop Chrome 3개 브레이크포인트 검증</t>
+          <t>PRD 8-1/8-2/8-3 사용자 플로우 기준 시나리오 작성</t>
         </is>
       </c>
       <c r="G94" s="5" t="inlineStr">
@@ -5859,12 +5859,12 @@
       </c>
       <c r="I94" s="3" t="inlineStr">
         <is>
-          <t>PRD12장(QA리소스제약)</t>
+          <t>PRD8장</t>
         </is>
       </c>
       <c r="J94" s="3" t="inlineStr">
         <is>
-          <t>주요 화면 시각 회귀 없음 확인</t>
+          <t>전체 시나리오 통과</t>
         </is>
       </c>
       <c r="K94" s="3" t="inlineStr">
@@ -5876,121 +5876,121 @@
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
+          <t>TEST-09</t>
+        </is>
+      </c>
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>테스트</t>
+        </is>
+      </c>
+      <c r="C95" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>전체 7화면</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>반응형 크로스브라우저 테스트</t>
+        </is>
+      </c>
+      <c r="F95" s="3" t="inlineStr">
+        <is>
+          <t>iOS Safari/Android Chrome/Desktop Chrome 3개 브레이크포인트 검증</t>
+        </is>
+      </c>
+      <c r="G95" s="5" t="inlineStr">
+        <is>
+          <t>필수</t>
+        </is>
+      </c>
+      <c r="H95" s="3" t="inlineStr">
+        <is>
+          <t>FE-03,FE-04,FE-05,FE-06,FE-07,FE-08,FE-09</t>
+        </is>
+      </c>
+      <c r="I95" s="3" t="inlineStr">
+        <is>
+          <t>PRD12장(QA리소스제약)</t>
+        </is>
+      </c>
+      <c r="J95" s="3" t="inlineStr">
+        <is>
+          <t>주요 화면 시각 회귀 없음 확인</t>
+        </is>
+      </c>
+      <c r="K95" s="3" t="inlineStr">
+        <is>
+          <t>해당 TASK 자체가 테스트 작성/실행 TASK의 산출물</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="5" t="inlineStr">
+        <is>
           <t>TEST-10</t>
         </is>
       </c>
-      <c r="B95" s="5" t="inlineStr">
+      <c r="B96" s="5" t="inlineStr">
         <is>
           <t>테스트</t>
         </is>
       </c>
-      <c r="C95" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D95" s="3" t="inlineStr">
+      <c r="C96" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
         <is>
           <t>공통</t>
         </is>
       </c>
-      <c r="E95" s="3" t="inlineStr">
+      <c r="E96" s="3" t="inlineStr">
         <is>
           <t>Rate Limiting/보안 테스트</t>
         </is>
       </c>
-      <c r="F95" s="3" t="inlineStr">
+      <c r="F96" s="3" t="inlineStr">
         <is>
           <t>요청 한도 초과·비정상 입력 처리 검증</t>
         </is>
       </c>
-      <c r="G95" s="5" t="inlineStr">
+      <c r="G96" s="5" t="inlineStr">
         <is>
           <t>권장</t>
         </is>
       </c>
-      <c r="H95" s="3" t="inlineStr">
+      <c r="H96" s="3" t="inlineStr">
         <is>
           <t>API-07</t>
         </is>
       </c>
-      <c r="I95" s="3" t="inlineStr">
+      <c r="I96" s="3" t="inlineStr">
         <is>
           <t>설계서4.2·6장</t>
         </is>
       </c>
-      <c r="J95" s="3" t="inlineStr">
+      <c r="J96" s="3" t="inlineStr">
         <is>
           <t>429 응답 및 로그 확인</t>
         </is>
       </c>
-      <c r="K95" s="3" t="inlineStr">
+      <c r="K96" s="3" t="inlineStr">
         <is>
           <t>해당 TASK 자체가 테스트 작성/실행 TASK의 산출물</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="6" t="inlineStr">
-        <is>
-          <t>REL-01</t>
-        </is>
-      </c>
-      <c r="B96" s="6" t="inlineStr">
-        <is>
-          <t>배포릴리즈</t>
-        </is>
-      </c>
-      <c r="C96" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D96" s="3" t="inlineStr">
-        <is>
-          <t>전체</t>
-        </is>
-      </c>
-      <c r="E96" s="3" t="inlineStr">
-        <is>
-          <t>스테이징 통합 배포 및 QA</t>
-        </is>
-      </c>
-      <c r="F96" s="3" t="inlineStr">
-        <is>
-          <t>전체 기능 스테이징 환경 배포 후 PM 검수</t>
-        </is>
-      </c>
-      <c r="G96" s="6" t="inlineStr">
-        <is>
-          <t>필수</t>
-        </is>
-      </c>
-      <c r="H96" s="3" t="inlineStr">
-        <is>
-          <t>TEST-01,TEST-02,TEST-03,TEST-04,TEST-05,TEST-06,TEST-07,TEST-08,TEST-09</t>
-        </is>
-      </c>
-      <c r="I96" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J96" s="3" t="inlineStr">
-        <is>
-          <t>PM 승인 획득</t>
-        </is>
-      </c>
-      <c r="K96" s="3" t="inlineStr">
-        <is>
-          <t>TEST-00~10 전체 그린 상태를 배포 전제조건으로 확인</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="6" t="inlineStr">
         <is>
-          <t>REL-02</t>
+          <t>REL-01</t>
         </is>
       </c>
       <c r="B97" s="6" t="inlineStr">
@@ -6010,12 +6010,12 @@
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>프로덕션 배포</t>
+          <t>스테이징 통합 배포 및 QA</t>
         </is>
       </c>
       <c r="F97" s="3" t="inlineStr">
         <is>
-          <t>Cloudflare Pages+Render 프로덕션 반영, PM 최종 승인 후 커밋/푸시</t>
+          <t>전체 기능 스테이징 환경 배포 후 PM 검수</t>
         </is>
       </c>
       <c r="G97" s="6" t="inlineStr">
@@ -6025,7 +6025,7 @@
       </c>
       <c r="H97" s="3" t="inlineStr">
         <is>
-          <t>REL-01</t>
+          <t>TEST-01,TEST-02,TEST-03,TEST-04,TEST-05,TEST-06,TEST-07,TEST-08,TEST-09</t>
         </is>
       </c>
       <c r="I97" s="3" t="inlineStr">
@@ -6035,19 +6035,19 @@
       </c>
       <c r="J97" s="3" t="inlineStr">
         <is>
-          <t>프로덕션 URL 정상 서비스 확인</t>
+          <t>PM 승인 획득</t>
         </is>
       </c>
       <c r="K97" s="3" t="inlineStr">
         <is>
-          <t>프로덕션 스모크 테스트: 핵심 URL 200 확인, 챗봇 질의 1회 왕복 확인</t>
+          <t>TEST-00~10 전체 그린 상태를 배포 전제조건으로 확인</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>REL-03</t>
+          <t>REL-02</t>
         </is>
       </c>
       <c r="B98" s="6" t="inlineStr">
@@ -6062,17 +6062,17 @@
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>전체</t>
         </is>
       </c>
       <c r="E98" s="3" t="inlineStr">
         <is>
-          <t>배포 후 모니터링 점검</t>
+          <t>프로덕션 배포</t>
         </is>
       </c>
       <c r="F98" s="3" t="inlineStr">
         <is>
-          <t>콜드스타트 비중·응답지연 p50/p95 확인</t>
+          <t>Cloudflare Pages+Render 프로덕션 반영, PM 최종 승인 후 커밋/푸시</t>
         </is>
       </c>
       <c r="G98" s="6" t="inlineStr">
@@ -6082,29 +6082,29 @@
       </c>
       <c r="H98" s="3" t="inlineStr">
         <is>
-          <t>REL-02,KPI-01</t>
+          <t>REL-01</t>
         </is>
       </c>
       <c r="I98" s="3" t="inlineStr">
         <is>
-          <t>PRD3-3</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J98" s="3" t="inlineStr">
         <is>
-          <t>초기 1주 지표 리뷰 완료</t>
+          <t>프로덕션 URL 정상 서비스 확인</t>
         </is>
       </c>
       <c r="K98" s="3" t="inlineStr">
         <is>
-          <t>해당 없음 — 모니터링 지표 수동 리뷰</t>
+          <t>프로덕션 스모크 테스트: 핵심 URL 200 확인, 챗봇 질의 1회 왕복 확인</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="6" t="inlineStr">
         <is>
-          <t>REL-04</t>
+          <t>REL-03</t>
         </is>
       </c>
       <c r="B99" s="6" t="inlineStr">
@@ -6124,92 +6124,149 @@
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>1.0 출시 회고 및 KPI 재보정 계획 수립</t>
+          <t>배포 후 모니터링 점검</t>
         </is>
       </c>
       <c r="F99" s="3" t="inlineStr">
         <is>
-          <t>2~4주 실측 데이터 수집 계획 및 재보정 일정 수립</t>
+          <t>콜드스타트 비중·응답지연 p50/p95 확인</t>
         </is>
       </c>
       <c r="G99" s="6" t="inlineStr">
         <is>
-          <t>권장</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="H99" s="3" t="inlineStr">
         <is>
-          <t>REL-03</t>
+          <t>REL-02,KPI-01</t>
         </is>
       </c>
       <c r="I99" s="3" t="inlineStr">
         <is>
-          <t>PRD3-2·3-3</t>
+          <t>PRD3-3</t>
         </is>
       </c>
       <c r="J99" s="3" t="inlineStr">
         <is>
-          <t>재보정 일정 문서화</t>
+          <t>초기 1주 지표 리뷰 완료</t>
         </is>
       </c>
       <c r="K99" s="3" t="inlineStr">
         <is>
-          <t>해당 없음 — 문서화 작업</t>
+          <t>해당 없음 — 모니터링 지표 수동 리뷰</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="6" t="inlineStr">
         <is>
+          <t>REL-04</t>
+        </is>
+      </c>
+      <c r="B100" s="6" t="inlineStr">
+        <is>
+          <t>배포릴리즈</t>
+        </is>
+      </c>
+      <c r="C100" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>공통</t>
+        </is>
+      </c>
+      <c r="E100" s="3" t="inlineStr">
+        <is>
+          <t>1.0 출시 회고 및 KPI 재보정 계획 수립</t>
+        </is>
+      </c>
+      <c r="F100" s="3" t="inlineStr">
+        <is>
+          <t>2~4주 실측 데이터 수집 계획 및 재보정 일정 수립</t>
+        </is>
+      </c>
+      <c r="G100" s="6" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H100" s="3" t="inlineStr">
+        <is>
+          <t>REL-03</t>
+        </is>
+      </c>
+      <c r="I100" s="3" t="inlineStr">
+        <is>
+          <t>PRD3-2·3-3</t>
+        </is>
+      </c>
+      <c r="J100" s="3" t="inlineStr">
+        <is>
+          <t>재보정 일정 문서화</t>
+        </is>
+      </c>
+      <c r="K100" s="3" t="inlineStr">
+        <is>
+          <t>해당 없음 — 문서화 작업</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="6" t="inlineStr">
+        <is>
           <t>REL-05</t>
         </is>
       </c>
-      <c r="B100" s="6" t="inlineStr">
+      <c r="B101" s="6" t="inlineStr">
         <is>
           <t>배포릴리즈</t>
         </is>
       </c>
-      <c r="C100" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D100" s="3" t="inlineStr">
+      <c r="C101" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D101" s="3" t="inlineStr">
         <is>
           <t>전체</t>
         </is>
       </c>
-      <c r="E100" s="3" t="inlineStr">
+      <c r="E101" s="3" t="inlineStr">
         <is>
           <t>포트폴리오 공개 전환 준비 체크리스트</t>
         </is>
       </c>
-      <c r="F100" s="3" t="inlineStr">
+      <c r="F101" s="3" t="inlineStr">
         <is>
           <t>저장소를 private에서 public으로 전환하기 전 확인·조치한다: (1) gitleaks 등으로 커밋 히스토리 전체에서 시크릿·API 키 잔존 여부 스캔 (2) 테스트 fixture 전수 조사 — 실제 Riot ID/PUUID/닉네임/매치 데이터가 아닌 합성 데이터로만 구성됐는지 확인, 실데이터가 섞여 있으면 fixture 재작성 후 필요시 git 히스토리 정리 (3) README에 'Riot Games와 무관한 비공식 팬 프로젝트' 디스클레이머 추가 (4) 라이브 배포 URL을 README/공개 자료에 노출할지 결정 (5) 노출하기로 하면 챗봇/전적조회 진입점에 Cloudflare Turnstile 등 경량 봇 방지 적용 검토. 무료 호스팅 비용에는 영향 없음(저장소 공개 여부와 인프라 비용은 무관)</t>
         </is>
       </c>
-      <c r="G100" s="6" t="inlineStr">
+      <c r="G101" s="6" t="inlineStr">
         <is>
           <t>권장</t>
         </is>
       </c>
-      <c r="H100" s="3" t="inlineStr">
+      <c r="H101" s="3" t="inlineStr">
         <is>
           <t>REL-04</t>
         </is>
       </c>
-      <c r="I100" s="3" t="inlineStr">
+      <c r="I101" s="3" t="inlineStr">
         <is>
           <t>PM 결정사항(2026-07-30 대화), policies.md 11번</t>
         </is>
       </c>
-      <c r="J100" s="3" t="inlineStr">
+      <c r="J101" s="3" t="inlineStr">
         <is>
           <t>체크리스트 5개 항목 모두 확인·조치 완료 및 PM 승인 후 저장소 visibility를 public으로 변경</t>
         </is>
       </c>
-      <c r="K100" s="3" t="inlineStr">
+      <c r="K101" s="3" t="inlineStr">
         <is>
           <t>정량 검증: gitleaks(또는 동급 도구) 스캔 결과 시크릿 탐지 0건, 전체 fixture 파일에서 실제 Riot ID 패턴(게임명#태그)·PUUID 패턴 검색 결과 0건</t>
         </is>

</xml_diff>

<commit_message>
feat(DATA-17): 메타 조합 소프트 삭제(is_active) 로직 구현
op.gg tft_list_meta_decks는 페이지네이션 없이 항상 현재 상위 10개 조합만
반환해, 같은 patch_version 내에서도 메타 회전으로 예전 상위 10위 조합이
응답에서 사라질 수 있음(opgg-schema.md 7·8번). 기존 upsert 로직은 삭제를
하지 않아 이런 조합이 comps 테이블에 영구히 남고 신규 필드(cell_x/cell_y
등)도 채울 방법이 없어 계속 휴리스틱 폴백 상태로 고착됨.

comp_champions/comp_augments FK·match_analyses.matched_comp_id FK·
meta_document_embeddings 참조가 있어 하드 삭제 대신 comps.is_active
플래그로 소프트 삭제(PM 결정): 이번 배치 응답에 없는 기존 조합은
is_active=false로 전환, 다시 나타나면 true로 복귀. GET /catalog/tierlist는
is_active=true만 반환하고, GET /catalog/comps/{id}는 비활성 조합도 그대로
조회 가능하게 유지.

batch/normalize.py에 mark_stale_comps_inactive() 신규(upsert_comps 직후
run_patch_batch.py에 배선). backend pytest 202/202(신규 3건)·batch pytest
87/87(신규 4건) 통과. 상세: docs/verification/DATA-17-작업결과.md
</commit_message>
<xml_diff>
--- a/TFT_Hideout_WBS.xlsx
+++ b/TFT_Hideout_WBS.xlsx
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K101"/>
+  <dimension ref="A1:K103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2397,66 +2397,66 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>API-01</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>코딩</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>백엔드API</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>공통</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr">
-        <is>
-          <t>FastAPI 프로젝트 스캐폴딩</t>
-        </is>
-      </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>단일 앱 + catalog/chat/analysis/kpi 4개 라우터 구조(kpi는 SET-11 취소로 Metabase 대신 자체 KPI 대시보드 백엔드용으로 v1.7에서 추가), 헬스체크 엔드포인트</t>
-        </is>
-      </c>
-      <c r="G34" s="4" t="inlineStr">
-        <is>
-          <t>필수</t>
-        </is>
-      </c>
-      <c r="H34" s="3" t="inlineStr">
-        <is>
-          <t>SET-02,SET-03</t>
-        </is>
-      </c>
-      <c r="I34" s="3" t="inlineStr">
-        <is>
-          <t>설계서 4.2</t>
-        </is>
-      </c>
-      <c r="J34" s="3" t="inlineStr">
-        <is>
-          <t>/health 200 응답 확인</t>
-        </is>
-      </c>
-      <c r="K34" s="3" t="inlineStr">
-        <is>
-          <t>pytest+FastAPI TestClient: /health 200 및 4개 라우터(catalog/chat/analysis/kpi) 마운트 확인</t>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>DATA-17</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>데이터파이프라인</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>티어리스트·조합상세</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>메타 조합 소프트 삭제(비활성화) 로직 구현</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>op.gg tft_list_meta_decks는 페이지네이션 없이 항상 현재 상위 10개 조합만 반환하는데(DATA-05/opgg-schema.md 7·8번), 같은 patch_version 내에서도 메타가 회전하면서 예전에 상위 10위였던 조합이 응답에서 사라질 수 있음(FE-14 실좌표 백필 중 10개 중 2개가 이렇게 누락된 것으로 확인, 2026-08-06 재조사로 확정). 기존 upsert 로직은 삭제를 하지 않아 이런 조합이 comps 테이블에 영구히 남고, cell_x/cell_y 등 신규 컬럼도 채울 방법이 없어 계속 휴리스틱 폴백 상태로 고착됨. comp_champions/comp_augments FK·match_analyses.matched_comp_id FK·meta_document_embeddings 참조가 있어 하드 삭제 대신 comps.is_active 플래그로 소프트 삭제한다(PM 결정 2026-08-06): 이번 배치 응답에 없는 기존 행은 is_active=false로 전환, 다시 나타나면 true로 복귀. 티어리스트 API는 is_active=true만 노출하고, 조합 상세·챗봇 인용·PGA 매칭 링크는 비활성 조합도 그대로 조회 가능하게 유지.</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>DATA-08</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>docs/spike/opgg-schema.md(7·8번), 이번 세션 재조사 결과(2026-08-06)</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>배치 실행 시 이번 op.gg 응답에 없는 기존 comps 행이 is_active=false로 전환되고, 응답에 다시 나타나면 is_active=true로 복귀. GET /catalog/tierlist는 is_active=true인 조합만 반환. GET /catalog/comps/{id}는 비활성 조합도 그대로 조회 가능(하드 삭제 아님, FK 참조 보존).</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>pytest: (1) 이번 배치 응답에 없는 riot_comp_id의 기존 comps 행이 is_active=false로 전환되는지, (2) 응답에 다시 나타나면 is_active=true로 복귀하는지, (3) GET /catalog/tierlist가 비활성 조합을 제외하는지, (4) GET /catalog/comps/{id}는 비활성 조합도 정상 응답하는지 확인</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>API-02</t>
+          <t>API-01</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
@@ -2471,17 +2471,17 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>티어리스트</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>GET /catalog/tierlist 구현</t>
+          <t>FastAPI 프로젝트 스캐폴딩</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>패치·랭크 필터 지원, comps 테이블 SQL 조회</t>
+          <t>단일 앱 + catalog/chat/analysis/kpi 4개 라우터 구조(kpi는 SET-11 취소로 Metabase 대신 자체 KPI 대시보드 백엔드용으로 v1.7에서 추가), 헬스체크 엔드포인트</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -2491,29 +2491,29 @@
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>DATA-02,API-01</t>
+          <t>SET-02,SET-03</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>PRD 7-1·설계서6장</t>
+          <t>설계서 4.2</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>응답 스키마·필터 동작 확인</t>
+          <t>/health 200 응답 확인</t>
         </is>
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>pytest: 패치/랭크 필터 조합별 응답, 빈 결과, 잘못된 파라미터 400 케이스</t>
+          <t>pytest+FastAPI TestClient: /health 200 및 4개 라우터(catalog/chat/analysis/kpi) 마운트 확인</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>API-03</t>
+          <t>API-02</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -2528,17 +2528,17 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>조합상세</t>
+          <t>티어리스트</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>GET /catalog/comps/{comp_id} 구현</t>
+          <t>GET /catalog/tierlist 구현</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>챔피언구성·증강체 우선순위 포함</t>
+          <t>패치·랭크 필터 지원, comps 테이블 SQL 조회</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -2553,24 +2553,24 @@
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>설계서 5.1·6장</t>
+          <t>PRD 7-1·설계서6장</t>
         </is>
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>응답 필드 검증</t>
+          <t>응답 스키마·필터 동작 확인</t>
         </is>
       </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
-          <t>pytest: 존재/미존재 comp_id 케이스, 캐리/서브 챔피언 구분 필드 정확성</t>
+          <t>pytest: 패치/랭크 필터 조합별 응답, 빈 결과, 잘못된 파라미터 400 케이스</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>API-04</t>
+          <t>API-03</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
@@ -2585,17 +2585,17 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>아이템빌드</t>
+          <t>조합상세</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>GET /catalog/items/builds 구현</t>
+          <t>GET /catalog/comps/{comp_id} 구현</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>챔피언 필터 지원</t>
+          <t>챔피언구성·증강체 우선순위 포함</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -2610,7 +2610,7 @@
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>설계서 6장</t>
+          <t>설계서 5.1·6장</t>
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr">
@@ -2620,14 +2620,14 @@
       </c>
       <c r="K37" s="3" t="inlineStr">
         <is>
-          <t>pytest: champion_id 필터 유무 케이스, 정렬 순서 검증</t>
+          <t>pytest: 존재/미존재 comp_id 케이스, 캐리/서브 챔피언 구분 필드 정확성</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>API-05</t>
+          <t>API-04</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
@@ -2642,17 +2642,17 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>증강체정보</t>
+          <t>아이템빌드</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>GET /catalog/augments 구현</t>
+          <t>GET /catalog/items/builds 구현</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>is_legend_related=true 승률 마스킹 포함</t>
+          <t>챔피언 필터 지원</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -2662,29 +2662,29 @@
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>DATA-07,API-01</t>
+          <t>DATA-02,API-01</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>PRD 10-1·설계서4.4.3</t>
+          <t>설계서 6장</t>
         </is>
       </c>
       <c r="J38" s="3" t="inlineStr">
         <is>
-          <t>마스킹 동작 단위 테스트 통과</t>
+          <t>응답 필드 검증</t>
         </is>
       </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
-          <t>pytest(필수·정책, TEST-00 시나리오 선적용): is_legend_related=true 데이터로 응답에 win_rate 필드 자체가 없는지(=null 아님) 검증</t>
+          <t>pytest: champion_id 필터 유무 케이스, 정렬 순서 검증</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>API-06</t>
+          <t>API-05</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
@@ -2699,17 +2699,17 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>공통(GNB)</t>
+          <t>증강체정보</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>GET /catalog/patches/current 구현</t>
+          <t>GET /catalog/augments 구현</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>현재 패치 조회</t>
+          <t>is_legend_related=true 승률 마스킹 포함</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
@@ -2719,29 +2719,29 @@
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>DATA-01,API-01</t>
+          <t>DATA-07,API-01</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>설계서 6장</t>
+          <t>PRD 10-1·설계서4.4.3</t>
         </is>
       </c>
       <c r="J39" s="3" t="inlineStr">
         <is>
-          <t>응답 검증</t>
+          <t>마스킹 동작 단위 테스트 통과</t>
         </is>
       </c>
       <c r="K39" s="3" t="inlineStr">
         <is>
-          <t>pytest: is_current=true 패치 1건만 반환되는지 확인</t>
+          <t>pytest(필수·정책, TEST-00 시나리오 선적용): is_legend_related=true 데이터로 응답에 win_rate 필드 자체가 없는지(=null 아님) 검증</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>API-07</t>
+          <t>API-06</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
@@ -2756,17 +2756,17 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>공통(GNB)</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Rate Limiting 미들웨어 구현</t>
+          <t>GET /catalog/patches/current 구현</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>IP 기준 catalog 분당60/chat 분당10</t>
+          <t>현재 패치 조회</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
@@ -2776,29 +2776,29 @@
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>API-01</t>
+          <t>DATA-01,API-01</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.2·6장</t>
+          <t>설계서 6장</t>
         </is>
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>초과 요청 429 응답 확인</t>
+          <t>응답 검증</t>
         </is>
       </c>
       <c r="K40" s="3" t="inlineStr">
         <is>
-          <t>pytest: 한도 초과 요청 시 429 응답 확인(catalog 60/분, chat 10/분 각각)</t>
+          <t>pytest: is_current=true 패치 1건만 반환되는지 확인</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>API-08</t>
+          <t>API-07</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
@@ -2813,17 +2813,17 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>챗봇위젯</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>session_id 발급/조회 로직 구현</t>
+          <t>Rate Limiting 미들웨어 구현</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>클라이언트 UUID 수신 및 대화 묶음 키로 사용</t>
+          <t>IP 기준 catalog 분당60/chat 분당10</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
@@ -2838,24 +2838,24 @@
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.2</t>
+          <t>설계서 4.2·6장</t>
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>세션별 대화 구분 확인</t>
+          <t>초과 요청 429 응답 확인</t>
         </is>
       </c>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>pytest: 동일 session_id 재사용 시 동일 대화로 묶이는지, 신규 UUID는 분리되는지 확인</t>
+          <t>pytest: 한도 초과 요청 시 429 응답 확인(catalog 60/분, chat 10/분 각각)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>API-09</t>
+          <t>API-08</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
@@ -2875,12 +2875,12 @@
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>POST /chat/message 뼈대 구현(SSE)</t>
+          <t>session_id 발급/조회 로직 구현</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>스트리밍 응답 인프라 구현(RAG 로직은 CHAT 그룹에서 연동)</t>
+          <t>클라이언트 UUID 수신 및 대화 묶음 키로 사용</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
@@ -2890,29 +2890,29 @@
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>API-08</t>
+          <t>API-01</t>
         </is>
       </c>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.2·4.4</t>
+          <t>설계서 4.2</t>
         </is>
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t>SSE 스트림 클라이언트 수신 확인</t>
+          <t>세션별 대화 구분 확인</t>
         </is>
       </c>
       <c r="K42" s="3" t="inlineStr">
         <is>
-          <t>pytest: SSE 스트림 청크 수신 순서 및 연결 종료 처리 확인(mock LLM 스트림)</t>
+          <t>pytest: 동일 session_id 재사용 시 동일 대화로 묶이는지, 신규 UUID는 분리되는지 확인</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>API-10</t>
+          <t>API-09</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
@@ -2932,12 +2932,12 @@
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>GET /chat/session/{id}/history 구현</t>
+          <t>POST /chat/message 뼈대 구현(SSE)</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>chat_logs 기반 대화이력 조회</t>
+          <t>스트리밍 응답 인프라 구현(RAG 로직은 CHAT 그룹에서 연동)</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
@@ -2947,29 +2947,29 @@
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>DATA-03,API-09</t>
+          <t>API-08</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.4</t>
+          <t>설계서 4.2·4.4</t>
         </is>
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>최근 3턴 조회 확인</t>
+          <t>SSE 스트림 클라이언트 수신 확인</t>
         </is>
       </c>
       <c r="K43" s="3" t="inlineStr">
         <is>
-          <t>pytest: 최근 3턴만 반환, 4턴 이상 시 오래된 턴 제외 확인</t>
+          <t>pytest: SSE 스트림 청크 수신 순서 및 연결 종료 처리 확인(mock LLM 스트림)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>API-11</t>
+          <t>API-10</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
@@ -2984,17 +2984,17 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석</t>
+          <t>챗봇위젯</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>POST /analysis/link 구현</t>
+          <t>GET /chat/session/{id}/history 구현</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>Riot ID→PUUID 변환, TTL 1시간 캐시(Postgres puuid_cache 테이블, v1.7)</t>
+          <t>chat_logs 기반 대화이력 조회</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
@@ -3004,29 +3004,29 @@
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>SET-16,API-01</t>
+          <t>DATA-03,API-09</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>PRD 9-1·설계서v1.7 4.5</t>
+          <t>설계서 4.4</t>
         </is>
       </c>
       <c r="J44" s="3" t="inlineStr">
         <is>
-          <t>변환 성공/실패 케이스 확인</t>
+          <t>최근 3턴 조회 확인</t>
         </is>
       </c>
       <c r="K44" s="3" t="inlineStr">
         <is>
-          <t>pytest: mock Riot API로 정상/미존재 계정/레이트리밋 초과 3케이스, TTL 1시간 캐시 hit 확인</t>
+          <t>pytest: 최근 3턴만 반환, 4턴 이상 시 오래된 턴 제외 확인</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>API-12</t>
+          <t>API-11</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
@@ -3046,12 +3046,12 @@
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>POST /analysis/recent 뼈대 구현</t>
+          <t>POST /analysis/link 구현</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>최신 매치ID 조회 및 캐시 재사용 분기(스코어링은 PGA 그룹에서 연동)</t>
+          <t>Riot ID→PUUID 변환, TTL 1시간 캐시(Postgres puuid_cache 테이블, v1.7)</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
@@ -3061,29 +3061,29 @@
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>API-11,DATA-03</t>
+          <t>SET-16,API-01</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>PRD 8-3·설계서4.5</t>
+          <t>PRD 9-1·설계서v1.7 4.5</t>
         </is>
       </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t>캐시 hit/miss 분기 확인</t>
+          <t>변환 성공/실패 케이스 확인</t>
         </is>
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>pytest: match_analyses 캐시 hit 시 Riot API mock 호출 0회 확인</t>
+          <t>pytest: mock Riot API로 정상/미존재 계정/레이트리밋 초과 3케이스, TTL 1시간 캐시 hit 확인</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>API-13</t>
+          <t>API-12</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
@@ -3098,17 +3098,17 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>분석리포트</t>
+          <t>사후패인분석</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>GET /analysis/{match_id}/report 구현</t>
+          <t>POST /analysis/recent 뼈대 구현</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>match_analyses 기반 리포트 응답</t>
+          <t>최신 매치ID 조회 및 캐시 재사용 분기(스코어링은 PGA 그룹에서 연동)</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
@@ -3118,29 +3118,29 @@
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>DATA-03,API-12</t>
+          <t>API-11,DATA-03</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
-          <t>PRD 8-3·설계서6장</t>
+          <t>PRD 8-3·설계서4.5</t>
         </is>
       </c>
       <c r="J46" s="3" t="inlineStr">
         <is>
-          <t>응답 스키마 검증</t>
+          <t>캐시 hit/miss 분기 확인</t>
         </is>
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>pytest: 존재/미존재 match_id 케이스, 응답 스키마 필드 전체 검증</t>
+          <t>pytest: match_analyses 캐시 hit 시 Riot API mock 호출 0회 확인</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>API-14</t>
+          <t>API-13</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
@@ -3155,17 +3155,17 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>분석리포트</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>KPI 계측 이벤트 API 구현</t>
+          <t>GET /analysis/{match_id}/report 구현</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>link_click_events, account_link_events 적재 엔드포인트/훅</t>
+          <t>match_analyses 기반 리포트 응답</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
@@ -3175,29 +3175,29 @@
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>DATA-03,API-01</t>
+          <t>DATA-03,API-12</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>PRD 3-3·설계서5.3</t>
+          <t>PRD 8-3·설계서6장</t>
         </is>
       </c>
       <c r="J47" s="3" t="inlineStr">
         <is>
-          <t>이벤트 적재 확인</t>
+          <t>응답 스키마 검증</t>
         </is>
       </c>
       <c r="K47" s="3" t="inlineStr">
         <is>
-          <t>pytest: 이벤트 적재 후 DB row 생성 및 필드 값 정확성 확인</t>
+          <t>pytest: 존재/미존재 match_id 케이스, 응답 스키마 필드 전체 검증</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>CHAT-01</t>
+          <t>API-14</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
@@ -3207,22 +3207,22 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>챗봇RAG</t>
+          <t>백엔드API</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>챗봇위젯</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>의도 분류 로직 구현</t>
+          <t>KPI 계측 이벤트 API 구현</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>1차 키워드/정규식, 2차 Groq LLM 분류(4종)</t>
+          <t>link_click_events, account_link_events 적재 엔드포인트/훅</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
@@ -3232,29 +3232,29 @@
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>API-09</t>
+          <t>DATA-03,API-01</t>
         </is>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
-          <t>PRD 7-2·설계서4.4</t>
+          <t>PRD 3-3·설계서5.3</t>
         </is>
       </c>
       <c r="J48" s="3" t="inlineStr">
         <is>
-          <t>4개 의도 분류 정확도 샘플 테스트</t>
+          <t>이벤트 적재 확인</t>
         </is>
       </c>
       <c r="K48" s="3" t="inlineStr">
         <is>
-          <t>pytest: 키워드 규칙 매칭 케이스(4종 각 2개 이상) + 애매한 질문의 mock LLM 분류 경로 확인</t>
+          <t>pytest: 이벤트 적재 후 DB row 생성 및 필드 값 정확성 확인</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>CHAT-02</t>
+          <t>CHAT-01</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
@@ -3274,12 +3274,12 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>하이브리드 검색 구현</t>
+          <t>의도 분류 로직 구현</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>SQL 필터 + pgvector top-k 코사인 검색</t>
+          <t>1차 키워드/정규식, 2차 Groq LLM 분류(4종)</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
@@ -3289,29 +3289,29 @@
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>DATA-11,CHAT-01</t>
+          <t>API-09</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>PRD 9-4·설계서4.4</t>
+          <t>PRD 7-2·설계서4.4</t>
         </is>
       </c>
       <c r="J49" s="3" t="inlineStr">
         <is>
-          <t>의도별 검색 결과 검증</t>
+          <t>4개 의도 분류 정확도 샘플 테스트</t>
         </is>
       </c>
       <c r="K49" s="3" t="inlineStr">
         <is>
-          <t>pytest: 의도별 SQL 필터 조건 반영 여부, mock pgvector top-k 결과 병합 확인</t>
+          <t>pytest: 키워드 규칙 매칭 케이스(4종 각 2개 이상) + 애매한 질문의 mock LLM 분류 경로 확인</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>CHAT-03</t>
+          <t>CHAT-02</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
@@ -3331,12 +3331,12 @@
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>프롬프트 조립 로직 구현</t>
+          <t>하이브리드 검색 구현</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>시스템프롬프트+검색문서+대화이력+질문 결합, few-shot 삽입</t>
+          <t>SQL 필터 + pgvector top-k 코사인 검색</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
@@ -3346,29 +3346,29 @@
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>CHAT-02,API-10</t>
+          <t>DATA-11,CHAT-01</t>
         </is>
       </c>
       <c r="I50" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.4.1</t>
+          <t>PRD 9-4·설계서4.4</t>
         </is>
       </c>
       <c r="J50" s="3" t="inlineStr">
         <is>
-          <t>프롬프트 스냅샷 테스트</t>
+          <t>의도별 검색 결과 검증</t>
         </is>
       </c>
       <c r="K50" s="3" t="inlineStr">
         <is>
-          <t>pytest: 프롬프트 스냅샷 테스트 — 시스템프롬프트/검색문서/대화이력/질문이 정해진 순서·구분자로 조립되는지 문자열 비교</t>
+          <t>pytest: 의도별 SQL 필터 조건 반영 여부, mock pgvector top-k 결과 병합 확인</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>CHAT-04</t>
+          <t>CHAT-03</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
@@ -3388,12 +3388,12 @@
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>입력 전처리 구현</t>
+          <t>프롬프트 조립 로직 구현</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>질문정규화·은어치환·인젝션방어·길이제한·범위밖질문 안내</t>
+          <t>시스템프롬프트+검색문서+대화이력+질문 결합, few-shot 삽입</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
@@ -3403,29 +3403,29 @@
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>CHAT-01</t>
+          <t>CHAT-02,API-10</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.4.2</t>
+          <t>설계서 4.4.1</t>
         </is>
       </c>
       <c r="J51" s="3" t="inlineStr">
         <is>
-          <t>각 케이스 단위 테스트 통과</t>
+          <t>프롬프트 스냅샷 테스트</t>
         </is>
       </c>
       <c r="K51" s="3" t="inlineStr">
         <is>
-          <t>pytest(필수·보안, TEST-00 시나리오 선적용): 인젝션 문구가 [사용자 메시지] 델리미터 내부로만 들어가는지, 범위밖 질문 안내 문구 반환, 초과 길이 입력 truncate 확인</t>
+          <t>pytest: 프롬프트 스냅샷 테스트 — 시스템프롬프트/검색문서/대화이력/질문이 정해진 순서·구분자로 조립되는지 문자열 비교</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>CHAT-05</t>
+          <t>CHAT-04</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
@@ -3445,12 +3445,12 @@
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>sLLM 답변 생성 및 SSE 스트리밍 연동</t>
+          <t>입력 전처리 구현</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>Groq Llama 3.3 70B 호출, 스트리밍 응답</t>
+          <t>질문정규화·은어치환·인젝션방어·길이제한·범위밖질문 안내</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr">
@@ -3460,29 +3460,29 @@
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>CHAT-03,API-09,SET-10</t>
+          <t>CHAT-01</t>
         </is>
       </c>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.4</t>
+          <t>설계서 4.4.2</t>
         </is>
       </c>
       <c r="J52" s="3" t="inlineStr">
         <is>
-          <t>스트리밍 응답 end-to-end 확인</t>
+          <t>각 케이스 단위 테스트 통과</t>
         </is>
       </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
-          <t>pytest: mock Groq 클라이언트로 SSE 스트리밍 조립 확인, 타임아웃 예외 처리 확인</t>
+          <t>pytest(필수·보안, TEST-00 시나리오 선적용): 인젝션 문구가 [사용자 메시지] 델리미터 내부로만 들어가는지, 범위밖 질문 안내 문구 반환, 초과 길이 입력 truncate 확인</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>CHAT-06</t>
+          <t>CHAT-05</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
@@ -3502,12 +3502,12 @@
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>출력 후처리 구현</t>
+          <t>sLLM 답변 생성 및 SSE 스트리밍 연동</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>근거검증·Legend승률이중방어·닉네임마스킹·구조화출력·재시도폴백</t>
+          <t>Groq Llama 3.3 70B 호출, 스트리밍 응답</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
@@ -3517,29 +3517,29 @@
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>CHAT-05</t>
+          <t>CHAT-03,API-09,SET-10</t>
         </is>
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.4.3</t>
+          <t>설계서 4.4</t>
         </is>
       </c>
       <c r="J53" s="3" t="inlineStr">
         <is>
-          <t>각 방어 로직 단위 테스트 통과</t>
+          <t>스트리밍 응답 end-to-end 확인</t>
         </is>
       </c>
       <c r="K53" s="3" t="inlineStr">
         <is>
-          <t>pytest(필수·정책, TEST-00 시나리오 선적용): 근거 없는 고유명사 재생성/경고 처리, Legend 문서 승률 수치 후처리 제거, 상대 닉네임 정규식 마스킹 3케이스 모두 검증</t>
+          <t>pytest: mock Groq 클라이언트로 SSE 스트리밍 조립 확인, 타임아웃 예외 처리 확인</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>CHAT-07</t>
+          <t>CHAT-06</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
@@ -3559,12 +3559,12 @@
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>웹사이트 링크 자동 삽입 구현</t>
+          <t>출력 후처리 구현</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>답변 내 조합/아이템/증강체 id 파싱→상세페이지 링크 삽입</t>
+          <t>근거검증·Legend승률이중방어·닉네임마스킹·구조화출력·재시도폴백</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
@@ -3574,29 +3574,29 @@
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>CHAT-06</t>
+          <t>CHAT-05</t>
         </is>
       </c>
       <c r="I54" s="3" t="inlineStr">
         <is>
-          <t>PRD 7-2·설계서4.4</t>
+          <t>설계서 4.4.3</t>
         </is>
       </c>
       <c r="J54" s="3" t="inlineStr">
         <is>
-          <t>링크 삽입 정확도 샘플 테스트</t>
+          <t>각 방어 로직 단위 테스트 통과</t>
         </is>
       </c>
       <c r="K54" s="3" t="inlineStr">
         <is>
-          <t>pytest: 답변 내 조합/아이템/증강체 언급 시 정확한 링크 삽입, 존재하지 않는 id 오탐 케이스 처리 확인</t>
+          <t>pytest(필수·정책, TEST-00 시나리오 선적용): 근거 없는 고유명사 재생성/경고 처리, Legend 문서 승률 수치 후처리 제거, 상대 닉네임 정규식 마스킹 3케이스 모두 검증</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>CHAT-08</t>
+          <t>CHAT-07</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
@@ -3616,12 +3616,12 @@
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>응답 캐싱 로직 구현</t>
+          <t>웹사이트 링크 자동 삽입 구현</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>첫턴 질문 Postgres(chat_answer_cache) 캐시, 후속턴 캐시제외, 패치갱신시 무효화</t>
+          <t>답변 내 조합/아이템/증강체 id 파싱→상세페이지 링크 삽입</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
@@ -3631,29 +3631,29 @@
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>CHAT-05,DATA-15</t>
+          <t>CHAT-06</t>
         </is>
       </c>
       <c r="I55" s="3" t="inlineStr">
         <is>
-          <t>PRD 9-6·설계서v1.7 4.4·4.6</t>
+          <t>PRD 7-2·설계서4.4</t>
         </is>
       </c>
       <c r="J55" s="3" t="inlineStr">
         <is>
-          <t>캐시 hit/무효화 시나리오 테스트</t>
+          <t>링크 삽입 정확도 샘플 테스트</t>
         </is>
       </c>
       <c r="K55" s="3" t="inlineStr">
         <is>
-          <t>pytest: 첫턴 캐시 hit, 후속턴 캐시 미적용, 패치갱신 후 캐시 무효화 확인</t>
+          <t>pytest: 답변 내 조합/아이템/증강체 언급 시 정확한 링크 삽입, 존재하지 않는 id 오탐 케이스 처리 확인</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>CHAT-09</t>
+          <t>CHAT-08</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
@@ -3673,12 +3673,12 @@
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>Q&amp;A 로깅 구현</t>
+          <t>응답 캐싱 로직 구현</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>chat_logs 적재(질의/의도/근거문서/patch/지연시간/콜드스타트)</t>
+          <t>첫턴 질문 Postgres(chat_answer_cache) 캐시, 후속턴 캐시제외, 패치갱신시 무효화</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
@@ -3688,29 +3688,29 @@
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>DATA-03,CHAT-05</t>
+          <t>CHAT-05,DATA-15</t>
         </is>
       </c>
       <c r="I56" s="3" t="inlineStr">
         <is>
-          <t>PRD 3-3·9-5</t>
+          <t>PRD 9-6·설계서v1.7 4.4·4.6</t>
         </is>
       </c>
       <c r="J56" s="3" t="inlineStr">
         <is>
-          <t>로그 적재 필드 확인</t>
+          <t>캐시 hit/무효화 시나리오 테스트</t>
         </is>
       </c>
       <c r="K56" s="3" t="inlineStr">
         <is>
-          <t>pytest: chat_logs row에 질의/의도/근거문서id/patch_version/답변/지연시간/콜드스타트 전체 필드 적재 확인</t>
+          <t>pytest: 첫턴 캐시 hit, 후속턴 캐시 미적용, 패치갱신 후 캐시 무효화 확인</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>CHAT-10</t>
+          <t>CHAT-09</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
@@ -3730,12 +3730,12 @@
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>사후분석 트리거 연동</t>
+          <t>Q&amp;A 로깅 구현</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>'방금 게임 분석해줘' 발화 시 분석 로직 호출 및 챗봇 답변 영역 요약 표시</t>
+          <t>chat_logs 적재(질의/의도/근거문서/patch/지연시간/콜드스타트)</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
@@ -3745,29 +3745,29 @@
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>CHAT-06,API-12</t>
+          <t>DATA-03,CHAT-05</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
         <is>
-          <t>PRD 8-3</t>
+          <t>PRD 3-3·9-5</t>
         </is>
       </c>
       <c r="J57" s="3" t="inlineStr">
         <is>
-          <t>트리거 발화 테스트 통과</t>
+          <t>로그 적재 필드 확인</t>
         </is>
       </c>
       <c r="K57" s="3" t="inlineStr">
         <is>
-          <t>pytest: '방금 게임 분석해줘' mock 발화 시 analysis 로직 호출(1회) 및 응답에 요약+링크 포함 확인</t>
+          <t>pytest: chat_logs row에 질의/의도/근거문서id/patch_version/답변/지연시간/콜드스타트 전체 필드 적재 확인</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>CHAT-11</t>
+          <t>CHAT-10</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
@@ -3787,44 +3787,44 @@
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>후속질문 동적 생성(LLM 기반) 구현</t>
+          <t>사후분석 트리거 연동</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>CHAT-05 답변 생성 이후 Groq에 맥락 기반 후속 질문 2~3개 생성을 추가 요청(프롬프트 설계), SSE에 신규 이벤트(event: followups) 추가해 FE-09가 만든 고정 4개 칩을 동적 목록으로 교체. 무료 티어 레이트리밋/응답 지연 영향 검토 포함(PM 결정 2026-08-06, LLM 기반 채택).</t>
+          <t>'방금 게임 분석해줘' 발화 시 분석 로직 호출 및 챗봇 답변 영역 요약 표시</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
-          <t>권장</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>CHAT-05,FE-09</t>
+          <t>CHAT-06,API-12</t>
         </is>
       </c>
       <c r="I58" s="3" t="inlineStr">
         <is>
-          <t>PRD7-4·화면설계서2.7(SuggestedFollowupChips)·개발설계서4.4(프롬프트 조립)</t>
+          <t>PRD 8-3</t>
         </is>
       </c>
       <c r="J58" s="3" t="inlineStr">
         <is>
-          <t>Groq 추가 호출로 후속 질문 2~3개 생성, SSE event: followups로 프론트에 전달, FE-09 정적 칩이 동적 목록으로 교체됨, 무료 티어 레이트리밋 영향(호출 증가율·콜드스타트 비중 변화) 검토 결과 기록</t>
+          <t>트리거 발화 테스트 통과</t>
         </is>
       </c>
       <c r="K58" s="3" t="inlineStr">
         <is>
-          <t>pytest: 후속질문 생성 함수 고정 fixture 입력 → 질문 형식/개수 검증, Groq 실패 시 후속질문 없이도 기존 답변 스트리밍은 정상 동작하는지(폴백) 확인 | Vitest+RTL: followups 이벤트 포함 mock SSE로 동적 칩 렌더링, 칩 클릭 시 해당 질문이 전송되는지 테스트</t>
+          <t>pytest: '방금 게임 분석해줘' mock 발화 시 analysis 로직 호출(1회) 및 응답에 요약+링크 포함 확인</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>PGA-01</t>
+          <t>CHAT-11</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
@@ -3834,54 +3834,54 @@
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>사후패인분석</t>
+          <t>챗봇RAG</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석</t>
+          <t>챗봇위젯</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>Riot ID 계정 연동 로직 구현</t>
+          <t>후속질문 동적 생성(LLM 기반) 구현</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>게임명#태그+지역 입력→PUUID 변환, 임의계정 조회 허용</t>
+          <t>CHAT-05 답변 생성 이후 Groq에 맥락 기반 후속 질문 2~3개 생성을 추가 요청(프롬프트 설계), SSE에 신규 이벤트(event: followups) 추가해 FE-09가 만든 고정 4개 칩을 동적 목록으로 교체. 무료 티어 레이트리밋/응답 지연 영향 검토 포함(PM 결정 2026-08-06, LLM 기반 채택).</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t>필수</t>
+          <t>권장</t>
         </is>
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>API-11</t>
+          <t>CHAT-05,FE-09</t>
         </is>
       </c>
       <c r="I59" s="3" t="inlineStr">
         <is>
-          <t>PRD 7-3·8-3·9-1</t>
+          <t>PRD7-4·화면설계서2.7(SuggestedFollowupChips)·개발설계서4.4(프롬프트 조립)</t>
         </is>
       </c>
       <c r="J59" s="3" t="inlineStr">
         <is>
-          <t>정상/비정상 계정 케이스 테스트</t>
+          <t>Groq 추가 호출로 후속 질문 2~3개 생성, SSE event: followups로 프론트에 전달, FE-09 정적 칩이 동적 목록으로 교체됨, 무료 티어 레이트리밋 영향(호출 증가율·콜드스타트 비중 변화) 검토 결과 기록</t>
         </is>
       </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t>pytest: 정상 Riot ID/형식 오류/미존재 계정 3케이스</t>
+          <t>pytest: 후속질문 생성 함수 고정 fixture 입력 → 질문 형식/개수 검증, Groq 실패 시 후속질문 없이도 기존 답변 스트리밍은 정상 동작하는지(폴백) 확인 | Vitest+RTL: followups 이벤트 포함 mock SSE로 동적 칩 렌더링, 칩 클릭 시 해당 질문이 전송되는지 테스트</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>PGA-02</t>
+          <t>PGA-01</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
@@ -3901,12 +3901,12 @@
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>최신 매치 조회 로직 구현</t>
+          <t>Riot ID 계정 연동 로직 구현</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>Match-V1으로 매치ID/매치상세 조회</t>
+          <t>게임명#태그+지역 입력→PUUID 변환, 임의계정 조회 허용</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
@@ -3916,29 +3916,29 @@
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>PGA-01</t>
+          <t>API-11</t>
         </is>
       </c>
       <c r="I60" s="3" t="inlineStr">
         <is>
-          <t>PRD 7-3·설계서4.5</t>
+          <t>PRD 7-3·8-3·9-1</t>
         </is>
       </c>
       <c r="J60" s="3" t="inlineStr">
         <is>
-          <t>매치 상세 파싱 검증</t>
+          <t>정상/비정상 계정 케이스 테스트</t>
         </is>
       </c>
       <c r="K60" s="3" t="inlineStr">
         <is>
-          <t>pytest: mock Match-V1 응답 기준 매치ID·매치상세 파싱 필드 전체 검증</t>
+          <t>pytest: 정상 Riot ID/형식 오류/미존재 계정 3케이스</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>PGA-03</t>
+          <t>PGA-02</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
@@ -3953,17 +3953,17 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석·분석리포트</t>
+          <t>사후패인분석</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>분석 결과 캐시 재사용 로직 구현</t>
+          <t>최신 매치 조회 로직 구현</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>match_analyses 조회 우선, 없으면 신규계산</t>
+          <t>Match-V1으로 매치ID/매치상세 조회</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
@@ -3973,29 +3973,29 @@
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>DATA-03,PGA-02</t>
+          <t>PGA-01</t>
         </is>
       </c>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.5·4.6·5.1</t>
+          <t>PRD 7-3·설계서4.5</t>
         </is>
       </c>
       <c r="J61" s="3" t="inlineStr">
         <is>
-          <t>재요청 시 캐시 히트 확인</t>
+          <t>매치 상세 파싱 검증</t>
         </is>
       </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>pytest: 동일 match_id+puuid 재요청 시 Riot API/Groq mock 호출 0회(캐시 hit), 신규 조합은 계산 경로 진입 확인</t>
+          <t>pytest: mock Match-V1 응답 기준 매치ID·매치상세 파싱 필드 전체 검증</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>PGA-04</t>
+          <t>PGA-03</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
@@ -4010,17 +4010,17 @@
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>분석리포트</t>
+          <t>사후패인분석·분석리포트</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>조합 이탈도 계산 로직 구현</t>
+          <t>분석 결과 캐시 재사용 로직 구현</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>가중 자카드 유사도(캐리 가중치2), 구간분류</t>
+          <t>match_analyses 조회 우선, 없으면 신규계산</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
@@ -4030,29 +4030,29 @@
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>PGA-02,DATA-02</t>
+          <t>DATA-03,PGA-02</t>
         </is>
       </c>
       <c r="I62" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.5.1</t>
+          <t>설계서 4.5·4.6·5.1</t>
         </is>
       </c>
       <c r="J62" s="3" t="inlineStr">
         <is>
-          <t>샘플 매치 계산값 수기검증 일치</t>
+          <t>재요청 시 캐시 히트 확인</t>
         </is>
       </c>
       <c r="K62" s="3" t="inlineStr">
         <is>
-          <t>pytest(필수·크리티컬, TEST-00 시나리오 선적용): 수기 계산한 샘플 보드 3~5개에 대해 이탈도 값이 소수점 둘째자리까지 일치, 구간분류 경계값(0.3/0.6) 케이스 포함</t>
+          <t>pytest: 동일 match_id+puuid 재요청 시 Riot API/Groq mock 호출 0회(캐시 hit), 신규 조합은 계산 경로 진입 확인</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>PGA-05</t>
+          <t>PGA-04</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
@@ -4072,12 +4072,12 @@
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>아이템 집중도 계산 로직 구현</t>
+          <t>조합 이탈도 계산 로직 구현</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>캐리 완성아이템 비율, 추천빌드 멀티셋 교집합</t>
+          <t>가중 자카드 유사도(캐리 가중치2), 구간분류</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr">
@@ -4087,7 +4087,7 @@
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>PGA-04</t>
+          <t>PGA-02,DATA-02</t>
         </is>
       </c>
       <c r="I63" s="3" t="inlineStr">
@@ -4097,19 +4097,19 @@
       </c>
       <c r="J63" s="3" t="inlineStr">
         <is>
-          <t>샘플 계산값 검증</t>
+          <t>샘플 매치 계산값 수기검증 일치</t>
         </is>
       </c>
       <c r="K63" s="3" t="inlineStr">
         <is>
-          <t>pytest: 샘플 보드 기준 집중도 값 수기 계산과 일치, 중복 아이템 멀티셋 케이스 포함</t>
+          <t>pytest(필수·크리티컬, TEST-00 시나리오 선적용): 수기 계산한 샘플 보드 3~5개에 대해 이탈도 값이 소수점 둘째자리까지 일치, 구간분류 경계값(0.3/0.6) 케이스 포함</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>PGA-06</t>
+          <t>PGA-05</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
@@ -4129,12 +4129,12 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>증강체 시너지 계산 로직 구현</t>
+          <t>아이템 집중도 계산 로직 구현</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>선택증강체 vs comp_augments 매칭 비율</t>
+          <t>캐리 완성아이템 비율, 추천빌드 멀티셋 교집합</t>
         </is>
       </c>
       <c r="G64" s="4" t="inlineStr">
@@ -4159,14 +4159,14 @@
       </c>
       <c r="K64" s="3" t="inlineStr">
         <is>
-          <t>pytest: 선택 증강체 0개/일부일치/전체일치 3케이스 시너지 점수 검증</t>
+          <t>pytest: 샘플 보드 기준 집중도 값 수기 계산과 일치, 중복 아이템 멀티셋 케이스 포함</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>PGA-07</t>
+          <t>PGA-06</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
@@ -4186,12 +4186,12 @@
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>코칭 문장 생성 로직 구현</t>
+          <t>증강체 시너지 계산 로직 구현</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>3개 지표+등수 근거로 잘한점/아쉬운점/제안 고정구조 생성, 수치 비노출. op.gg tft_get_play_style(PUUID 필요, DATA-08에서 이동)을 호출해 코칭 근거로 활용</t>
+          <t>선택증강체 vs comp_augments 매칭 비율</t>
         </is>
       </c>
       <c r="G65" s="4" t="inlineStr">
@@ -4201,29 +4201,29 @@
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
-          <t>PGA-04,PGA-05,PGA-06,SET-10</t>
+          <t>PGA-04</t>
         </is>
       </c>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>PRD 7-3·설계서4.5.2</t>
+          <t>설계서 4.5.1</t>
         </is>
       </c>
       <c r="J65" s="3" t="inlineStr">
         <is>
-          <t>출력 포맷 규칙 준수 확인</t>
+          <t>샘플 계산값 검증</t>
         </is>
       </c>
       <c r="K65" s="3" t="inlineStr">
         <is>
-          <t>pytest(필수·정책, TEST-00 시나리오 선적용): mock LLM 출력에 원 수치(예: '이탈도 0.42')가 노출되면 실패 처리되는 검증 로직 자체 테스트, 고정 3단 구조 파싱 확인</t>
+          <t>pytest: 선택 증강체 0개/일부일치/전체일치 3케이스 시너지 점수 검증</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>PGA-08</t>
+          <t>PGA-07</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
@@ -4243,12 +4243,12 @@
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>다음 게임 제안 근거 조회 로직 구현</t>
+          <t>코칭 문장 생성 로직 구현</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>matched_comp_id 기준 추천아이템·증강체 조회</t>
+          <t>3개 지표+등수 근거로 잘한점/아쉬운점/제안 고정구조 생성, 수치 비노출. op.gg tft_get_play_style(PUUID 필요, DATA-08에서 이동)을 호출해 코칭 근거로 활용</t>
         </is>
       </c>
       <c r="G66" s="4" t="inlineStr">
@@ -4258,29 +4258,29 @@
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>PGA-04,DATA-02</t>
+          <t>PGA-04,PGA-05,PGA-06,SET-10</t>
         </is>
       </c>
       <c r="I66" s="3" t="inlineStr">
         <is>
-          <t>설계서 4.5.3</t>
+          <t>PRD 7-3·설계서4.5.2</t>
         </is>
       </c>
       <c r="J66" s="3" t="inlineStr">
         <is>
-          <t>추천 근거 정확성 검증</t>
+          <t>출력 포맷 규칙 준수 확인</t>
         </is>
       </c>
       <c r="K66" s="3" t="inlineStr">
         <is>
-          <t>pytest: matched_comp_id 기준 추천아이템/증강체 조회 결과가 champion_item_builds/comp_augments와 일치하는지 확인</t>
+          <t>pytest(필수·정책, TEST-00 시나리오 선적용): mock LLM 출력에 원 수치(예: '이탈도 0.42')가 노출되면 실패 처리되는 검증 로직 자체 테스트, 고정 3단 구조 파싱 확인</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>PGA-09</t>
+          <t>PGA-08</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
@@ -4300,12 +4300,12 @@
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>프라이버시 마스킹 로직 구현</t>
+          <t>다음 게임 제안 근거 조회 로직 구현</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>상대 닉네임 마스킹 전처리+정규식 재마스킹 이중방어</t>
+          <t>matched_comp_id 기준 추천아이템·증강체 조회</t>
         </is>
       </c>
       <c r="G67" s="4" t="inlineStr">
@@ -4315,29 +4315,29 @@
       </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
-          <t>PGA-07</t>
+          <t>PGA-04,DATA-02</t>
         </is>
       </c>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>PRD 7-3·설계서4.4.3·4.5.3</t>
+          <t>설계서 4.5.3</t>
         </is>
       </c>
       <c r="J67" s="3" t="inlineStr">
         <is>
-          <t>마스킹 누락 케이스 없음 확인</t>
+          <t>추천 근거 정확성 검증</t>
         </is>
       </c>
       <c r="K67" s="3" t="inlineStr">
         <is>
-          <t>pytest(필수·보안, TEST-00 시나리오 선적용): 상대 Riot ID 포함 mock LLM 출력에서 정규식 마스킹 후 원본 문자열이 전혀 남지 않는지(부분 마스킹 실패 케이스 포함) 확인</t>
+          <t>pytest: matched_comp_id 기준 추천아이템/증강체 조회 결과가 champion_item_builds/comp_augments와 일치하는지 확인</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>PGA-10</t>
+          <t>PGA-09</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
@@ -4352,17 +4352,17 @@
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석·분석리포트</t>
+          <t>분석리포트</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>상세 리포트 데이터 조립 로직 구현</t>
+          <t>프라이버시 마스킹 로직 구현</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>코칭요약·매칭조합·등수변화·아이템타임라인 응답 조립</t>
+          <t>상대 닉네임 마스킹 전처리+정규식 재마스킹 이중방어</t>
         </is>
       </c>
       <c r="G68" s="4" t="inlineStr">
@@ -4372,29 +4372,29 @@
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>PGA-07,PGA-08,PGA-09,API-13</t>
+          <t>PGA-07</t>
         </is>
       </c>
       <c r="I68" s="3" t="inlineStr">
         <is>
-          <t>PRD 8-3·IA4.6</t>
+          <t>PRD 7-3·설계서4.4.3·4.5.3</t>
         </is>
       </c>
       <c r="J68" s="3" t="inlineStr">
         <is>
-          <t>API-13 응답 필드 전체 채움 확인</t>
+          <t>마스킹 누락 케이스 없음 확인</t>
         </is>
       </c>
       <c r="K68" s="3" t="inlineStr">
         <is>
-          <t>pytest: API-13 응답 스키마 전체 필드가 null 없이 채워지는지 통합 테스트</t>
+          <t>pytest(필수·보안, TEST-00 시나리오 선적용): 상대 Riot ID 포함 mock LLM 출력에서 정규식 마스킹 후 원본 문자열이 전혀 남지 않는지(부분 마스킹 실패 케이스 포함) 확인</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>FE-01</t>
+          <t>PGA-10</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
@@ -4404,22 +4404,22 @@
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>프론트엔드</t>
+          <t>사후패인분석</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>사후패인분석·분석리포트</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Next.js 프로젝트 스캐폴딩 및 Tailwind 설정</t>
+          <t>상세 리포트 데이터 조립 로직 구현</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>App Router, Tailwind 브레이크포인트(md768/lg1024) 매핑, 디자인가이드 토큰(컬러/타이포/spacing) 반영</t>
+          <t>코칭요약·매칭조합·등수변화·아이템타임라인 응답 조립</t>
         </is>
       </c>
       <c r="G69" s="4" t="inlineStr">
@@ -4429,29 +4429,29 @@
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>SET-07</t>
+          <t>PGA-07,PGA-08,PGA-09,API-13</t>
         </is>
       </c>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>설계서4.1.1·디자인가이드</t>
+          <t>PRD 8-3·IA4.6</t>
         </is>
       </c>
       <c r="J69" s="3" t="inlineStr">
         <is>
-          <t>기본 레이아웃 렌더링 확인</t>
+          <t>API-13 응답 필드 전체 채움 확인</t>
         </is>
       </c>
       <c r="K69" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: Tailwind 브레이크포인트 클래스 적용 여부, 디자인 토큰 색상값 매칭 확인</t>
+          <t>pytest: API-13 응답 스키마 전체 필드가 null 없이 채워지는지 통합 테스트</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>FE-02</t>
+          <t>FE-01</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
@@ -4466,17 +4466,17 @@
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>공통(GNB)</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>GNB 컴포넌트 구현</t>
+          <t>Next.js 프로젝트 스캐폴딩 및 Tailwind 설정</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>데스크톱/태블릿 가로바, 모바일 햄버거+드로어, 4개 진입점</t>
+          <t>App Router, Tailwind 브레이크포인트(md768/lg1024) 매핑, 디자인가이드 토큰(컬러/타이포/spacing) 반영</t>
         </is>
       </c>
       <c r="G70" s="4" t="inlineStr">
@@ -4486,29 +4486,29 @@
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>FE-01</t>
+          <t>SET-07</t>
         </is>
       </c>
       <c r="I70" s="3" t="inlineStr">
         <is>
-          <t>PRD7-4·IA6.1·디자인가이드6.1</t>
+          <t>설계서4.1.1·디자인가이드</t>
         </is>
       </c>
       <c r="J70" s="3" t="inlineStr">
         <is>
-          <t>3개 브레이크포인트 시각 확인</t>
+          <t>기본 레이아웃 렌더링 확인</t>
         </is>
       </c>
       <c r="K70" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: 3개 브레이크포인트에서 GNB 렌더링 분기(가로바/드로어) 테스트 + Playwright 스모크(클릭 시 드로어 오픈)</t>
+          <t>Vitest+RTL: Tailwind 브레이크포인트 클래스 적용 여부, 디자인 토큰 색상값 매칭 확인</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>FE-03</t>
+          <t>FE-02</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
@@ -4523,17 +4523,17 @@
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>티어리스트</t>
+          <t>공통(GNB)</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>티어리스트(홈) 페이지 구현</t>
+          <t>GNB 컴포넌트 구현</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>필터바/카드그리드/챗봇슬롯, 정적 export(FE-01 결정) + 클라이언트 사이드 fetch(CSR), 반응형(3~4열→2열→1열)</t>
+          <t>데스크톱/태블릿 가로바, 모바일 햄버거+드로어, 4개 진입점</t>
         </is>
       </c>
       <c r="G71" s="4" t="inlineStr">
@@ -4543,29 +4543,29 @@
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
-          <t>FE-02,API-02,API-06</t>
+          <t>FE-01</t>
         </is>
       </c>
       <c r="I71" s="3" t="inlineStr">
         <is>
-          <t>PRD7-1·7-4·화면설계서2.1</t>
+          <t>PRD7-4·IA6.1·디자인가이드6.1</t>
         </is>
       </c>
       <c r="J71" s="3" t="inlineStr">
         <is>
-          <t>데스크톱/태블릿/모바일 와이어프레임 대비 시각 검증</t>
+          <t>3개 브레이크포인트 시각 확인</t>
         </is>
       </c>
       <c r="K71" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: 카드 그리드 컬럼 수 브레이크포인트별 렌더링, mock API 응답 데이터 바인딩 테스트(E2E는 TEST-08)</t>
+          <t>Vitest+RTL: 3개 브레이크포인트에서 GNB 렌더링 분기(가로바/드로어) 테스트 + Playwright 스모크(클릭 시 드로어 오픈)</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>FE-04</t>
+          <t>FE-03</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
@@ -4580,17 +4580,17 @@
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>조합상세</t>
+          <t>티어리스트</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>조합 상세 페이지 구현</t>
+          <t>티어리스트(홈) 페이지 구현</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>개요/챔피언구성(캐리강조)/증강체목록/CTA버튼, 모바일 full-width CTA</t>
+          <t>필터바/카드그리드/챗봇슬롯, 정적 export(FE-01 결정) + 클라이언트 사이드 fetch(CSR), 반응형(3~4열→2열→1열)</t>
         </is>
       </c>
       <c r="G72" s="4" t="inlineStr">
@@ -4600,29 +4600,29 @@
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>FE-02,API-03</t>
+          <t>FE-02,API-02,API-06</t>
         </is>
       </c>
       <c r="I72" s="3" t="inlineStr">
         <is>
-          <t>화면설계서2.2</t>
+          <t>PRD7-1·7-4·화면설계서2.1</t>
         </is>
       </c>
       <c r="J72" s="3" t="inlineStr">
         <is>
-          <t>링크이동·반응형 검증</t>
+          <t>데스크톱/태블릿/모바일 와이어프레임 대비 시각 검증</t>
         </is>
       </c>
       <c r="K72" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: 캐리/서브 챔피언 보더 스타일 분기, CTA 버튼 모바일 full-width 렌더링 테스트</t>
+          <t>Vitest+RTL: 카드 그리드 컬럼 수 브레이크포인트별 렌더링, mock API 응답 데이터 바인딩 테스트(E2E는 TEST-08)</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>FE-05</t>
+          <t>FE-04</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
@@ -4637,17 +4637,17 @@
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>아이템빌드</t>
+          <t>조합상세</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>아이템 빌드 페이지 구현</t>
+          <t>조합 상세 페이지 구현</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>챔피언필터/조합리스트/상세패널(모바일 바텀시트)</t>
+          <t>개요/챔피언구성(캐리강조)/증강체목록/CTA버튼, 모바일 full-width CTA</t>
         </is>
       </c>
       <c r="G73" s="4" t="inlineStr">
@@ -4657,29 +4657,29 @@
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>FE-02,API-04</t>
+          <t>FE-02,API-03</t>
         </is>
       </c>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>화면설계서2.3</t>
+          <t>화면설계서2.2</t>
         </is>
       </c>
       <c r="J73" s="3" t="inlineStr">
         <is>
-          <t>필터-URL쿼리 동기화 검증</t>
+          <t>링크이동·반응형 검증</t>
         </is>
       </c>
       <c r="K73" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: 챔피언 필터 선택 시 URL 쿼리 동기화, 모바일 바텀시트 오픈/클로즈 테스트</t>
+          <t>Vitest+RTL: 캐리/서브 챔피언 보더 스타일 분기, CTA 버튼 모바일 full-width 렌더링 테스트</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>FE-06</t>
+          <t>FE-05</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
@@ -4694,17 +4694,17 @@
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>증강체정보</t>
+          <t>아이템빌드</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>증강체 정보 페이지 구현</t>
+          <t>아이템 빌드 페이지 구현</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>티어필터/카드리스트, Legend 승률 숨김 표시</t>
+          <t>챔피언필터/조합리스트/상세패널(모바일 바텀시트)</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr">
@@ -4714,29 +4714,29 @@
       </c>
       <c r="H74" s="3" t="inlineStr">
         <is>
-          <t>FE-02,API-05</t>
+          <t>FE-02,API-04</t>
         </is>
       </c>
       <c r="I74" s="3" t="inlineStr">
         <is>
-          <t>PRD10-1·화면설계서2.4</t>
+          <t>화면설계서2.3</t>
         </is>
       </c>
       <c r="J74" s="3" t="inlineStr">
         <is>
-          <t>Legend 항목 승률 미노출 확인</t>
+          <t>필터-URL쿼리 동기화 검증</t>
         </is>
       </c>
       <c r="K74" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL(필수·정책): is_legend_related=true 카드에 '승률 표시 안함' 텍스트만 렌더링되고 숫자가 DOM에 없는지 확인</t>
+          <t>Vitest+RTL: 챔피언 필터 선택 시 URL 쿼리 동기화, 모바일 바텀시트 오픈/클로즈 테스트</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>FE-07</t>
+          <t>FE-06</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
@@ -4751,17 +4751,17 @@
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석</t>
+          <t>증강체정보</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>사후 패인 분석 페이지 구현</t>
+          <t>증강체 정보 페이지 구현</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>Riot ID 폼/최근계정목록(localStorage)/전적불러오기 버튼/진행상태</t>
+          <t>티어필터/카드리스트, Legend 승률 숨김 표시</t>
         </is>
       </c>
       <c r="G75" s="4" t="inlineStr">
@@ -4771,29 +4771,29 @@
       </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
-          <t>FE-02,API-11,API-12</t>
+          <t>FE-02,API-05</t>
         </is>
       </c>
       <c r="I75" s="3" t="inlineStr">
         <is>
-          <t>PRD8-3·화면설계서2.5</t>
+          <t>PRD10-1·화면설계서2.4</t>
         </is>
       </c>
       <c r="J75" s="3" t="inlineStr">
         <is>
-          <t>로컬스토리지 저장/재사용 확인</t>
+          <t>Legend 항목 승률 미노출 확인</t>
         </is>
       </c>
       <c r="K75" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: localStorage mock 기준 최근 계정 목록 추가/조회/전환 테스트, 폼 검증 에러 메시지 테스트</t>
+          <t>Vitest+RTL(필수·정책): is_legend_related=true 카드에 '승률 표시 안함' 텍스트만 렌더링되고 숫자가 DOM에 없는지 확인</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>FE-08</t>
+          <t>FE-07</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
@@ -4808,17 +4808,17 @@
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>분석리포트</t>
+          <t>사후패인분석</t>
         </is>
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>분석 리포트 상세 페이지 구현</t>
+          <t>사후 패인 분석 페이지 구현</t>
         </is>
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>코칭요약/매칭조합카드/등수변화그래프/아이템타임라인</t>
+          <t>Riot ID 폼/최근계정목록(localStorage)/전적불러오기 버튼/진행상태</t>
         </is>
       </c>
       <c r="G76" s="4" t="inlineStr">
@@ -4828,29 +4828,29 @@
       </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
-          <t>API-13,FE-02</t>
+          <t>FE-02,API-11,API-12</t>
         </is>
       </c>
       <c r="I76" s="3" t="inlineStr">
         <is>
-          <t>PRD8-3·화면설계서2.6</t>
+          <t>PRD8-3·화면설계서2.5</t>
         </is>
       </c>
       <c r="J76" s="3" t="inlineStr">
         <is>
-          <t>그래프/타임라인 렌더링 확인</t>
+          <t>로컬스토리지 저장/재사용 확인</t>
         </is>
       </c>
       <c r="K76" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: 그래프/타임라인 mock 데이터 렌더링, opponent-info 마스킹 텍스트 렌더링 확인</t>
+          <t>Vitest+RTL: localStorage mock 기준 최근 계정 목록 추가/조회/전환 테스트, 폼 검증 에러 메시지 테스트</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>FE-09</t>
+          <t>FE-08</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
@@ -4865,17 +4865,17 @@
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>챗봇위젯</t>
+          <t>분석리포트</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>챗봇 위젯 전역 컴포넌트 구현</t>
+          <t>분석 리포트 상세 페이지 구현</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>collapsed/expanded, SSE 연동, 모바일 바텀시트 전환, 후속질문칩</t>
+          <t>코칭요약/매칭조합카드/등수변화그래프/아이템타임라인</t>
         </is>
       </c>
       <c r="G77" s="4" t="inlineStr">
@@ -4885,29 +4885,29 @@
       </c>
       <c r="H77" s="3" t="inlineStr">
         <is>
-          <t>FE-01,API-09,CHAT-05</t>
+          <t>API-13,FE-02</t>
         </is>
       </c>
       <c r="I77" s="3" t="inlineStr">
         <is>
-          <t>PRD7-4·화면설계서2.7·디자인가이드6.6</t>
+          <t>PRD8-3·화면설계서2.6</t>
         </is>
       </c>
       <c r="J77" s="3" t="inlineStr">
         <is>
-          <t>전 페이지 삽입 및 반응형 동작 확인</t>
+          <t>그래프/타임라인 렌더링 확인</t>
         </is>
       </c>
       <c r="K77" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: collapsed/expanded 상태 전환, 모바일 바텀시트 전환, mock SSE 스트림 렌더링 테스트</t>
+          <t>Vitest+RTL: 그래프/타임라인 mock 데이터 렌더링, opponent-info 마스킹 텍스트 렌더링 확인</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>FE-10</t>
+          <t>FE-09</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
@@ -4922,49 +4922,49 @@
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>챗봇위젯</t>
         </is>
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>이미지 최적화 및 반응형 sizes 적용</t>
+          <t>챗봇 위젯 전역 컴포넌트 구현</t>
         </is>
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>Next Image 컴포넌트, 브레이크포인트별 해상도 서빙</t>
+          <t>collapsed/expanded, SSE 연동, 모바일 바텀시트 전환, 후속질문칩</t>
         </is>
       </c>
       <c r="G78" s="4" t="inlineStr">
         <is>
-          <t>권장</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
-          <t>FE-03,FE-04,FE-05,FE-06,FE-07,FE-08</t>
+          <t>FE-01,API-09,CHAT-05</t>
         </is>
       </c>
       <c r="I78" s="3" t="inlineStr">
         <is>
-          <t>PRD7-4·설계서4.1.1</t>
+          <t>PRD7-4·화면설계서2.7·디자인가이드6.6</t>
         </is>
       </c>
       <c r="J78" s="3" t="inlineStr">
         <is>
-          <t>모바일 이미지 로딩 성능 확인</t>
+          <t>전 페이지 삽입 및 반응형 동작 확인</t>
         </is>
       </c>
       <c r="K78" s="3" t="inlineStr">
         <is>
-          <t>해당 없음 — Lighthouse 모바일 성능 점수로 갈음(수동 측정)</t>
+          <t>Vitest+RTL: collapsed/expanded 상태 전환, 모바일 바텀시트 전환, mock SSE 스트림 렌더링 테스트</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>FE-11</t>
+          <t>FE-10</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
@@ -4984,44 +4984,44 @@
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>필터 UI 반응형 공용 컴포넌트 구현</t>
+          <t>이미지 최적화 및 반응형 sizes 적용</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>데스크톱/태블릿 Dropdown, 모바일 BottomSheet 공용 컴포넌트</t>
+          <t>Next Image 컴포넌트, 브레이크포인트별 해상도 서빙</t>
         </is>
       </c>
       <c r="G79" s="4" t="inlineStr">
         <is>
-          <t>필수</t>
+          <t>권장</t>
         </is>
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
-          <t>FE-01</t>
+          <t>FE-03,FE-04,FE-05,FE-06,FE-07,FE-08</t>
         </is>
       </c>
       <c r="I79" s="3" t="inlineStr">
         <is>
-          <t>디자인가이드6.2</t>
+          <t>PRD7-4·설계서4.1.1</t>
         </is>
       </c>
       <c r="J79" s="3" t="inlineStr">
         <is>
-          <t>3개 화면(티어리스트/아이템빌드/증강체)에서 재사용 확인</t>
+          <t>모바일 이미지 로딩 성능 확인</t>
         </is>
       </c>
       <c r="K79" s="3" t="inlineStr">
         <is>
-          <t>Vitest+RTL: 동일 필터 상태를 Dropdown/BottomSheet 두 컴포넌트가 공유하는지 상태 동기화 테스트</t>
+          <t>해당 없음 — Lighthouse 모바일 성능 점수로 갈음(수동 측정)</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>FE-12</t>
+          <t>FE-11</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
@@ -5036,17 +5036,17 @@
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>KPI 대시보드(비공개)</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>KPI 대시보드 페이지 구현(비공개)</t>
+          <t>필터 UI 반응형 공용 컴포넌트 구현</t>
         </is>
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>/kpi 페이지 — 비밀번호 입력 폼(미인증 시) + 5개 지표 카드/차트(최신성/근거율/전환율/이용률/응답지연). GNB·모바일 드로어에는 노출하지 않음(URL 직접 접근 전용)</t>
+          <t>데스크톱/태블릿 Dropdown, 모바일 BottomSheet 공용 컴포넌트</t>
         </is>
       </c>
       <c r="G80" s="4" t="inlineStr">
@@ -5056,29 +5056,29 @@
       </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
-          <t>KPI-01</t>
+          <t>FE-01</t>
         </is>
       </c>
       <c r="I80" s="3" t="inlineStr">
         <is>
-          <t>IA v1.2 4.7절</t>
+          <t>디자인가이드6.2</t>
         </is>
       </c>
       <c r="J80" s="3" t="inlineStr">
         <is>
-          <t>비밀번호 게이트 통과 후 5개 지표 정상 렌더링 확인, 오답 시 게이트 재노출 확인</t>
+          <t>3개 화면(티어리스트/아이템빌드/증강체)에서 재사용 확인</t>
         </is>
       </c>
       <c r="K80" s="3" t="inlineStr">
         <is>
-          <t>Vitest: 비밀번호 게이트 컴포넌트 성공/실패 케이스, 지표 카드 렌더링 테스트</t>
+          <t>Vitest+RTL: 동일 필터 상태를 Dropdown/BottomSheet 두 컴포넌트가 공유하는지 상태 동기화 테스트</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>FE-13</t>
+          <t>FE-12</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
@@ -5093,49 +5093,49 @@
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>티어리스트</t>
+          <t>KPI 대시보드(비공개)</t>
         </is>
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>티어리스트 카드 챔피언 이미지 표시</t>
+          <t>KPI 대시보드 페이지 구현(비공개)</t>
         </is>
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>CompCard의 캐리 챔피언 점(●) placeholder를 Community Dragon 실제 챔피언 아이콘 이미지로 교체. champions 테이블에 square_icon_url 컬럼 추가(배치, Community Dragon squareIcon .tex 경로를 raw.communitydragon.org PNG URL로 변환), GET /catalog/tierlist 응답(CompSummary)에 캐리 챔피언 이름·이미지 URL 포함하도록 확장(API-02), CompCard에 next/image로 렌더링(이미지 없으면 기존 placeholder 폴백).</t>
+          <t>/kpi 페이지 — 비밀번호 입력 폼(미인증 시) + 5개 지표 카드/차트(최신성/근거율/전환율/이용률/응답지연). GNB·모바일 드로어에는 노출하지 않음(URL 직접 접근 전용)</t>
         </is>
       </c>
       <c r="G81" s="4" t="inlineStr">
         <is>
-          <t>권장</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
-          <t>FE-03</t>
+          <t>KPI-01</t>
         </is>
       </c>
       <c r="I81" s="3" t="inlineStr">
         <is>
-          <t>PM 요청 2026-08-05, Community Dragon squareIcon 필드 실호출로 URL 변환 가능 확인</t>
+          <t>IA v1.2 4.7절</t>
         </is>
       </c>
       <c r="J81" s="3" t="inlineStr">
         <is>
-          <t>티어리스트 카드에 캐리 챔피언 실제 이미지가 표시됨(이미지 URL 없으면 기존 placeholder로 폴백)</t>
+          <t>비밀번호 게이트 통과 후 5개 지표 정상 렌더링 확인, 오답 시 게이트 재노출 확인</t>
         </is>
       </c>
       <c r="K81" s="3" t="inlineStr">
         <is>
-          <t>pytest(batch): squareIcon .tex 경로 -&gt; PNG URL 변환 함수 단위 테스트 / pytest(backend): GET /catalog/tierlist 응답에 캐리 챔피언 이름·이미지 URL 포함 확인 / Vitest+RTL: CompCard가 이미지 URL 있으면 이미지, 없으면 placeholder 렌더링 확인</t>
+          <t>Vitest: 비밀번호 게이트 컴포넌트 성공/실패 케이스, 지표 카드 렌더링 테스트</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>FE-14</t>
+          <t>FE-13</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
@@ -5150,17 +5150,17 @@
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>조합상세</t>
+          <t>티어리스트</t>
         </is>
       </c>
       <c r="E82" s="3" t="inlineStr">
         <is>
-          <t>조합 상세 헥스 배치도 실좌표 반영</t>
+          <t>티어리스트 카드 챔피언 이미지 표시</t>
         </is>
       </c>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>HexBoard의 is_carry 기반 전열/후열 휴리스틱 배치를 op.gg tft_list_meta_decks 응답의 units[].cell.{x,y}(실제 랭커 배치 좌표, 4행x7열, 2026-08-06 실호출로 확인)로 교체. comp_champions 테이블에 cell_x/cell_y 컬럼 추가(배치, comp_champion_rows()에서 unit.cell 추출), GET /comps/{comp_id} 응답(ChampionInComp)에 cell_x/cell_y 포함(API-03), HexBoard가 좌표 있으면 실제 4x7 헥스 그리드(오프셋 스태거)로 렌더링하고 좌표 없는 기존 데이터는 기존 휴리스틱 배치로 폴백.</t>
+          <t>CompCard의 캐리 챔피언 점(●) placeholder를 Community Dragon 실제 챔피언 아이콘 이미지로 교체. champions 테이블에 square_icon_url 컬럼 추가(배치, Community Dragon squareIcon .tex 경로를 raw.communitydragon.org PNG URL로 변환), GET /catalog/tierlist 응답(CompSummary)에 캐리 챔피언 이름·이미지 URL 포함하도록 확장(API-02), CompCard에 next/image로 렌더링(이미지 없으면 기존 placeholder 폴백).</t>
         </is>
       </c>
       <c r="G82" s="4" t="inlineStr">
@@ -5170,29 +5170,29 @@
       </c>
       <c r="H82" s="3" t="inlineStr">
         <is>
-          <t>FE-04</t>
+          <t>FE-03</t>
         </is>
       </c>
       <c r="I82" s="3" t="inlineStr">
         <is>
-          <t>PM 요청 2026-08-06, op.gg tft_list_meta_decks 실호출로 units[].cell 필드(x:1-7, y:1-4) 확인</t>
+          <t>PM 요청 2026-08-05, Community Dragon squareIcon 필드 실호출로 URL 변환 가능 확인</t>
         </is>
       </c>
       <c r="J82" s="3" t="inlineStr">
         <is>
-          <t>조합 상세 페이지 태블릿/데스크톱에서 실제 좌표 기반 헥스 배치도가 표시됨(좌표 없는 구 데이터는 기존 휴리스틱 폴백 유지, 콘솔 에러 0건)</t>
+          <t>티어리스트 카드에 캐리 챔피언 실제 이미지가 표시됨(이미지 URL 없으면 기존 placeholder로 폴백)</t>
         </is>
       </c>
       <c r="K82" s="3" t="inlineStr">
         <is>
-          <t>pytest(batch): comp_champion_rows()가 unit.cell에서 cell_x/cell_y를 추출하는 단위 테스트 / pytest(backend): GET /comps/{comp_id} 응답에 cell_x/cell_y 포함 및 null 폴백 확인 / Vitest+RTL: HexBoard가 좌표 있으면 실좌표 그리드, 없으면(cell_x/y null) 기존 휴리스틱 렌더링 확인</t>
+          <t>pytest(batch): squareIcon .tex 경로 -&gt; PNG URL 변환 함수 단위 테스트 / pytest(backend): GET /catalog/tierlist 응답에 캐리 챔피언 이름·이미지 URL 포함 확인 / Vitest+RTL: CompCard가 이미지 URL 있으면 이미지, 없으면 placeholder 렌더링 확인</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>KPI-01</t>
+          <t>FE-14</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
@@ -5202,54 +5202,54 @@
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>KPI모니터링</t>
+          <t>프론트엔드</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>조합상세</t>
         </is>
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>KPI 대시보드 백엔드 API 구현(자체, Metabase 대체)</t>
+          <t>조합 상세 헥스 배치도 실좌표 반영</t>
         </is>
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>5개 지표(최신성/근거율/전환율/이용률/응답지연) 집계 GET /kpi/summary 구현 + POST /kpi/auth 비밀번호 게이트(환경변수 KPI_DASHBOARD_PASSWORD 대조, 서명 토큰 발급) 구현. Metabase 대신 자체 페이지(FE-12)로 제공 (PM 결정 2026-08-03)</t>
+          <t>HexBoard의 is_carry 기반 전열/후열 휴리스틱 배치를 op.gg tft_list_meta_decks 응답의 units[].cell.{x,y}(실제 랭커 배치 좌표, 4행x7열, 2026-08-06 실호출로 확인)로 교체. comp_champions 테이블에 cell_x/cell_y 컬럼 추가(배치, comp_champion_rows()에서 unit.cell 추출), GET /comps/{comp_id} 응답(ChampionInComp)에 cell_x/cell_y 포함(API-03), HexBoard가 좌표 있으면 실제 4x7 헥스 그리드(오프셋 스태거)로 렌더링하고 좌표 없는 기존 데이터는 기존 휴리스틱 배치로 폴백.</t>
         </is>
       </c>
       <c r="G83" s="4" t="inlineStr">
         <is>
-          <t>필수</t>
+          <t>권장</t>
         </is>
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>DATA-03</t>
+          <t>FE-04</t>
         </is>
       </c>
       <c r="I83" s="3" t="inlineStr">
         <is>
-          <t>PRD 3-3 / IA v1.2 4.7절 (자체구현 결정 2026-08-03)</t>
+          <t>PM 요청 2026-08-06, op.gg tft_list_meta_decks 실호출로 units[].cell 필드(x:1-7, y:1-4) 확인</t>
         </is>
       </c>
       <c r="J83" s="3" t="inlineStr">
         <is>
-          <t>5개 지표 API 정상 응답 확인, 비밀번호 게이트 통과/실패 동작 확인</t>
+          <t>조합 상세 페이지 태블릿/데스크톱에서 실제 좌표 기반 헥스 배치도가 표시됨(좌표 없는 구 데이터는 기존 휴리스틱 폴백 유지, 콘솔 에러 0건)</t>
         </is>
       </c>
       <c r="K83" s="3" t="inlineStr">
         <is>
-          <t>pytest: 비밀번호 게이트 성공/실패 케이스, mock 로그 데이터로 5개 지표 집계 쿼리 결과 검증</t>
+          <t>pytest(batch): comp_champion_rows()가 unit.cell에서 cell_x/cell_y를 추출하는 단위 테스트 / pytest(backend): GET /comps/{comp_id} 응답에 cell_x/cell_y 포함 및 null 폴백 확인 / Vitest+RTL: HexBoard가 좌표 있으면 실좌표 그리드, 없으면(cell_x/y null) 기존 휴리스틱 렌더링 확인</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>KPI-02</t>
+          <t>KPI-01</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
@@ -5269,12 +5269,12 @@
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>RAGAS 주간 배치 평가 파이프라인 구현</t>
+          <t>KPI 대시보드 백엔드 API 구현(자체, Metabase 대체)</t>
         </is>
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>GitHub Actions 주간 배치로 Faithfulness/Answer Relevancy 산출, ragas_eval_results 적재</t>
+          <t>5개 지표(최신성/근거율/전환율/이용률/응답지연) 집계 GET /kpi/summary 구현 + POST /kpi/auth 비밀번호 게이트(환경변수 KPI_DASHBOARD_PASSWORD 대조, 서명 토큰 발급) 구현. Metabase 대신 자체 페이지(FE-12)로 제공 (PM 결정 2026-08-03)</t>
         </is>
       </c>
       <c r="G84" s="4" t="inlineStr">
@@ -5284,143 +5284,143 @@
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
-          <t>CHAT-09,SET-08</t>
+          <t>DATA-03</t>
         </is>
       </c>
       <c r="I84" s="3" t="inlineStr">
         <is>
-          <t>PRD3-3·설계서4.7</t>
+          <t>PRD 3-3 / IA v1.2 4.7절 (자체구현 결정 2026-08-03)</t>
         </is>
       </c>
       <c r="J84" s="3" t="inlineStr">
         <is>
-          <t>배치 실행 후 결과 적재 확인</t>
+          <t>5개 지표 API 정상 응답 확인, 비밀번호 게이트 통과/실패 동작 확인</t>
         </is>
       </c>
       <c r="K84" s="3" t="inlineStr">
         <is>
-          <t>pytest: mock 질의-답변 샘플로 RAGAS 스코어러 호출 및 ragas_eval_results 적재 필드 확인</t>
+          <t>pytest: 비밀번호 게이트 성공/실패 케이스, mock 로그 데이터로 5개 지표 집계 쿼리 결과 검증</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
+          <t>KPI-02</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>KPI모니터링</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>공통</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>RAGAS 주간 배치 평가 파이프라인 구현</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>GitHub Actions 주간 배치로 Faithfulness/Answer Relevancy 산출, ragas_eval_results 적재</t>
+        </is>
+      </c>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>필수</t>
+        </is>
+      </c>
+      <c r="H85" s="3" t="inlineStr">
+        <is>
+          <t>CHAT-09,SET-08</t>
+        </is>
+      </c>
+      <c r="I85" s="3" t="inlineStr">
+        <is>
+          <t>PRD3-3·설계서4.7</t>
+        </is>
+      </c>
+      <c r="J85" s="3" t="inlineStr">
+        <is>
+          <t>배치 실행 후 결과 적재 확인</t>
+        </is>
+      </c>
+      <c r="K85" s="3" t="inlineStr">
+        <is>
+          <t>pytest: mock 질의-답변 샘플로 RAGAS 스코어러 호출 및 ragas_eval_results 적재 필드 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
           <t>KPI-03</t>
         </is>
       </c>
-      <c r="B85" s="4" t="inlineStr">
-        <is>
-          <t>코딩</t>
-        </is>
-      </c>
-      <c r="C85" s="4" t="inlineStr">
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="inlineStr">
         <is>
           <t>KPI모니터링</t>
         </is>
       </c>
-      <c r="D85" s="3" t="inlineStr">
+      <c r="D86" s="3" t="inlineStr">
         <is>
           <t>공통</t>
         </is>
       </c>
-      <c r="E85" s="3" t="inlineStr">
+      <c r="E86" s="3" t="inlineStr">
         <is>
           <t>목표 미달 알림 로직 구현</t>
         </is>
       </c>
-      <c r="F85" s="3" t="inlineStr">
+      <c r="F86" s="3" t="inlineStr">
         <is>
           <t>2주 연속 목표 미달 감지 시 알림 발송</t>
         </is>
       </c>
-      <c r="G85" s="4" t="inlineStr">
+      <c r="G86" s="4" t="inlineStr">
         <is>
           <t>권장</t>
         </is>
       </c>
-      <c r="H85" s="3" t="inlineStr">
+      <c r="H86" s="3" t="inlineStr">
         <is>
           <t>KPI-01</t>
         </is>
       </c>
-      <c r="I85" s="3" t="inlineStr">
+      <c r="I86" s="3" t="inlineStr">
         <is>
           <t>PRD3-3</t>
         </is>
       </c>
-      <c r="J85" s="3" t="inlineStr">
+      <c r="J86" s="3" t="inlineStr">
         <is>
           <t>알림 트리거 테스트 통과</t>
         </is>
       </c>
-      <c r="K85" s="3" t="inlineStr">
+      <c r="K86" s="3" t="inlineStr">
         <is>
           <t>pytest: 2주 연속 미달 mock 데이터 주입 시 알림 함수 호출 확인</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="5" t="inlineStr">
-        <is>
-          <t>TEST-00</t>
-        </is>
-      </c>
-      <c r="B86" s="5" t="inlineStr">
-        <is>
-          <t>테스트</t>
-        </is>
-      </c>
-      <c r="C86" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D86" s="3" t="inlineStr">
-        <is>
-          <t>공통(정책·로직 크리티컬 TASK)</t>
-        </is>
-      </c>
-      <c r="E86" s="3" t="inlineStr">
-        <is>
-          <t>핵심 정책/로직 테스트 시나리오 사전 정의</t>
-        </is>
-      </c>
-      <c r="F86" s="3" t="inlineStr">
-        <is>
-          <t>API-05, CHAT-04, CHAT-06, PGA-04~09, DATA-13 등 정책 준수·크리티컬 계산 로직이 걸린 TASK에 한해, 코딩 착수 전 입력값·기대출력·경계값을 포함한 테스트 시나리오를 문서화하고 PM과 합의한다. 해당 TASK의 구현자는 이 문서를 기준으로 단위 테스트를 먼저 작성한 뒤 구현한다</t>
-        </is>
-      </c>
-      <c r="G86" s="5" t="inlineStr">
-        <is>
-          <t>필수</t>
-        </is>
-      </c>
-      <c r="H86" s="3" t="inlineStr">
-        <is>
-          <t>SET-01</t>
-        </is>
-      </c>
-      <c r="I86" s="3" t="inlineStr">
-        <is>
-          <t>요구사항정의서 NFR-SEC·FR-PGA, 설계서 4.4.2·4.4.3·4.5.1·4.5.2</t>
-        </is>
-      </c>
-      <c r="J86" s="3" t="inlineStr">
-        <is>
-          <t>/docs/test-scenarios.md에 대상 TASK별 시나리오 표 작성 및 PM 승인 완료</t>
-        </is>
-      </c>
-      <c r="K86" s="3" t="inlineStr">
-        <is>
-          <t>해당 TASK 자체가 산출물 — /docs/test-scenarios.md 표 작성</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>TEST-01</t>
+          <t>TEST-00</t>
         </is>
       </c>
       <c r="B87" s="5" t="inlineStr">
@@ -5435,17 +5435,17 @@
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>공통(정책·로직 크리티컬 TASK)</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>DB 스키마/마이그레이션 검증</t>
+          <t>핵심 정책/로직 테스트 시나리오 사전 정의</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>전체 테이블·인덱스·제약조건 검증</t>
+          <t>API-05, CHAT-04, CHAT-06, PGA-04~09, DATA-13 등 정책 준수·크리티컬 계산 로직이 걸린 TASK에 한해, 코딩 착수 전 입력값·기대출력·경계값을 포함한 테스트 시나리오를 문서화하고 PM과 합의한다. 해당 TASK의 구현자는 이 문서를 기준으로 단위 테스트를 먼저 작성한 뒤 구현한다</t>
         </is>
       </c>
       <c r="G87" s="5" t="inlineStr">
@@ -5455,29 +5455,29 @@
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
-          <t>DATA-01,DATA-02,DATA-03,DATA-04</t>
+          <t>SET-01</t>
         </is>
       </c>
       <c r="I87" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>요구사항정의서 NFR-SEC·FR-PGA, 설계서 4.4.2·4.4.3·4.5.1·4.5.2</t>
         </is>
       </c>
       <c r="J87" s="3" t="inlineStr">
         <is>
-          <t>마이그레이션 재실행 무결성 확인</t>
+          <t>/docs/test-scenarios.md에 대상 TASK별 시나리오 표 작성 및 PM 승인 완료</t>
         </is>
       </c>
       <c r="K87" s="3" t="inlineStr">
         <is>
-          <t>해당 TASK 자체가 테스트 작성/실행 TASK의 산출물</t>
+          <t>해당 TASK 자체가 산출물 — /docs/test-scenarios.md 표 작성</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>TEST-02</t>
+          <t>TEST-01</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
@@ -5492,17 +5492,17 @@
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>티어리스트~증강체정보</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>catalog API 단위/통합 테스트</t>
+          <t>DB 스키마/마이그레이션 검증</t>
         </is>
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>API-02~06 엔드포인트 테스트 코드 작성 및 실행</t>
+          <t>전체 테이블·인덱스·제약조건 검증</t>
         </is>
       </c>
       <c r="G88" s="5" t="inlineStr">
@@ -5512,7 +5512,7 @@
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>API-02,API-03,API-04,API-05,API-06</t>
+          <t>DATA-01,DATA-02,DATA-03,DATA-04</t>
         </is>
       </c>
       <c r="I88" s="3" t="inlineStr">
@@ -5522,7 +5522,7 @@
       </c>
       <c r="J88" s="3" t="inlineStr">
         <is>
-          <t>전체 테스트 통과</t>
+          <t>마이그레이션 재실행 무결성 확인</t>
         </is>
       </c>
       <c r="K88" s="3" t="inlineStr">
@@ -5534,7 +5534,7 @@
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>TEST-03</t>
+          <t>TEST-02</t>
         </is>
       </c>
       <c r="B89" s="5" t="inlineStr">
@@ -5549,17 +5549,17 @@
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>챗봇위젯</t>
+          <t>티어리스트~증강체정보</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>chat API 및 RAG 파이프라인 테스트</t>
+          <t>catalog API 단위/통합 테스트</t>
         </is>
       </c>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>의도분류/검색/생성/후처리/캐싱 테스트</t>
+          <t>API-02~06 엔드포인트 테스트 코드 작성 및 실행</t>
         </is>
       </c>
       <c r="G89" s="5" t="inlineStr">
@@ -5569,7 +5569,7 @@
       </c>
       <c r="H89" s="3" t="inlineStr">
         <is>
-          <t>CHAT-01,CHAT-02,CHAT-03,CHAT-04,CHAT-05,CHAT-06,CHAT-07,CHAT-08,CHAT-09</t>
+          <t>API-02,API-03,API-04,API-05,API-06</t>
         </is>
       </c>
       <c r="I89" s="3" t="inlineStr">
@@ -5579,7 +5579,7 @@
       </c>
       <c r="J89" s="3" t="inlineStr">
         <is>
-          <t>전체 통과, 근거율 샘플 검증</t>
+          <t>전체 테스트 통과</t>
         </is>
       </c>
       <c r="K89" s="3" t="inlineStr">
@@ -5591,7 +5591,7 @@
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>TEST-04</t>
+          <t>TEST-03</t>
         </is>
       </c>
       <c r="B90" s="5" t="inlineStr">
@@ -5606,17 +5606,17 @@
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석·분석리포트</t>
+          <t>챗봇위젯</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>analysis API 및 스코어링 로직 테스트</t>
+          <t>chat API 및 RAG 파이프라인 테스트</t>
         </is>
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>PUUID변환/매치조회/3개지표계산/코칭생성 테스트</t>
+          <t>의도분류/검색/생성/후처리/캐싱 테스트</t>
         </is>
       </c>
       <c r="G90" s="5" t="inlineStr">
@@ -5626,7 +5626,7 @@
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>PGA-01,PGA-02,PGA-03,PGA-04,PGA-05,PGA-06,PGA-07,PGA-08,PGA-09,PGA-10</t>
+          <t>CHAT-01,CHAT-02,CHAT-03,CHAT-04,CHAT-05,CHAT-06,CHAT-07,CHAT-08,CHAT-09</t>
         </is>
       </c>
       <c r="I90" s="3" t="inlineStr">
@@ -5636,7 +5636,7 @@
       </c>
       <c r="J90" s="3" t="inlineStr">
         <is>
-          <t>전체 통과</t>
+          <t>전체 통과, 근거율 샘플 검증</t>
         </is>
       </c>
       <c r="K90" s="3" t="inlineStr">
@@ -5648,7 +5648,7 @@
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>TEST-05</t>
+          <t>TEST-04</t>
         </is>
       </c>
       <c r="B91" s="5" t="inlineStr">
@@ -5663,17 +5663,17 @@
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>사후패인분석·분석리포트</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>배치 파이프라인 통합 테스트</t>
+          <t>analysis API 및 스코어링 로직 테스트</t>
         </is>
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>패치감지→수집→정규화→임베딩→원자적전환 end-to-end 테스트</t>
+          <t>PUUID변환/매치조회/3개지표계산/코칭생성 테스트</t>
         </is>
       </c>
       <c r="G91" s="5" t="inlineStr">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="H91" s="3" t="inlineStr">
         <is>
-          <t>DATA-05,DATA-08,DATA-09,DATA-10,DATA-11,DATA-12,DATA-13,DATA-14,DATA-15</t>
+          <t>PGA-01,PGA-02,PGA-03,PGA-04,PGA-05,PGA-06,PGA-07,PGA-08,PGA-09,PGA-10</t>
         </is>
       </c>
       <c r="I91" s="3" t="inlineStr">
@@ -5693,7 +5693,7 @@
       </c>
       <c r="J91" s="3" t="inlineStr">
         <is>
-          <t>정상/중간실패 시나리오 모두 검증</t>
+          <t>전체 통과</t>
         </is>
       </c>
       <c r="K91" s="3" t="inlineStr">
@@ -5705,7 +5705,7 @@
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
         <is>
-          <t>TEST-06</t>
+          <t>TEST-05</t>
         </is>
       </c>
       <c r="B92" s="5" t="inlineStr">
@@ -5720,17 +5720,17 @@
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>챗봇위젯</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>챗봇 정책 준수 테스트</t>
+          <t>배치 파이프라인 통합 테스트</t>
         </is>
       </c>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>Legend 승률 비노출·프롬프트 인젝션 방어·범위밖 질문 안내 검증</t>
+          <t>패치감지→수집→정규화→임베딩→원자적전환 end-to-end 테스트</t>
         </is>
       </c>
       <c r="G92" s="5" t="inlineStr">
@@ -5740,17 +5740,17 @@
       </c>
       <c r="H92" s="3" t="inlineStr">
         <is>
-          <t>CHAT-04,CHAT-06</t>
+          <t>DATA-05,DATA-08,DATA-09,DATA-10,DATA-11,DATA-12,DATA-13,DATA-14,DATA-15</t>
         </is>
       </c>
       <c r="I92" s="3" t="inlineStr">
         <is>
-          <t>PRD10-1·12장</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J92" s="3" t="inlineStr">
         <is>
-          <t>정책 위반 케이스 0건</t>
+          <t>정상/중간실패 시나리오 모두 검증</t>
         </is>
       </c>
       <c r="K92" s="3" t="inlineStr">
@@ -5762,7 +5762,7 @@
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>TEST-07</t>
+          <t>TEST-06</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
@@ -5777,17 +5777,17 @@
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>사후패인분석·분석리포트</t>
+          <t>챗봇위젯</t>
         </is>
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>프라이버시 마스킹 테스트</t>
+          <t>챗봇 정책 준수 테스트</t>
         </is>
       </c>
       <c r="F93" s="3" t="inlineStr">
         <is>
-          <t>상대 닉네임 마스킹 누락 케이스 점검</t>
+          <t>Legend 승률 비노출·프롬프트 인젝션 방어·범위밖 질문 안내 검증</t>
         </is>
       </c>
       <c r="G93" s="5" t="inlineStr">
@@ -5797,17 +5797,17 @@
       </c>
       <c r="H93" s="3" t="inlineStr">
         <is>
-          <t>PGA-09</t>
+          <t>CHAT-04,CHAT-06</t>
         </is>
       </c>
       <c r="I93" s="3" t="inlineStr">
         <is>
-          <t>PRD7-3·12장</t>
+          <t>PRD10-1·12장</t>
         </is>
       </c>
       <c r="J93" s="3" t="inlineStr">
         <is>
-          <t>마스킹 누락 0건</t>
+          <t>정책 위반 케이스 0건</t>
         </is>
       </c>
       <c r="K93" s="3" t="inlineStr">
@@ -5819,7 +5819,7 @@
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>TEST-08</t>
+          <t>TEST-07</t>
         </is>
       </c>
       <c r="B94" s="5" t="inlineStr">
@@ -5834,17 +5834,17 @@
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>전체 7화면</t>
+          <t>사후패인분석·분석리포트</t>
         </is>
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>프론트엔드 E2E 테스트(Playwright)</t>
+          <t>프라이버시 마스킹 테스트</t>
         </is>
       </c>
       <c r="F94" s="3" t="inlineStr">
         <is>
-          <t>PRD 8-1/8-2/8-3 사용자 플로우 기준 시나리오 작성</t>
+          <t>상대 닉네임 마스킹 누락 케이스 점검</t>
         </is>
       </c>
       <c r="G94" s="5" t="inlineStr">
@@ -5854,17 +5854,17 @@
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>FE-03,FE-04,FE-05,FE-06,FE-07,FE-08,FE-09</t>
+          <t>PGA-09</t>
         </is>
       </c>
       <c r="I94" s="3" t="inlineStr">
         <is>
-          <t>PRD8장</t>
+          <t>PRD7-3·12장</t>
         </is>
       </c>
       <c r="J94" s="3" t="inlineStr">
         <is>
-          <t>전체 시나리오 통과</t>
+          <t>마스킹 누락 0건</t>
         </is>
       </c>
       <c r="K94" s="3" t="inlineStr">
@@ -5876,7 +5876,7 @@
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>TEST-09</t>
+          <t>TEST-08</t>
         </is>
       </c>
       <c r="B95" s="5" t="inlineStr">
@@ -5896,12 +5896,12 @@
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>반응형 크로스브라우저 테스트</t>
+          <t>프론트엔드 E2E 테스트(Playwright)</t>
         </is>
       </c>
       <c r="F95" s="3" t="inlineStr">
         <is>
-          <t>iOS Safari/Android Chrome/Desktop Chrome 3개 브레이크포인트 검증</t>
+          <t>PRD 8-1/8-2/8-3 사용자 플로우 기준 시나리오 작성</t>
         </is>
       </c>
       <c r="G95" s="5" t="inlineStr">
@@ -5916,12 +5916,12 @@
       </c>
       <c r="I95" s="3" t="inlineStr">
         <is>
-          <t>PRD12장(QA리소스제약)</t>
+          <t>PRD8장</t>
         </is>
       </c>
       <c r="J95" s="3" t="inlineStr">
         <is>
-          <t>주요 화면 시각 회귀 없음 확인</t>
+          <t>전체 시나리오 통과</t>
         </is>
       </c>
       <c r="K95" s="3" t="inlineStr">
@@ -5933,121 +5933,121 @@
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
         <is>
+          <t>TEST-09</t>
+        </is>
+      </c>
+      <c r="B96" s="5" t="inlineStr">
+        <is>
+          <t>테스트</t>
+        </is>
+      </c>
+      <c r="C96" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>전체 7화면</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>반응형 크로스브라우저 테스트</t>
+        </is>
+      </c>
+      <c r="F96" s="3" t="inlineStr">
+        <is>
+          <t>iOS Safari/Android Chrome/Desktop Chrome 3개 브레이크포인트 검증</t>
+        </is>
+      </c>
+      <c r="G96" s="5" t="inlineStr">
+        <is>
+          <t>필수</t>
+        </is>
+      </c>
+      <c r="H96" s="3" t="inlineStr">
+        <is>
+          <t>FE-03,FE-04,FE-05,FE-06,FE-07,FE-08,FE-09</t>
+        </is>
+      </c>
+      <c r="I96" s="3" t="inlineStr">
+        <is>
+          <t>PRD12장(QA리소스제약)</t>
+        </is>
+      </c>
+      <c r="J96" s="3" t="inlineStr">
+        <is>
+          <t>주요 화면 시각 회귀 없음 확인</t>
+        </is>
+      </c>
+      <c r="K96" s="3" t="inlineStr">
+        <is>
+          <t>해당 TASK 자체가 테스트 작성/실행 TASK의 산출물</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="5" t="inlineStr">
+        <is>
           <t>TEST-10</t>
         </is>
       </c>
-      <c r="B96" s="5" t="inlineStr">
+      <c r="B97" s="5" t="inlineStr">
         <is>
           <t>테스트</t>
         </is>
       </c>
-      <c r="C96" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D96" s="3" t="inlineStr">
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
         <is>
           <t>공통</t>
         </is>
       </c>
-      <c r="E96" s="3" t="inlineStr">
+      <c r="E97" s="3" t="inlineStr">
         <is>
           <t>Rate Limiting/보안 테스트</t>
         </is>
       </c>
-      <c r="F96" s="3" t="inlineStr">
+      <c r="F97" s="3" t="inlineStr">
         <is>
           <t>요청 한도 초과·비정상 입력 처리 검증</t>
         </is>
       </c>
-      <c r="G96" s="5" t="inlineStr">
+      <c r="G97" s="5" t="inlineStr">
         <is>
           <t>권장</t>
         </is>
       </c>
-      <c r="H96" s="3" t="inlineStr">
+      <c r="H97" s="3" t="inlineStr">
         <is>
           <t>API-07</t>
         </is>
       </c>
-      <c r="I96" s="3" t="inlineStr">
+      <c r="I97" s="3" t="inlineStr">
         <is>
           <t>설계서4.2·6장</t>
         </is>
       </c>
-      <c r="J96" s="3" t="inlineStr">
+      <c r="J97" s="3" t="inlineStr">
         <is>
           <t>429 응답 및 로그 확인</t>
         </is>
       </c>
-      <c r="K96" s="3" t="inlineStr">
+      <c r="K97" s="3" t="inlineStr">
         <is>
           <t>해당 TASK 자체가 테스트 작성/실행 TASK의 산출물</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="6" t="inlineStr">
-        <is>
-          <t>REL-01</t>
-        </is>
-      </c>
-      <c r="B97" s="6" t="inlineStr">
-        <is>
-          <t>배포릴리즈</t>
-        </is>
-      </c>
-      <c r="C97" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D97" s="3" t="inlineStr">
-        <is>
-          <t>전체</t>
-        </is>
-      </c>
-      <c r="E97" s="3" t="inlineStr">
-        <is>
-          <t>스테이징 통합 배포 및 QA</t>
-        </is>
-      </c>
-      <c r="F97" s="3" t="inlineStr">
-        <is>
-          <t>전체 기능 스테이징 환경 배포 후 PM 검수</t>
-        </is>
-      </c>
-      <c r="G97" s="6" t="inlineStr">
-        <is>
-          <t>필수</t>
-        </is>
-      </c>
-      <c r="H97" s="3" t="inlineStr">
-        <is>
-          <t>TEST-01,TEST-02,TEST-03,TEST-04,TEST-05,TEST-06,TEST-07,TEST-08,TEST-09</t>
-        </is>
-      </c>
-      <c r="I97" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J97" s="3" t="inlineStr">
-        <is>
-          <t>PM 승인 획득</t>
-        </is>
-      </c>
-      <c r="K97" s="3" t="inlineStr">
-        <is>
-          <t>TEST-00~10 전체 그린 상태를 배포 전제조건으로 확인</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>REL-02</t>
+          <t>REL-01</t>
         </is>
       </c>
       <c r="B98" s="6" t="inlineStr">
@@ -6067,12 +6067,12 @@
       </c>
       <c r="E98" s="3" t="inlineStr">
         <is>
-          <t>프로덕션 배포</t>
+          <t>스테이징 통합 배포 및 QA</t>
         </is>
       </c>
       <c r="F98" s="3" t="inlineStr">
         <is>
-          <t>Cloudflare Pages+Render 프로덕션 반영, PM 최종 승인 후 커밋/푸시</t>
+          <t>전체 기능 스테이징 환경 배포 후 PM 검수</t>
         </is>
       </c>
       <c r="G98" s="6" t="inlineStr">
@@ -6082,7 +6082,7 @@
       </c>
       <c r="H98" s="3" t="inlineStr">
         <is>
-          <t>REL-01</t>
+          <t>TEST-01,TEST-02,TEST-03,TEST-04,TEST-05,TEST-06,TEST-07,TEST-08,TEST-09</t>
         </is>
       </c>
       <c r="I98" s="3" t="inlineStr">
@@ -6092,19 +6092,19 @@
       </c>
       <c r="J98" s="3" t="inlineStr">
         <is>
-          <t>프로덕션 URL 정상 서비스 확인</t>
+          <t>PM 승인 획득</t>
         </is>
       </c>
       <c r="K98" s="3" t="inlineStr">
         <is>
-          <t>프로덕션 스모크 테스트: 핵심 URL 200 확인, 챗봇 질의 1회 왕복 확인</t>
+          <t>TEST-00~10 전체 그린 상태를 배포 전제조건으로 확인</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="6" t="inlineStr">
         <is>
-          <t>REL-03</t>
+          <t>REL-02</t>
         </is>
       </c>
       <c r="B99" s="6" t="inlineStr">
@@ -6119,17 +6119,17 @@
       </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>전체</t>
         </is>
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>배포 후 모니터링 점검</t>
+          <t>프로덕션 배포</t>
         </is>
       </c>
       <c r="F99" s="3" t="inlineStr">
         <is>
-          <t>콜드스타트 비중·응답지연 p50/p95 확인</t>
+          <t>Cloudflare Pages+Render 프로덕션 반영, PM 최종 승인 후 커밋/푸시</t>
         </is>
       </c>
       <c r="G99" s="6" t="inlineStr">
@@ -6139,29 +6139,29 @@
       </c>
       <c r="H99" s="3" t="inlineStr">
         <is>
-          <t>REL-02,KPI-01</t>
+          <t>REL-01</t>
         </is>
       </c>
       <c r="I99" s="3" t="inlineStr">
         <is>
-          <t>PRD3-3</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J99" s="3" t="inlineStr">
         <is>
-          <t>초기 1주 지표 리뷰 완료</t>
+          <t>프로덕션 URL 정상 서비스 확인</t>
         </is>
       </c>
       <c r="K99" s="3" t="inlineStr">
         <is>
-          <t>해당 없음 — 모니터링 지표 수동 리뷰</t>
+          <t>프로덕션 스모크 테스트: 핵심 URL 200 확인, 챗봇 질의 1회 왕복 확인</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="6" t="inlineStr">
         <is>
-          <t>REL-04</t>
+          <t>REL-03</t>
         </is>
       </c>
       <c r="B100" s="6" t="inlineStr">
@@ -6181,94 +6181,208 @@
       </c>
       <c r="E100" s="3" t="inlineStr">
         <is>
-          <t>1.0 출시 회고 및 KPI 재보정 계획 수립</t>
+          <t>배포 후 모니터링 점검</t>
         </is>
       </c>
       <c r="F100" s="3" t="inlineStr">
         <is>
-          <t>2~4주 실측 데이터 수집 계획 및 재보정 일정 수립</t>
+          <t>콜드스타트 비중·응답지연 p50/p95 확인</t>
         </is>
       </c>
       <c r="G100" s="6" t="inlineStr">
         <is>
-          <t>권장</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="H100" s="3" t="inlineStr">
         <is>
-          <t>REL-03</t>
+          <t>REL-02,KPI-01</t>
         </is>
       </c>
       <c r="I100" s="3" t="inlineStr">
         <is>
-          <t>PRD3-2·3-3</t>
+          <t>PRD3-3</t>
         </is>
       </c>
       <c r="J100" s="3" t="inlineStr">
         <is>
-          <t>재보정 일정 문서화</t>
+          <t>초기 1주 지표 리뷰 완료</t>
         </is>
       </c>
       <c r="K100" s="3" t="inlineStr">
         <is>
-          <t>해당 없음 — 문서화 작업</t>
+          <t>해당 없음 — 모니터링 지표 수동 리뷰</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="6" t="inlineStr">
         <is>
+          <t>REL-04</t>
+        </is>
+      </c>
+      <c r="B101" s="6" t="inlineStr">
+        <is>
+          <t>배포릴리즈</t>
+        </is>
+      </c>
+      <c r="C101" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D101" s="3" t="inlineStr">
+        <is>
+          <t>공통</t>
+        </is>
+      </c>
+      <c r="E101" s="3" t="inlineStr">
+        <is>
+          <t>1.0 출시 회고 및 KPI 재보정 계획 수립</t>
+        </is>
+      </c>
+      <c r="F101" s="3" t="inlineStr">
+        <is>
+          <t>2~4주 실측 데이터 수집 계획 및 재보정 일정 수립</t>
+        </is>
+      </c>
+      <c r="G101" s="6" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H101" s="3" t="inlineStr">
+        <is>
+          <t>REL-03</t>
+        </is>
+      </c>
+      <c r="I101" s="3" t="inlineStr">
+        <is>
+          <t>PRD3-2·3-3</t>
+        </is>
+      </c>
+      <c r="J101" s="3" t="inlineStr">
+        <is>
+          <t>재보정 일정 문서화</t>
+        </is>
+      </c>
+      <c r="K101" s="3" t="inlineStr">
+        <is>
+          <t>해당 없음 — 문서화 작업</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="6" t="inlineStr">
+        <is>
           <t>REL-05</t>
         </is>
       </c>
-      <c r="B101" s="6" t="inlineStr">
+      <c r="B102" s="6" t="inlineStr">
         <is>
           <t>배포릴리즈</t>
         </is>
       </c>
-      <c r="C101" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D101" s="3" t="inlineStr">
+      <c r="C102" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D102" s="3" t="inlineStr">
         <is>
           <t>전체</t>
         </is>
       </c>
-      <c r="E101" s="3" t="inlineStr">
+      <c r="E102" s="3" t="inlineStr">
         <is>
           <t>포트폴리오 공개 전환 준비 체크리스트</t>
         </is>
       </c>
-      <c r="F101" s="3" t="inlineStr">
+      <c r="F102" s="3" t="inlineStr">
         <is>
           <t>저장소를 private에서 public으로 전환하기 전 확인·조치한다: (1) gitleaks 등으로 커밋 히스토리 전체에서 시크릿·API 키 잔존 여부 스캔 (2) 테스트 fixture 전수 조사 — 실제 Riot ID/PUUID/닉네임/매치 데이터가 아닌 합성 데이터로만 구성됐는지 확인, 실데이터가 섞여 있으면 fixture 재작성 후 필요시 git 히스토리 정리 (3) README에 'Riot Games와 무관한 비공식 팬 프로젝트' 디스클레이머 추가 (4) 라이브 배포 URL을 README/공개 자료에 노출할지 결정 (5) 노출하기로 하면 챗봇/전적조회 진입점에 Cloudflare Turnstile 등 경량 봇 방지 적용 검토. 무료 호스팅 비용에는 영향 없음(저장소 공개 여부와 인프라 비용은 무관)</t>
         </is>
       </c>
-      <c r="G101" s="6" t="inlineStr">
+      <c r="G102" s="6" t="inlineStr">
         <is>
           <t>권장</t>
         </is>
       </c>
-      <c r="H101" s="3" t="inlineStr">
+      <c r="H102" s="3" t="inlineStr">
         <is>
           <t>REL-04</t>
         </is>
       </c>
-      <c r="I101" s="3" t="inlineStr">
+      <c r="I102" s="3" t="inlineStr">
         <is>
           <t>PM 결정사항(2026-07-30 대화), policies.md 11번</t>
         </is>
       </c>
-      <c r="J101" s="3" t="inlineStr">
+      <c r="J102" s="3" t="inlineStr">
         <is>
           <t>체크리스트 5개 항목 모두 확인·조치 완료 및 PM 승인 후 저장소 visibility를 public으로 변경</t>
         </is>
       </c>
-      <c r="K101" s="3" t="inlineStr">
+      <c r="K102" s="3" t="inlineStr">
         <is>
           <t>정량 검증: gitleaks(또는 동급 도구) 스캔 결과 시크릿 탐지 0건, 전체 fixture 파일에서 실제 Riot ID 패턴(게임명#태그)·PUUID 패턴 검색 결과 0건</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="4" t="inlineStr">
+        <is>
+          <t>FE-15</t>
+        </is>
+      </c>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C103" s="4" t="inlineStr">
+        <is>
+          <t>프론트엔드</t>
+        </is>
+      </c>
+      <c r="D103" s="3" t="inlineStr">
+        <is>
+          <t>조합상세</t>
+        </is>
+      </c>
+      <c r="E103" s="3" t="inlineStr">
+        <is>
+          <t>조합 상세 헥스 배치도 성급(★) 표시</t>
+        </is>
+      </c>
+      <c r="F103" s="3" t="inlineStr">
+        <is>
+          <t>HexBoard 챔피언 타일에 op.gg tft_list_meta_decks 응답 units[].tier(2 또는 3, 2026-08-06 실호출로 확인 — FE-14 cell_x/y와 같은 unit 객체 필드)를 성급으로 매핑해 별 아이콘 표시. comp_champions 테이블에 star_level 컬럼 추가(배치, comp_champion_rows()에서 unit.tier 추출, 없으면 None), GET /comps/{comp_id} 응답(ChampionInComp)에 star_level 포함(API-03), 실좌표 그리드(HexBoard)에서 챔피언 타일 위에 star_level개의 별 아이콘을 표시하되 색상은 3성=레드, 2성=골드로 고정(PM 결정 2026-08-06 — op.gg 원본의 색상 체계(초록/파랑/핑크/회색 등)는 근거 데이터가 없어 재현하지 않고 2단계 고정 색상만 적용). star_level이 없는 구 데이터/휴리스틱 폴백 모드에서는 별 표시를 생략한다.</t>
+        </is>
+      </c>
+      <c r="G103" s="4" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H103" s="3" t="inlineStr">
+        <is>
+          <t>FE-14</t>
+        </is>
+      </c>
+      <c r="I103" s="3" t="inlineStr">
+        <is>
+          <t>PM 요청 2026-08-06, op.gg tft_list_meta_decks 실호출로 units[].tier 필드(값 2/3) 확인, 색상 고정은 PM 결정(2026-08-06, 3성=레드/2성=골드)</t>
+        </is>
+      </c>
+      <c r="J103" s="3" t="inlineStr">
+        <is>
+          <t>조합 상세 페이지에서 실좌표 그리드로 렌더링되는 챔피언 타일에 star_level(2 또는 3)만큼 별 아이콘이 3성=레드/2성=골드 고정 색상으로 표시됨, star_level 없는 챔피언/휴리스틱 폴백 모드는 별 미표시로 정상 동작(콘솔 에러 0건)</t>
+        </is>
+      </c>
+      <c r="K103" s="3" t="inlineStr">
+        <is>
+          <t>pytest(batch): comp_champion_rows()가 unit.tier에서 star_level을 추출하는 단위 테스트(2/3/누락 케이스) / pytest(backend): GET /comps/{comp_id} 응답에 star_level 포함 및 null 폴백 확인 / Vitest+RTL: HexBoard가 star_level만큼 별 아이콘(3성=레드, 2성=골드)을 렌더링하고, star_level 없으면 별 미표시함을 확인</t>
         </is>
       </c>
     </row>
@@ -6366,7 +6480,7 @@
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6">
@@ -6452,7 +6566,7 @@
       </c>
       <c r="B11" s="8" t="inlineStr"/>
       <c r="C11" s="8" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: CHAT-12/CHAT-13 완료 반영, DATA-19·CHAT-14 신규 TASK 등록
- 진행현황.md: CHAT-12·CHAT-13 상태를 완료로 갱신(PM 승인 2026-08-08),
  진행률 요약 수치 갱신
- CHAT-12(답변 마크다운 서식)·CHAT-13(아이템 이름 근거검증 인식 개선,
  PM 재검증 중 발견한 링크 회귀 2건 포함)·DATA-19(아이템 효과 설명 데이터
  확보·정제)·CHAT-14(아이템 효과 설명 RAG 연동·이름 줄임말 인식) 신규
  TASK를 WBS.xlsx에 반영
- opgg-schema.md: DATA-19/CHAT-14 착수 전 확인한 아이템 desc 필드 실측
  결과(완성 아이템 96% 정리만으로 사용 가능, 재사용 키워드는 4종뿐) 기록
</commit_message>
<xml_diff>
--- a/TFT_Hideout_WBS.xlsx
+++ b/TFT_Hideout_WBS.xlsx
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K104"/>
+  <dimension ref="A1:K108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6440,6 +6440,234 @@
       <c r="K104" s="3" t="inlineStr">
         <is>
           <t>pytest(batch): comp_champion_rows()가 unit.tier에서 star_level을 추출하는 단위 테스트(2/3/누락 케이스) / pytest(backend): GET /comps/{comp_id} 응답에 star_level 포함 및 null 폴백 확인 / Vitest+RTL: HexBoard가 star_level만큼 별 아이콘(3성=레드, 2성=골드)을 렌더링하고, star_level 없으면 별 미표시함을 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>CHAT-12</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>챗봇RAG</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>챗봇위젯</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>답변 마크다운 서식(목록/강조) 렌더링 구현</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>CHAT-03 시스템 프롬프트에 목록(-)·강조(**) 서식 규칙과 few-shot 예시를 추가하고, FE-09 renderAnswerText()가 링크 문법만 파싱하던 것을 목록/굵게까지 파싱하도록 확장해 답변이 길 때 줄바꿈·글머리로 가독성 있게 표시되게 한다(PM 요청 2026-08-08).</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>CHAT-03,FE-09</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>PM 요청(2026-08-08, 챗봇 답변 가독성 개선), 설계서 4.4.1</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>답변에 2개 이상 항목이 나열될 때 각 항목이 줄바꿈된 '-' 목록으로, 강조 문구는 **굵게**로 표시되어 프론트에서 실제 리스트/볼드로 렌더링됨(스크린샷과 유사한 산문형 나열이 더는 발생하지 않음)</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>pytest: SYSTEM_PROMPT_BASE에 목록/강조 서식 규칙 문자열 포함 확인, few-shot 예시에 형식 반영 확인 | Vitest+RTL: '- ' 접두 줄이 &lt;ul&gt;&lt;li&gt; 목록으로, '**텍스트**'가 &lt;strong&gt;으로 렌더링되는지 mock 텍스트로 확인, 기존 링크 파싱·타이핑 인디케이터 테스트 무회귀</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>CHAT-13</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>챗봇RAG</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>챗봇위젯</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>아이템 이름 근거검증 인식 개선</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>CHAT-06 verify_grounding()의 _known_names()가 챔피언/조합 이름(doc_metadata name/champion 키)만 인식하고 아이템 이름은 전혀 인식하지 못해, 8번 규칙(작은따옴표 인용)에 따라 정상적으로 인용된 아이템 이름도 항상 "(주의: 위 답변 중 일부 명칭은 검색된 문서에서 확인되지 않았습니다.)" 경고를 유발하는 구조적 오탐을 수정한다(PM 제보 2026-08-08, CHAT-12 작업결과 참고). item_build 문서 doc_metadata에 아이템 이름 목록을 추가하고, verify_grounding()·insert_links() 양쪽이 이를 인식하도록 확장한다(아이템 이름도 CHAT-07처럼 링크 대상이 될 수 있음).</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>CHAT-06,CHAT-07,DATA-11</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>PM 제보(2026-08-08), docs/verification/CHAT-12-작업결과.md</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>아이템 이름만 인용된 정확한 답변에서 근거검증 경고가 더 이상 뜨지 않고, 실제로 근거 없는 이름(챔피언/조합/아이템 불문)은 여전히 경고가 뜸. 아이템 이름도 가능하면 /items/builds 링크로 렌더링됨</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>pytest: item_build 문서 doc_metadata에 items 목록이 포함되는지(batch), _known_names()/verify_grounding()이 아이템 이름을 인식해 경고를 안 붙이는지, 여전히 미확인 이름은 경고가 붙는지, insert_links()가 아이템 이름도 링크로 치환하는지 각각 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>DATA-19</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>데이터파이프라인</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>아이템빌드</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>아이템 효과 설명 데이터 확보·정제</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>op.gg tft_list_item_combinations의 desc 필드(Community Dragon 원본, 실호출로 확인 완료)를 활용해 items.description 컬럼을 채운다. DATA-16의 clean_augment_description() 패턴을 재사용/일반화해 &lt;br&gt;·&lt;tftitemrules&gt; 등 HTML 유사 태그와 @TFTUnitProperty...@ 미해석 수치 템플릿을 정리한다. {{TFT_Keyword_Precision}} 등 재사용 키워드 참조(실측 4종: 정밀/화상/냉각/상처)는 op.gg·Community Dragon 어디에도 해석된 텍스트가 없어(cdragon/tft 전체 덤프 top-level 키가 items/setData/sets뿐, 별도 키워드 글로서리 없음 확인) DATA-07 Legend 목록과 동일한 수동 유지 사전으로 보강한다(PM 요청 2026-08-08).</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>DATA-08</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>PM 요청(2026-08-08), docs/verification/CHAT-12-작업결과.md</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>items.description이 채워지고 HTML 태그·미해석 수치 템플릿이 남지 않음, 4개 재사용 키워드는 수동 사전으로 완전한 문장으로 대체됨(실측: 전체 838개 중 약 84개(10%)가 원문 그대로는 불완전, 나머지는 태그 정리만으로 사용 가능)</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>pytest: desc 클렌징 함수 단위 테스트(태그 제거, 수치 플레이스홀더 처리 — DATA-16 기존 테스트 패턴 재사용), 4개 키워드 수동 사전 치환 테스트, 합성 fixture로 items.description 컬럼 채움 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>CHAT-14</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>챗봇RAG</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>챗봇위젯</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>아이템 효과 설명 RAG 연동 및 이름 줄임말 인식</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>(1) DATA-19가 채운 items.description을 신규 'item' 문서 타입(champion doc_type과 동일 패턴, 2026-08-07 신설분 참고)으로 임베딩해 '보석 건틀릿 효과가 뭐야?' 같은 질문에 검색되게 하고, CHAT-02 하이브리드 검색의 의도별 doc_type 필터에 반영한다. (2) CHAT-04 SLANG_DICTIONARY(현재 '아뎃'→애쉬 1건뿐)에 커뮤니티에서 흔히 쓰는 아이템 줄임말(예: 보건→보석 건틀릿, 무대→무한의 대검)을 확장해 줄임말 질문도 정규화되게 한다. 정확한 줄임말 목록은 PM 확인 필요(제안 초안으로 착수, 착수 시 PM과 확정).</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>DATA-19,CHAT-02,CHAT-04</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>PM 요청(2026-08-08), docs/verification/CHAT-12-작업결과.md</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>아이템 효과를 묻거나 특정 아이템을 쓰는 챔피언을 물을 때 답변에 아이템 효과 설명이 함께 포함됨, 등록된 줄임말로 질문해도 정규화되어 정상 검색·답변됨</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>pytest: item 문서타입이 하이브리드 검색 의도별 필터에 포함되는지, 프롬프트 조립 시 item 문서 content_text가 포함되는지, SLANG_DICTIONARY 줄임말 다건 치환 테스트(정규화 후 검색 문구가 원래 이름으로 바뀌는지)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: DATA-20·CHAT-14·CHAT-15 완료 반영(PM 승인)
진행현황.md 상태 갱신(진행중 -> 완료, 커밋 링크·작업결과 문서 반영),
WBS.xlsx에 DATA-20·CHAT-15 신규 등록 반영. 세 TASK 모두 2026-08-09
PM 확인·승인.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TFT_Hideout_WBS.xlsx
+++ b/TFT_Hideout_WBS.xlsx
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6668,6 +6668,120 @@
       <c r="K108" t="inlineStr">
         <is>
           <t>pytest: item 문서타입이 하이브리드 검색 의도별 필터에 포함되는지, 프롬프트 조립 시 item 문서 content_text가 포함되는지, SLANG_DICTIONARY 줄임말 다건 치환 테스트(정규화 후 검색 문구가 원래 이름으로 바뀌는지)</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>DATA-20</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>데이터파이프라인</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>아이템빌드</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>아이템 핵심 수치 스탯 RAG 노출</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>CHAT-14 PM 검증 중 발견 — items.stats(op.gg/Community Dragon 원본 툴팁 변수 그대로, distinct 키 500개 이상, CritDamageToGive처럼 값이 None인 키·"{해시}" 형태 미해석 키 다수)가 챗봇 RAG 문서(item_chunk_text)에 전혀 포함되지 않아, "치명타 확률이 얼마나 증가하나요?" 같은 수치 질문에 항상 "정보가 확인되지 않았다"로만 답하는 한계를 실측 확인('보석 건틀릿' CritChance=35가 DB엔 있으나 임베딩 텍스트엔 없었음). 전체 키를 다 노출하는 대신, 게임적으로 의미가 명확하고 흔히 쓰이는 핵심 스탯(공격력/주문력/방어력/마법저항력/체력/공격속도/치명타확률/치명타피해/생명흡수/마나회복 등) 한정 화이트리스트를 DATA-07·DATA-19와 동일 패턴(수동 유지 목록)으로 두고 "이름: 값" 형태로 정리해 item_chunk_text에 덧붙여 임베딩한다. 화이트리스트 밖 키(단위·의미가 불분명한 어빌리티 변수·미해석 해시 키 다수)는 이번 범위에서 제외한다.</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>DATA-19</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>CHAT-14 PM 검증 중 발견(2026-08-09), docs/verification/CHAT-14-작업결과.md</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>화이트리스트에 포함된 핵심 스탯이 non-null로 존재하는 아이템은 RAG 문서에 "스탯: 치명타 확률 +35" 같은 형태로 수치가 포함되어 챗봇이 문서 근거로 정확한 수치를 답변할 수 있음, 화이트리스트 밖 키는 노출하지 않아 의미 불명 수치로 인한 오답 위험이 없음</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>pytest: 스탯 화이트리스트 포맷 함수 단위 테스트(값 존재/None/화이트리스트 밖 키 스킵, 퍼센트·정수 표기 규칙), item_chunk_text 출력에 포맷된 스탯 문자열이 포함되는지, 배치 임베딩 스냅샷 갱신 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>CHAT-15</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>챗봇RAG</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>챗봇위젯</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>검색 결과 최소 유사도 신뢰도 임계값 도입</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>CHAT-14 PM 검증 중 발견("죽무 효과는?"에 전혀 다른 아이템 '절멸자'의 효과를 확신에 찬 문장으로 답한 사례) — hybrid_search()가 pgvector 코사인 거리를 순위 정렬에만 쓰고 값 자체는 버려서, 사전(SLANG_DICTIONARY)에 없는 줄임말·오타처럼 의미상 애매한 질의도 top-k 안에 들어오면 무조건 근거 문서로 채택돼 LLM이 그걸 사실처럼 답한다. 실측(2026-08-09): item doc_type에서 정상 매칭 거리는 0.38~0.46, 오매칭('죽무'-&gt;'절멸자')은 0.59, 실제 정답 문서('죽음의 저항')는 0.65(52위)로 확연히 분리됨 — item·augment doc_type은 이 분리가 확인돼 최소 유사도 임계값(불합격 시 검색 결과 자체를 비움 → "정보 없음" 답변으로 처리, 완전히 새 방어선이 아니라 기존 retrieved_docs 빈 턴 처리와 동일 경로 재사용)을 둘 수 있다. champion doc_type은 정상적인 특정 챔피언 이름 질의도 거리 0.507로 item의 "나쁜 매칭" 수준과 겹쳐 위험하고, comp doc_type은 특정 조합명이 아닌 일반 "메타 추천" 질의가 정상인데도 거리 0.48~0.49로 나와 임계값 적용 시 정상 케이스가 깨질 위험이 실측으로 확인돼, 이번 TASK 범위에서는 item·augment 두 doc_type에만 한정 적용한다(champion·comp·playstyle·item_build는 제외, 근거는 위 실측치).</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>CHAT-02,CHAT-14</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>CHAT-14 PM 검증 중 발견(2026-08-09), docs/verification/CHAT-14-작업결과.md</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>item·augment doc_type 검색에서 최소 유사도(코사인 거리) 임계값을 넘는(=너무 먼) 결과는 후보에서 제외됨, 임계값을 만족하는 결과가 하나도 없으면 해당 doc_type은 빈 결과로 처리되어 기존 "근거 문서 없음" 경로(정보 없음 답변, 후속질문 미생성)를 그대로 탐, champion·comp 등 실측상 임계값 적용이 위험한 doc_type은 이번 범위에서 제외됨이 문서화됨</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>pytest: item/augment doc_type에서 임계값 초과 결과가 실제로 걸러지는지(가까운 문서는 포함, 먼 문서는 제외), 임계값 미달로 결과가 전부 없어져도 에러 없이 빈 리스트를 반환하는지, champion/comp doc_type은 먼 거리 문서도 그대로 반환되는지(회귀 없음) 확인</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: CHAT-16·SET-17 완료 반영, CHAT-17 신설(PM 승인)
진행현황.md 상태 갱신(대기/진행중 -> 완료, 커밋 링크·작업결과 문서 반영),
WBS.xlsx에 CHAT-16·SET-17·CHAT-17 신규 등록 반영. CHAT-16·SET-17은
2026-08-12 PM 확인·승인, CHAT-17은 대기 상태로 신설만 반영.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TFT_Hideout_WBS.xlsx
+++ b/TFT_Hideout_WBS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="WBS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="요약" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'WBS'!$A$1:$K$95</definedName>
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K110"/>
+  <dimension ref="A1:K113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6782,6 +6782,177 @@
       <c r="K110" t="inlineStr">
         <is>
           <t>pytest: item/augment doc_type에서 임계값 초과 결과가 실제로 걸러지는지(가까운 문서는 포함, 먼 문서는 제외), 임계값 미달로 결과가 전부 없어져도 에러 없이 빈 리스트를 반환하는지, champion/comp doc_type은 먼 거리 문서도 그대로 반환되는지(회귀 없음) 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>CHAT-16</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>챗봇RAG</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>챗봇위젯</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>오프토픽 판별 2차 LLM 검증 도입</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>chat_preprocessing.py의 is_off_topic()이 _TFT_DOMAIN_PATTERN 키워드 정규식 미스만으로 즉시 범위 밖 처리해, "시즌 종료는 언제?"처럼 TFT 관련이지만 조합/아이템/증강체/메타 키워드가 없는 질문이 오분류되는 문제를 CHAT-01 의도 분류와 동일한 "1차 키워드 → 애매하면 2차 Groq LLM" 패턴으로 확장해 개선한다(PM 제보 2026-08-12, CHAT-17 웹검색 스코프 검토 중 발견). 키워드 매칭 성공 시 기존과 동일하게 즉시 on-topic 처리(LLM 미호출, 속도·비용 유지), 키워드 매칭 실패 시에만 Groq에 "이 질문이 TFT(전략적 팀 전투) 게임과 관련 있는가"만 판별시켜(예/아니오만 출력), 관련 있음이면 on-topic으로 넘겨 CHAT-17(5번째 의도) 분류로 이어지게 하고, 관련 없음이면 기존 OFF_TOPIC_MESSAGE로 처리한다. 2차 LLM 호출 실패 시 안전 기본값(관련없음 폴백 vs on-topic 통과)은 착수 시 PM과 확정.</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>CHAT-01,CHAT-04</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>PM 요청(2026-08-12, 웹검색 스코프 검토), policies.md 8번</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>"시즌 종료는 언제?" 같이 키워드는 없지만 TFT 관련인 질문이 더 이상 즉시 거부되지 않고 on-topic으로 통과함, "오늘 점심 뭐 먹지" 같은 순수 무관 질문은 여전히 거부됨(TEST-00 CHAT-04 6번 시나리오 무회귀), test-scenarios.md CHAT-04 섹션에 2차 검증 케이스 추가 및 PM 재승인 완료</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>pytest: 키워드 매칭 성공 시 LLM 미호출 확인(mock 호출 카운트 0), 키워드 미스+LLM "관련있음" 응답 시 on-topic 통과 확인, 키워드 미스+LLM "관련없음" 응답 시 기존 거부 문구 확인, LLM 실패 시 확정된 안전 기본값대로 동작하는지 확인 — TEST-00 갱신 시나리오를 그대로 옮김</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>SET-17</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>시스템설정</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>웹 검색 API 키 발급 및 검증(Tavily)</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>CHAT-17(웹검색 기반 일반 게임 정보 답변)에 필요한 Tavily API 키를 발급하고 .env(로컬)·GitHub Secrets·Render 환경변수에 등록한다. SET-16(Riot Personal Key) 발급 절차와 동일 패턴(무료 티어 확인 → 1회성 스모크 호출로 실제 검색 응답 확인 → smoke-tests.md 기록). Tavily 무료 티어는 월 1,000 크레딧(기본 검색 1건=1크레딧) 매월 갱신, 카드 등록 불요(2026-08-12 확인).</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>PM 결정(2026-08-12, 웹검색 스코프 검토), SET-10 발급 절차 패턴</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>Tavily API 키 발급 완료, .env/GitHub Secrets/Render 환경변수 등록 완료, 실제 검색 API 1회 호출로 200 응답 및 검색 결과 스니펫 확인</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>해당 없음(인프라·시크릿) — 1회성 스모크 테스트 결과를 docs/verification/smoke-tests.md에 기록하는 것으로 갈음(policies.md 12번과 동일 패턴)</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>CHAT-17</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>챗봇RAG</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>챗봇위젯</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>웹검색 기반 일반 게임 정보 답변 경로 신설</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>CHAT-16이 on-topic으로 판별했지만 기존 4개 의도(조합/아이템/증강체/일반전략) RAG 검색 대상이 아닌 질문(시즌 일정, 정식 출시 예정 콘텐츠, 공식 이벤트 일정 등)을 위해 5번째 의도 general_game_info를 신설한다(PM 결정 2026-08-12, 5번째 의도 신설 방식 채택 — 기존 RAG 실패시 폴백 방식 대비 트리거 범위가 명확하고 비용 통제가 쉬움). intent_classification.py에 이 카테고리를 추가하고, 해당 의도로 분류되면 기존 pgvector 하이브리드 검색(CHAT-02) 대신 Tavily 웹 검색(SET-17)을 호출해 상위 스니펫을 근거로 사용한다. 근거 형식이 기존 [검색된 문서](내부 DB, 패치 버전 명시)와 근본적으로 달라 별도 프롬프트 섹션([웹 검색 결과], 출처 URL 포함)과 별도 시스템 규칙("웹 검색 결과에 없는 내용은 추측 금지, 반드시 출처 URL을 답변에 포함하라")을 신설한다. CHAT-06 근거검증(verify_grounding)·CHAT-07 링크삽입 패턴을 재사용해 답변에 포함된 출처 URL이 실제 검색 결과에 있던 URL인지 사후 검증한다. Tavily 호출 실패/무료 티어 소진 시 기존 FALLBACK_MESSAGE 경로로 폴백(policies.md 9번, 재시도 1회 후 폴백).</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>CHAT-16,CHAT-03,CHAT-06,SET-17</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>PM 요청(2026-08-12), policies.md 5번(RAG 근거 원칙 — 웹검색용 별도 원칙 신설 필요)</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>"시즌 종료는 언제?" 같은 질문이 웹 검색 결과를 근거로 출처 URL과 함께 답변됨, 검색 결과에 없는 내용은 추측하지 않고 "확인되지 않았습니다"로 답함(기존 원칙과 동일 수준 유지), Tavily 실패 시 기존 폴백 메시지로 안전하게 대체됨, policies.md에 "웹 검색 근거 원칙" 신설 반영</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>pytest: general_game_info 의도 분류 확인, 해당 의도일 때 CHAT-02(내부검색) 대신 Tavily 호출 경로를 타는지, 검색 결과 없음/API 실패 시 폴백 메시지로 처리되는지, 답변 내 URL이 실제 검색 결과 URL과 일치하는지(근거검증) — 외부 API는 fixture로 mock(CLAUDE.md 10.2 외부 API 목 정책, 실제 Tavily 미호출)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: CHAT-18 완료 반영(PM 승인)
진행현황.md 상태 갱신, WBS.xlsx에 CHAT-18 신규 등록 반영.
2026-08-12 PM 확인·승인.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TFT_Hideout_WBS.xlsx
+++ b/TFT_Hideout_WBS.xlsx
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K113"/>
+  <dimension ref="A1:K114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6953,6 +6953,63 @@
       <c r="K113" t="inlineStr">
         <is>
           <t>pytest: general_game_info 의도 분류 확인, 해당 의도일 때 CHAT-02(내부검색) 대신 Tavily 호출 경로를 타는지, 검색 결과 없음/API 실패 시 폴백 메시지로 처리되는지, 답변 내 URL이 실제 검색 결과 URL과 일치하는지(근거검증) — 외부 API는 fixture로 mock(CLAUDE.md 10.2 외부 API 목 정책, 실제 Tavily 미호출)</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>CHAT-18</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>챗봇RAG</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>챗봇위젯</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>비활성 조합 근거검증·랭킹 정합성 개선</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>CHAT-17 실사용 검증 중 PM 제보(2026-08-12) — "룰루는 어떤덱으로?"에 챗봇이 comps.is_active=false(DATA-17 소프트 삭제, op.gg 상위 10위 밖으로 밀려나 사이트 티어리스트엔 안 보임)인 "별돌보미 룰루"를 티어 S로 추천. batch/embeddings.py의 comp_chunk_text()/playstyle_chunk_text()가 is_active를 전혀 반영하지 않아 통계가 얼어붙은 비활성 조합도 현재형 문구로 재임베딩되고, hybrid_search.py가 tier_rank만 1차 정렬 기준으로 써서 얼어붙은 옛 티어가 실제 활성 조합보다 랭킹에서 앞서던 것이 원인. is_active=false면 임베딩 본문에 "상위 10위 밖으로 밀려남" 문구 추가, SYSTEM_PROMPT_BASE 11번 규칙으로 LLM이 캐비엇을 달도록 지시, hybrid_search.py에 is_active 기반 _ACTIVE_PRIORITY를 tier_rank보다 앞선 1차 정렬 기준으로 추가. 검증 중 comp/playstyle 메타데이터에 구성 챔피언 이름이 없어 정상 인용도 근거검증 오탐을 내는 것을 추가 발견(CHAT-13이 item_build에 이미 고친 것과 동일한 문제) — "champions" 메타데이터 키 추가로 함께 수정. CHAT-17의 웹검색 링크 오버플로우(원문 URL 노출)도 같이 제보돼 [출처](URL) 마크다운 형식 전환 + 채팅 버블 wrap-break-word CSS로 함께 수정, 그 과정에서 웹검색 경로가 CHAT-06 근거검증을 잘못 재사용해 오탐을 내던 버그도 함께 발견·수정.</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>CHAT-17</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>PM 제보(2026-08-12, CHAT-17 실사용 검증 중)</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>"룰루는 어떤덱으로?" 같은 질문에 비활성(is_active=false) 조합 대신 활성 조합이 추천됨, 부득이 비활성 조합을 언급할 때는 상위권 밖으로 밀려났다는 캐비엇이 함께 표시됨, comp 답변에서 챔피언 이름을 정상 인용해도 근거검증 오탐이 붙지 않음, 웹검색 출처 링크가 채팅 버블 밖으로 넘치지 않고 짧은 링크로 표시됨</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>pytest(backend): hybrid_search가 비활성 조합을 활성 조합보다 항상 뒤로 정렬하는지, SYSTEM_PROMPT_BASE에 캐비엇 규칙 문구가 있는지, verify_grounding이 comp metadata의 champions 목록으로 챔피언 인용을 검증하는지, 웹검색 답변이 postprocess_answer(CHAT-06 근거검증)를 타지 않는지 확인 | pytest(batch): comp_chunk_text/playstyle_chunk_text가 is_active=false일 때만 상태 문구를 추가하는지, collect_chunks의 comp/playstyle metadata에 champions 키가 포함되는지 확인 | Vitest 대신 로컬 Playwright로 채팅 버블 가로 오버플로우 없음 실측 확인(자동화 테스트 미작성, 수동 스크린샷 검증)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(CHAT-19): 패치 버전 질문 general_game_info 오분류 수정
"현재 패치버전은?"류 질문이 1차 키워드 매칭에 걸리지 않아 2차 LLM
의도분류에서 general_game_info(Tavily 웹검색 전용)로 오분류되고,
이미 조회해둔 patch_version은 쓰지 않은 채 무관한 웹검색 결과로
답하던 문제를 수정. 의도분류 이전에 패치 버전 질문을 감지해
patches.is_current 값으로 검색/LLM 호출 없이 즉답하는 조기 반환
경로를 신설(PM 제보 2026-08-14, CHAT-19 신규 등록).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TFT_Hideout_WBS.xlsx
+++ b/TFT_Hideout_WBS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="WBS" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="요약" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'WBS'!$A$1:$K$95</definedName>
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K114"/>
+  <dimension ref="A1:K115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7010,6 +7010,63 @@
       <c r="K114" t="inlineStr">
         <is>
           <t>pytest(backend): hybrid_search가 비활성 조합을 활성 조합보다 항상 뒤로 정렬하는지, SYSTEM_PROMPT_BASE에 캐비엇 규칙 문구가 있는지, verify_grounding이 comp metadata의 champions 목록으로 챔피언 인용을 검증하는지, 웹검색 답변이 postprocess_answer(CHAT-06 근거검증)를 타지 않는지 확인 | pytest(batch): comp_chunk_text/playstyle_chunk_text가 is_active=false일 때만 상태 문구를 추가하는지, collect_chunks의 comp/playstyle metadata에 champions 키가 포함되는지 확인 | Vitest 대신 로컬 Playwright로 채팅 버블 가로 오버플로우 없음 실측 확인(자동화 테스트 미작성, 수동 스크린샷 검증)</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>CHAT-19</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>챗봇RAG</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>챗봇위젯</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>패치 버전 질문 직접 답변 경로 신설</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>PM이 실사용 중 "현재 패치버전은?" 질문에 챗봇이 패치 정보를 확인할 수 없다고 답하며 LoL/Windows 핫패치 같은 무관한 웹검색 결과를 인용하는 문제를 제보(2026-08-14). 원인 조사 결과 intent_classification.py의 1차 키워드 패턴(조합/아이템/증강체/메타)에 "패치"가 없어 2차 Groq LLM 분류로 넘어가고, LLM이 "게임 운영 정보 질문"으로 보고 general_game_info(CHAT-17, Tavily 웹검색 전용)로 오분류함을 확인. 정작 patch_version(patches.is_current)은 chat_stream.py의 generate_answer_stream()이 의도분류 이전에 이미 조회해두는데, 이 값이 general_game_info 경로(_generate_web_search_answer)에는 로깅용으로만 전달되고 프롬프트/답변 생성에는 전혀 쓰이지 않아 굳이 웹검색을 돌리는 구조적 공백이었음. "패치버전이 몇이냐"류 질문은 의도분류·검색·LLM 호출 없이 이미 알고 있는 patch_version으로 결정론적으로 즉답하는 조기 반환 경로를 신설한다(CLARIFICATION_MESSAGE/OFF_TOPIC_MESSAGE/NO_CURRENT_PATCH_MESSAGE와 동일한 패턴).</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>CHAT-01,CHAT-04,CHAT-05</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>PM 제보(2026-08-14), glossary.md 챗봇 의도 분류(5종)</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>"현재 패치버전은?"/"지금 몇 패치야?"/"패치 버전이 뭐야?" 류 질문이 웹검색·LLM 호출 없이 patches.is_current 값으로 즉답됨, "이번 패치에 뭐가 바뀌었어?" 같이 버전이 아닌 패치노트류 질문은 기존 general_game_info 경로로 정상 동작(회귀 없음)</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>pytest: is_patch_version_query()가 '패치버전'/'몇 패치'류 질의는 True, '이번 패치에 뭐가 바뀌었어?' 등 패치노트류 질의는 False를 반환하는지, generate_answer_stream이 패치 버전 질의를 감지하면 classify_fn/search_fn/web_search_fn/stream_fn을 전혀 호출하지 않고 patch_version 값을 포함한 고정 문구로 즉답하는지(patch_version이 None일 때는 기존 NO_CURRENT_PATCH_MESSAGE가 우선함을 확인)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: TEST-11 카테고리 G 결과 논의 반영 — CHAT-26/API-15/FE-17 신규 등록
TEST-11 카테고리 G(챗봇 기능·서비스 메타 질문) 결과를 PM과 논의:

- G9("한국 서버 기준이야, 글로벌 기준이야?") 오답의 실제 정답을
  docs/spike/opgg-schema.md(DATA-05 스파이크)로 재확인 — op.gg MCP
  통계 도구는 region 파라미터 자체가 없어 리전 구분 없는 전 세계
  통합 집계임.
- G8(신고/피드백 경로 없음)에 대해 PM이 신규 기능(작성자 이메일+내용
  등록/공개 목록조회/삭제, 수정 없음)을 결정.

신규 TASK 3개 등록(착수는 보류, 시점 추후 결정):
- CHAT-26: 챗봇 자기소개/메타 질문 전용 의도(chatbot_meta) 신설
- API-15: 신고(피드백) 게시판 API 구현
- FE-17: 신고(피드백) 게시판 페이지 구현

전체 TASK 수 123 -> 126개(활성 120 -> 123개).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TFT_Hideout_WBS.xlsx
+++ b/TFT_Hideout_WBS.xlsx
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K121"/>
+  <dimension ref="A1:K124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7409,6 +7409,177 @@
       <c r="K121" t="inlineStr">
         <is>
           <t>Vitest+RTL: 티어리스트 페이지/조합 카드에 안내 문구 텍스트가 렌더링되는지 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>CHAT-26</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>챗봇RAG</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>챗봇위젯</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>챗봇 자기소개/메타 질문 전용 의도(chatbot_meta) 신설</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>TEST-11 카테고리 G(챗봇 기능·서비스, 15문항) 채점 중 발견(2026-08-18) — "너는 어떤 걸 도와줄 수 있어?", "이전에 물어본 내용을 계속 기억해?", "너는 라이엇게임즈 소속이야?" 등 챗봇 자기 자신에 대한 메타 질문이 오프토픽 판별기에 걸려 정형 거절 메시지로 일괄 회피되거나(11/15), 우연히 키워드가 걸리면 웹검색으로 새서 무관한 정보를 인용(G9 — "한국 서버 기준으로 답하냐"는 질문에 무관한 실제 서버 오픈일 정보로 답변). op.gg MCP 통계 도구(tft_list_meta_decks 등)는 region 파라미터 자체가 없어(docs/spike/opgg-schema.md 4·7번 항목, tft_get_play_style 개인조회 도구만 region+puuid 필요) 이 서비스의 메타 통계는 리전 구분 없는 전 세계 통합 집계임을 재확인 — G9은 이 사실로 정정. intent_classification 단계(또는 오프토픽 판별과 병렬)에 챗봇 자기참조 키워드("너는"/"챗봇은"/"기억해"/"안전해"/"라이엇"/"신고" 등)를 감지하는 chatbot_meta 의도를 신설하고, LLM/RAG 생성 없이 미리 정의한 정적 FAQ 답변(CHAT-19 패치버전 조기 반환과 동일하게 검색·LLM 호출 없는 결정론적 즉답)으로 응답한다. 답변에 담을 사실: 기능 범위(CLAUDE.md 1~3장 스코프, 룰 설명·아이템/시너지 정보·공략 팁), 데이터 최신성(패치 자동 갱신, DATA-12~14), 전적 분석 기능 부재(PGA-* 미구현 상태, 추후 지원 예정), 리전(전 세계 통합 집계, 특정 서버 기준 아님 — 위 재확인 내용), 세션 대화 기억 범위(같은 세션 내 최근 3턴, CHAT-04), 개인정보(로그인 없음, session_id는 회원식별자 아님, 불필요한 개인정보 입력 비권장), 정체성(라이엇 공식 아닌 개인/비상업 팬 프로젝트), 음성/이미지/다국어 미지원, 오류 신고 경로(API-15/FE-17 신고 게시판 안내, 해당 TASK 완료 전까지는 문구 보류 또는 "추후 지원 예정"으로 임시 처리 — 착수 시 API-15/FE-17 상태 확인).</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>CHAT-01,CHAT-16</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>PM 결정(2026-08-18, TEST-11 카테고리 G 결과 논의), docs/verification/TEST-11-작업결과.md(카테고리 G 결과 상세), docs/spike/opgg-schema.md</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>TFT_챗봇_테스트_예상질문지.docx 카테고리 G 15문항 재질의 시 정답지 채점기준(docs/spike/TFT_챗봇_테스트_정답지.docx, 테이블 index 6)을 각각 충족하는 고정 답변이 검색·LLM 생성 없이 즉답됨, G9(리전 오답)이 더 이상 재현되지 않음, 일반 TFT 게임 질문 분류에는 회귀 없음</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>pytest: 챗봇 자기참조 키워드 감지 함수 단위 테스트(15문항 각각 chatbot_meta로 분류되는지), 각 메타 질문 유형별 고정 답변 매핑 테스트, chatbot_meta 분류 시 classify_fn(2차 LLM)/search_fn/web_search_fn이 전혀 호출되지 않는지(mock 카운트 0), 기존 4~5개 의도 분류에 회귀 없는지(키워드 겹침 케이스 포함)</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>API-15</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>백엔드API</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>공통(신고)</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>신고(피드백) 게시판 API 구현</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>TEST-11 카테고리 G8("답변이 틀렸을 때 어떻게 신고하거나 고칠 수 있어?") 채점 중 신고/피드백 경로가 전혀 없다는 공백이 확인되어 PM이 신규 기능으로 결정(2026-08-18) — 작성자 이메일·내용을 입력해 등록하고, 누구나 목록을 조회할 수 있으며, 수정 기능은 두지 않고 삭제만 지원하는 간단한 신고 게시판. 신규 테이블(feedback_reports: id, author_email, content, created_at 등)을 만들고 등록(POST)·목록조회(GET)·삭제(DELETE) 3개 엔드포인트를 구현한다. 프로젝트 전체가 인증 시스템이 없는 정책(CLAUDE.md 7장)이라 삭제 권한 범위(작성자만 가능하게 할 방법이 마땅치 않음 vs 누구나 삭제 가능 — 개인/지인 10명 규모 MVP라 리스크 낮음)는 착수 시 PM과 확정. Rate limiting(API-07 패턴 재사용) 적용.</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>API-01</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>PM 결정(2026-08-18, TEST-11 카테고리 G8 결과 논의)</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>POST로 작성자 이메일+내용 등록 가능, GET으로 전체 목록(누구나) 조회 가능, DELETE로 특정 신고 삭제 가능(권한 범위는 착수 시 확정한 대로 동작), 수정 엔드포인트는 존재하지 않음, 이메일 형식 등 최소 입력 검증 포함</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>pytest: 등록/목록조회/삭제 각 엔드포인트 정상 동작, 잘못된 이메일 형식 400 처리, 존재하지 않는 신고 삭제 시 404, rate limiting 적용 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>FE-17</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>프론트엔드</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>공통(신고)</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>신고(피드백) 게시판 페이지 구현</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>API-15가 제공하는 신고 게시판 API를 사용하는 프론트엔드 페이지 — 작성자 이메일·내용 입력 폼, 등록된 신고 전체 목록(공개), 삭제 버튼으로 구성. GNB 진입점 배치(신규 메뉴 항목 vs 챗봇 위젯 내 링크 vs 푸터)는 착수 시 PM과 확정, 화면설계서 v1.2에 없는 신규 화면이라 IA 반영 여부도 함께 논의.</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>FE-01,API-15</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>PM 결정(2026-08-18, TEST-11 카테고리 G8 결과 논의)</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>이메일+내용 입력 후 등록하면 목록에 즉시 반영됨, 목록이 누구나 조회 가능하게 노출됨, 삭제 버튼으로 개별 신고 삭제 가능, 수정 UI는 존재하지 않음, 모바일/태블릿/데스크톱 반응형 레이아웃 깨짐 없음</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>Vitest+RTL: 등록 폼 제출·목록 렌더링·삭제 동작 테스트, Playwright e2e로 등록→목록노출→삭제 흐름 스모크</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(TEST-11): 카테고리 H 채점 완료(157/157) 및 후속 CHAT-2x 9개 신규 등록
카테고리 H(경계/예외 상황, 22문항) 채점 완료로 A~H 전체 157/157 완료.
발견 8건(미래정보 환각 H15 최우선, 슬랭인식실패, 복합질의누락, 언어무시,
의도오분류재발, 커버리지공백, 미검증환각목록) 문서화.

A~H 전체 발견사항을 5개 교차 패턴으로 종합 정리해 PM에게 보고, PM 결정에
따라 CHAT-27~35(패턴1~5 우선순위 + 기타 단발성) 9개 신규 등록. 패턴4는
기존 CHAT-26에 H10 사례를 추가로 포함. 조사 중 발견한 기존 드리프트
(CHAT-23/24/25가 WBS.xlsx에는 누락돼 있던 것)도 함께 동기화.

전체 TASK 수 130→139개(활성 127→136개).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TFT_Hideout_WBS.xlsx
+++ b/TFT_Hideout_WBS.xlsx
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K128"/>
+  <dimension ref="A1:K140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7440,7 +7440,7 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>TEST-11 카테고리 G(챗봇 기능·서비스, 15문항) 채점 중 발견(2026-08-18) — "너는 어떤 걸 도와줄 수 있어?", "이전에 물어본 내용을 계속 기억해?", "너는 라이엇게임즈 소속이야?" 등 챗봇 자기 자신에 대한 메타 질문이 오프토픽 판별기에 걸려 정형 거절 메시지로 일괄 회피되거나(11/15), 우연히 키워드가 걸리면 웹검색으로 새서 무관한 정보를 인용(G9 — "한국 서버 기준으로 답하냐"는 질문에 무관한 실제 서버 오픈일 정보로 답변). op.gg MCP 통계 도구(tft_list_meta_decks 등)는 region 파라미터 자체가 없어(docs/spike/opgg-schema.md 4·7번 항목, tft_get_play_style 개인조회 도구만 region+puuid 필요) 이 서비스의 메타 통계는 리전 구분 없는 전 세계 통합 집계임을 재확인 — G9은 이 사실로 정정. intent_classification 단계(또는 오프토픽 판별과 병렬)에 챗봇 자기참조 키워드("너는"/"챗봇은"/"기억해"/"안전해"/"라이엇"/"신고" 등)를 감지하는 chatbot_meta 의도를 신설하고, LLM/RAG 생성 없이 미리 정의한 정적 FAQ 답변(CHAT-19 패치버전 조기 반환과 동일하게 검색·LLM 호출 없는 결정론적 즉답)으로 응답한다. 답변에 담을 사실: 기능 범위(CLAUDE.md 1~3장 스코프, 룰 설명·아이템/시너지 정보·공략 팁), 데이터 최신성(패치 자동 갱신, DATA-12~14), 전적 분석 기능 부재(PGA-* 미구현 상태, 추후 지원 예정), 리전(전 세계 통합 집계, 특정 서버 기준 아님 — 위 재확인 내용), 세션 대화 기억 범위(같은 세션 내 최근 3턴, CHAT-04), 개인정보(로그인 없음, session_id는 회원식별자 아님, 불필요한 개인정보 입력 비권장), 정체성(라이엇 공식 아닌 개인/비상업 팬 프로젝트), 음성/이미지/다국어 미지원, 오류 신고 경로(API-15/FE-17 신고 게시판 안내, 해당 TASK 완료 전까지는 문구 보류 또는 "추후 지원 예정"으로 임시 처리 — 착수 시 API-15/FE-17 상태 확인).</t>
+          <t>TEST-11 카테고리 G(챗봇 기능·서비스, 15문항) 채점 중 발견(2026-08-18) — "너는 어떤 걸 도와줄 수 있어?", "이전에 물어본 내용을 계속 기억해?", "너는 라이엇게임즈 소속이야?" 등 챗봇 자기 자신에 대한 메타 질문이 오프토픽 판별기에 걸려 정형 거절 메시지로 일괄 회피되거나(11/15), 우연히 키워드가 걸리면 웹검색으로 새서 무관한 정보를 인용(G9 — "한국 서버 기준으로 답하냐"는 질문에 무관한 실제 서버 오픈일 정보로 답변). op.gg MCP 통계 도구(tft_list_meta_decks 등)는 region 파라미터 자체가 없어(docs/spike/opgg-schema.md 4·7번 항목, tft_get_play_style 개인조회 도구만 region+puuid 필요) 이 서비스의 메타 통계는 리전 구분 없는 전 세계 통합 집계임을 재확인 — G9은 이 사실로 정정. intent_classification 단계(또는 오프토픽 판별과 병렬)에 챗봇 자기참조 키워드("너는"/"챗봇은"/"기억해"/"안전해"/"라이엇"/"신고" 등)를 감지하는 chatbot_meta 의도를 신설하고, LLM/RAG 생성 없이 미리 정의한 정적 FAQ 답변(CHAT-19 패치버전 조기 반환과 동일하게 검색·LLM 호출 없는 결정론적 즉답)으로 응답한다. 답변에 담을 사실: 기능 범위(CLAUDE.md 1~3장 스코프, 룰 설명·아이템/시너지 정보·공략 팁), 데이터 최신성(패치 자동 갱신, DATA-12~14), 전적 분석 기능 부재(PGA-* 미구현 상태, 추후 지원 예정), 리전(전 세계 통합 집계, 특정 서버 기준 아님 — 위 재확인 내용), 세션 대화 기억 범위(같은 세션 내 최근 3턴, CHAT-04), 개인정보(로그인 없음, session_id는 회원식별자 아님, 불필요한 개인정보 입력 비권장), 정체성(라이엇 공식 아닌 개인/비상업 팬 프로젝트), 음성/이미지/다국어 미지원, 오류 신고 경로(API-15/FE-17 신고 게시판 안내, 해당 TASK 완료 전까지는 문구 보류 또는 "추후 지원 예정"으로 임시 처리 — 착수 시 API-15/FE-17 상태 확인). [2026-08-19 추가] TEST-11 카테고리 H에서도 같은 계열 재확인 — H10("너 진짜 도움이 하나도 안 되네"라는 메타 피드백/불만)이 날씨 질문(H1)과 동일한 정형 오프토픽 거절 문구로 응대됨(방어적이지 않다는 기준은 충족하나 무엇이 부족한지 되묻거나 개선 방향을 제시하지 않음). 착수 시 chatbot_meta 의도에 "불만/피드백 표현" 감지 케이스도 포함해 침착하게 응대하고 개선 방향을 되묻는 고정 응답을 추가할 것.</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
@@ -7808,6 +7808,690 @@
       <c r="K128" t="inlineStr">
         <is>
           <t>pytest(batch): 새 op_score 기반 클러스터링 함수 단위 테스트(격차 임계값 경계 케이스, 3~5단계로 가변적으로 나뉘는 케이스, 모든 조합이 비슷한 점수일 때 단일 그룹으로 뭉치는 케이스), 여러 스냅샷 fixture로 재현성 확인, 기존 DATA-21 assign_self_tiers 테스트 교체</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>CHAT-27</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>챗봇RAG</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>챗봇위젯</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>일반 게임 규칙/개념 설명 RAG 커버리지 확충</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>TEST-11 카테고리 B~E·H 채점(2026-08-15~08-19) 중 반복 확인된 가장 큰 규모의 커버리지 공백 — 패치와 무관한 불변 게임 규칙/개념(아이템 조합 방식, 아이템 가방/장착 개념, 마나 시스템, 챔피언 성급별 스킬 강화, 스킨-밸런스 무관, 랭크 티어 단계 수·LP 계산·매칭 기준·지원 서버, 시즌 종료 시 랭크 초기화, 세트 교체 시 랭크 유지 여부, 일반 전략 상담 등)을 물으면 근거 문서가 없어 전부 "정보가 확인되지 않았습니다"로 회피. 카테고리별 비중: B 8/25(32%) · C 15/20(75%, 아이템 영역 특히 심각) · D 5/15(33%) · E 4/15(27%) · H20(장문 실전 전략 상담) 1건. 해당 질문번호: B4,10,12,13,15,21,23,25 / C1,2,6,7,8,9,10,12,13,14,15,16,18,19,20 / D2,5,12,13,15 / E1,3,6,12 / H20. 근본 원인 추정 — 내부 벡터DB(comps/item_builds/augments)에는 승률·통계 데이터만 있고 "게임이 어떻게 동작하는지" 설명하는 규칙 문서 자체가 없어 검색 결과가 항상 빈 문자열에 가까움. 착수 시 PM과 해결 방식부터 확정 필요: (a) 일반 게임 규칙 설명 문서를 신규 작성해 RAG에 추가, (b) 새 의도(예: general_rules)를 신설해 검색 없이 LLM 상식 기반 답변을 제한적으로 허용, (c) 두 방식 절충. 방식에 따라 DATA-* TASK 신설이 필요할 수 있음(문서 신설 시).</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>CHAT-01,CHAT-02,CHAT-16</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>TEST-11 카테고리 B/C/D/E/H 결과 상세(docs/verification/TEST-11-작업결과.md), PM 종합보고 논의(2026-08-19)</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>착수 시 PM과 확정한 해결 방식으로 위 목록 질문(B4,10,12,13,15,21,23,25/C1,2,6,7,8,9,10,12,13,14,15,16,18,19,20/D2,5,12,13,15/E1,3,6,12/H20) 재질의 시 각 정답지 채점기준(내용상 일치 또는 정직한 확인경로 안내)을 충족, 기존 4~5개 의도 분류 및 A~H 정상 판정 케이스에 회귀 없음</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>pytest — 해결 방식이 RAG 문서 신설이면 해당 문서 검색 시 관련 chunk가 top-k에 포함되는지, 새 의도 신설이면 분류 함수 단위 테스트+search_fn/web_search_fn 호출 여부 검증, 위 질문 목록 대표 샘플 재질의 스냅샷 테스트, 기존 의도 분류 회귀 테스트</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>CHAT-28</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>챗봇RAG</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>챗봇위젯</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>키워드 기반 의도 과잉분류 재발 방지(분류 로직 재설계 검토)</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>카테고리 키워드가 포함되면 실제 질문 의도(메커니즘 설명/일반 문의)와 무관하게 해당 카테고리의 "추천 요청"으로 오분류되는 패턴이 A~H 전 카테고리에 걸쳐 반복 재발 — A13(증강 메커니즘 질문→augment_recommendation 오분류, CHAT-21에서 A1만 좁게 수정하고 문서화만 함), B5·B11(comps 데이터 무관 질문에 조합 통계 혼입), C3·C11(아이템 조합표 질문에 무관 증강체/일반론 혼입), G9(리전 질문이 "한국 서버" 키워드로 웹검색 오검색), H16(패치 예측 질문이 "패치" 키워드로 CHAT-19 패치버전 조기반환 경로에 오분류). CHAT-21이 A1 사례 하나만 정규식 예외처리로 좁게 막았을 뿐 근본적인 분류 로직(카테고리 키워드 1차 매칭 방식) 자체는 그대로라 계속 재발 중.</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>CHAT-01,CHAT-21</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>TEST-11 A13/B5·11/C3·11/G9/H16 발견 상세(docs/verification/TEST-11-작업결과.md), CHAT-21 작업결과(기존 좁은 수정 사례)</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>A13, B5, B11, C3, C11, G9, H16 질문 재질의 시 더 이상 무관한 카테고리로 오분류되지 않고 정답지 채점기준 충족, 기존 정상 분류 케이스(A1 포함)에 회귀 없음</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>pytest — 위 7개 질문 각각 올바른 의도로 분류되는지, "메커니즘 설명 질문" vs "추천 요청" 구분 대표 사례 단위 테스트 세트 신설, 기존 의도 분류 회귀 스위트 전체 통과</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>CHAT-29</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>챗봇RAG</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>챗봇위젯</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>웹검색(general_game_info) 출처 해석 정확도·품질 개선</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>CHAT-20/22가 출처 신뢰도 라벨링·쿼리 스코핑을 도입했음에도, 저품질/무관 출처를 오독하거나 그대로 이어붙여 확정적으로 틀린 결론을 내리는 문제가 카테고리를 가리지 않고 재발 — B1·B2·B6·B24(동일 나무위키/블로그 반복 인용, B1 세트 번호 모순), D4(듀오랭크 결론 반대로 오독 — duo.op.gg를 "듀오 큐 가능"으로 오해), D8·D14(핵심 답 대신 저신뢰 출처의 산발적 정보 나열), D10(강등방지 보호와 "순방" 개념 혼동), E4·E5(패치 빈도 오답, 출처가 구버전 패치 링크), E9·E15(세트 식별 혼동 — 현재/과거 세트를 다음 세트인 것처럼 답변). CHAT-20/22가 도입한 is_authoritative_source()/출처 라벨링은 "신뢰도 라벨 부착"까지만 하고, 라벨이 낮은 출처의 내용을 얼마나 신뢰해 결론에 반영할지·복수 출처 간 모순을 어떻게 처리할지는 다루지 않아 이 계열 오류가 계속 발생하는 것으로 추정.</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>CHAT-17,CHAT-20,CHAT-22</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>TEST-11 B/D/E 결과 상세(docs/verification/TEST-11-작업결과.md)</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>B1,B2,B6,B24,D4,D8,D10,D14,E4,E5,E9,E15 재질의 시 각 정답지 채점기준 충족(사실관계 정반대 결론 금지, 핵심 질문 회피 없이 답변, 세트 식별 혼동 없음), CHAT-20/22 도입 로직에 회귀 없음</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>pytest — 위 12개 질문 대표 케이스 재현 fixture로 오독 방지 로직 단위 테스트, [커뮤니티/미검증] 라벨 출처만으로 확정적 결론을 내리지 못하도록 프롬프트 지시 준수 여부 검증(모의 저신뢰 출처 fixture), 기존 CHAT-20/22 테스트 회귀 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>CHAT-30</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>챗봇RAG</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>챗봇위젯</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>미확정/미래 정보 환각 방지(생성 그라운딩 강화)</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>TEST-11 카테고리 H 채점(2026-08-19) 중 발견된 가장 심각한 유형 — 미공개·미확정 정보(다음 세트 번호·컨셉·출시일, 과거 세트 챔피언 목록 등)를 근거 문서 없이 구체적 수치까지 붙여 확신에 차게 생성. H15(다음다음 세트를 "세트15/소년만화 배틀물/2025년 말~2026년 초"로 단정, 오늘 2026-08-19 기준 이미 지난 시점으로 서술하는 시점 모순까지 포함)가 가장 심각. E9·E15(세트 식별 혼동 — 현재/과거 세트 내용을 다음 세트인 것처럼 답변), E2(이미 공지된 정식 출시일을 "미공개"로 오답), H18(구버전 챔피언 목록을 "미검증 자료"로 자체 라벨링하며 사실상 지어냄)도 같은 계열. 답변 끝에 붙는 "출처 링크 일부가 실제 검색 결과에서 확인되지 않았습니다"라는 자동 경고(CHAT-18 근거검증 계열)는 URL 존재 여부만 사후검증할 뿐, 본문 내용(세트 번호·컨셉·시기 등) 자체가 근거 없이 생성됐다는 더 근본적인 문제는 걸러내지 못함 — SYSTEM_PROMPT_BASE 1번 원칙(문서에 없으면 추측 금지) 위반이 general_game_info(웹검색) 경로에서 본문 콘텐츠 레벨로 반복 발생.</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>CHAT-01,CHAT-17,CHAT-18</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>TEST-11 카테고리 H 결과 상세(docs/verification/TEST-11-작업결과.md), 카테고리 E 결과 상세(E2·E9·E15)</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>H15, E2, E9, E15, H18 재질의 시 미확정 정보를 구체적으로 단정하지 않고 정답지 채점기준(모른다고 정직하게 답변) 충족, 근거검증(CHAT-18)이 URL 존재 여부뿐 아니라 본문 핵심 주장(세트 번호·날짜 등 구체적 사실)이 실제 검색 결과에 등장하는지까지 확인하도록 확장</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>pytest — 위 5개 질문 대표 케이스 재현, "검색 결과에 없는 구체적 사실(세트 번호/날짜)을 본문에 포함하면 안 됨" 검증하는 사후 필터 단위 테스트, 검색 결과 fixture에 실제로 있는 사실은 정상적으로 답변에 포함되는지(과잉 차단 방지) 회귀 테스트</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>CHAT-31</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>챗봇RAG</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>챗봇위젯</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>증강체·전략 은어(슬랭)·줄임말 인식 확장</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>TEST-11 카테고리 H에서 발견 — "오구먼트"(증강체 줄임말, H13), "하이롤"·"각 잡다"(고성급 확률 성공/전략 준비를 뜻하는 커뮤니티 은어, H14)를 인식하지 못해 검색 자체가 실패하고 "확인되지 않았습니다"로 종료. CHAT-13(아이템 이름 근거검증 인식 개선)·CHAT-14(아이템 이름 줄임말 인식)가 아이템 영역에서 다뤘던 것과 같은 문제 유형이 증강체·전략 용어에도 존재함을 확인 — 아이템 전용으로 좁게 구현된 줄임말 정규화 로직을 증강체·전략 용어까지 확장하거나, 공통 슬랭 사전으로 일반화할 필요.</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>CHAT-13,CHAT-14</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>TEST-11 카테고리 H 결과 상세(docs/verification/TEST-11-작업결과.md), CHAT-13/CHAT-14 작업결과(기존 아이템 줄임말 처리 로직)</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>H13("티에프티 오구먼트가 뭐임?"), H14("롤체 하이롤 각 어캐 잡음?") 재질의 시 각각 증강체 설명, 하이롤 전략 관련 정상 답변(정답지 채점기준 충족), 기존 아이템 줄임말 인식(CHAT-13/14)에 회귀 없음</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>pytest — "오구먼트"→"증강체", "하이롤"→하이롤/고확률 관련 검색어 정규화 단위 테스트, 두 질문 재질의 스냅샷 테스트, 기존 아이템 줄임말 테스트 회귀 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>CHAT-32</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>챗봇RAG</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>챗봇위젯</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>다중 주제 복합질의 항목별 분해 응답</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>TEST-11 H12 발견 — "아이템 조합표랑 이번 패치노트랑 랭크 시스템 다 한 번에 알려줘"처럼 서로 다른 topic 3개를 한 질문에 요청하면, 실제 응답은 아이템 이름 나열(조합표 형태 아님) 1개 + 질문과 무관한 특정 조합("운명술사 트위스티드 페이트") 설명뿐이고 패치노트·랭크 시스템 항목은 통째로 누락됨. 다중 주제 질의를 항목별로 분해해 각각 답하는 로직이 없어 의도분류가 잡은 첫 항목(또는 우연히 매칭된 조합)만 답하고 나머지는 침묵하는 것으로 추정.</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>CHAT-01</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>TEST-11 카테고리 H 결과 상세(docs/verification/TEST-11-작업결과.md)</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>H12 재질의 시 요청된 3개 항목(아이템 조합표, 패치노트, 랭크 시스템)을 각각 구분해 빠짐없이 답변(정답지 채점기준 충족), 단일 주제 질문에는 회귀 없음</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>pytest — 다중 주제 질의 감지 로직 단위 테스트(2개 이상 topic 키워드 동시 포함 시), 항목별 분해 응답 조립 테스트, H12 재질의 스냅샷 테스트, 단일 주제 질문 기존 동작 회귀 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>CHAT-33</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>챗봇RAG</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>챗봇위젯</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>비한국어(영어) 질문 언어 대응</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>TEST-11 H17 발견 — "Can you explain the best comp in English?"처럼 영어로 질문해도 전부 한국어로만 답하고 "한국어 우선 지원"이라는 안내조차 없음(정답지는 영어 응답 또는 한국어 우선 지원 안내 중 하나를 기대). 현재 시스템 프롬프트·의도분류가 질문 언어를 전혀 감지하지 않는 것으로 추정. MVP 스코프(개인/지인 10명, 한국어 사용자 중심)상 완전한 다국어 지원보다 "한국어 우선 안내"만으로 충족 가능한지 착수 시 PM과 확정 필요(과잉 구현 방지).</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>CHAT-01</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>TEST-11 카테고리 H 결과 상세(docs/verification/TEST-11-작업결과.md)</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>H17 재질의 시 영어로 답변하거나 최소한 "한국어를 우선 지원한다"는 안내를 명시(정답지 채점기준 충족), 한국어 질문 응답 품질에 회귀 없음</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>pytest — 영어 질문 입력 시 언어 감지 로직 단위 테스트, H17 재질의 스냅샷 테스트, 한국어 질문 기존 동작 회귀 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>CHAT-34</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>챗봇RAG</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>챗봇위젯</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>목록형 답변 중도 절단(불완전 열거) 수정</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>TEST-11 D1 발견 — "TFT 랭크 티어는 몇 단계로 나뉘나요?"에 정답 10단계 중 4개(아이언·브론즈·실버·골드)만 나열하고 "몇 단계"라는 질문 자체엔 답하지 않은 채 "자세한 정보 확인 안됨"으로 마무리. 출처(namu.wiki)가 있었음에도 목록을 끝까지 읽지 않고 중도에 잘라낸 것으로 추정 — CHAT-24가 다뤘던 gpt-oss-120b 리즈닝 토큰 소비로 인한 응답 절단(max_tokens 부족)과 유사한 근본 원인일 가능성이 있어 우선 실측 필요.</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>CHAT-01,CHAT-24</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>TEST-11 카테고리 D 결과 상세(docs/verification/TEST-11-작업결과.md), CHAT-24 작업결과(gpt-oss-120b 리즈닝 토큰 회귀 사례)</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>착수 시 D1 재현 확인 후 원인 규명(max_tokens 부족/검색 결과 자체가 불완전/기타), 원인에 따라 수정하고 D1 재질의 시 10단계 전체 열거하며 "몇 단계"라는 질문에 직접 답변(정답지 채점기준 충족), 다른 목록형 답변에 회귀 없음</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>pytest — D1 재현·수정 확인 스냅샷 테스트, 목록형 질문(예: 다른 다단계 열거 질문) 회귀 테스트, max_tokens 원인이면 CHAT-24 방식대로 토큰 여유 실측 근거 기록</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>CHAT-35</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>챗봇RAG</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>챗봇위젯</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>답변 텍스트 한자 혼입 재현 확인 및 수정</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>TEST-11 B24 발견 — "금색은最高 등급을", "강度나 효율성" 등 답변 문장 중간에 한글이 아닌 한자가 섞여 나온 사례 1건 관찰(재현성 미확인). Groq/LLM 생성 결함 또는 소스 인코딩 문제로 추정.</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>CHAT-01</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>TEST-11 카테고리 B 결과 상세(docs/verification/TEST-11-작업결과.md)</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>착수 시 B24 및 유사 질문 반복 재질의로 재현 여부부터 확인 — 재현되면 원인(인코딩/생성 결함) 규명 후 수정, 재현 안 되면 관찰 종료로 문서화하고 TASK 종결(수정 불필요)</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>재현 시 pytest 회귀 테스트 신설(한자 혼입 방지 후처리 필터 등), 재현 안 되면 별도 자동화 테스트 불필요(관찰 종료 근거만 문서화)</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>CHAT-23</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>챗봇RAG</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>챗봇위젯</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Groq LLM 모델 마이그레이션(llama-3.3-70b-versatile 폐기 대응)</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Groq가 2026-06-17 공지, 2026-08-16 실제 폐기한 llama-3.3-70b-versatile 모델에 대응. PM이 Groq 폐기 공지를 제보해 긴급 신설. 대체 모델을 openai/gpt-oss-120b(프로덕션 등급, 무료 티어 TPD 200,000으로 기존 100,000 대비 2배)로 교체, 프리뷰 등급인 qwen/qwen3.6-27b는 비채택. 코드 변경은 backend/services/groq_client.py의 GROQ_MODEL 상수 한 곳뿐(모든 Groq 호출 경로가 공유).</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>필수</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>CHAT-01</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>Groq 공식 모델 폐기 공지(PM 제보, 2026-08-16), docs/verification/CHAT-23-작업결과.md</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>GROQ_MODEL을 openai/gpt-oss-120b로 교체 후 챗봇 전체 응답 경로(의도분류/오프토픽/본답변/후속질문)가 정상 동작, 기존 pytest 전체 통과, 프로덕션에서 실제 질의 확인</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>pytest 전체 회귀, 프로덕션 실제 질의 스모크 테스트(정상 응답 확인)</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>CHAT-24</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>챗봇RAG</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>챗봇위젯</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>gpt-oss-120b 리즈닝 토큰으로 인한 의도분류/오프토픽/후속질문 회귀 수정</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>CHAT-23 배포 후 TEST-11 재개 중 발견(2026-08-16 긴급 신설) — gpt-oss-120b는 리즈닝 모델이라 답변 전 별도 reasoning 토큰을 소비하는데, 기존 max_tokens=20(구모델 llama-3.3-70b-versatile 기준으로 설정된 값)이 reasoning만으로 소진돼 의도분류·오프토픽 판별 결과가 빈 문자열로 잘리는 회귀를 실측 확인. reasoning_effort="low"+max_tokens=100으로 수정.</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>필수</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>CHAT-23</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>docs/verification/CHAT-24-작업결과.md</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>의도분류/오프토픽 판별/후속질문 생성 등 짧은 응답을 기대하는 모든 Groq 호출 경로에서 reasoning 토큰 소진으로 인한 빈 응답 회귀가 재현되지 않음, 기존 pytest 전체 통과</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>pytest 전체 회귀, 의도분류·오프토픽 판별 대표 케이스 재실행 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>CHAT-25</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>코딩</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>챗봇RAG</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>챗봇위젯</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>경제·로우롤 전략 질문의 오프토픽 오탐 수정</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>TEST-11 카테고리 F 실행 중 발견(2026-08-17 신설) — "경제 운영", "그리핑" 같은 커뮤니티 용어가 1차 키워드 목록에 없어 2차 LLM 오프토픽 판별기가 잡담으로 오판. 키워드 목록 추가 + 2차 판별 프롬프트 보강으로 수정.</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>권장</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>CHAT-01,CHAT-16</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>TEST-11 카테고리 F 결과 상세(docs/verification/TEST-11-작업결과.md), docs/verification/CHAT-25-작업결과.md</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>"경제 운영", "그리핑" 등 커뮤니티 전략 용어를 포함한 질문이 더 이상 오프토픽으로 오분류되지 않음, 기존 오프토픽 판별 정상 케이스에 회귀 없음</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>pytest — 신규 키워드 포함 질문 분류 단위 테스트, 기존 오프토픽 판별 회귀 스위트 통과</t>
         </is>
       </c>
     </row>

</xml_diff>